<commit_message>
Modul PDV: prijava, periodi, podešavanja, export knjiga i kontrole
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -411,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -476,19 +476,19 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIF/KUF uvoz</v>
+        <v>KIF/KUF uvoz/export</v>
       </c>
       <c r="B7" t="str">
         <v>Core implementiran</v>
       </c>
       <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA.</v>
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
       </c>
       <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata.</v>
+        <v>Kontrole iznosa i duplikata; XML export.</v>
       </c>
       <c r="E7" t="str">
-        <v>QA uvoznih knjizenja.</v>
+        <v>QA uvoznih knjizenja i export fajlova.</v>
       </c>
     </row>
     <row r="8">
@@ -508,16 +508,33 @@
         <v>Azurirati uz svaku vecu promjenu.</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Prva implementacija</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z332"/>
+  <dimension ref="A1:Z336"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2743,16 +2760,132 @@
         <v>Dodati su MAPR/SEP import, KIF/KUF print, edit/delete neproknjiženih i automatsko knjiženje knjiga.</v>
       </c>
     </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>API-081</v>
+      </c>
+      <c r="B333" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C333" t="str">
+        <v>/api/racuni/export/kif</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Excel export KIF pregleda po aktivnoj firmi/godini i datumskom filteru.</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Računi / KIF-KUF</v>
+      </c>
+      <c r="F333" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G333" t="str">
+        <v>F-071</v>
+      </c>
+      <c r="H333" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="I333" t="str">
+        <v>Provjerava export pravo na modulu izlazni_racuni.</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>API-082</v>
+      </c>
+      <c r="B334" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C334" t="str">
+        <v>/api/racuni/export/kuf</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Excel export KUF pregleda po aktivnoj firmi/godini i datumskom filteru.</v>
+      </c>
+      <c r="E334" t="str">
+        <v>Računi / KIF-KUF</v>
+      </c>
+      <c r="F334" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G334" t="str">
+        <v>F-071</v>
+      </c>
+      <c r="H334" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="I334" t="str">
+        <v>Provjerava export pravo na modulu ulazni_racuni.</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>API-083</v>
+      </c>
+      <c r="B335" t="str">
+        <v>SERVER_ACTION</v>
+      </c>
+      <c r="C335" t="str">
+        <v>/agencija/pdv</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Kreiranje PDV perioda, osvježavanje prijave iz KIF/KUF, čuvanje korekcija, podešavanja i knjiženje.</v>
+      </c>
+      <c r="E335" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="F335" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G335" t="str">
+        <v>F-072,F-074,F-075</v>
+      </c>
+      <c r="H335" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="I335" t="str">
+        <v>Server actions u src/app/agencija/pdv/actions.ts.</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>API-084</v>
+      </c>
+      <c r="B336" t="str">
+        <v>GET</v>
+      </c>
+      <c r="C336" t="str">
+        <v>/api/pdv/xml</v>
+      </c>
+      <c r="D336" t="str">
+        <v>XML export PDV prijave za izabrani mjesec.</v>
+      </c>
+      <c r="E336" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="F336" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G336" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H336" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="I336" t="str">
+        <v>MVP XML snapshot redova prijave; finalno IRMS mapiranje ostaje.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z332"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z336"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z331"/>
+  <dimension ref="A1:AB333"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4211,9 +4344,73 @@
         <v>Treba doraditi širinu/kolone i provjeriti PDF/štampu na više redova.</v>
       </c>
     </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>T-062</v>
+      </c>
+      <c r="B332" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C332" t="str">
+        <v>PDV period po datumu knjige</v>
+      </c>
+      <c r="D332" t="str">
+        <v>KIF koristi kif_date a KUF kuf_date za izbor mjeseca PDV prijave.</v>
+      </c>
+      <c r="E332" t="str">
+        <v>F-072,F-073</v>
+      </c>
+      <c r="F332" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="G332" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="H332">
+        <v>46201.083333333336</v>
+      </c>
+      <c r="I332" t="str">
+        <v>Provjereno TypeScript i migracija; potreban ručni test na primjeru majskog računa u junskom KUF-u.</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>T-063</v>
+      </c>
+      <c r="B333" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C333" t="str">
+        <v>PDV prijava i knjiženje</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Prijava se osvježi iz KIF/KUF i može se proknjižiti na podešenu vrstu naloga/konta.</v>
+      </c>
+      <c r="E333" t="str">
+        <v>F-074,F-075</v>
+      </c>
+      <c r="F333" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="G333" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="H333">
+        <v>46201.083333333336</v>
+      </c>
+      <c r="I333" t="str">
+        <v>Provjereno TypeScript; PDV podešavanja sada prikazuju cijeli kontni plan</v>
+      </c>
+      <c r="J333" t="str">
+        <v xml:space="preserve"> kontrole porede PDV evidenciju sa glavnom knjigom</v>
+      </c>
+      <c r="K333" t="str">
+        <v xml:space="preserve"> a brisanje PDV naloga vraća prijavu u nacrt. Potreban ručni test sa stvarnim kontima 2700/4700 i nalogom.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z331"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB333"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6253,7 +6450,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="E11" t="str">
-        <v>Djelimično kroz KIF/KUF</v>
+        <v>Implementirano djelimicno</v>
       </c>
       <c r="F11" t="str">
         <v>Računovođa</v>
@@ -6262,7 +6459,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H11" t="str">
-        <v>PDV stope i osnovne KIF/KUF PDV razrade postoje. PDV prijava, kontrole i XML nisu implementirani.</v>
+        <v>PDV stope, mjesečni periodi, ulazni/izlazni PDV evidencije, nacrt PDV prijave, korekcije, podešavanja knjiženja, XML snapshot i osnovno knjiženje su implementirani. Ostaju finalno IRMS XML mapiranje, zaključavanje perioda i jači QA.</v>
       </c>
     </row>
     <row r="12">
@@ -6340,7 +6537,7 @@
         <v>MVP 1</v>
       </c>
       <c r="H301" t="str">
-        <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa i print su implementirani. Ostaju kontrole, export, PDV zaključavanje i QA.</v>
+        <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa, print i Excel export su implementirani. Ostaju kontrole, XML export, PDV zaključavanje i QA.</v>
       </c>
     </row>
   </sheetData>
@@ -6352,7 +6549,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z332"/>
+  <dimension ref="A1:Z337"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -8793,7 +8990,7 @@
         <v>F-062</v>
       </c>
       <c r="L325" t="str">
-        <v>KIF/KUF imaju mjesečne knjige, vrste, unos računa, PDV razradu, MAPR/SEP import, seme kontiranja, automatsko knjiženje, edit/delete za neproknjižene i print. Ostaju kontrole/export/lock/testovi.</v>
+        <v>KIF/KUF imaju mjesečne knjige, vrste, unos računa, PDV razradu, MAPR/SEP import, seme kontiranja, automatsko knjiženje, edit/delete neproknjiženih, print i Excel export. Ostaju kontrole/XML/lock/testovi.</v>
       </c>
     </row>
     <row r="326">
@@ -8869,7 +9066,7 @@
         <v>F-063</v>
       </c>
       <c r="L327" t="str">
-        <v>Šema čuva pravila za ukupno, osnovice, PDV po stopama i oslobođeni promet.</v>
+        <v>Šema čuva pravila za ukupno, osnovice, PDV po stopama i oslobođeni promet. Pravila su odvojena po vrsti knjige; UI remount-uje redove po vrsti da se KIF/KUF šeme ne prelivaju.</v>
       </c>
     </row>
     <row r="328">
@@ -9062,9 +9259,199 @@
         <v>Za proknjižene račune ostaje definisati stroga pravila korekcije/storna.</v>
       </c>
     </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>F-071</v>
+      </c>
+      <c r="B333" t="str">
+        <v>Računi / KIF-KUF</v>
+      </c>
+      <c r="C333" t="str">
+        <v>Excel export KIF/KUF pregleda</v>
+      </c>
+      <c r="D333" t="str">
+        <v>KIF/KUF pregledi se izvoze u XLSX po aktivnoj firmi, poslovnoj godini i filteru datuma knjige.</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F333" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G333" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H333" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I333" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J333" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="K333" t="str">
+        <v>F-063</v>
+      </c>
+      <c r="L333" t="str">
+        <v>Export uključuje partnera, tip prometa, iznose, status knjiženja i PDV razradu; backend provjerava export pravo.</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>F-072</v>
+      </c>
+      <c r="B334" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C334" t="str">
+        <v>PDV periodi po mjesecu</v>
+      </c>
+      <c r="D334" t="str">
+        <v>PDV periodi se vode za aktivnu firmu i poslovnu godinu; na PDV ekranima bira se samo mjesec.</v>
+      </c>
+      <c r="E334" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F334" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G334" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H334" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I334" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J334" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="K334" t="str">
+        <v>F-063</v>
+      </c>
+      <c r="L334" t="str">
+        <v>Period KIF/KUF računa određuje datum knjige: kif_date odnosno kuf_date.</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>F-073</v>
+      </c>
+      <c r="B335" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C335" t="str">
+        <v>Ulazni i izlazni PDV evidencije</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Ulazni PDV prikazuje KUF račune, a izlazni PDV KIF račune koji ulaze u izabrani mjesec.</v>
+      </c>
+      <c r="E335" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F335" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G335" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H335" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I335" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J335" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="K335" t="str">
+        <v>F-063,F-072</v>
+      </c>
+      <c r="L335" t="str">
+        <v>Evidencije su dokazni pregled iza prijave i linkuju na KIF/KUF knjige.</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="B336" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C336" t="str">
+        <v>PDV prijava po IRMS obrascu</v>
+      </c>
+      <c r="D336" t="str">
+        <v>Prijava se automatski puni iz KIF/KUF, ima redove obrasca i automatske preračune PDV-a i zbirnih redova.</v>
+      </c>
+      <c r="E336" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F336" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G336" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H336" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I336" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J336" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="K336" t="str">
+        <v>F-072,F-073</v>
+      </c>
+      <c r="L336" t="str">
+        <v>Dodat nacrt prijave, osvježavanje iz KIF/KUF, portal layout, XML export i osnovno zbirno knjiženje; brisanje PDV naloga vraća prijavu u nacrt. Ostaje finalno mapiranje IRMS XML-a i zaključavanje.</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>F-075</v>
+      </c>
+      <c r="B337" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C337" t="str">
+        <v>Podešavanja knjiženja PDV prijave</v>
+      </c>
+      <c r="D337" t="str">
+        <v>Firma za aktivnu godinu bira vrstu naloga i šemu D/P + konto za zatvaranje kartica PDV-a.</v>
+      </c>
+      <c r="E337" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F337" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G337" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H337" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I337" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J337" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="K337" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="L337" t="str">
+        <v>Pravila se generišu po aktivnim PDV stopama iz baze za ulazni/izlazni PDV, plus carinski, paušalni, obaveza i kredit. Dropdown konta prikazuje cijeli spojeni kontni plan; izbor globalnog konta se pri čuvanju veže kao firmi konto. Kontrole porede PDV evidenciju sa glavnom knjigom.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z332"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z337"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -12615,7 +13002,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z318"/>
+  <dimension ref="A1:Z325"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -13498,16 +13885,198 @@
         <v>/agencija/racuni/podesavanja, /agencija/racuni/kuf, /agencija/racuni/kuf/[id], /agencija/racuni/kif/[id], /agencija/racuni/neproknjizeno, /agencija/racuni/pregled-kuf i /agencija/racuni/pregled-kuf/[id]. Dodato knjiženje/dopuna naloga po knjizi.</v>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>E-035</v>
+      </c>
+      <c r="B319" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C319" t="str">
+        <v>PDV pregled</v>
+      </c>
+      <c r="D319" t="str">
+        <v>Lista mjesečnih PDV perioda za aktivnu firmu/godinu sa statusom i zbirnim iznosima.</v>
+      </c>
+      <c r="E319" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F319" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G319" t="str">
+        <v>F-072</v>
+      </c>
+      <c r="H319" t="str">
+        <v>/agencija/pdv</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>E-036</v>
+      </c>
+      <c r="B320" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C320" t="str">
+        <v>Ulazni PDV</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Dokazna evidencija KUF računa za izabrani mjesec po datumu KUF knjige.</v>
+      </c>
+      <c r="E320" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F320" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G320" t="str">
+        <v>F-073</v>
+      </c>
+      <c r="H320" t="str">
+        <v>/agencija/pdv/ulazni</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>E-037</v>
+      </c>
+      <c r="B321" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C321" t="str">
+        <v>Izlazni PDV</v>
+      </c>
+      <c r="D321" t="str">
+        <v>Dokazna evidencija KIF računa za izabrani mjesec po datumu KIF knjige.</v>
+      </c>
+      <c r="E321" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F321" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G321" t="str">
+        <v>F-073</v>
+      </c>
+      <c r="H321" t="str">
+        <v>/agencija/pdv/izlazni</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>E-038</v>
+      </c>
+      <c r="B322" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C322" t="str">
+        <v>PDV prijava</v>
+      </c>
+      <c r="D322" t="str">
+        <v>IRMS-like obrazac prijave sa lijevom/desnom PDV kolonom i automatskim preračunima.</v>
+      </c>
+      <c r="E322" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F322" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G322" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H322" t="str">
+        <v>/agencija/pdv/prijava</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>E-039</v>
+      </c>
+      <c r="B323" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C323" t="str">
+        <v>PDV kontrole</v>
+      </c>
+      <c r="D323" t="str">
+        <v>Kontrole prije XML izvoza i knjiženja prijave; uključuje neproknjižene/rasknjižene KIF/KUF stavke i poređenje sa glavnom knjigom.</v>
+      </c>
+      <c r="E323" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F323" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G323" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H323" t="str">
+        <v>/agencija/pdv/kontrole</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>E-040</v>
+      </c>
+      <c r="B324" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C324" t="str">
+        <v>Arhiva PDV prijava</v>
+      </c>
+      <c r="D324" t="str">
+        <v>Lista sačuvanih/proknjiženih prijava i linkovi na XML/nalog.</v>
+      </c>
+      <c r="E324" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F324" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G324" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H324" t="str">
+        <v>/agencija/pdv/arhiva</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>E-041</v>
+      </c>
+      <c r="B325" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C325" t="str">
+        <v>Podešavanja PDV-a</v>
+      </c>
+      <c r="D325" t="str">
+        <v>Vrsta naloga i šema D/P + konto za knjiženje PDV prijave po aktivnim stopama; konto dropdown prikazuje cijeli spojeni kontni plan.</v>
+      </c>
+      <c r="E325" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F325" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G325" t="str">
+        <v>F-075</v>
+      </c>
+      <c r="H325" t="str">
+        <v>/agencija/pdv/podesavanja</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z318"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z325"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z328"/>
+  <dimension ref="A1:Z333"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -14776,9 +15345,139 @@
         <v>Osnovni unos KIF računa je povezan sa šemom kontiranja.</v>
       </c>
     </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>DB-054</v>
+      </c>
+      <c r="B329" t="str">
+        <v>pdv_periodi</v>
+      </c>
+      <c r="C329" t="str">
+        <v>PDV periodi po mjesecu aktivne firme/godine.</v>
+      </c>
+      <c r="D329" t="str">
+        <v>agencija_id, firma_id, poslovna_godina_id, mjesec, datum_od, datum_do, status</v>
+      </c>
+      <c r="E329" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="F329" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G329" t="str">
+        <v>F-072</v>
+      </c>
+      <c r="H329" t="str">
+        <v>Migracija 20260628150000_pdv_periodi_prijave_podesavanja.</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>DB-055</v>
+      </c>
+      <c r="B330" t="str">
+        <v>pdv_prijave</v>
+      </c>
+      <c r="C330" t="str">
+        <v>PDV prijava za period.</v>
+      </c>
+      <c r="D330" t="str">
+        <v>pdv_period_id, totals, status, journal_id, xml_generated_at</v>
+      </c>
+      <c r="E330" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="F330" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G330" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H330" t="str">
+        <v>Jedna prijava po periodu; pamti zbirne iznose i nalog knjiženja.</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>DB-056</v>
+      </c>
+      <c r="B331" t="str">
+        <v>pdv_prijava_stavke</v>
+      </c>
+      <c r="C331" t="str">
+        <v>Redovi PDV prijave.</v>
+      </c>
+      <c r="D331" t="str">
+        <v>pdv_prijava_id, sifra, opis, kolona, sistemska_vrijednost, rucna_vrijednost, razlog_korekcije</v>
+      </c>
+      <c r="E331" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="F331" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G331" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H331" t="str">
+        <v>Čuva sistemsku i ručnu vrijednost po redu obrasca.</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>DB-057</v>
+      </c>
+      <c r="B332" t="str">
+        <v>pdv_podesavanja</v>
+      </c>
+      <c r="C332" t="str">
+        <v>Podešavanja knjiženja PDV prijave.</v>
+      </c>
+      <c r="D332" t="str">
+        <v>vrsta_naloga_id, izlazni/ulazni/obaveza/kredit/neodbitni konta i smjerovi D/P</v>
+      </c>
+      <c r="E332" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="F332" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G332" t="str">
+        <v>F-075</v>
+      </c>
+      <c r="H332" t="str">
+        <v>Jedan zapis po firmi i poslovnoj godini; migracija 20260628162000 dodaje smjerove.</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>DB-058</v>
+      </c>
+      <c r="B333" t="str">
+        <v>pdv_podesavanja_pravila</v>
+      </c>
+      <c r="C333" t="str">
+        <v>Pravila knjiženja PDV prijave po poljima.</v>
+      </c>
+      <c r="D333" t="str">
+        <v>pdv_podesavanja_id, polje_sifra, polje_naziv, pdv_stopa_sifra, smjer, konto_id</v>
+      </c>
+      <c r="E333" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="F333" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G333" t="str">
+        <v>F-075</v>
+      </c>
+      <c r="H333" t="str">
+        <v>Pravila po aktivnim PDV stopama iz baze i posebna pravila za carinski/paušalni/obaveza/kredit.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z328"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z333"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement bank statements workflow
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,22 +3,23 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-06-29" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-06-28" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-06-25" sheetId="3" r:id="rId3"/>
-    <sheet name="Dashboard" sheetId="4" r:id="rId4"/>
-    <sheet name="Moduli" sheetId="5" r:id="rId5"/>
-    <sheet name="Funkcionalnosti" sheetId="6" r:id="rId6"/>
-    <sheet name="Pravila" sheetId="7" r:id="rId7"/>
-    <sheet name="Zavisnosti" sheetId="8" r:id="rId8"/>
-    <sheet name="Ekrani" sheetId="9" r:id="rId9"/>
-    <sheet name="Baza" sheetId="10" r:id="rId10"/>
-    <sheet name="API" sheetId="11" r:id="rId11"/>
-    <sheet name="Testovi" sheetId="12" r:id="rId12"/>
-    <sheet name="Bugovi" sheetId="13" r:id="rId13"/>
-    <sheet name="Ideje" sheetId="14" r:id="rId14"/>
-    <sheet name="Odluke" sheetId="15" r:id="rId15"/>
-    <sheet name="Kategorije" sheetId="16" r:id="rId16"/>
+    <sheet name="Status 2026-06-30" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-06-29" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-06-28" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-06-25" sheetId="4" r:id="rId4"/>
+    <sheet name="Dashboard" sheetId="5" r:id="rId5"/>
+    <sheet name="Moduli" sheetId="6" r:id="rId6"/>
+    <sheet name="Funkcionalnosti" sheetId="7" r:id="rId7"/>
+    <sheet name="Pravila" sheetId="8" r:id="rId8"/>
+    <sheet name="Zavisnosti" sheetId="9" r:id="rId9"/>
+    <sheet name="Ekrani" sheetId="10" r:id="rId10"/>
+    <sheet name="Baza" sheetId="11" r:id="rId11"/>
+    <sheet name="API" sheetId="12" r:id="rId12"/>
+    <sheet name="Testovi" sheetId="13" r:id="rId13"/>
+    <sheet name="Bugovi" sheetId="14" r:id="rId14"/>
+    <sheet name="Ideje" sheetId="15" r:id="rId15"/>
+    <sheet name="Odluke" sheetId="16" r:id="rId16"/>
+    <sheet name="Kategorije" sheetId="17" r:id="rId17"/>
   </sheets>
 </workbook>
 </file>
@@ -412,11 +413,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-29</v>
+        <v>Status projekta na dan 2026-06-30</v>
       </c>
     </row>
     <row r="2">
@@ -443,98 +444,1285 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nalozi</v>
+        <v>Izvodi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core zaokruzen</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
+        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
       </c>
       <c r="D5" t="str">
-        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
       </c>
       <c r="E5" t="str">
-        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
+        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PDV</v>
+        <v>Nalozi</v>
       </c>
       <c r="B6" t="str">
-        <v>Core zaokruzen</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C6" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
       </c>
       <c r="D6" t="str">
-        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
+        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E6" t="str">
-        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
+        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Izvodi</v>
+        <v>PDV</v>
       </c>
       <c r="B7" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C7" t="str">
-        <v>Procitana finalna specifikacija 07_Izvodi_i_Automatsko_Knjizenje_FINAL.md; docs i planer azurirani. pdfjs-dist je ranije instaliran.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D7" t="str">
-        <v>Implementacija tabela, upload PDF/HTML, parser, preview, prepoznavanje po ziro racunu, alokacije na KIF/KUF, pravila i knjiženje.</v>
+        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
       </c>
       <c r="E7" t="str">
-        <v>Krenuti od migracija/modela i import/preview toka, ne od posebnog rucnog izvoda.</v>
+        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>KIF/KUF</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B8" t="str">
-        <v>Core implementiran</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C8" t="str">
-        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
+        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
       </c>
       <c r="D8" t="str">
-        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
+        <v>Redovno održavanje.</v>
       </c>
       <c r="E8" t="str">
-        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C9" t="str">
-        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Regenerisati Excel nakon svake vece promjene.</v>
+        <v>Regenerisati Excel nakon svake veće promjene.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Z330"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Ekrani aplikacije</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Plan UI ekrana za prva 3 zaključena modula.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ID ekrana</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Naziv ekrana</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Opis</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Prioritet</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Povezane funkcije</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>UI-001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Super admin — Agencije</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Pregled agencija, pretplata, statusa aktivacije i isteka.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G5" t="str">
+        <v>F-001,F-003,F-004</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Pregled agencija postoji; pretplate nisu kompletno UI zaokruzene.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>UI-002</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Agencijski admin — Radnici</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Kreiranje radnika i dodjela prava.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G6" t="str">
+        <v>F-005,F-008</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Kreiranje radnika i dodjela prava postoje.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>UI-003</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Agencijski admin — Prava pristupa</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Matrica prava po firmama, modulima i akcijama.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G7" t="str">
+        <v>F-007,F-008</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Matrica prava postoji; enforcement prava treba dodatno zakljucati.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>UI-004</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Učinak radnika</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Dnevni/nedjeljni/mjesečni pregled aktivnosti po radniku.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F8" t="str">
+        <v>U izradi</v>
+      </c>
+      <c r="G8" t="str">
+        <v>F-009,F-010</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Postoji audit/aktivnost osnova; puni ekran ucinka jos nije implementiran.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>UI-005</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Firme i kontni plan</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Lista firmi</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Naziv, PIB, tip, PDV status, godina, glavni radnik, status.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G9" t="str">
+        <v>F-012,F-014,F-019</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Lista firmi postoji kao /agencija/firme.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>UI-006</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Firme i kontni plan</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Dodavanje firme</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Unos PIB-a, IRMS pretraga, provjera podataka i snimanje.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G10" t="str">
+        <v>F-012,F-013</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Dodavanje firme sa IRMS pretragom postoji kao /agencija/firme/nova.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>UI-007</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Firme i kontni plan</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Profil firme</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Tabovi: podaci, lica, banke, godine, podešavanja, radnici, klijenti, ugovor, kontni plan.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G11" t="str">
+        <v>F-012-F-023</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Detalj firme sada prikazuje osnovne podatke, godine, bankovne racune, ugovor/cijenu i korisnike; odgovorna lica, kontni plan i podesavanja jos nisu kompletirani.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>UI-008</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Firme i kontni plan</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Poslovne godine</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Otvaranje, zaključavanje, otključavanje i arhiva godina.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G12" t="str">
+        <v>F-014,F-015</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Centralna stranica poslovnih godina postoji.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>UI-009</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Firme i kontni plan</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Kontni plan firme</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Kombinovani prikaz osnovnog plana i firmi specifičnih izmjena.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G13" t="str">
+        <v>F-021,F-022,F-023</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Postoje dva ekrana: globalni osnovni kontni plan u podesavanjima i kontni plan firme za specificne izmjene i default konta. Kontni plan firme ima pretragu po sifri/nazivu direktno iznad tabele.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>UI-010</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Lista naloga</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Pregled naloga po firmi, godini, vrsti, broju, statusu, korisniku.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G14" t="str">
+        <v>F-024-F-031</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Lista naloga po aktivnoj firmi/godini postoji na /agencija/nalozi, sa filterom statusa.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>UI-011</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Unos naloga</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Zaglavlje + tabelarni unos stavki.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G15" t="str">
+        <v>F-026,F-027,F-029</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Unos novog naloga postoji na /agencija/nalozi/novi; izmjena nacrta ostaje za naredni korak.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>UI-012</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Nacrti naloga</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Lista nacrta koji nijesu proknjiženi.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G16" t="str">
+        <v>F-028</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Nacrti su dostupni preko /agencija/nalozi/nacrti odnosno status filtera.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>UI-013</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Početno stanje</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Pregled/generisanje/proknjižavanje početnog stanja.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Nije poceto</v>
+      </c>
+      <c r="G17" t="str">
+        <v>F-034,F-035</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Početno stanje jos nije posebna funkcionalnost.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>UI-014</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Partneri</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Lista partnera, kupac/dobavljač oznake, PIB, kontakt podaci.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G18" t="str">
+        <v>F-036</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Agencijski ekran za dodatne partnere i admin ekran za globalne partnere podrzavaju unos, IRMS pretragu i izmjenu.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>UI-015</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Bruto bilans</v>
+      </c>
+      <c r="D19" t="str">
+        <v>PS, promet, ukupno, saldo; filter po firmi, godini, poslovnoj jedinici.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Nije poceto</v>
+      </c>
+      <c r="G19" t="str">
+        <v>F-038</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Bruto bilans jos nije implementiran.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>UI-016</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Kartica partnera</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Detaljna kartica i zbirni saldo kupaca/dobavljača.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G20" t="str">
+        <v>F-037</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Analiticka kartica je implementirana u /agencija/nalozi/analiticke-kartice; zbir kupaca/dobavljaca po partneru u /agencija/nalozi/kupci-dobavljaci. Ostaju stampa/export.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>UI-017</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Uvoz izvoda</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Upload PDF/HTML/XML izvoda za aktivnu firmu/godinu i bankovni račun firme.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="G21" t="str">
+        <v>F-076</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, XML/tekst fajla i paste teksta; NLB XML radi, ostale banke ostaju otvorene.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>UI-018</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Preview parsiranja</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Pregled zaglavlja, parsiranih stavki, grešaka i kontrole početnog/krajnjeg stanja.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="G22" t="str">
+        <v>F-078</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Postoji tab Stavke izvoda sa kontrolom stanja; edit parsiranih iznosa/datuma ostaje otvoren.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>UI-019</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Povezivanje i obrada stavki</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Tabela stavki sa komitentom, fakturom, predlogom knjiženja, confidence score-om i akcijama.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="G23" t="str">
+        <v>F-079,F-080,F-081,F-083</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Postoji izbor partnera i konta, ignorisanje stavki i posebna stranica Obrada stavki; fakture, učenje računa i trajna pravila ostaju otvoreni.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>UI-020</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Preview naloga izvoda</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Prije knjiženja prikazuje stavke naloga duguje/potražuje, konto, partner, opis i iznos.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="G24" t="str">
+        <v>F-084</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Postoji tab Predlog naloga; banka se knjiži zbirno po ukupnom prilivu/odlivu, a stavke idu na kontra konta; knjiženje READY izvoda u IZV nalog postoji.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>UI-021</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Kartica banke</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Pregled prometa bankovnog računa iz proknjiženih izvoda/naloga.</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="G25" t="str">
+        <v>F-084</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Dodata stranica Kartica banke sa filterom bankovnog računa i pregledom uvezenih izvoda, priliva, odliva i naloga.</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>E-017</v>
+      </c>
+      <c r="B306" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C306" t="str">
+        <v>Artikli</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Lista i unos artikala/usluga.</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F306" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G306" t="str">
+        <v>F-039</v>
+      </c>
+      <c r="H306" t="str">
+        <v>Checkbox usluga.</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>E-018</v>
+      </c>
+      <c r="B307" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C307" t="str">
+        <v>Grupe artikala</v>
+      </c>
+      <c r="D307" t="str">
+        <v>Šifarnik grupa artikala.</v>
+      </c>
+      <c r="E307" t="str">
+        <v>Srednji</v>
+      </c>
+      <c r="F307" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G307" t="str">
+        <v>F-039</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>E-019</v>
+      </c>
+      <c r="B308" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C308" t="str">
+        <v>Cijene artikala</v>
+      </c>
+      <c r="D308" t="str">
+        <v>Upravljanje više cijena artikla.</v>
+      </c>
+      <c r="E308" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F308" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G308" t="str">
+        <v>F-040</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>E-020</v>
+      </c>
+      <c r="B309" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C309" t="str">
+        <v>Magacini</v>
+      </c>
+      <c r="D309" t="str">
+        <v>Lista i podešavanje magacina.</v>
+      </c>
+      <c r="E309" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F309" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G309" t="str">
+        <v>F-041</v>
+      </c>
+      <c r="H309" t="str">
+        <v>Negativan lager opciono po magacinu.</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>E-021</v>
+      </c>
+      <c r="B310" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C310" t="str">
+        <v>Lager lista</v>
+      </c>
+      <c r="D310" t="str">
+        <v>Stanje robe po magacinu.</v>
+      </c>
+      <c r="E310" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F310" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G310" t="str">
+        <v>F-042,F-060</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>E-022</v>
+      </c>
+      <c r="B311" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C311" t="str">
+        <v>Kartica artikla</v>
+      </c>
+      <c r="D311" t="str">
+        <v>Ulazi, izlazi i saldo artikla.</v>
+      </c>
+      <c r="E311" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F311" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G311" t="str">
+        <v>F-060</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>E-023</v>
+      </c>
+      <c r="B312" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C312" t="str">
+        <v>Kalkulacije</v>
+      </c>
+      <c r="D312" t="str">
+        <v>Unos i knjiženje kalkulacija.</v>
+      </c>
+      <c r="E312" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F312" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G312" t="str">
+        <v>F-045</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>E-024</v>
+      </c>
+      <c r="B313" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C313" t="str">
+        <v>Uvozna kalkulacija</v>
+      </c>
+      <c r="D313" t="str">
+        <v>Kalkulacija sa carinskom deklaracijom.</v>
+      </c>
+      <c r="E313" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F313" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G313" t="str">
+        <v>F-051</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>E-025</v>
+      </c>
+      <c r="B314" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C314" t="str">
+        <v>Povrat dobavljaču</v>
+      </c>
+      <c r="D314" t="str">
+        <v>Slobodan ili povezan povrat robe dobavljaču.</v>
+      </c>
+      <c r="E314" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F314" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G314" t="str">
+        <v>F-052</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>E-026</v>
+      </c>
+      <c r="B315" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C315" t="str">
+        <v>Prenos robe</v>
+      </c>
+      <c r="D315" t="str">
+        <v>Prenos između magacina.</v>
+      </c>
+      <c r="E315" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F315" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G315" t="str">
+        <v>F-054</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>E-027</v>
+      </c>
+      <c r="B316" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C316" t="str">
+        <v>Popis robe</v>
+      </c>
+      <c r="D316" t="str">
+        <v>Unos stvarnog stanja, višak i manjak.</v>
+      </c>
+      <c r="E316" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F316" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G316" t="str">
+        <v>F-055</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>E-028</v>
+      </c>
+      <c r="B317" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C317" t="str">
+        <v>Otpis robe</v>
+      </c>
+      <c r="D317" t="str">
+        <v>Otpis i razduženje robe.</v>
+      </c>
+      <c r="E317" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F317" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G317" t="str">
+        <v>F-058</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>E-029</v>
+      </c>
+      <c r="B318" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C318" t="str">
+        <v>Nivelacija</v>
+      </c>
+      <c r="D318" t="str">
+        <v>Promjena maloprodajnih cijena.</v>
+      </c>
+      <c r="E318" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F318" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G318" t="str">
+        <v>F-059</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>E-030</v>
+      </c>
+      <c r="B319" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C319" t="str">
+        <v>Robni izvještaji</v>
+      </c>
+      <c r="D319" t="str">
+        <v>Vrijednost zaliha, lager i pregledi po magacinima.</v>
+      </c>
+      <c r="E319" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F319" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G319" t="str">
+        <v>F-060</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>E-031</v>
+      </c>
+      <c r="B320" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C320" t="str">
+        <v>Podešavanje negativnog lagera</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Blokiranje ili dozvola zaliha u minus.</v>
+      </c>
+      <c r="E320" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F320" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G320" t="str">
+        <v>F-043</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>E-032</v>
+      </c>
+      <c r="B321" t="str">
+        <v>Izlazne fakture</v>
+      </c>
+      <c r="C321" t="str">
+        <v>Izlazne fakture bez fiskalizacije</v>
+      </c>
+      <c r="D321" t="str">
+        <v>Ekran za kreiranje faktura koje mogu razdužiti magacin i kasnije se automatski knjižiti.</v>
+      </c>
+      <c r="E321" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F321" t="str">
+        <v>Za razradu</v>
+      </c>
+      <c r="G321" t="str">
+        <v>M-005</v>
+      </c>
+      <c r="H321" t="str">
+        <v>Fiskalizacija nije dio prve verzije.</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>E-033</v>
+      </c>
+      <c r="B322" t="str">
+        <v>Podešavanja / PDV</v>
+      </c>
+      <c r="C322" t="str">
+        <v>PDV stope</v>
+      </c>
+      <c r="D322" t="str">
+        <v>Ekran za unos, pregled, izmjenu i aktivaciju/deaktivaciju PDV stopa.</v>
+      </c>
+      <c r="E322" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F322" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G322" t="str">
+        <v>F-062</v>
+      </c>
+      <c r="H322" t="str">
+        <v>/agencija/podesavanja/pdv-stope</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>E-034</v>
+      </c>
+      <c r="B323" t="str">
+        <v>Računi / KUF</v>
+      </c>
+      <c r="C323" t="str">
+        <v>KUF knjige i detalj KUF-a</v>
+      </c>
+      <c r="D323" t="str">
+        <v>Računi / Podešavanja prikazuju vrste KIF/KUF i šemu kontiranja po poljima. KUF i KIF imaju otvaranje knjige i unos računa; KIF konto prihoda zavisi od šeme.</v>
+      </c>
+      <c r="E323" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F323" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G323" t="str">
+        <v>F-063</v>
+      </c>
+      <c r="H323" t="str">
+        <v>/agencija/racuni/podesavanja, /agencija/racuni/kuf, /agencija/racuni/kuf/[id], /agencija/racuni/kif/[id], /agencija/racuni/neproknjizeno, /agencija/racuni/pregled-kuf i /agencija/racuni/pregled-kuf/[id]. Dodato knjiženje/dopuna naloga po knjizi i uvoz podešavanja iz druge firme.</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>E-035</v>
+      </c>
+      <c r="B324" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C324" t="str">
+        <v>PDV pregled</v>
+      </c>
+      <c r="D324" t="str">
+        <v>Lista mjesečnih PDV perioda za aktivnu firmu/godinu sa statusom i zbirnim iznosima.</v>
+      </c>
+      <c r="E324" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F324" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G324" t="str">
+        <v>F-072</v>
+      </c>
+      <c r="H324" t="str">
+        <v>/agencija/pdv</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>E-036</v>
+      </c>
+      <c r="B325" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C325" t="str">
+        <v>Ulazni PDV</v>
+      </c>
+      <c r="D325" t="str">
+        <v>Dokazna evidencija KUF računa za izabrani mjesec po datumu KUF knjige.</v>
+      </c>
+      <c r="E325" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F325" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G325" t="str">
+        <v>F-073</v>
+      </c>
+      <c r="H325" t="str">
+        <v>/agencija/pdv/ulazni</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>E-037</v>
+      </c>
+      <c r="B326" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C326" t="str">
+        <v>Izlazni PDV</v>
+      </c>
+      <c r="D326" t="str">
+        <v>Dokazna evidencija KIF računa za izabrani mjesec po datumu KIF knjige.</v>
+      </c>
+      <c r="E326" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F326" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G326" t="str">
+        <v>F-073</v>
+      </c>
+      <c r="H326" t="str">
+        <v>/agencija/pdv/izlazni</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>E-038</v>
+      </c>
+      <c r="B327" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C327" t="str">
+        <v>PDV prijava</v>
+      </c>
+      <c r="D327" t="str">
+        <v>IRMS-like obrazac prijave sa lijevom/desnom PDV kolonom i automatskim preračunima.</v>
+      </c>
+      <c r="E327" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F327" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G327" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H327" t="str">
+        <v>/agencija/pdv/prijava</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>E-039</v>
+      </c>
+      <c r="B328" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C328" t="str">
+        <v>PDV kontrole</v>
+      </c>
+      <c r="D328" t="str">
+        <v>Kontrole prije XML izvoza i knjiženja prijave; uključuje neproknjižene/rasknjižene KIF/KUF stavke i poređenje sa glavnom knjigom.</v>
+      </c>
+      <c r="E328" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F328" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="G328" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H328" t="str">
+        <v>/agencija/pdv/kontrole</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>E-040</v>
+      </c>
+      <c r="B329" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C329" t="str">
+        <v>Arhiva PDV prijava</v>
+      </c>
+      <c r="D329" t="str">
+        <v>Lista sačuvanih/proknjiženih prijava i linkovi na XML/nalog.</v>
+      </c>
+      <c r="E329" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F329" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G329" t="str">
+        <v>F-074</v>
+      </c>
+      <c r="H329" t="str">
+        <v>/agencija/pdv/arhiva</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>E-041</v>
+      </c>
+      <c r="B330" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C330" t="str">
+        <v>Podešavanja PDV-a</v>
+      </c>
+      <c r="D330" t="str">
+        <v>Vrsta naloga i šema D/P + konto za knjiženje PDV prijave po aktivnim stopama; konto dropdown prikazuje cijeli spojeni kontni plan.</v>
+      </c>
+      <c r="E330" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F330" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G330" t="str">
+        <v>F-075</v>
+      </c>
+      <c r="H330" t="str">
+        <v>/agencija/pdv/podesavanja</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z330"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z341"/>
   <sheetData>
     <row r="1">
@@ -2003,13 +3191,13 @@
         <v>Izvodi</v>
       </c>
       <c r="F336" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Implementirano</v>
       </c>
       <c r="G336" t="str">
         <v>F-084</v>
       </c>
       <c r="H336" t="str">
-        <v>Jedan izvod u pravilu kreira jedan nalog.</v>
+        <v>Dodato migracijom 20260629190000_bank_statements_mvp; jedan izvod u pravilu kreira jedan nalog.</v>
       </c>
     </row>
     <row r="337">
@@ -2029,13 +3217,13 @@
         <v>Izvodi</v>
       </c>
       <c r="F337" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Implementirano</v>
       </c>
       <c r="G337" t="str">
         <v>F-078,F-079,F-081</v>
       </c>
       <c r="H337" t="str">
-        <v>Stavke nose prepoznavanje, status i ručno kontiranje.</v>
+        <v>Dodato migracijom 20260629190000_bank_statements_mvp; stavke nose prepoznavanje, status i ručno kontiranje.</v>
       </c>
     </row>
     <row r="338">
@@ -2055,13 +3243,13 @@
         <v>Izvodi</v>
       </c>
       <c r="F338" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Implementirano</v>
       </c>
       <c r="G338" t="str">
         <v>F-079</v>
       </c>
       <c r="H338" t="str">
-        <v>Komitent se prepoznaje primarno po normalizovanom računu; source može biti MANUAL, BANK_STATEMENT_LEARNED ili IMPORT.</v>
+        <v>Dodato migracijom 20260629190000_bank_statements_mvp; UI za učenje računa ostaje otvoren.</v>
       </c>
     </row>
     <row r="339">
@@ -2149,7 +3337,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z350"/>
   <sheetData>
@@ -4906,7 +6094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB344"/>
   <sheetData>
@@ -6448,7 +7636,7 @@
         <v>F-076,R-104</v>
       </c>
       <c r="F334" t="str">
-        <v>Nije poceto</v>
+        <v>Ručni QA potreban</v>
       </c>
     </row>
     <row r="335">
@@ -6468,7 +7656,7 @@
         <v>F-077,F-078</v>
       </c>
       <c r="F335" t="str">
-        <v>Nije poceto</v>
+        <v>Ručni QA potreban</v>
       </c>
     </row>
     <row r="336">
@@ -6488,7 +7676,7 @@
         <v>F-084,R-106</v>
       </c>
       <c r="F336" t="str">
-        <v>Nije poceto</v>
+        <v>Ručni QA potreban</v>
       </c>
     </row>
     <row r="337">
@@ -6588,7 +7776,7 @@
         <v>F-081,F-084</v>
       </c>
       <c r="F341" t="str">
-        <v>Nije poceto</v>
+        <v>Ručni QA potreban</v>
       </c>
     </row>
     <row r="342">
@@ -6628,7 +7816,7 @@
         <v>F-084,R-105,R-110</v>
       </c>
       <c r="F343" t="str">
-        <v>Nije poceto</v>
+        <v>Ručni QA potreban</v>
       </c>
     </row>
     <row r="344">
@@ -6658,7 +7846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -6708,7 +7896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -7145,7 +8333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z319"/>
   <sheetData>
@@ -7871,7 +9059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -8066,12 +9254,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-28</v>
+        <v>Status projekta na dan 2026-06-29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
       </c>
     </row>
     <row r="4">
@@ -8093,87 +9281,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Performanse partnera</v>
+        <v>Nalozi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core implementiran</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C5" t="str">
-        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
       </c>
       <c r="D5" t="str">
-        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E5" t="str">
-        <v>Pratiti brzinu na produkciji.</v>
+        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Indeksi baze</v>
+        <v>PDV</v>
       </c>
       <c r="B6" t="str">
-        <v>Implementirano</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C6" t="str">
-        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D6" t="str">
-        <v>-</v>
+        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
       </c>
       <c r="E6" t="str">
-        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIF/KUF uvoz/export</v>
+        <v>Izvodi</v>
       </c>
       <c r="B7" t="str">
-        <v>Core implementiran</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
       </c>
       <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata; XML export.</v>
+        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
       </c>
       <c r="E7" t="str">
-        <v>QA uvoznih knjizenja i export fajlova.</v>
+        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dokumentacija</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="B8" t="str">
-        <v>Uspostavljeno</v>
+        <v>Core implementiran</v>
       </c>
       <c r="C8" t="str">
-        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
       </c>
       <c r="D8" t="str">
-        <v>Redovno odrzavanje.</v>
+        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
       </c>
       <c r="E8" t="str">
-        <v>Azurirati uz svaku vecu promjenu.</v>
+        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PDV</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B9" t="str">
-        <v>Prva implementacija</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C9" t="str">
-        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
       </c>
       <c r="D9" t="str">
-        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+        <v>Redovno odrzavanje.</v>
       </c>
       <c r="E9" t="str">
-        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+        <v>Regenerisati Excel nakon svake vece promjene.</v>
       </c>
     </row>
   </sheetData>
@@ -8185,6 +9373,129 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Performanse partnera</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pratiti brzinu na produkciji.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Indeksi baze</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KIF/KUF uvoz/export</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kontrole iznosa i duplikata; XML export.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>QA uvoznih knjizenja i export fajlova.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Dokumentacija</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Uspostavljeno</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Redovno odrzavanje.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Azurirati uz svaku vecu promjenu.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Prva implementacija</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
@@ -8357,7 +9668,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -8652,7 +9963,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z301"/>
   <sheetData>
@@ -8810,7 +10121,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="E9" t="str">
-        <v>Specifikacija spremna / nije implementirano</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="F9" t="str">
         <v>Računovođa</v>
@@ -8819,7 +10130,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H9" t="str">
-        <v>Finalna specifikacija je u zadaci/07_Izvodi_i_Automatsko_Knjizenje_FINAL.md. Modul ne treba duplirati ručni nalog IZV, nego raditi kao import/preview/povezivanje/knjiženje sloj koji generiše jedan nalog po izvodu.</v>
+        <v>Prva MVP osnova postoji: tabele, NLB XML uvoz/paste teksta, preview stavki, predlog naloga, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila i alokacije KIF/KUF.</v>
       </c>
     </row>
     <row r="10">
@@ -8959,7 +10270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z347"/>
   <sheetData>
@@ -11878,7 +13189,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F338" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G338" t="str">
         <v>Ne</v>
@@ -11896,7 +13207,7 @@
         <v>M-005,F-017</v>
       </c>
       <c r="L338" t="str">
-        <v>Ne praviti paralelni ručni izvod; ručno knjiženje ostaje kroz nalog IZV. Modul izvoda počinje od import/preview toka.</v>
+        <v>Postoji upload/paste tekst i čuvanje izvoda; puna import sesija i parseri po bankama ostaju otvoreni.</v>
       </c>
     </row>
     <row r="339">
@@ -11916,7 +13227,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F339" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G339" t="str">
         <v>Ne</v>
@@ -11934,7 +13245,7 @@
         <v>F-076</v>
       </c>
       <c r="L339" t="str">
-        <v>Parser mora vratiti preview; sistem ne smije knjižiti bez korisničke potvrde.</v>
+        <v>Implementiran NLB XML parser za UTF-16 XML izvode i fallback tekstualni format; parseri za ostale banke su otvoreni.</v>
       </c>
     </row>
     <row r="340">
@@ -11954,7 +13265,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F340" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G340" t="str">
         <v>Ne</v>
@@ -11972,7 +13283,7 @@
         <v>F-077</v>
       </c>
       <c r="L340" t="str">
-        <v>Preview prikazuje datum, opis, račun, komitenta, priliv/odliv, predlog, confidence i status.</v>
+        <v>Postoji tab Stavke izvoda i kontrola stanja; korekcije iznosa/datuma ostaju za doradu.</v>
       </c>
     </row>
     <row r="341">
@@ -11992,7 +13303,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F341" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G341" t="str">
         <v>Ne</v>
@@ -12010,7 +13321,7 @@
         <v>F-078</v>
       </c>
       <c r="L341" t="str">
-        <v>Sistem mora moći naučiti žiro račun komitenta iz ručno riješene stavke.</v>
+        <v>Automatski predlog po partner_bank_accounts i komitent_ziro_racuni postoji; UI za učenje računa ostaje otvoren.</v>
       </c>
     </row>
     <row r="342">
@@ -12068,7 +13379,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F343" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G343" t="str">
         <v>Ne</v>
@@ -12086,7 +13397,7 @@
         <v>F-078</v>
       </c>
       <c r="L343" t="str">
-        <v>Primjeri: provizije, kamate, porezi, zarade, lizing, interni prenosi.</v>
+        <v>Tab Predlog naloga omogućava izbor partnera i duguje/potražuje konta; izbor konta ide preko šifre i automatskog firma_konta linka; napredna pravila ostaju otvorena.</v>
       </c>
     </row>
     <row r="344">
@@ -12182,7 +13493,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F346" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G346" t="str">
         <v>Ne</v>
@@ -12200,7 +13511,7 @@
         <v>F-078,F-080,F-081</v>
       </c>
       <c r="L346" t="str">
-        <v>Kontrola početno stanje + prilivi - odlivi = krajnje stanje mora proći prije knjiženja.</v>
+        <v>Postoji preview i knjiženje READY izvoda u poseban proknjižen IZV nalog; banka se knjiži zbirno po ukupnom prilivu/odlivu, pojedinačne stavke idu samo na kontra konta; alokacije KIF/KUF nisu još uključene.</v>
       </c>
     </row>
     <row r="347">
@@ -12248,7 +13559,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z362"/>
   <sheetData>
@@ -15573,7 +16884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z309"/>
   <sheetData>
@@ -16103,1208 +17414,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:Z309"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z330"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Ekrani aplikacije</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Plan UI ekrana za prva 3 zaključena modula.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ID ekrana</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Naziv ekrana</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Opis</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Prioritet</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Status</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Povezane funkcije</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>UI-001</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Korisnici, agencije i prava</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Super admin — Agencije</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Pregled agencija, pretplata, statusa aktivacije i isteka.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="G5" t="str">
-        <v>F-001,F-003,F-004</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Pregled agencija postoji; pretplate nisu kompletno UI zaokruzene.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>UI-002</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Korisnici, agencije i prava</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Agencijski admin — Radnici</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Kreiranje radnika i dodjela prava.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G6" t="str">
-        <v>F-005,F-008</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Kreiranje radnika i dodjela prava postoje.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>UI-003</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Korisnici, agencije i prava</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Agencijski admin — Prava pristupa</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Matrica prava po firmama, modulima i akcijama.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="G7" t="str">
-        <v>F-007,F-008</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Matrica prava postoji; enforcement prava treba dodatno zakljucati.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>UI-004</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Korisnici, agencije i prava</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Učinak radnika</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Dnevni/nedjeljni/mjesečni pregled aktivnosti po radniku.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F8" t="str">
-        <v>U izradi</v>
-      </c>
-      <c r="G8" t="str">
-        <v>F-009,F-010</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Postoji audit/aktivnost osnova; puni ekran ucinka jos nije implementiran.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>UI-005</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Firme i kontni plan</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Lista firmi</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Naziv, PIB, tip, PDV status, godina, glavni radnik, status.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G9" t="str">
-        <v>F-012,F-014,F-019</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Lista firmi postoji kao /agencija/firme.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>UI-006</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Firme i kontni plan</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Dodavanje firme</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Unos PIB-a, IRMS pretraga, provjera podataka i snimanje.</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G10" t="str">
-        <v>F-012,F-013</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Dodavanje firme sa IRMS pretragom postoji kao /agencija/firme/nova.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>UI-007</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Firme i kontni plan</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Profil firme</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Tabovi: podaci, lica, banke, godine, podešavanja, radnici, klijenti, ugovor, kontni plan.</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="G11" t="str">
-        <v>F-012-F-023</v>
-      </c>
-      <c r="H11" t="str">
-        <v>Detalj firme sada prikazuje osnovne podatke, godine, bankovne racune, ugovor/cijenu i korisnike; odgovorna lica, kontni plan i podesavanja jos nisu kompletirani.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>UI-008</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Firme i kontni plan</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Poslovne godine</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Otvaranje, zaključavanje, otključavanje i arhiva godina.</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G12" t="str">
-        <v>F-014,F-015</v>
-      </c>
-      <c r="H12" t="str">
-        <v>Centralna stranica poslovnih godina postoji.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>UI-009</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Firme i kontni plan</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Kontni plan firme</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Kombinovani prikaz osnovnog plana i firmi specifičnih izmjena.</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G13" t="str">
-        <v>F-021,F-022,F-023</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Postoje dva ekrana: globalni osnovni kontni plan u podesavanjima i kontni plan firme za specificne izmjene i default konta. Kontni plan firme ima pretragu po sifri/nazivu direktno iznad tabele.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>UI-010</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Lista naloga</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Pregled naloga po firmi, godini, vrsti, broju, statusu, korisniku.</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G14" t="str">
-        <v>F-024-F-031</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Lista naloga po aktivnoj firmi/godini postoji na /agencija/nalozi, sa filterom statusa.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>UI-011</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Unos naloga</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Zaglavlje + tabelarni unos stavki.</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="G15" t="str">
-        <v>F-026,F-027,F-029</v>
-      </c>
-      <c r="H15" t="str">
-        <v>Unos novog naloga postoji na /agencija/nalozi/novi; izmjena nacrta ostaje za naredni korak.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>UI-012</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Nacrti naloga</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Lista nacrta koji nijesu proknjiženi.</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G16" t="str">
-        <v>F-028</v>
-      </c>
-      <c r="H16" t="str">
-        <v>Nacrti su dostupni preko /agencija/nalozi/nacrti odnosno status filtera.</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>UI-013</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Početno stanje</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Pregled/generisanje/proknjižavanje početnog stanja.</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F17" t="str">
-        <v>Nije poceto</v>
-      </c>
-      <c r="G17" t="str">
-        <v>F-034,F-035</v>
-      </c>
-      <c r="H17" t="str">
-        <v>Početno stanje jos nije posebna funkcionalnost.</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>UI-014</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Partneri</v>
-      </c>
-      <c r="D18" t="str">
-        <v>Lista partnera, kupac/dobavljač oznake, PIB, kontakt podaci.</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F18" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G18" t="str">
-        <v>F-036</v>
-      </c>
-      <c r="H18" t="str">
-        <v>Agencijski ekran za dodatne partnere i admin ekran za globalne partnere podrzavaju unos, IRMS pretragu i izmjenu.</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>UI-015</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="C19" t="str">
-        <v>Bruto bilans</v>
-      </c>
-      <c r="D19" t="str">
-        <v>PS, promet, ukupno, saldo; filter po firmi, godini, poslovnoj jedinici.</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F19" t="str">
-        <v>Nije poceto</v>
-      </c>
-      <c r="G19" t="str">
-        <v>F-038</v>
-      </c>
-      <c r="H19" t="str">
-        <v>Bruto bilans jos nije implementiran.</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>UI-016</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Kartica partnera</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Detaljna kartica i zbirni saldo kupaca/dobavljača.</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F20" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="G20" t="str">
-        <v>F-037</v>
-      </c>
-      <c r="H20" t="str">
-        <v>Analiticka kartica je implementirana u /agencija/nalozi/analiticke-kartice; zbir kupaca/dobavljaca po partneru u /agencija/nalozi/kupci-dobavljaci. Ostaju stampa/export.</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>UI-017</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Uvoz izvoda</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Upload PDF/HTML izvoda za aktivnu firmu/godinu i bankovni račun firme.</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F21" t="str">
-        <v>Specifikacija spremna</v>
-      </c>
-      <c r="G21" t="str">
-        <v>F-076</v>
-      </c>
-      <c r="H21" t="str">
-        <v>Ekran bira bankovni račun/banku i fajl, kreira import sesiju.</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>UI-018</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="C22" t="str">
-        <v>Preview parsiranja</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Pregled zaglavlja, parsiranih stavki, grešaka i kontrole početnog/krajnjeg stanja.</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F22" t="str">
-        <v>Specifikacija spremna</v>
-      </c>
-      <c r="G22" t="str">
-        <v>F-078</v>
-      </c>
-      <c r="H22" t="str">
-        <v>Korisnik može ispraviti pogrešno pročitane podatke prije povezivanja.</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>UI-019</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="C23" t="str">
-        <v>Povezivanje i obrada stavki</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Tabela stavki sa komitentom, fakturom, predlogom knjiženja, confidence score-om i akcijama.</v>
-      </c>
-      <c r="E23" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F23" t="str">
-        <v>Specifikacija spremna</v>
-      </c>
-      <c r="G23" t="str">
-        <v>F-079,F-080,F-081,F-083</v>
-      </c>
-      <c r="H23" t="str">
-        <v>Akcije: izaberi komitenta, poveži fakturu, rasporedi iznos, ručno kontiraj, ignoriši, zapamti račun, napravi pravilo.</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>UI-020</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="C24" t="str">
-        <v>Preview naloga izvoda</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Prije knjiženja prikazuje stavke naloga duguje/potražuje, konto, partner, opis i iznos.</v>
-      </c>
-      <c r="E24" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F24" t="str">
-        <v>Specifikacija spremna</v>
-      </c>
-      <c r="G24" t="str">
-        <v>F-084</v>
-      </c>
-      <c r="H24" t="str">
-        <v>Sistem knjiži tek kada su sve stavke READY ili IGNORED.</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>UI-021</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="C25" t="str">
-        <v>Kartica banke</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Pregled prometa bankovnog računa iz proknjiženih izvoda/naloga.</v>
-      </c>
-      <c r="E25" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F25" t="str">
-        <v>Specifikacija spremna</v>
-      </c>
-      <c r="G25" t="str">
-        <v>F-084</v>
-      </c>
-      <c r="H25" t="str">
-        <v>Zavisi od pravilnog povezivanja izvoda sa bankovnim računom firme.</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="str">
-        <v>E-017</v>
-      </c>
-      <c r="B306" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C306" t="str">
-        <v>Artikli</v>
-      </c>
-      <c r="D306" t="str">
-        <v>Lista i unos artikala/usluga.</v>
-      </c>
-      <c r="E306" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F306" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G306" t="str">
-        <v>F-039</v>
-      </c>
-      <c r="H306" t="str">
-        <v>Checkbox usluga.</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="str">
-        <v>E-018</v>
-      </c>
-      <c r="B307" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C307" t="str">
-        <v>Grupe artikala</v>
-      </c>
-      <c r="D307" t="str">
-        <v>Šifarnik grupa artikala.</v>
-      </c>
-      <c r="E307" t="str">
-        <v>Srednji</v>
-      </c>
-      <c r="F307" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G307" t="str">
-        <v>F-039</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="str">
-        <v>E-019</v>
-      </c>
-      <c r="B308" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C308" t="str">
-        <v>Cijene artikala</v>
-      </c>
-      <c r="D308" t="str">
-        <v>Upravljanje više cijena artikla.</v>
-      </c>
-      <c r="E308" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F308" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G308" t="str">
-        <v>F-040</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="str">
-        <v>E-020</v>
-      </c>
-      <c r="B309" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C309" t="str">
-        <v>Magacini</v>
-      </c>
-      <c r="D309" t="str">
-        <v>Lista i podešavanje magacina.</v>
-      </c>
-      <c r="E309" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F309" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G309" t="str">
-        <v>F-041</v>
-      </c>
-      <c r="H309" t="str">
-        <v>Negativan lager opciono po magacinu.</v>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="str">
-        <v>E-021</v>
-      </c>
-      <c r="B310" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C310" t="str">
-        <v>Lager lista</v>
-      </c>
-      <c r="D310" t="str">
-        <v>Stanje robe po magacinu.</v>
-      </c>
-      <c r="E310" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F310" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G310" t="str">
-        <v>F-042,F-060</v>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="str">
-        <v>E-022</v>
-      </c>
-      <c r="B311" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C311" t="str">
-        <v>Kartica artikla</v>
-      </c>
-      <c r="D311" t="str">
-        <v>Ulazi, izlazi i saldo artikla.</v>
-      </c>
-      <c r="E311" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F311" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G311" t="str">
-        <v>F-060</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="str">
-        <v>E-023</v>
-      </c>
-      <c r="B312" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C312" t="str">
-        <v>Kalkulacije</v>
-      </c>
-      <c r="D312" t="str">
-        <v>Unos i knjiženje kalkulacija.</v>
-      </c>
-      <c r="E312" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F312" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G312" t="str">
-        <v>F-045</v>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="str">
-        <v>E-024</v>
-      </c>
-      <c r="B313" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C313" t="str">
-        <v>Uvozna kalkulacija</v>
-      </c>
-      <c r="D313" t="str">
-        <v>Kalkulacija sa carinskom deklaracijom.</v>
-      </c>
-      <c r="E313" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F313" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G313" t="str">
-        <v>F-051</v>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="str">
-        <v>E-025</v>
-      </c>
-      <c r="B314" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C314" t="str">
-        <v>Povrat dobavljaču</v>
-      </c>
-      <c r="D314" t="str">
-        <v>Slobodan ili povezan povrat robe dobavljaču.</v>
-      </c>
-      <c r="E314" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F314" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G314" t="str">
-        <v>F-052</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="str">
-        <v>E-026</v>
-      </c>
-      <c r="B315" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C315" t="str">
-        <v>Prenos robe</v>
-      </c>
-      <c r="D315" t="str">
-        <v>Prenos između magacina.</v>
-      </c>
-      <c r="E315" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F315" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G315" t="str">
-        <v>F-054</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="str">
-        <v>E-027</v>
-      </c>
-      <c r="B316" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C316" t="str">
-        <v>Popis robe</v>
-      </c>
-      <c r="D316" t="str">
-        <v>Unos stvarnog stanja, višak i manjak.</v>
-      </c>
-      <c r="E316" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F316" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G316" t="str">
-        <v>F-055</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="str">
-        <v>E-028</v>
-      </c>
-      <c r="B317" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C317" t="str">
-        <v>Otpis robe</v>
-      </c>
-      <c r="D317" t="str">
-        <v>Otpis i razduženje robe.</v>
-      </c>
-      <c r="E317" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F317" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G317" t="str">
-        <v>F-058</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="str">
-        <v>E-029</v>
-      </c>
-      <c r="B318" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C318" t="str">
-        <v>Nivelacija</v>
-      </c>
-      <c r="D318" t="str">
-        <v>Promjena maloprodajnih cijena.</v>
-      </c>
-      <c r="E318" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F318" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G318" t="str">
-        <v>F-059</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="str">
-        <v>E-030</v>
-      </c>
-      <c r="B319" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C319" t="str">
-        <v>Robni izvještaji</v>
-      </c>
-      <c r="D319" t="str">
-        <v>Vrijednost zaliha, lager i pregledi po magacinima.</v>
-      </c>
-      <c r="E319" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F319" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G319" t="str">
-        <v>F-060</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="str">
-        <v>E-031</v>
-      </c>
-      <c r="B320" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C320" t="str">
-        <v>Podešavanje negativnog lagera</v>
-      </c>
-      <c r="D320" t="str">
-        <v>Blokiranje ili dozvola zaliha u minus.</v>
-      </c>
-      <c r="E320" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F320" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G320" t="str">
-        <v>F-043</v>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="str">
-        <v>E-032</v>
-      </c>
-      <c r="B321" t="str">
-        <v>Izlazne fakture</v>
-      </c>
-      <c r="C321" t="str">
-        <v>Izlazne fakture bez fiskalizacije</v>
-      </c>
-      <c r="D321" t="str">
-        <v>Ekran za kreiranje faktura koje mogu razdužiti magacin i kasnije se automatski knjižiti.</v>
-      </c>
-      <c r="E321" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F321" t="str">
-        <v>Za razradu</v>
-      </c>
-      <c r="G321" t="str">
-        <v>M-005</v>
-      </c>
-      <c r="H321" t="str">
-        <v>Fiskalizacija nije dio prve verzije.</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="str">
-        <v>E-033</v>
-      </c>
-      <c r="B322" t="str">
-        <v>Podešavanja / PDV</v>
-      </c>
-      <c r="C322" t="str">
-        <v>PDV stope</v>
-      </c>
-      <c r="D322" t="str">
-        <v>Ekran za unos, pregled, izmjenu i aktivaciju/deaktivaciju PDV stopa.</v>
-      </c>
-      <c r="E322" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F322" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G322" t="str">
-        <v>F-062</v>
-      </c>
-      <c r="H322" t="str">
-        <v>/agencija/podesavanja/pdv-stope</v>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="str">
-        <v>E-034</v>
-      </c>
-      <c r="B323" t="str">
-        <v>Računi / KUF</v>
-      </c>
-      <c r="C323" t="str">
-        <v>KUF knjige i detalj KUF-a</v>
-      </c>
-      <c r="D323" t="str">
-        <v>Računi / Podešavanja prikazuju vrste KIF/KUF i šemu kontiranja po poljima. KUF i KIF imaju otvaranje knjige i unos računa; KIF konto prihoda zavisi od šeme.</v>
-      </c>
-      <c r="E323" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F323" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="G323" t="str">
-        <v>F-063</v>
-      </c>
-      <c r="H323" t="str">
-        <v>/agencija/racuni/podesavanja, /agencija/racuni/kuf, /agencija/racuni/kuf/[id], /agencija/racuni/kif/[id], /agencija/racuni/neproknjizeno, /agencija/racuni/pregled-kuf i /agencija/racuni/pregled-kuf/[id]. Dodato knjiženje/dopuna naloga po knjizi i uvoz podešavanja iz druge firme.</v>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="str">
-        <v>E-035</v>
-      </c>
-      <c r="B324" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="C324" t="str">
-        <v>PDV pregled</v>
-      </c>
-      <c r="D324" t="str">
-        <v>Lista mjesečnih PDV perioda za aktivnu firmu/godinu sa statusom i zbirnim iznosima.</v>
-      </c>
-      <c r="E324" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F324" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G324" t="str">
-        <v>F-072</v>
-      </c>
-      <c r="H324" t="str">
-        <v>/agencija/pdv</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="str">
-        <v>E-036</v>
-      </c>
-      <c r="B325" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="C325" t="str">
-        <v>Ulazni PDV</v>
-      </c>
-      <c r="D325" t="str">
-        <v>Dokazna evidencija KUF računa za izabrani mjesec po datumu KUF knjige.</v>
-      </c>
-      <c r="E325" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F325" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G325" t="str">
-        <v>F-073</v>
-      </c>
-      <c r="H325" t="str">
-        <v>/agencija/pdv/ulazni</v>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="str">
-        <v>E-037</v>
-      </c>
-      <c r="B326" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="C326" t="str">
-        <v>Izlazni PDV</v>
-      </c>
-      <c r="D326" t="str">
-        <v>Dokazna evidencija KIF računa za izabrani mjesec po datumu KIF knjige.</v>
-      </c>
-      <c r="E326" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F326" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G326" t="str">
-        <v>F-073</v>
-      </c>
-      <c r="H326" t="str">
-        <v>/agencija/pdv/izlazni</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="str">
-        <v>E-038</v>
-      </c>
-      <c r="B327" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="C327" t="str">
-        <v>PDV prijava</v>
-      </c>
-      <c r="D327" t="str">
-        <v>IRMS-like obrazac prijave sa lijevom/desnom PDV kolonom i automatskim preračunima.</v>
-      </c>
-      <c r="E327" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F327" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="G327" t="str">
-        <v>F-074</v>
-      </c>
-      <c r="H327" t="str">
-        <v>/agencija/pdv/prijava</v>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="str">
-        <v>E-039</v>
-      </c>
-      <c r="B328" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="C328" t="str">
-        <v>PDV kontrole</v>
-      </c>
-      <c r="D328" t="str">
-        <v>Kontrole prije XML izvoza i knjiženja prijave; uključuje neproknjižene/rasknjižene KIF/KUF stavke i poređenje sa glavnom knjigom.</v>
-      </c>
-      <c r="E328" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F328" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="G328" t="str">
-        <v>F-074</v>
-      </c>
-      <c r="H328" t="str">
-        <v>/agencija/pdv/kontrole</v>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="str">
-        <v>E-040</v>
-      </c>
-      <c r="B329" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="C329" t="str">
-        <v>Arhiva PDV prijava</v>
-      </c>
-      <c r="D329" t="str">
-        <v>Lista sačuvanih/proknjiženih prijava i linkovi na XML/nalog.</v>
-      </c>
-      <c r="E329" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="F329" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G329" t="str">
-        <v>F-074</v>
-      </c>
-      <c r="H329" t="str">
-        <v>/agencija/pdv/arhiva</v>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="str">
-        <v>E-041</v>
-      </c>
-      <c r="B330" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="C330" t="str">
-        <v>Podešavanja PDV-a</v>
-      </c>
-      <c r="D330" t="str">
-        <v>Vrsta naloga i šema D/P + konto za knjiženje PDV prijave po aktivnim stopama; konto dropdown prikazuje cijeli spojeni kontni plan.</v>
-      </c>
-      <c r="E330" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="F330" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G330" t="str">
-        <v>F-075</v>
-      </c>
-      <c r="H330" t="str">
-        <v>/agencija/pdv/podesavanja</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z330"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Expand bank statement import and rules
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,23 +3,24 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-06-30" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-06-29" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-06-28" sheetId="3" r:id="rId3"/>
-    <sheet name="Status 2026-06-25" sheetId="4" r:id="rId4"/>
-    <sheet name="Dashboard" sheetId="5" r:id="rId5"/>
-    <sheet name="Moduli" sheetId="6" r:id="rId6"/>
-    <sheet name="Funkcionalnosti" sheetId="7" r:id="rId7"/>
-    <sheet name="Pravila" sheetId="8" r:id="rId8"/>
-    <sheet name="Zavisnosti" sheetId="9" r:id="rId9"/>
-    <sheet name="Ekrani" sheetId="10" r:id="rId10"/>
-    <sheet name="Baza" sheetId="11" r:id="rId11"/>
-    <sheet name="API" sheetId="12" r:id="rId12"/>
-    <sheet name="Testovi" sheetId="13" r:id="rId13"/>
-    <sheet name="Bugovi" sheetId="14" r:id="rId14"/>
-    <sheet name="Ideje" sheetId="15" r:id="rId15"/>
-    <sheet name="Odluke" sheetId="16" r:id="rId16"/>
-    <sheet name="Kategorije" sheetId="17" r:id="rId17"/>
+    <sheet name="Status 2026-07-02" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-06-30" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-06-29" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-06-28" sheetId="4" r:id="rId4"/>
+    <sheet name="Status 2026-06-25" sheetId="5" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="6" r:id="rId6"/>
+    <sheet name="Moduli" sheetId="7" r:id="rId7"/>
+    <sheet name="Funkcionalnosti" sheetId="8" r:id="rId8"/>
+    <sheet name="Pravila" sheetId="9" r:id="rId9"/>
+    <sheet name="Zavisnosti" sheetId="10" r:id="rId10"/>
+    <sheet name="Ekrani" sheetId="11" r:id="rId11"/>
+    <sheet name="Baza" sheetId="12" r:id="rId12"/>
+    <sheet name="API" sheetId="13" r:id="rId13"/>
+    <sheet name="Testovi" sheetId="14" r:id="rId14"/>
+    <sheet name="Bugovi" sheetId="15" r:id="rId15"/>
+    <sheet name="Ideje" sheetId="16" r:id="rId16"/>
+    <sheet name="Odluke" sheetId="17" r:id="rId17"/>
+    <sheet name="Kategorije" sheetId="18" r:id="rId18"/>
   </sheets>
 </workbook>
 </file>
@@ -417,7 +418,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-30</v>
+        <v>Status projekta na dan 2026-07-02</v>
       </c>
     </row>
     <row r="2">
@@ -450,13 +451,13 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
+        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
       </c>
       <c r="D5" t="str">
-        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
+        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
       </c>
       <c r="E5" t="str">
-        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
+        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
       </c>
     </row>
     <row r="6">
@@ -519,6 +520,538 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Z309"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Zavisnosti</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Šta zavisi od čega, da se razvoj radi pravilnim redosljedom.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Tip stavke</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Stavka</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Zavisi od</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Razlog / napomena</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Rizik ako nije gotovo</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Faza</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Z-001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Firme i kontni plan</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Firma mora pripadati agenciji; korisnici moraju imati prava.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Bez ovoga nema izolacije podataka.</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H5" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Z-002</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Firme, poslovne godine i kontni plan</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Nalog mora znati firmu, godinu i konto.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Nalozi bi bili nevalidni.</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H6" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Z-003</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Funkcionalnost</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Dodjela firmi radnicima</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Radnici agencije + firme</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Mora postojati radnik i firma.</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Ne može se ograničiti pristup.</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H7" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Z-004</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Funkcionalnost</v>
+      </c>
+      <c r="C8" t="str">
+        <v>PDV pravila knjiženja</v>
+      </c>
+      <c r="D8" t="str">
+        <v>PDV status firme + kontni plan</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Da bi se znalo da li knjižiti PDV stavku.</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Pogrešno knjiženje računa.</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H8" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Z-005</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Funkcionalnost</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Numeracija naloga</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Vrste naloga + poslovna godina</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Brojač se vodi po vrsti i godini.</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Dupli brojevi naloga.</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H9" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Z-006</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Funkcionalnost</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Knjiženje naloga</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Stavke naloga + kontni plan + poslovna godina</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Mora se provjeriti balans, konto i status godine.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Neispravni izvještaji.</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H10" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Z-007</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Funkcionalnost</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Početno stanje</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Bruto bilans prethodne godine</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Prenos PS zavisi od krajnjeg stanja prethodne godine.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Pogrešan početak nove godine.</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H11" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Z-008</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Funkcionalnost</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Analitičke kartice</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Nalozi + partneri + analitička konta</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Za kupce/dobavljače treba partner po stavci.</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Nema tačnih kartica.</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H12" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Z-009</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Funkcionalnost</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Bruto bilans</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Proknjiženi nalozi + početno stanje</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Bruto bilans se računa iz POSTED naloga.</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Netačni bilansi.</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H13" t="str">
+        <v>MVP 1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Z-010</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Budući modul</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Nalozi + firma + kontni plan + partneri</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Kalkulacije/fakture/zalihe moraju kreirati naloge.</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Automatska knjiženja neće raditi.</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Sljedeće</v>
+      </c>
+      <c r="H14" t="str">
+        <v>MVP 1/2</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>Z-011</v>
+      </c>
+      <c r="B301" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C301" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Firme, poslovne godine, kontni plan</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Robni dokument mora znati firmu, godinu, PDV status i konta.</v>
+      </c>
+      <c r="F301" t="str">
+        <v>Bez toga nema pravilnog knjiženja.</v>
+      </c>
+      <c r="G301" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H301" t="str">
+        <v>MVP 1/2</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>Z-012</v>
+      </c>
+      <c r="B302" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C302" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="D302" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Svi proknjiženi robni dokumenti kreiraju naloge.</v>
+      </c>
+      <c r="F302" t="str">
+        <v>Nema glavne knjige i bruto bilansa.</v>
+      </c>
+      <c r="G302" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H302" t="str">
+        <v>MVP 1/2</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>Z-013</v>
+      </c>
+      <c r="B303" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C303" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="D303" t="str">
+        <v>Korisnici i prava</v>
+      </c>
+      <c r="E303" t="str">
+        <v>Prava određuju ko može unositi, knjižiti, vraćati i brisati robne dokumente.</v>
+      </c>
+      <c r="F303" t="str">
+        <v>Neovlašćen pristup robnim podacima.</v>
+      </c>
+      <c r="G303" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H303" t="str">
+        <v>MVP 1/2</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>Z-014</v>
+      </c>
+      <c r="B304" t="str">
+        <v>Budući modul</v>
+      </c>
+      <c r="C304" t="str">
+        <v>Izlazne fakture</v>
+      </c>
+      <c r="D304" t="str">
+        <v>Fakture razdužuju robu iz magacina.</v>
+      </c>
+      <c r="E304" t="str">
+        <v>Fakturisanje bez robnog razduženja.</v>
+      </c>
+      <c r="F304" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G304" t="str">
+        <v>MVP 2</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>Z-015</v>
+      </c>
+      <c r="B305" t="str">
+        <v>Budući modul</v>
+      </c>
+      <c r="C305" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="D305" t="str">
+        <v>Kalkulacije, uvoz i fakture utiču na PDV evidencije.</v>
+      </c>
+      <c r="E305" t="str">
+        <v>Neispravna PDV prijava.</v>
+      </c>
+      <c r="F305" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G305" t="str">
+        <v>MVP 2</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>Z-016</v>
+      </c>
+      <c r="B306" t="str">
+        <v>Izvještaji</v>
+      </c>
+      <c r="C306" t="str">
+        <v>Lager i kartice</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Robni izvještaji zavise od stock_movements i stock_balances.</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Neispravni lager izvještaji.</v>
+      </c>
+      <c r="F306" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G306" t="str">
+        <v>MVP 1/2</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>Z-017</v>
+      </c>
+      <c r="B307" t="str">
+        <v>Buduća integracija</v>
+      </c>
+      <c r="C307" t="str">
+        <v>Fiskalizacija</v>
+      </c>
+      <c r="D307" t="str">
+        <v>Izlazne fakture</v>
+      </c>
+      <c r="E307" t="str">
+        <v>Fiskalizacija se ne radi u prvoj verziji, ali fakture treba projektovati tako da se kasnije mogu povezati sa fiskalnim API-jem.</v>
+      </c>
+      <c r="F307" t="str">
+        <v>Ako model fakture nije dobro projektovan, kasnija integracija će biti teža.</v>
+      </c>
+      <c r="G307" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="H307" t="str">
+        <v>MVP 3 / Kasnije</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>Z-018</v>
+      </c>
+      <c r="B308" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C308" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="D308" t="str">
+        <v>Firme, poslovne godine, bankovni računi firme, komitenti, kontni plan, nalozi, KIF/KUF</v>
+      </c>
+      <c r="E308" t="str">
+        <v>Izvod mora znati firmu/godinu/banku, prepoznati komitenta i zatvoriti fakture kroz nalog.</v>
+      </c>
+      <c r="F308" t="str">
+        <v>Bez toga nema pouzdanog knjiženja izvoda ni zatvaranja stavki.</v>
+      </c>
+      <c r="G308" t="str">
+        <v>Sljedeće</v>
+      </c>
+      <c r="H308" t="str">
+        <v>MVP 2</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>Z-019</v>
+      </c>
+      <c r="B309" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C309" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="D309" t="str">
+        <v>Partner bank accounts</v>
+      </c>
+      <c r="E309" t="str">
+        <v>Prepoznavanje komitenta zavisi od normalizovanih žiro računa komitenata.</v>
+      </c>
+      <c r="F309" t="str">
+        <v>Bez toga bi sistem nepouzdano pogađao po nazivu iz banke.</v>
+      </c>
+      <c r="G309" t="str">
+        <v>Sljedeće</v>
+      </c>
+      <c r="H309" t="str">
+        <v>MVP 2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z309"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z330"/>
   <sheetData>
     <row r="1">
@@ -996,7 +1529,7 @@
         <v>F-076</v>
       </c>
       <c r="H21" t="str">
-        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, XML/tekst fajla i paste teksta; NLB XML radi, ostale banke ostaju otvorene.</v>
+        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML, Erste HTM i CKB PDF rade, ostale banke ostaju otvorene.</v>
       </c>
     </row>
     <row r="22">
@@ -1721,7 +2254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z341"/>
   <sheetData>
@@ -3289,19 +3822,19 @@
         <v>Pravila automatskog knjiženja izvoda.</v>
       </c>
       <c r="D340" t="str">
-        <v>agency_id, company_id, bank_account_id, rule_name, priority, match_type, match_value, direction, amount_condition, debit_account_id, credit_account_id, partner_id, auto_apply, requires_review</v>
+        <v>agencija_id, firma_id nullable, direction, counterparty_account_number, description_contains, reference_contains, payment_code, priority, account_code, account_id, partner_id, auto_apply, requires_review</v>
       </c>
       <c r="E340" t="str">
         <v>Izvodi</v>
       </c>
       <c r="F340" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Implementirano</v>
       </c>
       <c r="G340" t="str">
         <v>F-082</v>
       </c>
       <c r="H340" t="str">
-        <v>Za MVP auto_apply=false i requires_review=true.</v>
+        <v>Pravila mogu biti zajednička za agenciju ili specifična za firmu; account_code čuva šifru konta za primjenu kroz firme.</v>
       </c>
     </row>
     <row r="341">
@@ -3337,7 +3870,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z350"/>
   <sheetData>
@@ -6094,7 +6627,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB344"/>
   <sheetData>
@@ -7846,7 +8379,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -7896,7 +8429,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -8333,7 +8866,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z319"/>
   <sheetData>
@@ -9059,7 +9592,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -9250,11 +9783,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-29</v>
+        <v>Status projekta na dan 2026-06-30</v>
       </c>
     </row>
     <row r="2">
@@ -9281,92 +9814,75 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nalozi</v>
+        <v>Izvodi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core zaokruzen</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
+        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
       </c>
       <c r="D5" t="str">
-        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
       </c>
       <c r="E5" t="str">
-        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
+        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PDV</v>
+        <v>Nalozi</v>
       </c>
       <c r="B6" t="str">
-        <v>Core zaokruzen</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C6" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
       </c>
       <c r="D6" t="str">
-        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
+        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E6" t="str">
-        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
+        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Izvodi</v>
+        <v>PDV</v>
       </c>
       <c r="B7" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C7" t="str">
-        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D7" t="str">
-        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
+        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
       </c>
       <c r="E7" t="str">
-        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
+        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>KIF/KUF</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B8" t="str">
-        <v>Core implementiran</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C8" t="str">
-        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
+        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
       </c>
       <c r="D8" t="str">
-        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
+        <v>Redovno održavanje.</v>
       </c>
       <c r="E8" t="str">
-        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C9" t="str">
-        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Regenerisati Excel nakon svake vece promjene.</v>
+        <v>Regenerisati Excel nakon svake veće promjene.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9377,12 +9893,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-28</v>
+        <v>Status projekta na dan 2026-06-29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
       </c>
     </row>
     <row r="4">
@@ -9404,87 +9920,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Performanse partnera</v>
+        <v>Nalozi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core implementiran</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C5" t="str">
-        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
       </c>
       <c r="D5" t="str">
-        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E5" t="str">
-        <v>Pratiti brzinu na produkciji.</v>
+        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Indeksi baze</v>
+        <v>PDV</v>
       </c>
       <c r="B6" t="str">
-        <v>Implementirano</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C6" t="str">
-        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D6" t="str">
-        <v>-</v>
+        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
       </c>
       <c r="E6" t="str">
-        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIF/KUF uvoz/export</v>
+        <v>Izvodi</v>
       </c>
       <c r="B7" t="str">
-        <v>Core implementiran</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
       </c>
       <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata; XML export.</v>
+        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
       </c>
       <c r="E7" t="str">
-        <v>QA uvoznih knjizenja i export fajlova.</v>
+        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dokumentacija</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="B8" t="str">
-        <v>Uspostavljeno</v>
+        <v>Core implementiran</v>
       </c>
       <c r="C8" t="str">
-        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
       </c>
       <c r="D8" t="str">
-        <v>Redovno odrzavanje.</v>
+        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
       </c>
       <c r="E8" t="str">
-        <v>Azurirati uz svaku vecu promjenu.</v>
+        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PDV</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B9" t="str">
-        <v>Prva implementacija</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C9" t="str">
-        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
       </c>
       <c r="D9" t="str">
-        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+        <v>Redovno odrzavanje.</v>
       </c>
       <c r="E9" t="str">
-        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+        <v>Regenerisati Excel nakon svake vece promjene.</v>
       </c>
     </row>
   </sheetData>
@@ -9496,6 +10012,129 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Performanse partnera</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pratiti brzinu na produkciji.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Indeksi baze</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KIF/KUF uvoz/export</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kontrole iznosa i duplikata; XML export.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>QA uvoznih knjizenja i export fajlova.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Dokumentacija</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Uspostavljeno</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Redovno odrzavanje.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Azurirati uz svaku vecu promjenu.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Prva implementacija</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
@@ -9668,7 +10307,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -9963,7 +10602,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z301"/>
   <sheetData>
@@ -10115,7 +10754,7 @@
         <v>Izvodi i automatsko knjiženje</v>
       </c>
       <c r="C9" t="str">
-        <v>Uvoz PDF/HTML izvoda, import sesije, preview, prepoznavanje komitenata po žiro računu, povezivanje sa KIF/KUF fakturama, pravila knjiženja i automatski nalog.</v>
+        <v>Uvoz PDF/HTML/XML izvoda, import sesije, preview, prepoznavanje komitenata po žiro računu, povezivanje sa KIF/KUF fakturama, pravila knjiženja i automatski nalog.</v>
       </c>
       <c r="D9" t="str">
         <v>Vrlo visok</v>
@@ -10130,7 +10769,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H9" t="str">
-        <v>Prva MVP osnova postoji: tabele, NLB XML uvoz/paste teksta, preview stavki, predlog naloga, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila i alokacije KIF/KUF.</v>
+        <v>Prva MVP osnova postoji: tabele, NLB XML, Erste HTM i CKB PDF uvoz/paste teksta, preview stavki, predlog naloga, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i alokacije KIF/KUF.</v>
       </c>
     </row>
     <row r="10">
@@ -10270,7 +10909,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z347"/>
   <sheetData>
@@ -13183,7 +13822,7 @@
         <v>Import sesija PDF/HTML izvoda</v>
       </c>
       <c r="D338" t="str">
-        <v>Korisnik učitava PDF/HTML izvod za aktivnu firmu/godinu i bankovni račun; sistem čuva fajl, raw text i status importa.</v>
+        <v>Korisnik učitava PDF/HTML/XML izvod za aktivnu firmu/godinu i bankovni račun; sistem čuva fajl, raw text i status importa.</v>
       </c>
       <c r="E338" t="str">
         <v>Vrlo visok</v>
@@ -13207,7 +13846,7 @@
         <v>M-005,F-017</v>
       </c>
       <c r="L338" t="str">
-        <v>Postoji upload/paste tekst i čuvanje izvoda; puna import sesija i parseri po bankama ostaju otvoreni.</v>
+        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML, Erste HTM i CKB PDF, a puna import sesija ostaje za kasnije.</v>
       </c>
     </row>
     <row r="339">
@@ -13221,7 +13860,7 @@
         <v>Parsiranje izvoda</v>
       </c>
       <c r="D339" t="str">
-        <v>Generički PDF/HTML parser čita zaglavlje i stavke, a arhitektura dozvoljava parsere po bankama.</v>
+        <v>Parser čita zaglavlje i stavke, a arhitektura dozvoljava parsere po bankama.</v>
       </c>
       <c r="E339" t="str">
         <v>Vrlo visok</v>
@@ -13245,7 +13884,7 @@
         <v>F-076</v>
       </c>
       <c r="L339" t="str">
-        <v>Implementiran NLB XML parser za UTF-16 XML izvode i fallback tekstualni format; parseri za ostale banke su otvoreni.</v>
+        <v>Implementirani NLB XML, Erste HTM i CKB PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; fallback tekstualni format ostaje aktivan.</v>
       </c>
     </row>
     <row r="340">
@@ -13321,7 +13960,7 @@
         <v>F-078</v>
       </c>
       <c r="L341" t="str">
-        <v>Automatski predlog po partner_bank_accounts i komitent_ziro_racuni postoji; UI za učenje računa ostaje otvoren.</v>
+        <v>Automatski predlog po partner_bank_accounts i komitent_ziro_racuni postoji; ručno povezivanje partnera na stavci izvoda pamti račun kao agencijski zajednički račun kad je moguće.</v>
       </c>
     </row>
     <row r="342">
@@ -13397,7 +14036,7 @@
         <v>F-078</v>
       </c>
       <c r="L343" t="str">
-        <v>Tab Predlog naloga omogućava izbor partnera i duguje/potražuje konta; izbor konta ide preko šifre i automatskog firma_konta linka; napredna pravila ostaju otvorena.</v>
+        <v>Tab Predlog naloga omogućava izbor partnera i duguje/potražuje konta; izbor konta ide preko šifre i automatskog firma_konta linka; interni prenosi između sopstvenih računa firme se prepoznaju po kontra računu.</v>
       </c>
     </row>
     <row r="344">
@@ -13417,7 +14056,7 @@
         <v>Visok</v>
       </c>
       <c r="F344" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="G344" t="str">
         <v>Ne</v>
@@ -13435,7 +14074,7 @@
         <v>F-081</v>
       </c>
       <c r="L344" t="str">
-        <v>Za MVP auto_apply=false i requires_review=true.</v>
+        <v>Pravila podržavaju smjer, žiro račun, opis, šifru plaćanja, poziv na broj, prioritet, zajednički scope agencije i firm-specific override; account_code omogućava primjenu kroz firme.</v>
       </c>
     </row>
     <row r="345">
@@ -13559,7 +14198,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z362"/>
   <sheetData>
@@ -16882,536 +17521,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:Z362"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z309"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Zavisnosti</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Šta zavisi od čega, da se razvoj radi pravilnim redosljedom.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Tip stavke</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Stavka</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Zavisi od</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Razlog / napomena</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Rizik ako nije gotovo</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Status</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Faza</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Z-001</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Firme i kontni plan</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Korisnici, agencije i prava</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Firma mora pripadati agenciji; korisnici moraju imati prava.</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Bez ovoga nema izolacije podataka.</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H5" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Z-002</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Firme, poslovne godine i kontni plan</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Nalog mora znati firmu, godinu i konto.</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Nalozi bi bili nevalidni.</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H6" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Z-003</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Funkcionalnost</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Dodjela firmi radnicima</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Radnici agencije + firme</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Mora postojati radnik i firma.</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Ne može se ograničiti pristup.</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H7" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Z-004</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Funkcionalnost</v>
-      </c>
-      <c r="C8" t="str">
-        <v>PDV pravila knjiženja</v>
-      </c>
-      <c r="D8" t="str">
-        <v>PDV status firme + kontni plan</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Da bi se znalo da li knjižiti PDV stavku.</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Pogrešno knjiženje računa.</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H8" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Z-005</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Funkcionalnost</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Numeracija naloga</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Vrste naloga + poslovna godina</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Brojač se vodi po vrsti i godini.</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Dupli brojevi naloga.</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H9" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Z-006</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Funkcionalnost</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Knjiženje naloga</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Stavke naloga + kontni plan + poslovna godina</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Mora se provjeriti balans, konto i status godine.</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Neispravni izvještaji.</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H10" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Z-007</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Funkcionalnost</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Početno stanje</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Bruto bilans prethodne godine</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Prenos PS zavisi od krajnjeg stanja prethodne godine.</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Pogrešan početak nove godine.</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H11" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Z-008</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Funkcionalnost</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Analitičke kartice</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Nalozi + partneri + analitička konta</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Za kupce/dobavljače treba partner po stavci.</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Nema tačnih kartica.</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H12" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Z-009</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Funkcionalnost</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Bruto bilans</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Proknjiženi nalozi + početno stanje</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Bruto bilans se računa iz POSTED naloga.</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Netačni bilansi.</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H13" t="str">
-        <v>MVP 1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Z-010</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Budući modul</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Nalozi + firma + kontni plan + partneri</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Kalkulacije/fakture/zalihe moraju kreirati naloge.</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Automatska knjiženja neće raditi.</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Sljedeće</v>
-      </c>
-      <c r="H14" t="str">
-        <v>MVP 1/2</v>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="str">
-        <v>Z-011</v>
-      </c>
-      <c r="B301" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C301" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="D301" t="str">
-        <v>Firme, poslovne godine, kontni plan</v>
-      </c>
-      <c r="E301" t="str">
-        <v>Robni dokument mora znati firmu, godinu, PDV status i konta.</v>
-      </c>
-      <c r="F301" t="str">
-        <v>Bez toga nema pravilnog knjiženja.</v>
-      </c>
-      <c r="G301" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H301" t="str">
-        <v>MVP 1/2</v>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="str">
-        <v>Z-012</v>
-      </c>
-      <c r="B302" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C302" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="D302" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="E302" t="str">
-        <v>Svi proknjiženi robni dokumenti kreiraju naloge.</v>
-      </c>
-      <c r="F302" t="str">
-        <v>Nema glavne knjige i bruto bilansa.</v>
-      </c>
-      <c r="G302" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H302" t="str">
-        <v>MVP 1/2</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="str">
-        <v>Z-013</v>
-      </c>
-      <c r="B303" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C303" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="D303" t="str">
-        <v>Korisnici i prava</v>
-      </c>
-      <c r="E303" t="str">
-        <v>Prava određuju ko može unositi, knjižiti, vraćati i brisati robne dokumente.</v>
-      </c>
-      <c r="F303" t="str">
-        <v>Neovlašćen pristup robnim podacima.</v>
-      </c>
-      <c r="G303" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H303" t="str">
-        <v>MVP 1/2</v>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="str">
-        <v>Z-014</v>
-      </c>
-      <c r="B304" t="str">
-        <v>Budući modul</v>
-      </c>
-      <c r="C304" t="str">
-        <v>Izlazne fakture</v>
-      </c>
-      <c r="D304" t="str">
-        <v>Fakture razdužuju robu iz magacina.</v>
-      </c>
-      <c r="E304" t="str">
-        <v>Fakturisanje bez robnog razduženja.</v>
-      </c>
-      <c r="F304" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G304" t="str">
-        <v>MVP 2</v>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="str">
-        <v>Z-015</v>
-      </c>
-      <c r="B305" t="str">
-        <v>Budući modul</v>
-      </c>
-      <c r="C305" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="D305" t="str">
-        <v>Kalkulacije, uvoz i fakture utiču na PDV evidencije.</v>
-      </c>
-      <c r="E305" t="str">
-        <v>Neispravna PDV prijava.</v>
-      </c>
-      <c r="F305" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G305" t="str">
-        <v>MVP 2</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="str">
-        <v>Z-016</v>
-      </c>
-      <c r="B306" t="str">
-        <v>Izvještaji</v>
-      </c>
-      <c r="C306" t="str">
-        <v>Lager i kartice</v>
-      </c>
-      <c r="D306" t="str">
-        <v>Robni izvještaji zavise od stock_movements i stock_balances.</v>
-      </c>
-      <c r="E306" t="str">
-        <v>Neispravni lager izvještaji.</v>
-      </c>
-      <c r="F306" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G306" t="str">
-        <v>MVP 1/2</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="str">
-        <v>Z-017</v>
-      </c>
-      <c r="B307" t="str">
-        <v>Buduća integracija</v>
-      </c>
-      <c r="C307" t="str">
-        <v>Fiskalizacija</v>
-      </c>
-      <c r="D307" t="str">
-        <v>Izlazne fakture</v>
-      </c>
-      <c r="E307" t="str">
-        <v>Fiskalizacija se ne radi u prvoj verziji, ali fakture treba projektovati tako da se kasnije mogu povezati sa fiskalnim API-jem.</v>
-      </c>
-      <c r="F307" t="str">
-        <v>Ako model fakture nije dobro projektovan, kasnija integracija će biti teža.</v>
-      </c>
-      <c r="G307" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="H307" t="str">
-        <v>MVP 3 / Kasnije</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="str">
-        <v>Z-018</v>
-      </c>
-      <c r="B308" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C308" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="D308" t="str">
-        <v>Firme, poslovne godine, bankovni računi firme, komitenti, kontni plan, nalozi, KIF/KUF</v>
-      </c>
-      <c r="E308" t="str">
-        <v>Izvod mora znati firmu/godinu/banku, prepoznati komitenta i zatvoriti fakture kroz nalog.</v>
-      </c>
-      <c r="F308" t="str">
-        <v>Bez toga nema pouzdanog knjiženja izvoda ni zatvaranja stavki.</v>
-      </c>
-      <c r="G308" t="str">
-        <v>Sljedeće</v>
-      </c>
-      <c r="H308" t="str">
-        <v>MVP 2</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="str">
-        <v>Z-019</v>
-      </c>
-      <c r="B309" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C309" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="D309" t="str">
-        <v>Partner bank accounts</v>
-      </c>
-      <c r="E309" t="str">
-        <v>Prepoznavanje komitenta zavisi od normalizovanih žiro računa komitenata.</v>
-      </c>
-      <c r="F309" t="str">
-        <v>Bez toga bi sistem nepouzdano pogađao po nazivu iz banke.</v>
-      </c>
-      <c r="G309" t="str">
-        <v>Sljedeće</v>
-      </c>
-      <c r="H309" t="str">
-        <v>MVP 2</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z309"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Lovcen bank statement parser
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -1529,7 +1529,7 @@
         <v>F-076</v>
       </c>
       <c r="H21" t="str">
-        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML, Erste HTM i CKB PDF rade, ostale banke ostaju otvorene.</v>
+        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF i Lovćen PDF rade, ostale banke ostaju otvorene.</v>
       </c>
     </row>
     <row r="22">
@@ -10769,7 +10769,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H9" t="str">
-        <v>Prva MVP osnova postoji: tabele, NLB XML, Erste HTM i CKB PDF uvoz/paste teksta, preview stavki, predlog naloga, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i alokacije KIF/KUF.</v>
+        <v>Prva MVP osnova postoji: tabele, NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF i Lovćen PDF uvoz/paste teksta, preview stavki, predlog naloga, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i alokacije KIF/KUF.</v>
       </c>
     </row>
     <row r="10">
@@ -13846,7 +13846,7 @@
         <v>M-005,F-017</v>
       </c>
       <c r="L338" t="str">
-        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML, Erste HTM i CKB PDF, a puna import sesija ostaje za kasnije.</v>
+        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF i Lovćen PDF, a puna import sesija ostaje za kasnije.</v>
       </c>
     </row>
     <row r="339">
@@ -13884,7 +13884,7 @@
         <v>F-076</v>
       </c>
       <c r="L339" t="str">
-        <v>Implementirani NLB XML, Erste HTM i CKB PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; fallback tekstualni format ostaje aktivan.</v>
+        <v>Implementirani NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF i Lovćen PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; Hipotekarna i Lovćen podržavaju kartične stavke bez žiro računa; fallback tekstualni format ostaje aktivan.</v>
       </c>
     </row>
     <row r="340">

</xml_diff>

<commit_message>
Add Prva banka statement parser
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -1529,7 +1529,7 @@
         <v>F-076</v>
       </c>
       <c r="H21" t="str">
-        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF i Lovćen PDF rade, ostale banke ostaju otvorene.</v>
+        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF rade, ostale banke ostaju otvorene.</v>
       </c>
     </row>
     <row r="22">
@@ -10769,7 +10769,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H9" t="str">
-        <v>Prva MVP osnova postoji: tabele, NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF i Lovćen PDF uvoz/paste teksta, preview stavki, predlog naloga, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i alokacije KIF/KUF.</v>
+        <v>Prva MVP osnova postoji: tabele, NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF uvoz/paste teksta, preview stavki, predlog naloga, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i alokacije KIF/KUF.</v>
       </c>
     </row>
     <row r="10">
@@ -13846,7 +13846,7 @@
         <v>M-005,F-017</v>
       </c>
       <c r="L338" t="str">
-        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF i Lovćen PDF, a puna import sesija ostaje za kasnije.</v>
+        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF, a puna import sesija ostaje za kasnije.</v>
       </c>
     </row>
     <row r="339">
@@ -13884,7 +13884,7 @@
         <v>F-076</v>
       </c>
       <c r="L339" t="str">
-        <v>Implementirani NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF i Lovćen PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; Hipotekarna i Lovćen podržavaju kartične stavke bez žiro računa; fallback tekstualni format ostaje aktivan.</v>
+        <v>Implementirani NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; Hipotekarna i Lovćen podržavaju kartične stavke bez žiro računa; fallback tekstualni format ostaje aktivan.</v>
       </c>
     </row>
     <row r="340">

</xml_diff>

<commit_message>
Dodaj NLB PDF parser izvoda
- Čita zaglavlje, račun firme, početno/krajnje stanje i rekapitulaciju
- Parsira tabelarne stavke po koordinatama, uključujući višestranične izvode
- Ažurirani docs/accounting/izvodi.md, CURRENT_STATE.md, SESSION_LOG.md i planer
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -1529,7 +1529,7 @@
         <v>F-076</v>
       </c>
       <c r="H21" t="str">
-        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF rade, ostale banke ostaju otvorene.</v>
+        <v>Na /agencija/izvodi postoji izbor bankovnog računa, konta banke, PDF/HTML/XML fajla i paste teksta; NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF rade, ostale banke ostaju otvorene.</v>
       </c>
     </row>
     <row r="22">
@@ -10769,7 +10769,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H9" t="str">
-        <v>Prva MVP osnova postoji: tabele, NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF uvoz/paste teksta, preview stavki, predlog naloga, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i alokacije KIF/KUF.</v>
+        <v>Prva MVP osnova postoji: tabele, NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF uvoz/paste teksta, preview stavki, predlog naloga, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i alokacije KIF/KUF.</v>
       </c>
     </row>
     <row r="10">
@@ -13846,7 +13846,7 @@
         <v>M-005,F-017</v>
       </c>
       <c r="L338" t="str">
-        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF, a puna import sesija ostaje za kasnije.</v>
+        <v>Postoji upload/paste tekst i čuvanje izvoda; podržani su NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF, a puna import sesija ostaje za kasnije.</v>
       </c>
     </row>
     <row r="339">
@@ -13884,7 +13884,7 @@
         <v>F-076</v>
       </c>
       <c r="L339" t="str">
-        <v>Implementirani NLB XML, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; Hipotekarna i Lovćen podržavaju kartične stavke bez žiro računa; fallback tekstualni format ostaje aktivan.</v>
+        <v>Implementirani NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri; CKB ukupni priliv/odliv uzima iz zaglavlja PDF izvoda; Hipotekarna i Lovćen podržavaju kartične stavke bez žiro računa; fallback tekstualni format ostaje aktivan.</v>
       </c>
     </row>
     <row r="340">

</xml_diff>

<commit_message>
Implementiraj obrasce zavrsnog racuna
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -415,7 +415,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -468,9 +468,26 @@
         <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Zavrsni racun</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Djelimicno implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -13912,13 +13929,13 @@
         <v>Završni račun</v>
       </c>
       <c r="H13" t="str">
-        <v>U planu</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="I13" t="str">
         <v>MVP 3</v>
       </c>
       <c r="J13" t="str">
-        <v>Nije implementirano. Zavisi od bruto bilansa, početnog stanja i zatvaranja konta.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statistički aneks su implementirani iz POSTED naloga sa sistemskim šemama, podešavanjima po firmi i print obrascima. Ostaju ručni iznosi, arhiva, XML/export i zaključna knjiženja.</v>
       </c>
     </row>
     <row r="14">
@@ -14226,7 +14243,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="E12" t="str">
-        <v>U planu</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="F12" t="str">
         <v>Računovođa</v>
@@ -14235,7 +14252,7 @@
         <v>MVP 3</v>
       </c>
       <c r="H12" t="str">
-        <v>Nije implementirano. Zavisi od bruto bilansa, početnog stanja i zatvaranja konta.</v>
+        <v>Prva implementacija Bilansa uspjeha, Bilansa stanja i Statističkog aneksa postoji: šabloni pozicija, obračun iz POSTED naloga, prethodne kolone, podešavanja konta/formula po firmi i print obrasci. Ostaju ručni iznosi, arhiva, XML/export i zaključna knjiženja.</v>
       </c>
     </row>
     <row r="13">
@@ -14299,7 +14316,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z347"/>
+  <dimension ref="A1:Z350"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17579,9 +17596,123 @@
         <v>Provjeriti prava, zaključanu godinu i upisati audit log.</v>
       </c>
     </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>F-086</v>
+      </c>
+      <c r="B348" t="str">
+        <v>Zavrsni racun</v>
+      </c>
+      <c r="C348" t="str">
+        <v>Bilans uspjeha</v>
+      </c>
+      <c r="D348" t="str">
+        <v>Bilans uspjeha se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
+      </c>
+      <c r="E348" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F348" t="str">
+        <v>Djelimicno implementirano</v>
+      </c>
+      <c r="G348" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H348" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I348" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J348" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="K348" t="str">
+        <v>M-003,M-008,F-038</v>
+      </c>
+      <c r="L348" t="str">
+        <v>Sistemska sema je seedovana u finansijski_izvjestaj_sabloni/pozicije; firma moze izmijeniti konta, izuzetke i formule kroz podesavanja. Rucni iznosi i arhiva ostaju za doradu.</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>F-087</v>
+      </c>
+      <c r="B349" t="str">
+        <v>Zavrsni racun</v>
+      </c>
+      <c r="C349" t="str">
+        <v>Bilans stanja</v>
+      </c>
+      <c r="D349" t="str">
+        <v>Bilans stanja se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu godinu, prethodnu godinu - krajnje stanje i prethodnu godinu - pocetno stanje.</v>
+      </c>
+      <c r="E349" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F349" t="str">
+        <v>Djelimicno implementirano</v>
+      </c>
+      <c r="G349" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H349" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I349" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J349" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="K349" t="str">
+        <v>M-003,M-008,F-038</v>
+      </c>
+      <c r="L349" t="str">
+        <v>Dodati sistemski sablon, obracun, podesavanja po firmi i HTML/CSS print obrazac. Rucni iznosi i arhiva ostaju za doradu.</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>F-088</v>
+      </c>
+      <c r="B350" t="str">
+        <v>Zavrsni racun</v>
+      </c>
+      <c r="C350" t="str">
+        <v>Statisticki aneks</v>
+      </c>
+      <c r="D350" t="str">
+        <v>Statisticki aneks se racuna iz POSTED naloga po podesivoj semi pozicija, prikazuje tekucu i prethodnu godinu i stampa formalni obrazac.</v>
+      </c>
+      <c r="E350" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F350" t="str">
+        <v>Djelimicno implementirano</v>
+      </c>
+      <c r="G350" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H350" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I350" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J350" t="str">
+        <v>Djelimicno</v>
+      </c>
+      <c r="K350" t="str">
+        <v>M-003,M-008,F-038</v>
+      </c>
+      <c r="L350" t="str">
+        <v>Dodat sistemski sablon, obracun, podesavanja po firmi i HTML/CSS print obrazac. Rucni podaci kao prosjecan broj zaposlenih ostaju za doradu.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z347"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z350"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dodaj arhivu i zakljucna knjizenja zavrsnog racuna
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,26 +3,27 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-07-06" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-07-05" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-07-02" sheetId="3" r:id="rId3"/>
-    <sheet name="Status 2026-06-30" sheetId="4" r:id="rId4"/>
-    <sheet name="Status 2026-06-29" sheetId="5" r:id="rId5"/>
-    <sheet name="Status 2026-06-28" sheetId="6" r:id="rId6"/>
-    <sheet name="Status 2026-06-25" sheetId="7" r:id="rId7"/>
-    <sheet name="Dashboard" sheetId="8" r:id="rId8"/>
-    <sheet name="Moduli" sheetId="9" r:id="rId9"/>
-    <sheet name="Funkcionalnosti" sheetId="10" r:id="rId10"/>
-    <sheet name="Pravila" sheetId="11" r:id="rId11"/>
-    <sheet name="Zavisnosti" sheetId="12" r:id="rId12"/>
-    <sheet name="Ekrani" sheetId="13" r:id="rId13"/>
-    <sheet name="Baza" sheetId="14" r:id="rId14"/>
-    <sheet name="API" sheetId="15" r:id="rId15"/>
-    <sheet name="Testovi" sheetId="16" r:id="rId16"/>
-    <sheet name="Bugovi" sheetId="17" r:id="rId17"/>
-    <sheet name="Ideje" sheetId="18" r:id="rId18"/>
-    <sheet name="Odluke" sheetId="19" r:id="rId19"/>
-    <sheet name="Kategorije" sheetId="20" r:id="rId20"/>
+    <sheet name="Status 2026-07-07" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-07-06" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-07-05" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-07-02" sheetId="4" r:id="rId4"/>
+    <sheet name="Status 2026-06-30" sheetId="5" r:id="rId5"/>
+    <sheet name="Status 2026-06-29" sheetId="6" r:id="rId6"/>
+    <sheet name="Status 2026-06-28" sheetId="7" r:id="rId7"/>
+    <sheet name="Status 2026-06-25" sheetId="8" r:id="rId8"/>
+    <sheet name="Dashboard" sheetId="9" r:id="rId9"/>
+    <sheet name="Moduli" sheetId="10" r:id="rId10"/>
+    <sheet name="Funkcionalnosti" sheetId="11" r:id="rId11"/>
+    <sheet name="Pravila" sheetId="12" r:id="rId12"/>
+    <sheet name="Zavisnosti" sheetId="13" r:id="rId13"/>
+    <sheet name="Ekrani" sheetId="14" r:id="rId14"/>
+    <sheet name="Baza" sheetId="15" r:id="rId15"/>
+    <sheet name="API" sheetId="16" r:id="rId16"/>
+    <sheet name="Testovi" sheetId="17" r:id="rId17"/>
+    <sheet name="Bugovi" sheetId="18" r:id="rId18"/>
+    <sheet name="Ideje" sheetId="19" r:id="rId19"/>
+    <sheet name="Odluke" sheetId="20" r:id="rId20"/>
+    <sheet name="Kategorije" sheetId="21" r:id="rId21"/>
   </sheets>
 </workbook>
 </file>
@@ -416,7 +417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,63 +438,336 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Partneri</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B2" t="str">
-        <v>Implementirano</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
       </c>
       <c r="D2" t="str">
-        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
       </c>
       <c r="E2" t="str">
-        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Zavrsni racun</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Djelimicno implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce i trajne rucne korekcije po AOP/koloni.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije i primjenjuju prije ponovnog racunanja formula.</v>
+        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Z301"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Moduli aplikacije</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Glavni moduli računovodstvenog programa. Prva 3 modula su popunjena zaključcima iz razrade.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Opis</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Prioritet</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Vlasnik</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Faza</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>M-001</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Multi-agency struktura, super admin, admin agencije, radnici, klijenti, pretplate, prava pristupa, audit log.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Admin sistema</v>
+      </c>
+      <c r="G5" t="str">
+        <v>MVP 1</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Autentifikacija, agencije, korisnici, radnici/klijenti, dodjela firmi, matrica prava i audit osnova postoje. Ostaju kompletan backend enforcement prava, pretplate/limiti i statistika radnika.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>M-002</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Firme, klijenti, poslovne godine i kontni plan</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Firma kao centralni entitet: PIB, IRMS, poslovne godine, PDV status, banke, klijenti, radnici, ugovor/cijena i osnovni kontni plan + override po firmi.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Admin agencije</v>
+      </c>
+      <c r="G6" t="str">
+        <v>MVP 1</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Firme, IRMS, poslovne godine, aktivni kontekst firma/godina, banke, ugovori, kontni plan globalni + override, partneri globalni/agencijski/firmski su implementirani. Ostaju fina podesavanja firme, odgovorna lica i default konta.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>M-003</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Srce knjigovodstva: vrste naloga, numeracija, zaglavlje, stavke, nacrti, proknjiženi nalozi, početno stanje, partneri, analitika i bruto bilans.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Računovođa / Backend</v>
+      </c>
+      <c r="G7" t="str">
+        <v>MVP 1</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke iz ručnog naloga, datumi stavki, prečice F9/F10, bruto bilans, analitičke kartice i print su implementirani. Ostaju početno stanje i dodatne kontrole/testovi.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>M-004</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Dokumenti, kalkulacije, ulazne/izlazne fakture, roba, zalihe, lager, marže, maloprodaja/veleprodaja i automatska knjiženja.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Specifikacija spremna / nije implementirano</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Računovođa</v>
+      </c>
+      <c r="G8" t="str">
+        <v>MVP 1/2</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Specifikacija je pročitana i unesena u planer, ali modul nije krenuo u kodu osim navigacionih placeholdera.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>M-005</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Izvodi i automatsko knjiženje</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Uvoz PDF/HTML/XML izvoda, import sesije, preview, prepoznavanje komitenata po žiro računu, povezivanje sa KIF/KUF fakturama, pravila knjiženja i automatski nalog.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Računovođa</v>
+      </c>
+      <c r="G9" t="str">
+        <v>MVP 2</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Prva MVP osnova postoji: tabele, NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF uvoz/paste teksta, preview stavki, predlog naloga, osnovno zatvaranje KIF/KUF računa, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i split alokacije jedne uplate na više računa.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>M-006</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Zaposleni, ugovori, obračun plata, IOPPD/JPR veze, obaveze, automatski nalog plata.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E10" t="str">
+        <v>U planu</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Računovođa</v>
+      </c>
+      <c r="G10" t="str">
+        <v>MVP 2</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Nije implementirano.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>M-007</v>
+      </c>
+      <c r="B11" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="C11" t="str">
+        <v>PDV evidencije, kontrole, PDV prijava, XML, ulazni/izlazni PDV, firme van PDV sistema.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Implementirano djelimicno</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Računovođa</v>
+      </c>
+      <c r="G11" t="str">
+        <v>MVP 2</v>
+      </c>
+      <c r="H11" t="str">
+        <v>PDV stope, mjesečni periodi, ulazni/izlazni PDV evidencije, nacrt PDV prijave, korekcije, podešavanja knjiženja, XML snapshot i osnovno knjiženje su implementirani. Ostaju finalno IRMS XML mapiranje, zaključavanje perioda i jači QA.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>M-008</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Završni račun</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Pravila završnog računa, šeme, automatska zatvaranja, prenos početnog stanja.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Računovođa</v>
+      </c>
+      <c r="G12" t="str">
+        <v>MVP 3</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Prva implementacija Bilansa uspjeha, Bilansa stanja i Statističkog aneksa postoji: šabloni pozicija, obračun iz POSTED naloga, prethodne kolone, podešavanja konta/formula po firmi, trajne ručne korekcije po AOP/koloni, print obrasci, predlog zaključnog naloga za klase 5/6 i arhiva snimljenih obrazaca. Ostaje XML/export.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>M-009</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Izvještaji i dashboard</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Bruto bilans, glavna knjiga, kartice, partneri, radni učinak, statusi firmi.</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Admin agencije</v>
+      </c>
+      <c r="G13" t="str">
+        <v>MVP 1/2</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Bruto bilans i analitičke kartice postoje. Dashboard i ostali izvještaji su uglavnom placeholderi.</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>M-010</v>
+      </c>
+      <c r="B301" t="str">
+        <v>Računi / KIF-KUF</v>
+      </c>
+      <c r="C301" t="str">
+        <v>Kreiranje izlaznih faktura bez fiskalizacije u prvoj verziji; fakture razdužuju magacin i kasnije se automatski knjiže.</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="F301" t="str">
+        <v>Računovođa / Backend</v>
+      </c>
+      <c r="G301" t="str">
+        <v>MVP 1</v>
+      </c>
+      <c r="H301" t="str">
+        <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa, print i Excel export su implementirani. Ostaju kontrole, XML export, PDV zaključavanje i QA.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z301"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z350"/>
   <sheetData>
@@ -3896,7 +4170,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z362"/>
   <sheetData>
@@ -7221,7 +7495,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z309"/>
   <sheetData>
@@ -7753,7 +8027,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z330"/>
   <sheetData>
@@ -8957,7 +9231,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z341"/>
   <sheetData>
@@ -10573,7 +10847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z350"/>
   <sheetData>
@@ -13330,7 +13604,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB344"/>
   <sheetData>
@@ -15082,7 +15356,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -15132,7 +15406,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -15565,732 +15839,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:Z308"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z319"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Odluke</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Ključne arhitektonske i poslovne odluke donesene tokom razrade.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ODL-003</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Partneri</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Globalni partneri su centralni i dodaje ih samo sistemski admin; agencije mogu dodavati AGENCY/COMPANY partnere.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Prihvaćeno</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Codex</v>
-      </c>
-      <c r="F3">
-        <v>46193.083333333336</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ID odluke</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Datum</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Odluka</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Zašto</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Važi za</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Status</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>O-001</v>
-      </c>
-      <c r="B5">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Aplikacija je multi-agency SaaS</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Program se prodaje agencijama, svaka agencija ima svoj prostor.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Cijeli sistem</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>O-002</v>
-      </c>
-      <c r="B6">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Super admin ne mora operativno ulaziti u podatke agencija</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Zbog privatnosti i odvajanja odgovornosti.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Korisnici i prava</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Tehnička podrška može biti posebno pravo.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>O-003</v>
-      </c>
-      <c r="B7">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Admin agencije može i operativno knjižiti</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Admin agencije nije samo administrator nego može raditi kao računovođa.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Korisnici i prava</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Njegov rad se evidentira.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>O-004</v>
-      </c>
-      <c r="B8">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C8" t="str">
-        <v>PIB je unique po agenciji, ne globalno</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Ista firma može preći kod druge agencije.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Firme</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G8" t="str">
-        <v>UNIQUE agency_id + pib.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>O-005</v>
-      </c>
-      <c r="B9">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Sve se vodi po poslovnoj godini</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Nalozi, dokumenti, PDV, plate, izvještaji i završni moraju biti po godini.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Firme / Nalozi</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>O-006</v>
-      </c>
-      <c r="B10">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Firma pri kreiranju dobija tekuću poslovnu godinu</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Da se odmah može početi rad.</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Firme</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>O-007</v>
-      </c>
-      <c r="B11">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Kontni plan se ne kopira po firmi</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Baza bi bila ogromna; koristi se osnovni plan + override.</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Kontni plan</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>O-008</v>
-      </c>
-      <c r="B12">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Nalozi imaju nacrt i proknjižen status</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Nacrt ne ulazi u knjige, POSTED ulazi.</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>O-009</v>
-      </c>
-      <c r="B13">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Nema storna u prvoj verziji</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Da se ne komplikuje MVP.</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Soft delete + audit log + vraćanje u nacrt.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>O-010</v>
-      </c>
-      <c r="B14">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Jedna firma/godina ima samo jedno početno stanje</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Početno stanje mora biti jasno i posebno u bruto bilansu.</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="F14" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>O-011</v>
-      </c>
-      <c r="B15">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Partneri su zajednička tabela</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Jedan partner može biti i kupac i dobavljač.</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Nalozi / Analitika</v>
-      </c>
-      <c r="F15" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>O-012</v>
-      </c>
-      <c r="B16">
-        <v>46183.083333333336</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Sljedeći modul je robno knjigovodstvo</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Dokumenti, kalkulacije, fakture, roba i zalihe čine robni dio i traže posebnu razradu.</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="F16" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="str">
-        <v>O-013</v>
-      </c>
-      <c r="B301">
-        <v>46190.083333333336</v>
-      </c>
-      <c r="C301" t="str">
-        <v>Aktivna firma i poslovna godina se biraju globalno u top baru</v>
-      </c>
-      <c r="D301" t="str">
-        <v>Korisnik mora uvijek znati na kojoj firmi i godini radi prije unosa naloga/dokumenata.</v>
-      </c>
-      <c r="E301" t="str">
-        <v>Firme, nalozi, svi operativni moduli</v>
-      </c>
-      <c r="F301" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="G301" t="str">
-        <v>Izbor se pamti u cookie-ju; radnik vidi samo dodijeljene firme.</v>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="str">
-        <v>O-014</v>
-      </c>
-      <c r="B302">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C302" t="str">
-        <v>Modul 4 je kompletno robno knjigovodstvo</v>
-      </c>
-      <c r="D302" t="str">
-        <v>Obuhvata više od samog lagera: artikle, kalkulacije, povrate, popis, otpis i nivelaciju.</v>
-      </c>
-      <c r="E302" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="F302" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="str">
-        <v>O-015</v>
-      </c>
-      <c r="B303">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C303" t="str">
-        <v>Artikli su po firmi</v>
-      </c>
-      <c r="D303" t="str">
-        <v>Ista šifra/naziv kod različitih firmi ne mora značiti isto.</v>
-      </c>
-      <c r="E303" t="str">
-        <v>Artikli</v>
-      </c>
-      <c r="F303" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="str">
-        <v>O-016</v>
-      </c>
-      <c r="B304">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C304" t="str">
-        <v>Zalihe se vode po magacinu</v>
-      </c>
-      <c r="D304" t="str">
-        <v>Firma može imati više magacina i stanja robe.</v>
-      </c>
-      <c r="E304" t="str">
-        <v>Magacini / Lager</v>
-      </c>
-      <c r="F304" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="str">
-        <v>O-017</v>
-      </c>
-      <c r="B305">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C305" t="str">
-        <v>Razduženje po prosječnoj ponderisanoj cijeni</v>
-      </c>
-      <c r="D305" t="str">
-        <v>To je osnovni metod za nabavnu vrijednost prodate robe.</v>
-      </c>
-      <c r="E305" t="str">
-        <v>Lager</v>
-      </c>
-      <c r="F305" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="str">
-        <v>O-018</v>
-      </c>
-      <c r="B306">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C306" t="str">
-        <v>Negativan lager je podesiv</v>
-      </c>
-      <c r="D306" t="str">
-        <v>Nekome treba blokada, a nekome mogućnost rada u minus.</v>
-      </c>
-      <c r="E306" t="str">
-        <v>Lager</v>
-      </c>
-      <c r="F306" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G306" t="str">
-        <v>Podešavanje po firmi i opciono po magacinu.</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="str">
-        <v>O-019</v>
-      </c>
-      <c r="B307">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C307" t="str">
-        <v>Kalkulacija uvijek zadužuje magacin</v>
-      </c>
-      <c r="D307" t="str">
-        <v>Ako ne zadužuje magacin, nije kalkulacija.</v>
-      </c>
-      <c r="E307" t="str">
-        <v>Kalkulacije</v>
-      </c>
-      <c r="F307" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="str">
-        <v>O-020</v>
-      </c>
-      <c r="B308">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C308" t="str">
-        <v>Uvozna kalkulacija je poseban tip</v>
-      </c>
-      <c r="D308" t="str">
-        <v>Kod uvoza je roba bez PDV-a, a PDV dolazi iz carinske deklaracije.</v>
-      </c>
-      <c r="E308" t="str">
-        <v>Uvoz</v>
-      </c>
-      <c r="F308" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G308" t="str">
-        <v>Ulazna PDV stopa stavki je 0%.</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="str">
-        <v>O-021</v>
-      </c>
-      <c r="B309">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C309" t="str">
-        <v>Povrat dobavljaču je poseban dokument</v>
-      </c>
-      <c r="D309" t="str">
-        <v>Jasniji lager, PDV i knjiženje nego minus kalkulacija.</v>
-      </c>
-      <c r="E309" t="str">
-        <v>Povrat dobavljaču</v>
-      </c>
-      <c r="F309" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G309" t="str">
-        <v>Može biti slobodan ili povezan sa kalkulacijom.</v>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="str">
-        <v>O-022</v>
-      </c>
-      <c r="B310">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C310" t="str">
-        <v>Faktura razdužuje robu</v>
-      </c>
-      <c r="D310" t="str">
-        <v>Izlazna faktura sa robom mora skinuti robu sa lagera.</v>
-      </c>
-      <c r="E310" t="str">
-        <v>Fakture / Robno</v>
-      </c>
-      <c r="F310" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="str">
-        <v>O-023</v>
-      </c>
-      <c r="B311">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C311" t="str">
-        <v>Prenos, popis, otpis i nivelacija su posebni dokumenti</v>
-      </c>
-      <c r="D311" t="str">
-        <v>Robno mora imati jasne dokumente za svaki promet i korekciju.</v>
-      </c>
-      <c r="E311" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="F311" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="str">
-        <v>O-024</v>
-      </c>
-      <c r="B312">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C312" t="str">
-        <v>Samo proknjiženi robni dokumenti utiču na lager</v>
-      </c>
-      <c r="D312" t="str">
-        <v>Nacrti ne smiju mijenjati stanje zaliha.</v>
-      </c>
-      <c r="E312" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="F312" t="str">
-        <v>Zaključeno</v>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="str">
-        <v>O-025</v>
-      </c>
-      <c r="B313">
-        <v>46193.083333333336</v>
-      </c>
-      <c r="C313" t="str">
-        <v>Fiskalizacija se ne radi u prvoj verziji</v>
-      </c>
-      <c r="D313" t="str">
-        <v>Fiskalizacija je složena i može usporiti MVP; prvo se rade izlazne fakture, razduženje magacina i automatsko knjiženje.</v>
-      </c>
-      <c r="E313" t="str">
-        <v>Izlazne fakture / Fiskalizacija</v>
-      </c>
-      <c r="F313" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G313" t="str">
-        <v>Kasnije kupiti gotov API ili razviti poseban modul.</v>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="str">
-        <v>ODL-004</v>
-      </c>
-      <c r="B314" t="str">
-        <v>Partneri</v>
-      </c>
-      <c r="C314" t="str">
-        <v>Globalni partneri se inicijalno pune importom iz stare MySQL/IRMS baze emails po PIB-u.</v>
-      </c>
-      <c r="D314" t="str">
-        <v>Prihvaćeno</v>
-      </c>
-      <c r="E314" t="str">
-        <v>Codex</v>
-      </c>
-      <c r="F314">
-        <v>46194.083333333336</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="str">
-        <v>O-025</v>
-      </c>
-      <c r="B315">
-        <v>46198.083333333336</v>
-      </c>
-      <c r="C315" t="str">
-        <v>KIF/KUF knjiga se knjiži u jedan nalog</v>
-      </c>
-      <c r="D315" t="str">
-        <v>Lakši pregled i dopunjavanje naknadno dodatih računa.</v>
-      </c>
-      <c r="E315" t="str">
-        <v>Računi / Nalozi</v>
-      </c>
-      <c r="F315" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G315" t="str">
-        <v>Ako se dodaju računi poslije prvog knjiženja, dopunjavaju se samo neproknjiženi računi na postojeći nalog.</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="str">
-        <v>O-026</v>
-      </c>
-      <c r="B316">
-        <v>46198.083333333336</v>
-      </c>
-      <c r="C316" t="str">
-        <v>Broj fiskalnog računa se prikazuje kao čisti broj</v>
-      </c>
-      <c r="D316" t="str">
-        <v>Korisniku ne trebaju kodovi kase/softvera u broju računa.</v>
-      </c>
-      <c r="E316" t="str">
-        <v>KIF/KUF/MAPR</v>
-      </c>
-      <c r="F316" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G316" t="str">
-        <v>Primjer: pt385eg871/1/2026/dl426pc243 se prikazuje i knjiži kao 1/2026.</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="str">
-        <v>O-027</v>
-      </c>
-      <c r="B317">
-        <v>46198.083333333336</v>
-      </c>
-      <c r="C317" t="str">
-        <v>Print izvještaji idu kao HTML/CSS print stranice</v>
-      </c>
-      <c r="D317" t="str">
-        <v>Jednostavnije od server-side PDF generisanja i dovoljno za Save as PDF.</v>
-      </c>
-      <c r="E317" t="str">
-        <v>Izvještaji/Štampa</v>
-      </c>
-      <c r="F317" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G317" t="str">
-        <v>PDF biblioteke koristiti primarno za čitanje PDF-a.</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="str">
-        <v>O-028</v>
-      </c>
-      <c r="B318">
-        <v>46202.083333333336</v>
-      </c>
-      <c r="C318" t="str">
-        <v>Izvodi ne dupliraju ručni nalog IZV</v>
-      </c>
-      <c r="D318" t="str">
-        <v>Ručni unos ostaje kroz postojeći nalog tipa Izvodi; modul izvoda je import/preview/povezivanje/knjiženje sloj koji generiše jedan nalog po izvodu.</v>
-      </c>
-      <c r="E318" t="str">
-        <v>Izvodi / Nalozi</v>
-      </c>
-      <c r="F318" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G318" t="str">
-        <v>Bez ove odluke bismo imali dva paralelna ručna toka za isti posao.</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="str">
-        <v>O-029</v>
-      </c>
-      <c r="B319">
-        <v>46202.083333333336</v>
-      </c>
-      <c r="C319" t="str">
-        <v>Komitent iz izvoda se primarno prepoznaje po žiro računu</v>
-      </c>
-      <c r="D319" t="str">
-        <v>Naziv iz banke je pomoćni signal jer banke često skraćuju ili mijenjaju nazive.</v>
-      </c>
-      <c r="E319" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="F319" t="str">
-        <v>Zaključeno</v>
-      </c>
-      <c r="G319" t="str">
-        <v>Koristi se normalized_account_number.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z319"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -16358,13 +15906,13 @@
         <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
       </c>
       <c r="D4" t="str">
-        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
+        <v>Arhiva generisanih obrazaca i XML/export.</v>
       </c>
       <c r="E4" t="str">
-        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
+        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
       </c>
     </row>
   </sheetData>
@@ -16376,6 +15924,732 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Z319"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Odluke</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Ključne arhitektonske i poslovne odluke donesene tokom razrade.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ODL-003</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Partneri</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Globalni partneri su centralni i dodaje ih samo sistemski admin; agencije mogu dodavati AGENCY/COMPANY partnere.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Prihvaćeno</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="F3">
+        <v>46193.083333333336</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ID odluke</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Datum</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Odluka</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Zašto</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Važi za</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>O-001</v>
+      </c>
+      <c r="B5">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Aplikacija je multi-agency SaaS</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Program se prodaje agencijama, svaka agencija ima svoj prostor.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Cijeli sistem</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>O-002</v>
+      </c>
+      <c r="B6">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Super admin ne mora operativno ulaziti u podatke agencija</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Zbog privatnosti i odvajanja odgovornosti.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Korisnici i prava</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Tehnička podrška može biti posebno pravo.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>O-003</v>
+      </c>
+      <c r="B7">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Admin agencije može i operativno knjižiti</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Admin agencije nije samo administrator nego može raditi kao računovođa.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Korisnici i prava</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Njegov rad se evidentira.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>O-004</v>
+      </c>
+      <c r="B8">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C8" t="str">
+        <v>PIB je unique po agenciji, ne globalno</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Ista firma može preći kod druge agencije.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Firme</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G8" t="str">
+        <v>UNIQUE agency_id + pib.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>O-005</v>
+      </c>
+      <c r="B9">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Sve se vodi po poslovnoj godini</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Nalozi, dokumenti, PDV, plate, izvještaji i završni moraju biti po godini.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Firme / Nalozi</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>O-006</v>
+      </c>
+      <c r="B10">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Firma pri kreiranju dobija tekuću poslovnu godinu</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Da se odmah može početi rad.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Firme</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>O-007</v>
+      </c>
+      <c r="B11">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Kontni plan se ne kopira po firmi</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Baza bi bila ogromna; koristi se osnovni plan + override.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Kontni plan</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>O-008</v>
+      </c>
+      <c r="B12">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Nalozi imaju nacrt i proknjižen status</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Nacrt ne ulazi u knjige, POSTED ulazi.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Nalozi</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>O-009</v>
+      </c>
+      <c r="B13">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Nema storna u prvoj verziji</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Da se ne komplikuje MVP.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Nalozi</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Soft delete + audit log + vraćanje u nacrt.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>O-010</v>
+      </c>
+      <c r="B14">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Jedna firma/godina ima samo jedno početno stanje</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Početno stanje mora biti jasno i posebno u bruto bilansu.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Nalozi</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>O-011</v>
+      </c>
+      <c r="B15">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Partneri su zajednička tabela</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Jedan partner može biti i kupac i dobavljač.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Nalozi / Analitika</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>O-012</v>
+      </c>
+      <c r="B16">
+        <v>46183.083333333336</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Sljedeći modul je robno knjigovodstvo</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Dokumenti, kalkulacije, fakture, roba i zalihe čine robni dio i traže posebnu razradu.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>O-013</v>
+      </c>
+      <c r="B301">
+        <v>46190.083333333336</v>
+      </c>
+      <c r="C301" t="str">
+        <v>Aktivna firma i poslovna godina se biraju globalno u top baru</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Korisnik mora uvijek znati na kojoj firmi i godini radi prije unosa naloga/dokumenata.</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Firme, nalozi, svi operativni moduli</v>
+      </c>
+      <c r="F301" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G301" t="str">
+        <v>Izbor se pamti u cookie-ju; radnik vidi samo dodijeljene firme.</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>O-014</v>
+      </c>
+      <c r="B302">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C302" t="str">
+        <v>Modul 4 je kompletno robno knjigovodstvo</v>
+      </c>
+      <c r="D302" t="str">
+        <v>Obuhvata više od samog lagera: artikle, kalkulacije, povrate, popis, otpis i nivelaciju.</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="F302" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>O-015</v>
+      </c>
+      <c r="B303">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C303" t="str">
+        <v>Artikli su po firmi</v>
+      </c>
+      <c r="D303" t="str">
+        <v>Ista šifra/naziv kod različitih firmi ne mora značiti isto.</v>
+      </c>
+      <c r="E303" t="str">
+        <v>Artikli</v>
+      </c>
+      <c r="F303" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>O-016</v>
+      </c>
+      <c r="B304">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C304" t="str">
+        <v>Zalihe se vode po magacinu</v>
+      </c>
+      <c r="D304" t="str">
+        <v>Firma može imati više magacina i stanja robe.</v>
+      </c>
+      <c r="E304" t="str">
+        <v>Magacini / Lager</v>
+      </c>
+      <c r="F304" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>O-017</v>
+      </c>
+      <c r="B305">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C305" t="str">
+        <v>Razduženje po prosječnoj ponderisanoj cijeni</v>
+      </c>
+      <c r="D305" t="str">
+        <v>To je osnovni metod za nabavnu vrijednost prodate robe.</v>
+      </c>
+      <c r="E305" t="str">
+        <v>Lager</v>
+      </c>
+      <c r="F305" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>O-018</v>
+      </c>
+      <c r="B306">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C306" t="str">
+        <v>Negativan lager je podesiv</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Nekome treba blokada, a nekome mogućnost rada u minus.</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Lager</v>
+      </c>
+      <c r="F306" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G306" t="str">
+        <v>Podešavanje po firmi i opciono po magacinu.</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>O-019</v>
+      </c>
+      <c r="B307">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C307" t="str">
+        <v>Kalkulacija uvijek zadužuje magacin</v>
+      </c>
+      <c r="D307" t="str">
+        <v>Ako ne zadužuje magacin, nije kalkulacija.</v>
+      </c>
+      <c r="E307" t="str">
+        <v>Kalkulacije</v>
+      </c>
+      <c r="F307" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>O-020</v>
+      </c>
+      <c r="B308">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C308" t="str">
+        <v>Uvozna kalkulacija je poseban tip</v>
+      </c>
+      <c r="D308" t="str">
+        <v>Kod uvoza je roba bez PDV-a, a PDV dolazi iz carinske deklaracije.</v>
+      </c>
+      <c r="E308" t="str">
+        <v>Uvoz</v>
+      </c>
+      <c r="F308" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G308" t="str">
+        <v>Ulazna PDV stopa stavki je 0%.</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>O-021</v>
+      </c>
+      <c r="B309">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C309" t="str">
+        <v>Povrat dobavljaču je poseban dokument</v>
+      </c>
+      <c r="D309" t="str">
+        <v>Jasniji lager, PDV i knjiženje nego minus kalkulacija.</v>
+      </c>
+      <c r="E309" t="str">
+        <v>Povrat dobavljaču</v>
+      </c>
+      <c r="F309" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G309" t="str">
+        <v>Može biti slobodan ili povezan sa kalkulacijom.</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>O-022</v>
+      </c>
+      <c r="B310">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C310" t="str">
+        <v>Faktura razdužuje robu</v>
+      </c>
+      <c r="D310" t="str">
+        <v>Izlazna faktura sa robom mora skinuti robu sa lagera.</v>
+      </c>
+      <c r="E310" t="str">
+        <v>Fakture / Robno</v>
+      </c>
+      <c r="F310" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>O-023</v>
+      </c>
+      <c r="B311">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C311" t="str">
+        <v>Prenos, popis, otpis i nivelacija su posebni dokumenti</v>
+      </c>
+      <c r="D311" t="str">
+        <v>Robno mora imati jasne dokumente za svaki promet i korekciju.</v>
+      </c>
+      <c r="E311" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="F311" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>O-024</v>
+      </c>
+      <c r="B312">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C312" t="str">
+        <v>Samo proknjiženi robni dokumenti utiču na lager</v>
+      </c>
+      <c r="D312" t="str">
+        <v>Nacrti ne smiju mijenjati stanje zaliha.</v>
+      </c>
+      <c r="E312" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="F312" t="str">
+        <v>Zaključeno</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>O-025</v>
+      </c>
+      <c r="B313">
+        <v>46193.083333333336</v>
+      </c>
+      <c r="C313" t="str">
+        <v>Fiskalizacija se ne radi u prvoj verziji</v>
+      </c>
+      <c r="D313" t="str">
+        <v>Fiskalizacija je složena i može usporiti MVP; prvo se rade izlazne fakture, razduženje magacina i automatsko knjiženje.</v>
+      </c>
+      <c r="E313" t="str">
+        <v>Izlazne fakture / Fiskalizacija</v>
+      </c>
+      <c r="F313" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G313" t="str">
+        <v>Kasnije kupiti gotov API ili razviti poseban modul.</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>ODL-004</v>
+      </c>
+      <c r="B314" t="str">
+        <v>Partneri</v>
+      </c>
+      <c r="C314" t="str">
+        <v>Globalni partneri se inicijalno pune importom iz stare MySQL/IRMS baze emails po PIB-u.</v>
+      </c>
+      <c r="D314" t="str">
+        <v>Prihvaćeno</v>
+      </c>
+      <c r="E314" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="F314">
+        <v>46194.083333333336</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>O-025</v>
+      </c>
+      <c r="B315">
+        <v>46198.083333333336</v>
+      </c>
+      <c r="C315" t="str">
+        <v>KIF/KUF knjiga se knjiži u jedan nalog</v>
+      </c>
+      <c r="D315" t="str">
+        <v>Lakši pregled i dopunjavanje naknadno dodatih računa.</v>
+      </c>
+      <c r="E315" t="str">
+        <v>Računi / Nalozi</v>
+      </c>
+      <c r="F315" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G315" t="str">
+        <v>Ako se dodaju računi poslije prvog knjiženja, dopunjavaju se samo neproknjiženi računi na postojeći nalog.</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>O-026</v>
+      </c>
+      <c r="B316">
+        <v>46198.083333333336</v>
+      </c>
+      <c r="C316" t="str">
+        <v>Broj fiskalnog računa se prikazuje kao čisti broj</v>
+      </c>
+      <c r="D316" t="str">
+        <v>Korisniku ne trebaju kodovi kase/softvera u broju računa.</v>
+      </c>
+      <c r="E316" t="str">
+        <v>KIF/KUF/MAPR</v>
+      </c>
+      <c r="F316" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G316" t="str">
+        <v>Primjer: pt385eg871/1/2026/dl426pc243 se prikazuje i knjiži kao 1/2026.</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>O-027</v>
+      </c>
+      <c r="B317">
+        <v>46198.083333333336</v>
+      </c>
+      <c r="C317" t="str">
+        <v>Print izvještaji idu kao HTML/CSS print stranice</v>
+      </c>
+      <c r="D317" t="str">
+        <v>Jednostavnije od server-side PDF generisanja i dovoljno za Save as PDF.</v>
+      </c>
+      <c r="E317" t="str">
+        <v>Izvještaji/Štampa</v>
+      </c>
+      <c r="F317" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G317" t="str">
+        <v>PDF biblioteke koristiti primarno za čitanje PDF-a.</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>O-028</v>
+      </c>
+      <c r="B318">
+        <v>46202.083333333336</v>
+      </c>
+      <c r="C318" t="str">
+        <v>Izvodi ne dupliraju ručni nalog IZV</v>
+      </c>
+      <c r="D318" t="str">
+        <v>Ručni unos ostaje kroz postojeći nalog tipa Izvodi; modul izvoda je import/preview/povezivanje/knjiženje sloj koji generiše jedan nalog po izvodu.</v>
+      </c>
+      <c r="E318" t="str">
+        <v>Izvodi / Nalozi</v>
+      </c>
+      <c r="F318" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G318" t="str">
+        <v>Bez ove odluke bismo imali dva paralelna ručna toka za isti posao.</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>O-029</v>
+      </c>
+      <c r="B319">
+        <v>46202.083333333336</v>
+      </c>
+      <c r="C319" t="str">
+        <v>Komitent iz izvoda se primarno prepoznaje po žiro računu</v>
+      </c>
+      <c r="D319" t="str">
+        <v>Naziv iz banke je pomoćni signal jer banke često skraćuju ili mijenjaju nazive.</v>
+      </c>
+      <c r="E319" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="F319" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="G319" t="str">
+        <v>Koristi se normalized_account_number.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z319"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
     <row r="1">
@@ -16565,106 +16839,79 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-07-02</v>
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
+        <v>Partneri</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Oblast</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B4" t="str">
-        <v>Status</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Sta je zavrseno</v>
+        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
       </c>
       <c r="D4" t="str">
-        <v>Sta ostaje</v>
+        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
       </c>
       <c r="E4" t="str">
-        <v>Preporuceni sljedeci korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C5" t="str">
-        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C7" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C8" t="str">
-        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Redovno održavanje.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Regenerisati Excel nakon svake veće promjene.</v>
+        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -16675,7 +16922,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-30</v>
+        <v>Status projekta na dan 2026-07-02</v>
       </c>
     </row>
     <row r="2">
@@ -16708,13 +16955,13 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
+        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
       </c>
       <c r="D5" t="str">
-        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
+        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
       </c>
       <c r="E5" t="str">
-        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
+        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
       </c>
     </row>
     <row r="6">
@@ -16777,11 +17024,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-29</v>
+        <v>Status projekta na dan 2026-06-30</v>
       </c>
     </row>
     <row r="2">
@@ -16808,92 +17055,75 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nalozi</v>
+        <v>Izvodi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core zaokruzen</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
+        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
       </c>
       <c r="D5" t="str">
-        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
       </c>
       <c r="E5" t="str">
-        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
+        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PDV</v>
+        <v>Nalozi</v>
       </c>
       <c r="B6" t="str">
-        <v>Core zaokruzen</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C6" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
       </c>
       <c r="D6" t="str">
-        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
+        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E6" t="str">
-        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
+        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Izvodi</v>
+        <v>PDV</v>
       </c>
       <c r="B7" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C7" t="str">
-        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D7" t="str">
-        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
+        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
       </c>
       <c r="E7" t="str">
-        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
+        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>KIF/KUF</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B8" t="str">
-        <v>Core implementiran</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C8" t="str">
-        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
+        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
       </c>
       <c r="D8" t="str">
-        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
+        <v>Redovno održavanje.</v>
       </c>
       <c r="E8" t="str">
-        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C9" t="str">
-        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Regenerisati Excel nakon svake vece promjene.</v>
+        <v>Regenerisati Excel nakon svake veće promjene.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -16904,12 +17134,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-28</v>
+        <v>Status projekta na dan 2026-06-29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
       </c>
     </row>
     <row r="4">
@@ -16931,87 +17161,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Performanse partnera</v>
+        <v>Nalozi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core implementiran</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C5" t="str">
-        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
       </c>
       <c r="D5" t="str">
-        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E5" t="str">
-        <v>Pratiti brzinu na produkciji.</v>
+        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Indeksi baze</v>
+        <v>PDV</v>
       </c>
       <c r="B6" t="str">
-        <v>Implementirano</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C6" t="str">
-        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D6" t="str">
-        <v>-</v>
+        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
       </c>
       <c r="E6" t="str">
-        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIF/KUF uvoz/export</v>
+        <v>Izvodi</v>
       </c>
       <c r="B7" t="str">
-        <v>Core implementiran</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
       </c>
       <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata; XML export.</v>
+        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
       </c>
       <c r="E7" t="str">
-        <v>QA uvoznih knjizenja i export fajlova.</v>
+        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dokumentacija</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="B8" t="str">
-        <v>Uspostavljeno</v>
+        <v>Core implementiran</v>
       </c>
       <c r="C8" t="str">
-        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
       </c>
       <c r="D8" t="str">
-        <v>Redovno odrzavanje.</v>
+        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
       </c>
       <c r="E8" t="str">
-        <v>Azurirati uz svaku vecu promjenu.</v>
+        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PDV</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B9" t="str">
-        <v>Prva implementacija</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C9" t="str">
-        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
       </c>
       <c r="D9" t="str">
-        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+        <v>Redovno odrzavanje.</v>
       </c>
       <c r="E9" t="str">
-        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+        <v>Regenerisati Excel nakon svake vece promjene.</v>
       </c>
     </row>
   </sheetData>
@@ -17023,6 +17253,129 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Performanse partnera</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pratiti brzinu na produkciji.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Indeksi baze</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KIF/KUF uvoz/export</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kontrole iznosa i duplikata; XML export.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>QA uvoznih knjizenja i export fajlova.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Dokumentacija</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Uspostavljeno</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Redovno odrzavanje.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Azurirati uz svaku vecu promjenu.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Prva implementacija</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
@@ -17195,7 +17548,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -17418,7 +17771,7 @@
         <v>MVP 3</v>
       </c>
       <c r="J13" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statistički aneks su implementirani iz POSTED naloga sa sistemskim šemama, podešavanjima po firmi, trajnim ručnim korekcijama po AOP/koloni i print obrascima. Ostaju arhiva, XML/export i zaključna knjiženja.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statistički aneks su implementirani iz POSTED naloga sa sistemskim šemama, podešavanjima po firmi, trajnim ručnim korekcijama po AOP/koloni, print obrascima, predlogom zaključnog naloga za klase 5/6 i arhivom snimljenih obrazaca. Ostaje XML/export.</v>
       </c>
     </row>
     <row r="14">
@@ -17488,311 +17841,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:Z300"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z301"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Moduli aplikacije</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Glavni moduli računovodstvenog programa. Prva 3 modula su popunjena zaključcima iz razrade.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ID</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Opis</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Prioritet</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Status</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Vlasnik</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Faza</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>M-001</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Korisnici, agencije i prava</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Multi-agency struktura, super admin, admin agencije, radnici, klijenti, pretplate, prava pristupa, audit log.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Admin sistema</v>
-      </c>
-      <c r="G5" t="str">
-        <v>MVP 1</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Autentifikacija, agencije, korisnici, radnici/klijenti, dodjela firmi, matrica prava i audit osnova postoje. Ostaju kompletan backend enforcement prava, pretplate/limiti i statistika radnika.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>M-002</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Firme, klijenti, poslovne godine i kontni plan</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Firma kao centralni entitet: PIB, IRMS, poslovne godine, PDV status, banke, klijenti, radnici, ugovor/cijena i osnovni kontni plan + override po firmi.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Admin agencije</v>
-      </c>
-      <c r="G6" t="str">
-        <v>MVP 1</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Firme, IRMS, poslovne godine, aktivni kontekst firma/godina, banke, ugovori, kontni plan globalni + override, partneri globalni/agencijski/firmski su implementirani. Ostaju fina podesavanja firme, odgovorna lica i default konta.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>M-003</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Srce knjigovodstva: vrste naloga, numeracija, zaglavlje, stavke, nacrti, proknjiženi nalozi, početno stanje, partneri, analitika i bruto bilans.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Računovođa / Backend</v>
-      </c>
-      <c r="G7" t="str">
-        <v>MVP 1</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke iz ručnog naloga, datumi stavki, prečice F9/F10, bruto bilans, analitičke kartice i print su implementirani. Ostaju početno stanje i dodatne kontrole/testovi.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>M-004</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Dokumenti, kalkulacije, ulazne/izlazne fakture, roba, zalihe, lager, marže, maloprodaja/veleprodaja i automatska knjiženja.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Specifikacija spremna / nije implementirano</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Računovođa</v>
-      </c>
-      <c r="G8" t="str">
-        <v>MVP 1/2</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Specifikacija je pročitana i unesena u planer, ali modul nije krenuo u kodu osim navigacionih placeholdera.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>M-005</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Izvodi i automatsko knjiženje</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Uvoz PDF/HTML/XML izvoda, import sesije, preview, prepoznavanje komitenata po žiro računu, povezivanje sa KIF/KUF fakturama, pravila knjiženja i automatski nalog.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Računovođa</v>
-      </c>
-      <c r="G9" t="str">
-        <v>MVP 2</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Prva MVP osnova postoji: tabele, NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF uvoz/paste teksta, preview stavki, predlog naloga, osnovno zatvaranje KIF/KUF računa, napredna pravila po računu/opisu/šifri/pozivu/prioritetu, zajednička i firm-specific pravila, prepoznavanje internih prenosa, knjiženje READY izvoda u poseban IZV nalog, te stranice obrada/parseri/žiro računi/kartica/kontrole. Otvoreno: parseri za ostale banke i split alokacije jedne uplate na više računa.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>M-006</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Plate i zaposleni</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Zaposleni, ugovori, obračun plata, IOPPD/JPR veze, obaveze, automatski nalog plata.</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E10" t="str">
-        <v>U planu</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Računovođa</v>
-      </c>
-      <c r="G10" t="str">
-        <v>MVP 2</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Nije implementirano.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>M-007</v>
-      </c>
-      <c r="B11" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="C11" t="str">
-        <v>PDV evidencije, kontrole, PDV prijava, XML, ulazni/izlazni PDV, firme van PDV sistema.</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Implementirano djelimicno</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Računovođa</v>
-      </c>
-      <c r="G11" t="str">
-        <v>MVP 2</v>
-      </c>
-      <c r="H11" t="str">
-        <v>PDV stope, mjesečni periodi, ulazni/izlazni PDV evidencije, nacrt PDV prijave, korekcije, podešavanja knjiženja, XML snapshot i osnovno knjiženje su implementirani. Ostaju finalno IRMS XML mapiranje, zaključavanje perioda i jači QA.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>M-008</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Završni račun</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Pravila završnog računa, šeme, automatska zatvaranja, prenos početnog stanja.</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Računovođa</v>
-      </c>
-      <c r="G12" t="str">
-        <v>MVP 3</v>
-      </c>
-      <c r="H12" t="str">
-        <v>Prva implementacija Bilansa uspjeha, Bilansa stanja i Statističkog aneksa postoji: šabloni pozicija, obračun iz POSTED naloga, prethodne kolone, podešavanja konta/formula po firmi, trajne ručne korekcije po AOP/koloni i print obrasci. Ostaju arhiva, XML/export i zaključna knjiženja.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>M-009</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Izvještaji i dashboard</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Bruto bilans, glavna knjiga, kartice, partneri, radni učinak, statusi firmi.</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Visok</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Admin agencije</v>
-      </c>
-      <c r="G13" t="str">
-        <v>MVP 1/2</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Bruto bilans i analitičke kartice postoje. Dashboard i ostali izvještaji su uglavnom placeholderi.</v>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="str">
-        <v>M-010</v>
-      </c>
-      <c r="B301" t="str">
-        <v>Računi / KIF-KUF</v>
-      </c>
-      <c r="C301" t="str">
-        <v>Kreiranje izlaznih faktura bez fiskalizacije u prvoj verziji; fakture razdužuju magacin i kasnije se automatski knjiže.</v>
-      </c>
-      <c r="D301" t="str">
-        <v>Vrlo visok</v>
-      </c>
-      <c r="E301" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="F301" t="str">
-        <v>Računovođa / Backend</v>
-      </c>
-      <c r="G301" t="str">
-        <v>MVP 1</v>
-      </c>
-      <c r="H301" t="str">
-        <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa, print i Excel export su implementirani. Ostaju kontrole, XML export, PDV zaključavanje i QA.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z301"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Dodaj MVP modul plata
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,27 +3,28 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-07-07" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-07-06" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-07-05" sheetId="3" r:id="rId3"/>
-    <sheet name="Status 2026-07-02" sheetId="4" r:id="rId4"/>
-    <sheet name="Status 2026-06-30" sheetId="5" r:id="rId5"/>
-    <sheet name="Status 2026-06-29" sheetId="6" r:id="rId6"/>
-    <sheet name="Status 2026-06-28" sheetId="7" r:id="rId7"/>
-    <sheet name="Status 2026-06-25" sheetId="8" r:id="rId8"/>
-    <sheet name="Dashboard" sheetId="9" r:id="rId9"/>
-    <sheet name="Moduli" sheetId="10" r:id="rId10"/>
-    <sheet name="Funkcionalnosti" sheetId="11" r:id="rId11"/>
-    <sheet name="Pravila" sheetId="12" r:id="rId12"/>
-    <sheet name="Zavisnosti" sheetId="13" r:id="rId13"/>
-    <sheet name="Ekrani" sheetId="14" r:id="rId14"/>
-    <sheet name="Baza" sheetId="15" r:id="rId15"/>
-    <sheet name="API" sheetId="16" r:id="rId16"/>
-    <sheet name="Testovi" sheetId="17" r:id="rId17"/>
-    <sheet name="Bugovi" sheetId="18" r:id="rId18"/>
-    <sheet name="Ideje" sheetId="19" r:id="rId19"/>
-    <sheet name="Odluke" sheetId="20" r:id="rId20"/>
-    <sheet name="Kategorije" sheetId="21" r:id="rId21"/>
+    <sheet name="Status 2026-07-09" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-07-07" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-07-06" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-07-05" sheetId="4" r:id="rId4"/>
+    <sheet name="Status 2026-07-02" sheetId="5" r:id="rId5"/>
+    <sheet name="Status 2026-06-30" sheetId="6" r:id="rId6"/>
+    <sheet name="Status 2026-06-29" sheetId="7" r:id="rId7"/>
+    <sheet name="Status 2026-06-28" sheetId="8" r:id="rId8"/>
+    <sheet name="Status 2026-06-25" sheetId="9" r:id="rId9"/>
+    <sheet name="Dashboard" sheetId="10" r:id="rId10"/>
+    <sheet name="Moduli" sheetId="11" r:id="rId11"/>
+    <sheet name="Funkcionalnosti" sheetId="12" r:id="rId12"/>
+    <sheet name="Pravila" sheetId="13" r:id="rId13"/>
+    <sheet name="Zavisnosti" sheetId="14" r:id="rId14"/>
+    <sheet name="Ekrani" sheetId="15" r:id="rId15"/>
+    <sheet name="Baza" sheetId="16" r:id="rId16"/>
+    <sheet name="API" sheetId="17" r:id="rId17"/>
+    <sheet name="Testovi" sheetId="18" r:id="rId18"/>
+    <sheet name="Bugovi" sheetId="19" r:id="rId19"/>
+    <sheet name="Ideje" sheetId="20" r:id="rId20"/>
+    <sheet name="Odluke" sheetId="21" r:id="rId21"/>
+    <sheet name="Kategorije" sheetId="22" r:id="rId22"/>
   </sheets>
 </workbook>
 </file>
@@ -438,19 +439,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Zavrsni racun</v>
+        <v>Plate</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimicno implementirano</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
+        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje i izmjenu zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za redovan obračun 001, pripremu radnika, ručne mjesečne korekcije i dodatne stavke; /agencija/plate/podesavanja za pregled šifarnika.</v>
       </c>
       <c r="D2" t="str">
-        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
+        <v>Ugovori, obustave, IOPPD/JPR, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
       </c>
       <c r="E2" t="str">
-        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
+        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki.</v>
       </c>
     </row>
   </sheetData>
@@ -462,6 +463,301 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Z300"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Računovodstveni program — Master planer</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Ažurirano 2026-06-25: Core modula 1-3 je upotrebljiv, KIF/KUF modul je implementiran za unos, import, automatsko knjiženje i štampu; ostaju kontrole, export, PDV zaključavanje, početno stanje i testovi.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Broj stavki</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Zaključeno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Napomena</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Status modula</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Moduli</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Prva 3 modula su zaključena.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>ID</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Status</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Faza</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Funkcionalnosti</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Za praćenje implementacije.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>M-001</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="I6" t="str">
+        <v>MVP 1</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Autentifikacija, agencije, korisnici, radnici/klijenti, dodjela firmi, matrica prava i audit osnova postoje. Ostaju kompletan backend enforcement prava, pretplate/limiti i statistika radnika.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Pravila</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Poslovna logika.</v>
+      </c>
+      <c r="F7" t="str">
+        <v>M-002</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Firme, klijenti, poslovne godine i kontni plan</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="I7" t="str">
+        <v>MVP 1</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Firme, IRMS, poslovne godine, aktivni kontekst firma/godina, banke, ugovori, kontni plan globalni + override, partneri globalni/agencijski/firmski su implementirani. Ostaju fina podesavanja firme, odgovorna lica i default konta.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Baza</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Predlog tabela.</v>
+      </c>
+      <c r="F8" t="str">
+        <v>M-003</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Nalozi za knjiženje</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="I8" t="str">
+        <v>MVP 1</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke iz ručnog naloga, datumi stavki, prečice F9/F10, bruto bilans, analitičke kartice i print su implementirani. Ostaju početno stanje i dodatne kontrole/testovi.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>API</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Predlog ruta.</v>
+      </c>
+      <c r="F9" t="str">
+        <v>M-004</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Robno knjigovodstvo</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Specifikacija spremna / nije implementirano</v>
+      </c>
+      <c r="I9" t="str">
+        <v>MVP 1/2</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Specifikacija je pročitana i unesena u planer, ali modul nije krenuo u kodu osim navigacionih placeholdera.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Testovi</v>
+      </c>
+      <c r="D10" t="str">
+        <v>QA scenariji.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>M-005</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Izvodi i automatsko knjiženje</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Specifikacija spremna / nije implementirano</v>
+      </c>
+      <c r="I10" t="str">
+        <v>MVP 2</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Finalna specifikacija je u zadaci/07_Izvodi_i_Automatsko_Knjizenje_FINAL.md. Sljedeće: import sesije, PDF/HTML parser, preview, povezivanje sa komitentima/fakturama i generisanje naloga.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Odluke</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Arhitektonske odluke.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>M-006</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="I11" t="str">
+        <v>MVP 2</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Prva MVP osnova postoji: zaposleni sa dodavanjem/izmjenom i tabovima aktivni/neaktivni, šifarnici plata, redovan obračun 001, priprema radnika u nacrtu, ručne korekcije stavki i dodatne stavke po radniku. Bruto/neto servis čita pravila iz baze. Ostaju ugovori, obustave, IOPPD/JPR, uplatnice, knjiženje i print/export.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="F12" t="str">
+        <v>M-007</v>
+      </c>
+      <c r="G12" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Djelimično kroz KIF/KUF</v>
+      </c>
+      <c r="I12" t="str">
+        <v>MVP 2</v>
+      </c>
+      <c r="J12" t="str">
+        <v>PDV stope i osnovne KIF/KUF PDV razrade postoje. PDV prijava, kontrole i XML nisu implementirani.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="F13" t="str">
+        <v>M-008</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Završni račun</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="I13" t="str">
+        <v>MVP 3</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Bilans uspjeha, Bilans stanja i Statistički aneks su implementirani iz POSTED naloga sa sistemskim šemama, podešavanjima po firmi, trajnim ručnim korekcijama po AOP/koloni, print obrascima, predlogom zaključnog naloga za klase 5/6 i arhivom snimljenih obrazaca. Ostaje XML/export.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Sljedeći prioritet</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Završiti KIF/KUF kontrole i testove, pa odlučiti PDV ili Robno</v>
+      </c>
+      <c r="F14" t="str">
+        <v>M-009</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Izvještaji i dashboard</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="I14" t="str">
+        <v>MVP 1/2</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Bruto bilans i analitičke kartice postoje. Dashboard i ostali izvještaji su uglavnom placeholderi.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Obuhvat</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Dokumenti, kalkulacije, ulazne/izlazne fakture, roba, zalihe, lager, maloprodaja/veleprodaja, automatska knjiženja.</v>
+      </c>
+      <c r="F15" t="str">
+        <v>M-010</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Računi / KIF-KUF</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="I15" t="str">
+        <v>MVP 1</v>
+      </c>
+      <c r="J15" t="str">
+        <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa i print su implementirani. Ostaju kontrole, export, PDV zaključavanje i QA.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Zašto sada</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Zavisi od firme, kontnog plana, partnera i naloga koje smo sada definisali.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Napomena</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Biće dosta pravila, zato je dobro da se radi odvojeno i temeljno.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z300"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z301"/>
   <sheetData>
     <row r="1">
@@ -644,7 +940,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="E10" t="str">
-        <v>U planu</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="F10" t="str">
         <v>Računovođa</v>
@@ -653,7 +949,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H10" t="str">
-        <v>Nije implementirano.</v>
+        <v>Prva MVP osnova postoji: tabele i šifarnici za IOPPD, vrste obračuna, poreze, doprinose, prirez i šifre primanja; stranice za zaposlene sa dodavanjem, izmjenom i tabovima aktivni/neaktivni, redovan obračun 001, priprema radnika u nacrtu, ručne mjesečne korekcije po radniku i dodatne stavke; bruto/neto obračun čita pravila iz baze. Ostaju ugovori, obustave, IOPPD/JPR, uplatnice, knjiženje i print/export.</v>
       </c>
     </row>
     <row r="11">
@@ -767,7 +1063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z350"/>
   <sheetData>
@@ -4170,7 +4466,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z362"/>
   <sheetData>
@@ -7495,7 +7791,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z309"/>
   <sheetData>
@@ -8027,7 +8323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z330"/>
   <sheetData>
@@ -9231,7 +9527,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z341"/>
   <sheetData>
@@ -10847,7 +11143,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z350"/>
   <sheetData>
@@ -13604,7 +13900,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB344"/>
   <sheetData>
@@ -15356,7 +15652,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -15406,7 +15702,52 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Zavrsni racun</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Djelimicno implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -15843,86 +16184,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Partneri</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Zavrsni racun</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Djelimicno implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Arhiva generisanih obrazaca i XML/export.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z319"/>
   <sheetData>
@@ -16648,7 +16910,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -16900,13 +17162,13 @@
         <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
       </c>
       <c r="D4" t="str">
-        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
+        <v>Arhiva generisanih obrazaca i XML/export.</v>
       </c>
       <c r="E4" t="str">
-        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
+        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
       </c>
     </row>
   </sheetData>
@@ -16918,106 +17180,79 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-07-02</v>
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
+        <v>Partneri</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Oblast</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B4" t="str">
-        <v>Status</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Sta je zavrseno</v>
+        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
       </c>
       <c r="D4" t="str">
-        <v>Sta ostaje</v>
+        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
       </c>
       <c r="E4" t="str">
-        <v>Preporuceni sljedeci korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C5" t="str">
-        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C7" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C8" t="str">
-        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Redovno održavanje.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Regenerisati Excel nakon svake veće promjene.</v>
+        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -17028,7 +17263,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-30</v>
+        <v>Status projekta na dan 2026-07-02</v>
       </c>
     </row>
     <row r="2">
@@ -17061,13 +17296,13 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
+        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
       </c>
       <c r="D5" t="str">
-        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
+        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
       </c>
       <c r="E5" t="str">
-        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
+        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
       </c>
     </row>
     <row r="6">
@@ -17130,11 +17365,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-29</v>
+        <v>Status projekta na dan 2026-06-30</v>
       </c>
     </row>
     <row r="2">
@@ -17161,92 +17396,75 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nalozi</v>
+        <v>Izvodi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core zaokruzen</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
+        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
       </c>
       <c r="D5" t="str">
-        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
       </c>
       <c r="E5" t="str">
-        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
+        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PDV</v>
+        <v>Nalozi</v>
       </c>
       <c r="B6" t="str">
-        <v>Core zaokruzen</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C6" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
       </c>
       <c r="D6" t="str">
-        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
+        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E6" t="str">
-        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
+        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Izvodi</v>
+        <v>PDV</v>
       </c>
       <c r="B7" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C7" t="str">
-        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D7" t="str">
-        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
+        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
       </c>
       <c r="E7" t="str">
-        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
+        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>KIF/KUF</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B8" t="str">
-        <v>Core implementiran</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C8" t="str">
-        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
+        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
       </c>
       <c r="D8" t="str">
-        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
+        <v>Redovno održavanje.</v>
       </c>
       <c r="E8" t="str">
-        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C9" t="str">
-        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Regenerisati Excel nakon svake vece promjene.</v>
+        <v>Regenerisati Excel nakon svake veće promjene.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -17257,12 +17475,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-28</v>
+        <v>Status projekta na dan 2026-06-29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
       </c>
     </row>
     <row r="4">
@@ -17284,87 +17502,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Performanse partnera</v>
+        <v>Nalozi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core implementiran</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C5" t="str">
-        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
       </c>
       <c r="D5" t="str">
-        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E5" t="str">
-        <v>Pratiti brzinu na produkciji.</v>
+        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Indeksi baze</v>
+        <v>PDV</v>
       </c>
       <c r="B6" t="str">
-        <v>Implementirano</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C6" t="str">
-        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D6" t="str">
-        <v>-</v>
+        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
       </c>
       <c r="E6" t="str">
-        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIF/KUF uvoz/export</v>
+        <v>Izvodi</v>
       </c>
       <c r="B7" t="str">
-        <v>Core implementiran</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
       </c>
       <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata; XML export.</v>
+        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
       </c>
       <c r="E7" t="str">
-        <v>QA uvoznih knjizenja i export fajlova.</v>
+        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dokumentacija</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="B8" t="str">
-        <v>Uspostavljeno</v>
+        <v>Core implementiran</v>
       </c>
       <c r="C8" t="str">
-        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
       </c>
       <c r="D8" t="str">
-        <v>Redovno odrzavanje.</v>
+        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
       </c>
       <c r="E8" t="str">
-        <v>Azurirati uz svaku vecu promjenu.</v>
+        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PDV</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B9" t="str">
-        <v>Prva implementacija</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C9" t="str">
-        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
       </c>
       <c r="D9" t="str">
-        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+        <v>Redovno odrzavanje.</v>
       </c>
       <c r="E9" t="str">
-        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+        <v>Regenerisati Excel nakon svake vece promjene.</v>
       </c>
     </row>
   </sheetData>
@@ -17376,16 +17594,16 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-25</v>
+        <v>Status projekta na dan 2026-06-28</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ovaj list je kratki pregled šta je stvarno implementirano u aplikaciji, nezavisno od početne specifikacije.</v>
+        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
       </c>
     </row>
     <row r="4">
@@ -17396,170 +17614,119 @@
         <v>Status</v>
       </c>
       <c r="C4" t="str">
-        <v>Šta je završeno</v>
+        <v>Sta je zavrseno</v>
       </c>
       <c r="D4" t="str">
-        <v>Šta ostaje</v>
+        <v>Sta ostaje</v>
       </c>
       <c r="E4" t="str">
-        <v>Preporučeni sljedeći korak</v>
+        <v>Preporuceni sljedeci korak</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Navigacija i kontekst</v>
+        <v>Performanse partnera</v>
       </c>
       <c r="B5" t="str">
         <v>Core implementiran</v>
       </c>
       <c r="C5" t="str">
-        <v>Fiksni lijevi meni, gornji podmeniji, globalni izbor agencije/firme/godine/korisnika, dodata sekcija Računi.</v>
+        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
       </c>
       <c r="D5" t="str">
-        <v>Sakriti/zaključati menije po pravima i dodati kompletne podmenije budućih modula.</v>
+        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
       </c>
       <c r="E5" t="str">
-        <v>Dorađivati po modulu kad se modul stvarno implementira.</v>
+        <v>Pratiti brzinu na produkciji.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>M-001 Korisnici/agencije/prava</v>
+        <v>Indeksi baze</v>
       </c>
       <c r="B6" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Implementirano</v>
       </c>
       <c r="C6" t="str">
-        <v>Login, admin/agencija korisnici, radnici/klijenti, dodjela firmi, matrica prava, audit osnova.</v>
+        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
       </c>
       <c r="D6" t="str">
-        <v>Backend enforcement prava kroz sve rute, pretplate/limiti, statistika radnika, testovi.</v>
+        <v>-</v>
       </c>
       <c r="E6" t="str">
-        <v>Zaključati prava na server actions prije šire produkcije.</v>
+        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>M-002 Firme/kontni plan/partneri</v>
+        <v>KIF/KUF uvoz/export</v>
       </c>
       <c r="B7" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Core implementiran</v>
       </c>
       <c r="C7" t="str">
-        <v>Firme, IRMS, poslovne godine, banke, ugovor/cijena, globalni kontni plan + override, globalni/agencijski/firmski partneri, import globalnih partnera.</v>
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
       </c>
       <c r="D7" t="str">
-        <v>Odgovorna lica, puna izmjena firme, default konta po firmi/dobavljaču, podešavanja firme.</v>
+        <v>Kontrole iznosa i duplikata; XML export.</v>
       </c>
       <c r="E7" t="str">
-        <v>Dovršiti default konta i partner/firma preference koje KIF/KUF već koriste.</v>
+        <v>QA uvoznih knjizenja i export fajlova.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>M-003 Nalozi</v>
+        <v>Dokumentacija</v>
       </c>
       <c r="B8" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Uspostavljeno</v>
       </c>
       <c r="C8" t="str">
-        <v>Novi/izmjena naloga, nacrt, proknjižavanje, brisanje, partner analitika, datumi stavki, F9/F10, bruto bilans, analitičke kartice, print naloga i bruto bilansa.</v>
+        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
       </c>
       <c r="D8" t="str">
-        <v>Formalni prenos početnog stanja, jači testovi, izvještaji po poslovnoj jedinici, permission checks.</v>
+        <v>Redovno odrzavanje.</v>
       </c>
       <c r="E8" t="str">
-        <v>Napisati testove za validaciju stavki i za automatsko knjiženje iz KIF/KUF.</v>
+        <v>Azurirati uz svaku vecu promjenu.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>M-006 Računi KIF/KUF</v>
+        <v>PDV</v>
       </c>
       <c r="B9" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Prva implementacija</v>
       </c>
       <c r="C9" t="str">
-        <v>PDV stope, KIF/KUF knjige po mjesecu/vrsti, šeme kontiranja, MAPR link/F8, batch import, SEP Excel import za KIF, automatsko knjiženje knjige, edit/delete neproknjiženih, statusi na srpskom, print KIF/KUF.</v>
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
       </c>
       <c r="D9" t="str">
-        <v>Kontrole/duplikati, export, PDV zaključavanje, payment status, cache MAPR-a, PDF/QR čitanje, završni QA printa.</v>
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
       </c>
       <c r="E9" t="str">
-        <v>Dovršiti kontrole i testove, zatim krenuti PDV prijavu iz KIF/KUF.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>M-004 Robno</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Nije implementirano</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Specifikacija pročitana i unesena u planer.</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Cijeli modul: artikli, magacini, lager, kalkulacije, popis, otpis, nivelacija, automatsko knjiženje.</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Poslije stabilizacije KIF/KUF i PDV osnove krenuti na artikle/magacine.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Izvodi/PDF</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Priprema</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Instaliran pdfjs-dist za buduće čitanje tekstualnih PDF izvoda.</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Parser izvoda, QR iz PDF/TIFF, automatsko knjiženje izvoda.</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Kada se krene na izvode, prvo napraviti parser za jednu banku.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>PDV/Plate/Završni/Reports</v>
-      </c>
-      <c r="B12" t="str">
-        <v>U planu / djelimično</v>
-      </c>
-      <c r="C12" t="str">
-        <v>PDV stope i bruto bilans postoje; ostalo uglavnom placeholder.</v>
-      </c>
-      <c r="D12" t="str">
-        <v>PDV prijava, plate, završni račun, dashboard i izvještaji.</v>
-      </c>
-      <c r="E12" t="str">
-        <v>PDV prijava treba da dođe poslije finalizacije KIF/KUF kontrola.</v>
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z300"/>
+  <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Računovodstveni program — Master planer</v>
+        <v>Status projekta na dan 2026-06-25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ažurirano 2026-06-25: Core modula 1-3 je upotrebljiv, KIF/KUF modul je implementiran za unos, import, automatsko knjiženje i štampu; ostaju kontrole, export, PDV zaključavanje, početno stanje i testovi.</v>
+        <v>Ovaj list je kratki pregled šta je stvarno implementirano u aplikaciji, nezavisno od početne specifikacije.</v>
       </c>
     </row>
     <row r="4">
@@ -17567,278 +17734,157 @@
         <v>Oblast</v>
       </c>
       <c r="B4" t="str">
-        <v>Broj stavki</v>
+        <v>Status</v>
       </c>
       <c r="C4" t="str">
-        <v>Zaključeno</v>
+        <v>Šta je završeno</v>
       </c>
       <c r="D4" t="str">
-        <v>Napomena</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Status modula</v>
+        <v>Šta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporučeni sljedeći korak</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Moduli</v>
+        <v>Navigacija i kontekst</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Fiksni lijevi meni, gornji podmeniji, globalni izbor agencije/firme/godine/korisnika, dodata sekcija Računi.</v>
       </c>
       <c r="D5" t="str">
-        <v>Prva 3 modula su zaključena.</v>
-      </c>
-      <c r="F5" t="str">
-        <v>ID</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Status</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Faza</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Napomena</v>
+        <v>Sakriti/zaključati menije po pravima i dodati kompletne podmenije budućih modula.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Dorađivati po modulu kad se modul stvarno implementira.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Funkcionalnosti</v>
+        <v>M-001 Korisnici/agencije/prava</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Login, admin/agencija korisnici, radnici/klijenti, dodjela firmi, matrica prava, audit osnova.</v>
       </c>
       <c r="D6" t="str">
-        <v>Za praćenje implementacije.</v>
-      </c>
-      <c r="F6" t="str">
-        <v>M-001</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Korisnici, agencije i prava</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="I6" t="str">
-        <v>MVP 1</v>
-      </c>
-      <c r="J6" t="str">
-        <v>Autentifikacija, agencije, korisnici, radnici/klijenti, dodjela firmi, matrica prava i audit osnova postoje. Ostaju kompletan backend enforcement prava, pretplate/limiti i statistika radnika.</v>
+        <v>Backend enforcement prava kroz sve rute, pretplate/limiti, statistika radnika, testovi.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Zaključati prava na server actions prije šire produkcije.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Pravila</v>
+        <v>M-002 Firme/kontni plan/partneri</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Firme, IRMS, poslovne godine, banke, ugovor/cijena, globalni kontni plan + override, globalni/agencijski/firmski partneri, import globalnih partnera.</v>
       </c>
       <c r="D7" t="str">
-        <v>Poslovna logika.</v>
-      </c>
-      <c r="F7" t="str">
-        <v>M-002</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Firme, klijenti, poslovne godine i kontni plan</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="I7" t="str">
-        <v>MVP 1</v>
-      </c>
-      <c r="J7" t="str">
-        <v>Firme, IRMS, poslovne godine, aktivni kontekst firma/godina, banke, ugovori, kontni plan globalni + override, partneri globalni/agencijski/firmski su implementirani. Ostaju fina podesavanja firme, odgovorna lica i default konta.</v>
+        <v>Odgovorna lica, puna izmjena firme, default konta po firmi/dobavljaču, podešavanja firme.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Dovršiti default konta i partner/firma preference koje KIF/KUF već koriste.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Baza</v>
+        <v>M-003 Nalozi</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Novi/izmjena naloga, nacrt, proknjižavanje, brisanje, partner analitika, datumi stavki, F9/F10, bruto bilans, analitičke kartice, print naloga i bruto bilansa.</v>
       </c>
       <c r="D8" t="str">
-        <v>Predlog tabela.</v>
-      </c>
-      <c r="F8" t="str">
-        <v>M-003</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Nalozi za knjiženje</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="I8" t="str">
-        <v>MVP 1</v>
-      </c>
-      <c r="J8" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke iz ručnog naloga, datumi stavki, prečice F9/F10, bruto bilans, analitičke kartice i print su implementirani. Ostaju početno stanje i dodatne kontrole/testovi.</v>
+        <v>Formalni prenos početnog stanja, jači testovi, izvještaji po poslovnoj jedinici, permission checks.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Napisati testove za validaciju stavki i za automatsko knjiženje iz KIF/KUF.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>API</v>
+        <v>M-006 Računi KIF/KUF</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C9" t="str">
+        <v>PDV stope, KIF/KUF knjige po mjesecu/vrsti, šeme kontiranja, MAPR link/F8, batch import, SEP Excel import za KIF, automatsko knjiženje knjige, edit/delete neproknjiženih, statusi na srpskom, print KIF/KUF.</v>
       </c>
       <c r="D9" t="str">
-        <v>Predlog ruta.</v>
-      </c>
-      <c r="F9" t="str">
-        <v>M-004</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Robno knjigovodstvo</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Specifikacija spremna / nije implementirano</v>
-      </c>
-      <c r="I9" t="str">
-        <v>MVP 1/2</v>
-      </c>
-      <c r="J9" t="str">
-        <v>Specifikacija je pročitana i unesena u planer, ali modul nije krenuo u kodu osim navigacionih placeholdera.</v>
+        <v>Kontrole/duplikati, export, PDV zaključavanje, payment status, cache MAPR-a, PDF/QR čitanje, završni QA printa.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Dovršiti kontrole i testove, zatim krenuti PDV prijavu iz KIF/KUF.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Testovi</v>
+        <v>M-004 Robno</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Nije implementirano</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Specifikacija pročitana i unesena u planer.</v>
       </c>
       <c r="D10" t="str">
-        <v>QA scenariji.</v>
-      </c>
-      <c r="F10" t="str">
-        <v>M-005</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Izvodi i automatsko knjiženje</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Specifikacija spremna / nije implementirano</v>
-      </c>
-      <c r="I10" t="str">
-        <v>MVP 2</v>
-      </c>
-      <c r="J10" t="str">
-        <v>Finalna specifikacija je u zadaci/07_Izvodi_i_Automatsko_Knjizenje_FINAL.md. Sljedeće: import sesije, PDF/HTML parser, preview, povezivanje sa komitentima/fakturama i generisanje naloga.</v>
+        <v>Cijeli modul: artikli, magacini, lager, kalkulacije, popis, otpis, nivelacija, automatsko knjiženje.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Poslije stabilizacije KIF/KUF i PDV osnove krenuti na artikle/magacine.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Odluke</v>
+        <v>Izvodi/PDF</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Priprema</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Instaliran pdfjs-dist za buduće čitanje tekstualnih PDF izvoda.</v>
       </c>
       <c r="D11" t="str">
-        <v>Arhitektonske odluke.</v>
-      </c>
-      <c r="F11" t="str">
-        <v>M-006</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Plate i zaposleni</v>
-      </c>
-      <c r="H11" t="str">
-        <v>U planu</v>
-      </c>
-      <c r="I11" t="str">
-        <v>MVP 2</v>
-      </c>
-      <c r="J11" t="str">
-        <v>Nije implementirano.</v>
+        <v>Parser izvoda, QR iz PDF/TIFF, automatsko knjiženje izvoda.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Kada se krene na izvode, prvo napraviti parser za jednu banku.</v>
       </c>
     </row>
     <row r="12">
-      <c r="F12" t="str">
-        <v>M-007</v>
-      </c>
-      <c r="G12" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="H12" t="str">
-        <v>Djelimično kroz KIF/KUF</v>
-      </c>
-      <c r="I12" t="str">
-        <v>MVP 2</v>
-      </c>
-      <c r="J12" t="str">
-        <v>PDV stope i osnovne KIF/KUF PDV razrade postoje. PDV prijava, kontrole i XML nisu implementirani.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="F13" t="str">
-        <v>M-008</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Završni račun</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="I13" t="str">
-        <v>MVP 3</v>
-      </c>
-      <c r="J13" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statistički aneks su implementirani iz POSTED naloga sa sistemskim šemama, podešavanjima po firmi, trajnim ručnim korekcijama po AOP/koloni, print obrascima, predlogom zaključnog naloga za klase 5/6 i arhivom snimljenih obrazaca. Ostaje XML/export.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Sljedeći prioritet</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Završiti KIF/KUF kontrole i testove, pa odlučiti PDV ili Robno</v>
-      </c>
-      <c r="F14" t="str">
-        <v>M-009</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Izvještaji i dashboard</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="I14" t="str">
-        <v>MVP 1/2</v>
-      </c>
-      <c r="J14" t="str">
-        <v>Bruto bilans i analitičke kartice postoje. Dashboard i ostali izvještaji su uglavnom placeholderi.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Obuhvat</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Dokumenti, kalkulacije, ulazne/izlazne fakture, roba, zalihe, lager, maloprodaja/veleprodaja, automatska knjiženja.</v>
-      </c>
-      <c r="F15" t="str">
-        <v>M-010</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Računi / KIF-KUF</v>
-      </c>
-      <c r="H15" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="I15" t="str">
-        <v>MVP 1</v>
-      </c>
-      <c r="J15" t="str">
-        <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa i print su implementirani. Ostaju kontrole, export, PDV zaključavanje i QA.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Zašto sada</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Zavisi od firme, kontnog plana, partnera i naloga koje smo sada definisali.</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Napomena</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Biće dosta pravila, zato je dobro da se radi odvojeno i temeljno.</v>
+      <c r="A12" t="str">
+        <v>PDV/Plate/Završni/Reports</v>
+      </c>
+      <c r="B12" t="str">
+        <v>U planu / djelimično</v>
+      </c>
+      <c r="C12" t="str">
+        <v>PDV stope i bruto bilans postoje; ostalo uglavnom placeholder.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>PDV prijava, plate, završni račun, dashboard i izvještaji.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>PDV prijava treba da dođe poslije finalizacije KIF/KUF kontrola.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z300"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement payroll calculation and IOPPD workflow
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -445,13 +445,13 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje i izmjenu zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za redovan obračun 001, pripremu radnika, ručne mjesečne korekcije i dodatne stavke; /agencija/plate/podesavanja za pregled šifarnika.</v>
+        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ugovori, obustave, IOPPD/JPR, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
+        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
       </c>
       <c r="E2" t="str">
-        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki.</v>
+        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
       </c>
     </row>
   </sheetData>
@@ -650,7 +650,7 @@
         <v>MVP 2</v>
       </c>
       <c r="J11" t="str">
-        <v>Prva MVP osnova postoji: zaposleni sa dodavanjem/izmjenom i tabovima aktivni/neaktivni, šifarnici plata, redovan obračun 001, priprema radnika u nacrtu, ručne korekcije stavki i dodatne stavke po radniku. Bruto/neto servis čita pravila iz baze. Ostaju ugovori, obustave, IOPPD/JPR, uplatnice, knjiženje i print/export.</v>
+        <v>Prva MVP osnova postoji: zaposleni sa dodavanjem/izmjenom, odjavom/reaktivacijom i tabovima aktivni/neaktivni, šifarnici plata, kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, priprema radnika u nacrtu, kontrole prije obrade, ručne korekcije stavki, dodatne stavke po radniku, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz obračuna. Dodata je IOPPD matrica osnova obračuna, importovano je svih 108 šifara iz zvaničnog Excel dokumenta i generisane su šifre primanja za izbor kod radnika. Bruto/neto servis čita važeće stope iz baze, a minuli rad računa progresivno po navršenim godinama staža. IOPPD pregled po mjesecima, HTML/CSS štampa i XML download su dodati; ostaje povezivanje osnova direktno u algoritme za zakup/ugovore, obustave, uplatnice, knjiženje i print/export.</v>
       </c>
     </row>
     <row r="12">
@@ -934,7 +934,7 @@
         <v>Plate i zaposleni</v>
       </c>
       <c r="C10" t="str">
-        <v>Zaposleni, ugovori, obračun plata, IOPPD/JPR veze, obaveze, automatski nalog plata.</v>
+        <v>Zaposleni, ugovori, obračun plata, IOPPD, obaveze, automatski nalog plata.</v>
       </c>
       <c r="D10" t="str">
         <v>Vrlo visok</v>
@@ -949,7 +949,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H10" t="str">
-        <v>Prva MVP osnova postoji: tabele i šifarnici za IOPPD, vrste obračuna, poreze, doprinose, prirez i šifre primanja; stranice za zaposlene sa dodavanjem, izmjenom i tabovima aktivni/neaktivni, redovan obračun 001, priprema radnika u nacrtu, ručne mjesečne korekcije po radniku i dodatne stavke; bruto/neto obračun čita pravila iz baze. Ostaju ugovori, obustave, IOPPD/JPR, uplatnice, knjiženje i print/export.</v>
+        <v>Prva MVP osnova postoji: tabele i šifarnici za IOPPD, vrste obračuna, poreze, doprinose, prirez, šifre primanja i osnove obračuna; stranice za zaposlene sa dodavanjem, izmjenom, odjavom/reaktivacijom i tabovima aktivni/neaktivni, kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, priprema radnika u nacrtu, kontrole prije obrade, ručne mjesečne korekcije po radniku, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz obračuna; bruto/neto obračun čita važeće stope iz baze i strukturisana pravila osnova za linearne šifre poput ugovora i zakupa, minuli rad se računa progresivno po navršenim godinama staža, a u bazu je importovano svih 108 osnova iz zvaničnog Excel šifarnika, sa originalnim redom sačuvanim u JSON-u pravila i šiframa primanja generisanim za izbor kod radnika. IOPPD pregled po mjesecima, HTML/CSS štampa i XML download su dodati. Ostaju obustave, opisna pravila koja traže ručne parametre, uplatnice, knjiženje i print/export.</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Dodaj kontiranje plata i OPP-ND obrasce
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -419,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -440,24 +440,41 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
         <v>Firme</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B3" t="str">
         <v>Core implementiran / dorada</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C3" t="str">
         <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D3" t="str">
         <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
       </c>
-      <c r="E2" t="str">
+      <c r="E3" t="str">
         <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1109,7 +1126,7 @@
         <v>Plate i zaposleni</v>
       </c>
       <c r="C10" t="str">
-        <v>Zaposleni, ugovori, obračun plata, IOPPD, M-4, obaveze i automatski nalog plata.</v>
+        <v>Zaposleni, ugovori, obračun plata, IOPPD, M-4, OPP-ND, obaveze i automatski nalog plata.</v>
       </c>
       <c r="D10" t="str">
         <v>Vrlo visok</v>
@@ -1124,7 +1141,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H10" t="str">
-        <v>Prva MVP osnova postoji: tabele i šifarnici za IOPPD, vrste obračuna, poreze, doprinose, prirez, šifre primanja i osnove obračuna; stranice za zaposlene sa dodavanjem, izmjenom, odjavom/reaktivacijom i tabovima aktivni/neaktivni, kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, priprema radnika u nacrtu, kontrole prije obrade, ručne mjesečne korekcije po radniku, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz obračuna; bruto/neto obračun čita važeće stope iz baze i strukturisana pravila osnova za linearne šifre poput ugovora i zakupa, minuli rad se računa progresivno po navršenim godinama staža, a u bazu je importovano svih 108 osnova iz zvaničnog Excel šifarnika, sa originalnim redom sačuvanim u JSON-u pravila i šiframa primanja generisanim za izbor kod radnika. Dodato je 25 obračunskih podšifara iz A_SifR sa hijerarhijom, koeficijentima iznosa/staža, posebnim osnovicama i fondom sati, bez preuzimanja zastarjelih stopa. Podešavanja plata su grupisana: IOPPD šifre otvaraju postojeći šifarnik, a podešavanje knjiženja je pripremljen placeholder. IOPPD pregled po mjesecima, HTML/CSS štampa i XML download su dodati. M-4 je završen u dogovorenom obimu: godišnji pregled, matični podaci iz firme, potvrđene uplate, pojedinačni obrazac, Tabela 1 i Tabela 2. Globalni šifarnik prireza sadrži 21 opštinu sa DJP šiframa, stopama i raspoloživim računima iz stare MDB baze i koristi ga obračun plata i M-4. U modulu plata ostaju obustave, opisna pravila koja traže ručne parametre, uplatnice, implementacija podešavanja knjiženja i automatskog naloga te print/export obračuna.</v>
+        <v>Prva MVP osnova postoji: tabele i šifarnici za IOPPD, vrste obračuna, poreze, doprinose, prirez, šifre primanja i osnove obračuna; stranice za zaposlene sa dodavanjem, izmjenom, odjavom/reaktivacijom i tabovima aktivni/neaktivni, kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, priprema radnika u nacrtu, kontrole prije obrade, ručne mjesečne korekcije po radniku, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz obračuna; bruto/neto obračun čita važeće stope iz baze i strukturisana pravila osnova za linearne šifre poput ugovora i zakupa, minuli rad se računa progresivno po navršenim godinama staža, a u bazu je importovano svih 108 osnova iz zvaničnog Excel šifarnika, sa originalnim redom sačuvanim u JSON-u pravila i šiframa primanja generisanim za izbor kod radnika. Dodato je 25 obračunskih podšifara iz A_SifR sa hijerarhijom, koeficijentima iznosa/staža, posebnim osnovicama i fondom sati, bez preuzimanja zastarjelih stopa. Podešavanja plata su grupisana: IOPPD šifre otvaraju postojeći šifarnik, a podešavanje knjiženja čuva posebnu šemu D/P konta za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun se akcijom Proknjiži transakcijski pretvara u izbalansiran i odmah POSTED PAYROLL nalog, uz trajnu vezu i blokadu duplog knjiženja. M-4, OPP-ND i IOPPD grupisani su u drugom nivou podmenija Obrasci. IOPPD ima mjesečni pregled, HTML/CSS štampu i XML download. M-4 je završen u dogovorenom obimu: godišnji pregled, matični podaci iz firme, potvrđene uplate, pojedinačni obrazac, Tabela 1 i Tabela 2. OPP-ND razvrstava porez na četiri službene vrste, primjenjuje važeću opštinsku stopu firme i generiše A4 prijavu prema zvaničnom PDF-u. Globalni šifarnik prireza sadrži 21 opštinu sa DJP šiframa, stopama i raspoloživim računima iz stare MDB baze i koristi ga obračun plata, M-4 i OPP-ND. U modulu plata ostaju obustave, opisna pravila koja traže ručne parametre, uplatnice, namjenski storno/vraćanje automatskog naloga te print/export obračuna.</v>
       </c>
     </row>
     <row r="11">
@@ -1240,7 +1257,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z353"/>
+  <dimension ref="A1:Z356"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4748,9 +4765,123 @@
         <v>Brisanje je jedna backend transakcija sa agencijskim scope-om, audit zapisom i čišćenjem aktivnog konteksta. Zajednički korisnici i globalni/agencijski šifarnici ostaju sačuvani.</v>
       </c>
     </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>F-092</v>
+      </c>
+      <c r="B354" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C354" t="str">
+        <v>Podešavanje knjiženja po kategoriji</v>
+      </c>
+      <c r="D354" t="str">
+        <v>Firma za aktivnu poslovnu godinu bira vrstu naloga i posebna duguje/potražuje konta za neto, porez, prirez, svaki doprinos i ostale komponente redovnog rada, ugovora o djelu, zakupa i ostalih ugovora.</v>
+      </c>
+      <c r="E354" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F354" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G354" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H354" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I354" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J354" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K354" t="str">
+        <v>M-003,M-006,F-024</v>
+      </c>
+      <c r="L354" t="str">
+        <v>Početna redovna šema izvedena je iz 001LP.mdb/ZAR_Kontir i ZAR_TipZB i prilagođena važećem kontnom planu. Šemu koristi automatsko knjiženje obračuna.</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>F-093</v>
+      </c>
+      <c r="B355" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C355" t="str">
+        <v>Proknjižavanje obračuna plata</v>
+      </c>
+      <c r="D355" t="str">
+        <v>Akcija Proknjiži na obrađenom obračunu transakcijski kreira numerisan, izbalansiran i odmah POSTED PAYROLL nalog iz kategorijske D/P šeme i povezuje ga sa obračunom.</v>
+      </c>
+      <c r="E355" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F355" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G355" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H355" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I355" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J355" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K355" t="str">
+        <v>M-003,M-006,F-092</v>
+      </c>
+      <c r="L355" t="str">
+        <v>Provjeravaju se scope, pravo plate/post, zaključana godina, aktivna analitička konta, duple zbirne komponente i balans. Ponovno knjiženje je blokirano; opšte vraćanje automatskog naloga u nacrt nije dozvoljeno.</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>F-094</v>
+      </c>
+      <c r="B356" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C356" t="str">
+        <v>OPP-ND prijava prireza</v>
+      </c>
+      <c r="D356" t="str">
+        <v>Mjesečna prijava razvrstava porez na lična primanja, samostalnu djelatnost, imovinu/imovinska prava i kapital, primjenjuje važeću stopu prireza opštine firme i generiše službeni A4 obrazac.</v>
+      </c>
+      <c r="E356" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F356" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G356" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H356" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I356" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J356" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K356" t="str">
+        <v>M-006,F-089</v>
+      </c>
+      <c r="L356" t="str">
+        <v>Redovan rad ide u lična primanja, ugovor o djelu i ostali ugovori u samostalnu djelatnost, a zakup u imovinu. Kapital ostaje prazan dok ne postoji odgovarajuća vrsta obračuna. Vizuelni render provjeren je prema zvaničnom PDF-u.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z353"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z356"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8614,7 +8745,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z332"/>
+  <dimension ref="A1:Z334"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9820,13 +9951,13 @@
         <v>Podešavanja plata</v>
       </c>
       <c r="D331" t="str">
-        <v>Pregled grupa podešavanja; IOPPD šifre otvaraju šifarnik osnova i pravila sa pripadajućim obračunskim podšiframa, koeficijentima, posebnim procentom osnovice i fondom sati, a podešavanje knjiženja je pripremljeno za buduću implementaciju.</v>
+        <v>Pregled grupa podešavanja; IOPPD šifre otvaraju šifarnik osnova i pravila sa pripadajućim obračunskim podšiframa, koeficijentima, posebnim procentom osnovice i fondom sati, a podešavanje knjiženja čuva kategorijsku D/P šemu.</v>
       </c>
       <c r="E331" t="str">
         <v>Visok</v>
       </c>
       <c r="F331" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Implementirano</v>
       </c>
       <c r="G331" t="str">
         <v>M-006</v>
@@ -9858,19 +9989,71 @@
         <v>M-006</v>
       </c>
       <c r="H332" t="str">
-        <v>/agencija/plate/m4, /stampa/plate/m4</v>
+        <v>/agencija/plate/obrasci/m4, /stampa/plate/m4</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>E-044</v>
+      </c>
+      <c r="B333" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C333" t="str">
+        <v>Obrasci plata</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Pregledna grupa i drugi nivo podmenija za M-4, OPP-ND i IOPPD, bez promjene postojećih funkcionalnosti obrazaca.</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F333" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G333" t="str">
+        <v>M-006</v>
+      </c>
+      <c r="H333" t="str">
+        <v>/agencija/plate/obrasci</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>E-045</v>
+      </c>
+      <c r="B334" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C334" t="str">
+        <v>OPP-ND</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Mjesečni pregled prireza po vrstama poreza i važećoj opštinskoj stopi firme, sa službenom A4 štampom prema dostavljenom PDF obrascu.</v>
+      </c>
+      <c r="E334" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F334" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G334" t="str">
+        <v>F-094</v>
+      </c>
+      <c r="H334" t="str">
+        <v>/agencija/plate/obrasci/opp-nd, /stampa/plate/opp-nd</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z332"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z334"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z343"/>
+  <dimension ref="A1:Z346"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11529,9 +11712,87 @@
         <v>Zvaničnih 108 osnova ostaje autoritativno; dodato je 25 podšifara i korisni obračunski parametri iz 001LP.mdb/A_SifR bez preuzimanja starih stopa.</v>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>DB-069</v>
+      </c>
+      <c r="B344" t="str">
+        <v>plate_kontiranje_podesavanja</v>
+      </c>
+      <c r="C344" t="str">
+        <v>Podešavanje knjiženja obračuna po firmi/godini i kategoriji.</v>
+      </c>
+      <c r="D344" t="str">
+        <v>agencija_id, firma_id, poslovna_godina_id, kategorija, vrsta_naloga_id, opis_naloga</v>
+      </c>
+      <c r="E344" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="F344" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G344" t="str">
+        <v>F-092</v>
+      </c>
+      <c r="H344" t="str">
+        <v>Jedna šema za svaku kategoriju: redovan rad, ugovor o djelu, zakup i ostali ugovori.</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>DB-070</v>
+      </c>
+      <c r="B345" t="str">
+        <v>plate_kontiranje_pravila</v>
+      </c>
+      <c r="C345" t="str">
+        <v>Pravila D/P kontiranja po komponenti obračuna.</v>
+      </c>
+      <c r="D345" t="str">
+        <v>podesavanje_id, komponenta, naziv, grupa, izvorno_polje, duguje_konto_id, potrazuje_konto_id, aktivan, redosljed</v>
+      </c>
+      <c r="E345" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="F345" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G345" t="str">
+        <v>F-092</v>
+      </c>
+      <c r="H345" t="str">
+        <v>Neto, porez, prirez, pojedinačni doprinosi i ostale obaveze imaju posebna konta; zbirni redovi su isključene alternative.</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>DB-071</v>
+      </c>
+      <c r="B346" t="str">
+        <v>plate_obracuni.nalog_id</v>
+      </c>
+      <c r="C346" t="str">
+        <v>Jedinstvena veza proknjiženog obračuna sa automatskim PAYROLL nalogom.</v>
+      </c>
+      <c r="D346" t="str">
+        <v>nalog_id unique nullable, posted_at, posted_by</v>
+      </c>
+      <c r="E346" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="F346" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G346" t="str">
+        <v>F-093</v>
+      </c>
+      <c r="H346" t="str">
+        <v>Strani ključ je ON DELETE SET NULL; aplikacija blokira ponovno knjiženje i opšte vraćanje PAYROLL naloga u nacrt.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z343"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z346"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Dodaj početno stanje i QR učitavanje računa
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,29 +3,30 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-07-24" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-07-09" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-07-07" sheetId="3" r:id="rId3"/>
-    <sheet name="Status 2026-07-06" sheetId="4" r:id="rId4"/>
-    <sheet name="Status 2026-07-05" sheetId="5" r:id="rId5"/>
-    <sheet name="Status 2026-07-02" sheetId="6" r:id="rId6"/>
-    <sheet name="Status 2026-06-30" sheetId="7" r:id="rId7"/>
-    <sheet name="Status 2026-06-29" sheetId="8" r:id="rId8"/>
-    <sheet name="Status 2026-06-28" sheetId="9" r:id="rId9"/>
-    <sheet name="Status 2026-06-25" sheetId="10" r:id="rId10"/>
-    <sheet name="Dashboard" sheetId="11" r:id="rId11"/>
-    <sheet name="Moduli" sheetId="12" r:id="rId12"/>
-    <sheet name="Funkcionalnosti" sheetId="13" r:id="rId13"/>
-    <sheet name="Pravila" sheetId="14" r:id="rId14"/>
-    <sheet name="Zavisnosti" sheetId="15" r:id="rId15"/>
-    <sheet name="Ekrani" sheetId="16" r:id="rId16"/>
-    <sheet name="Baza" sheetId="17" r:id="rId17"/>
-    <sheet name="API" sheetId="18" r:id="rId18"/>
-    <sheet name="Testovi" sheetId="19" r:id="rId19"/>
-    <sheet name="Bugovi" sheetId="20" r:id="rId20"/>
-    <sheet name="Ideje" sheetId="21" r:id="rId21"/>
-    <sheet name="Odluke" sheetId="22" r:id="rId22"/>
-    <sheet name="Kategorije" sheetId="23" r:id="rId23"/>
+    <sheet name="Status 2026-07-25" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-07-24" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-07-09" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-07-07" sheetId="4" r:id="rId4"/>
+    <sheet name="Status 2026-07-06" sheetId="5" r:id="rId5"/>
+    <sheet name="Status 2026-07-05" sheetId="6" r:id="rId6"/>
+    <sheet name="Status 2026-07-02" sheetId="7" r:id="rId7"/>
+    <sheet name="Status 2026-06-30" sheetId="8" r:id="rId8"/>
+    <sheet name="Status 2026-06-29" sheetId="9" r:id="rId9"/>
+    <sheet name="Status 2026-06-28" sheetId="10" r:id="rId10"/>
+    <sheet name="Status 2026-06-25" sheetId="11" r:id="rId11"/>
+    <sheet name="Dashboard" sheetId="12" r:id="rId12"/>
+    <sheet name="Moduli" sheetId="13" r:id="rId13"/>
+    <sheet name="Funkcionalnosti" sheetId="14" r:id="rId14"/>
+    <sheet name="Pravila" sheetId="15" r:id="rId15"/>
+    <sheet name="Zavisnosti" sheetId="16" r:id="rId16"/>
+    <sheet name="Ekrani" sheetId="17" r:id="rId17"/>
+    <sheet name="Baza" sheetId="18" r:id="rId18"/>
+    <sheet name="API" sheetId="19" r:id="rId19"/>
+    <sheet name="Testovi" sheetId="20" r:id="rId20"/>
+    <sheet name="Bugovi" sheetId="21" r:id="rId21"/>
+    <sheet name="Ideje" sheetId="22" r:id="rId22"/>
+    <sheet name="Odluke" sheetId="23" r:id="rId23"/>
+    <sheet name="Kategorije" sheetId="24" r:id="rId24"/>
   </sheets>
 </workbook>
 </file>
@@ -440,36 +441,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Plate i zaposleni</v>
+        <v>M-003 Nalozi</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Početno stanje završeno</v>
       </c>
       <c r="C2" t="str">
-        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
       </c>
       <c r="D2" t="str">
-        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Firme</v>
+        <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B3" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>QR čitanje računa završeno</v>
       </c>
       <c r="C3" t="str">
-        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
       </c>
       <c r="E3" t="str">
-        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
+        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
       </c>
     </row>
   </sheetData>
@@ -481,6 +482,129 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Performanse partnera</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pratiti brzinu na produkciji.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Indeksi baze</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KIF/KUF uvoz/export</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kontrole iznosa i duplikata; XML export.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>QA uvoznih knjizenja i export fajlova.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Dokumentacija</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Uspostavljeno</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Redovno odrzavanje.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Azurirati uz svaku vecu promjenu.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Prva implementacija</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
@@ -653,7 +777,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -773,7 +897,7 @@
         <v>MVP 1</v>
       </c>
       <c r="J8" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke iz ručnog naloga, datumi stavki, prečice F9/F10, bruto bilans, analitičke kartice i print su implementirani. Ostaju početno stanje i dodatne kontrole/testovi.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke, prečice F9/F10, bruto bilans, analitičke kartice, print i automatski DRAFT prenos početnog stanja klasa 0-4 su implementirani. Ostaju kontrole po poslovnoj jedinici i dodatni automatizovani testovi.</v>
       </c>
     </row>
     <row r="9">
@@ -948,7 +1072,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z301"/>
   <sheetData>
@@ -1063,7 +1187,7 @@
         <v>MVP 1</v>
       </c>
       <c r="H7" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke iz ručnog naloga, datumi stavki, prečice F9/F10, bruto bilans, analitičke kartice i print su implementirani. Ostaju početno stanje i dodatne kontrole/testovi.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke, prečice F9/F10, bruto bilans, analitičke kartice, print i automatski DRAFT prenos početnog stanja klasa 0-4 su implementirani. Ostaju kontrole po poslovnoj jedinici i dodatni automatizovani testovi.</v>
       </c>
     </row>
     <row r="8">
@@ -1245,7 +1369,7 @@
         <v>MVP 1</v>
       </c>
       <c r="H301" t="str">
-        <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa, print i Excel export su implementirani. Ostaju kontrole, XML export, PDV zaključavanje i QA.</v>
+        <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, lokalno QR čitanje PDF/TIFF/JPG/PNG računa, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa, print i Excel export su implementirani. Ostaju kontrole, XML export, PDV zaključavanje i QA.</v>
       </c>
     </row>
   </sheetData>
@@ -1255,7 +1379,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z356"/>
   <sheetData>
@@ -2578,25 +2702,25 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F38" t="str">
-        <v>U izradi</v>
+        <v>Implementirano</v>
       </c>
       <c r="G38" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J38" t="str">
         <v>Djelimicno</v>
-      </c>
-      <c r="H38" t="str">
-        <v>Djelimicno</v>
-      </c>
-      <c r="I38" t="str">
-        <v>Da</v>
-      </c>
-      <c r="J38" t="str">
-        <v>Ne</v>
       </c>
       <c r="K38" t="str">
         <v>F-014,F-026</v>
       </c>
       <c r="L38" t="str">
-        <v>Bruto bilans ima odvojene kolone početnog stanja, ali unos/prenos početnog stanja nije kompletiran.</v>
+        <v>Generator i ručni unos backend provjerom i transakcijskim advisory lockom sprečavaju drugi aktivni nalog početnog stanja.</v>
       </c>
     </row>
     <row r="39">
@@ -2616,25 +2740,25 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F39" t="str">
-        <v>Nije poceto</v>
+        <v>Implementirano</v>
       </c>
       <c r="G39" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H39" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I39" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J39" t="str">
         <v>Djelimicno</v>
-      </c>
-      <c r="J39" t="str">
-        <v>Ne</v>
       </c>
       <c r="K39" t="str">
         <v>F-034</v>
       </c>
       <c r="L39" t="str">
-        <v>Specifikacija postoji; implementacija Modula 3 jos nije krenula osim ranijih osnovnih tabela.</v>
+        <v>Prenose se POSTED salda klasa 0-4 zbirno po kontu i partneru u numerisan DRAFT nalog; klase 5/6 se ne prenose i prikazuju upozorenje. Neizbalansirane klase 0-4 blokiraju kreiranje.</v>
       </c>
     </row>
     <row r="40">
@@ -3812,7 +3936,7 @@
         <v>F-063</v>
       </c>
       <c r="L328" t="str">
-        <v>KUF koristi dobavljača, KIF kupca; broj računa se normalizuje na čisti dio npr. 1/2026.</v>
+        <v>KUF forma lokalno čita MAPR QR iz PDF/TIFF/JPG/PNG računa bez čuvanja originala, uz visoku PDF rezoluciju, zone, uvećavanje i kontrast. Import stranica prihvata više takvih fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije postojećeg KUF/KIF importa.</v>
       </c>
     </row>
     <row r="329">
@@ -4886,7 +5010,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z362"/>
   <sheetData>
@@ -8211,7 +8335,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z309"/>
   <sheetData>
@@ -8743,7 +8867,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z334"/>
   <sheetData>
@@ -9112,13 +9236,13 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F17" t="str">
-        <v>Nije poceto</v>
+        <v>Implementirano</v>
       </c>
       <c r="G17" t="str">
         <v>F-034,F-035</v>
       </c>
       <c r="H17" t="str">
-        <v>Početno stanje jos nije posebna funkcionalnost.</v>
+        <v>Ekran prikazuje izvor iz prethodne godine, kontrole i pregled stavki; kreira DRAFT nalog koji se proknjižava kroz standardni detalj naloga.</v>
       </c>
     </row>
     <row r="18">
@@ -9755,7 +9879,7 @@
         <v>F-063</v>
       </c>
       <c r="H323" t="str">
-        <v>/agencija/racuni/podesavanja, /agencija/racuni/kuf, /agencija/racuni/kuf/[id], /agencija/racuni/kif/[id], /agencija/racuni/neproknjizeno, /agencija/racuni/pregled-kuf i /agencija/racuni/pregled-kuf/[id]. Dodato knjiženje/dopuna naloga po knjizi i uvoz podešavanja iz druge firme.</v>
+        <v>/agencija/racuni/podesavanja, /agencija/racuni/kuf, /agencija/racuni/kuf/[id], /agencija/racuni/kif/[id], /agencija/racuni/import, /agencija/racuni/neproknjizeno, /agencija/racuni/pregled-kuf i /agencija/racuni/pregled-kuf/[id]. Dodato knjiženje/dopuna naloga, uvoz podešavanja i pojedinačno/višestruko lokalno čitanje MAPR QR koda iz PDF/TIFF/JPG/PNG računa.</v>
       </c>
     </row>
     <row r="324">
@@ -10051,7 +10175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z346"/>
   <sheetData>
@@ -11797,7 +11921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z350"/>
   <sheetData>
@@ -13030,16 +13154,16 @@
         <v>Nalozi</v>
       </c>
       <c r="F47" t="str">
-        <v>Nije poceto</v>
+        <v>Implementirano</v>
       </c>
       <c r="G47" t="str">
         <v>F-035</v>
       </c>
       <c r="H47" t="str">
-        <v>Ne</v>
+        <v>Djelimicno</v>
       </c>
       <c r="I47" t="str">
-        <v>Generisanje pocetnog stanja jos nije implementirano.</v>
+        <v>Implementirano kao Next.js server action sa scope/permission/lock kontrolama, provjerom balansa i zaštitom od duplikata.</v>
       </c>
     </row>
     <row r="48">
@@ -14554,7 +14678,69 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Firme</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB345"/>
   <sheetData>
@@ -15225,10 +15411,16 @@
         <v>F-035,R-046</v>
       </c>
       <c r="F30" t="str">
-        <v>Nije poceto</v>
+        <v>Djelimicno testirano</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="H30">
+        <v>46228.083333333336</v>
       </c>
       <c r="I30" t="str">
-        <v>Generisanje pocetnog stanja jos nije implementirano.</v>
+        <v>TypeScript/lint, runtime pregled i rollback integracioni test potvrđuju prenos 0-4, partner analitiku, isključenje 5/6 i balans; trajni automatizovani test ostaje.</v>
       </c>
     </row>
     <row r="31">
@@ -15248,10 +15440,16 @@
         <v>F-034,R-044</v>
       </c>
       <c r="F31" t="str">
-        <v>Nije poceto</v>
+        <v>Djelimicno testirano</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="H31">
+        <v>46228.083333333336</v>
       </c>
       <c r="I31" t="str">
-        <v>Posebna zabrana drugog pocetnog stanja jos nije implementirana.</v>
+        <v>Backend provjera i transakcijski advisory lock postoje u generatoru i ručnom unosu; ostaje automatizovani test konkurentnih zahtjeva.</v>
       </c>
     </row>
     <row r="32">
@@ -16335,52 +16533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Plate</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -16430,7 +16583,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -16867,7 +17020,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z319"/>
   <sheetData>
@@ -17593,7 +17746,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -17805,19 +17958,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Zavrsni racun</v>
+        <v>Plate</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimicno implementirano</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
+        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
       </c>
       <c r="D2" t="str">
-        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
+        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
       </c>
       <c r="E2" t="str">
-        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
+        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
       </c>
     </row>
   </sheetData>
@@ -17829,7 +17982,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17850,58 +18003,24 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Partneri</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B2" t="str">
-        <v>Implementirano</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
       </c>
       <c r="D2" t="str">
-        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
       </c>
       <c r="E2" t="str">
-        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Zavrsni racun</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Djelimicno implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Arhiva generisanih obrazaca i XML/export.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
+        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -17969,13 +18088,13 @@
         <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
       </c>
       <c r="D4" t="str">
-        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
+        <v>Arhiva generisanih obrazaca i XML/export.</v>
       </c>
       <c r="E4" t="str">
-        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
+        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
       </c>
     </row>
   </sheetData>
@@ -17987,106 +18106,79 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-07-02</v>
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
+        <v>Partneri</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Oblast</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B4" t="str">
-        <v>Status</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Sta je zavrseno</v>
+        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
       </c>
       <c r="D4" t="str">
-        <v>Sta ostaje</v>
+        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
       </c>
       <c r="E4" t="str">
-        <v>Preporuceni sljedeci korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C5" t="str">
-        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C7" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C8" t="str">
-        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Redovno održavanje.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Regenerisati Excel nakon svake veće promjene.</v>
+        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -18097,7 +18189,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-30</v>
+        <v>Status projekta na dan 2026-07-02</v>
       </c>
     </row>
     <row r="2">
@@ -18130,13 +18222,13 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
+        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
       </c>
       <c r="D5" t="str">
-        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
+        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
       </c>
       <c r="E5" t="str">
-        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
+        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
       </c>
     </row>
     <row r="6">
@@ -18199,11 +18291,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-29</v>
+        <v>Status projekta na dan 2026-06-30</v>
       </c>
     </row>
     <row r="2">
@@ -18230,92 +18322,75 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nalozi</v>
+        <v>Izvodi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core zaokruzen</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
+        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
       </c>
       <c r="D5" t="str">
-        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
       </c>
       <c r="E5" t="str">
-        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
+        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PDV</v>
+        <v>Nalozi</v>
       </c>
       <c r="B6" t="str">
-        <v>Core zaokruzen</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C6" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
       </c>
       <c r="D6" t="str">
-        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
+        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E6" t="str">
-        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
+        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Izvodi</v>
+        <v>PDV</v>
       </c>
       <c r="B7" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C7" t="str">
-        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D7" t="str">
-        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
+        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
       </c>
       <c r="E7" t="str">
-        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
+        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>KIF/KUF</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B8" t="str">
-        <v>Core implementiran</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C8" t="str">
-        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
+        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
       </c>
       <c r="D8" t="str">
-        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
+        <v>Redovno održavanje.</v>
       </c>
       <c r="E8" t="str">
-        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C9" t="str">
-        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Regenerisati Excel nakon svake vece promjene.</v>
+        <v>Regenerisati Excel nakon svake veće promjene.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -18326,12 +18401,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-28</v>
+        <v>Status projekta na dan 2026-06-29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
       </c>
     </row>
     <row r="4">
@@ -18353,87 +18428,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Performanse partnera</v>
+        <v>Nalozi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core implementiran</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C5" t="str">
-        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
       </c>
       <c r="D5" t="str">
-        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E5" t="str">
-        <v>Pratiti brzinu na produkciji.</v>
+        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Indeksi baze</v>
+        <v>PDV</v>
       </c>
       <c r="B6" t="str">
-        <v>Implementirano</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C6" t="str">
-        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D6" t="str">
-        <v>-</v>
+        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
       </c>
       <c r="E6" t="str">
-        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIF/KUF uvoz/export</v>
+        <v>Izvodi</v>
       </c>
       <c r="B7" t="str">
-        <v>Core implementiran</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
       </c>
       <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata; XML export.</v>
+        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
       </c>
       <c r="E7" t="str">
-        <v>QA uvoznih knjizenja i export fajlova.</v>
+        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dokumentacija</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="B8" t="str">
-        <v>Uspostavljeno</v>
+        <v>Core implementiran</v>
       </c>
       <c r="C8" t="str">
-        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
       </c>
       <c r="D8" t="str">
-        <v>Redovno odrzavanje.</v>
+        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
       </c>
       <c r="E8" t="str">
-        <v>Azurirati uz svaku vecu promjenu.</v>
+        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PDV</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B9" t="str">
-        <v>Prva implementacija</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C9" t="str">
-        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
       </c>
       <c r="D9" t="str">
-        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+        <v>Redovno odrzavanje.</v>
       </c>
       <c r="E9" t="str">
-        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+        <v>Regenerisati Excel nakon svake vece promjene.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement fiscal platform and outgoing invoices
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,33 +3,35 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-07-30" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-07-29" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-07-26" sheetId="3" r:id="rId3"/>
-    <sheet name="Status 2026-07-25" sheetId="4" r:id="rId4"/>
-    <sheet name="Status 2026-07-24" sheetId="5" r:id="rId5"/>
-    <sheet name="Status 2026-07-09" sheetId="6" r:id="rId6"/>
-    <sheet name="Status 2026-07-07" sheetId="7" r:id="rId7"/>
-    <sheet name="Status 2026-07-06" sheetId="8" r:id="rId8"/>
-    <sheet name="Status 2026-07-05" sheetId="9" r:id="rId9"/>
-    <sheet name="Status 2026-07-02" sheetId="10" r:id="rId10"/>
-    <sheet name="Status 2026-06-30" sheetId="11" r:id="rId11"/>
-    <sheet name="Status 2026-06-29" sheetId="12" r:id="rId12"/>
-    <sheet name="Status 2026-06-28" sheetId="13" r:id="rId13"/>
-    <sheet name="Status 2026-06-25" sheetId="14" r:id="rId14"/>
-    <sheet name="Dashboard" sheetId="15" r:id="rId15"/>
-    <sheet name="Moduli" sheetId="16" r:id="rId16"/>
-    <sheet name="Funkcionalnosti" sheetId="17" r:id="rId17"/>
-    <sheet name="Pravila" sheetId="18" r:id="rId18"/>
-    <sheet name="Zavisnosti" sheetId="19" r:id="rId19"/>
-    <sheet name="Ekrani" sheetId="20" r:id="rId20"/>
-    <sheet name="Baza" sheetId="21" r:id="rId21"/>
-    <sheet name="API" sheetId="22" r:id="rId22"/>
-    <sheet name="Testovi" sheetId="23" r:id="rId23"/>
-    <sheet name="Bugovi" sheetId="24" r:id="rId24"/>
-    <sheet name="Ideje" sheetId="25" r:id="rId25"/>
-    <sheet name="Odluke" sheetId="26" r:id="rId26"/>
-    <sheet name="Kategorije" sheetId="27" r:id="rId27"/>
+    <sheet name="Status 2026-08-07" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-08-04" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-07-30" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-07-29" sheetId="4" r:id="rId4"/>
+    <sheet name="Status 2026-07-26" sheetId="5" r:id="rId5"/>
+    <sheet name="Status 2026-07-25" sheetId="6" r:id="rId6"/>
+    <sheet name="Status 2026-07-24" sheetId="7" r:id="rId7"/>
+    <sheet name="Status 2026-07-09" sheetId="8" r:id="rId8"/>
+    <sheet name="Status 2026-07-07" sheetId="9" r:id="rId9"/>
+    <sheet name="Status 2026-07-06" sheetId="10" r:id="rId10"/>
+    <sheet name="Status 2026-07-05" sheetId="11" r:id="rId11"/>
+    <sheet name="Status 2026-07-02" sheetId="12" r:id="rId12"/>
+    <sheet name="Status 2026-06-30" sheetId="13" r:id="rId13"/>
+    <sheet name="Status 2026-06-29" sheetId="14" r:id="rId14"/>
+    <sheet name="Status 2026-06-28" sheetId="15" r:id="rId15"/>
+    <sheet name="Status 2026-06-25" sheetId="16" r:id="rId16"/>
+    <sheet name="Dashboard" sheetId="17" r:id="rId17"/>
+    <sheet name="Moduli" sheetId="18" r:id="rId18"/>
+    <sheet name="Funkcionalnosti" sheetId="19" r:id="rId19"/>
+    <sheet name="Pravila" sheetId="20" r:id="rId20"/>
+    <sheet name="Zavisnosti" sheetId="21" r:id="rId21"/>
+    <sheet name="Ekrani" sheetId="22" r:id="rId22"/>
+    <sheet name="Baza" sheetId="23" r:id="rId23"/>
+    <sheet name="API" sheetId="24" r:id="rId24"/>
+    <sheet name="Testovi" sheetId="25" r:id="rId25"/>
+    <sheet name="Bugovi" sheetId="26" r:id="rId26"/>
+    <sheet name="Ideje" sheetId="27" r:id="rId27"/>
+    <sheet name="Odluke" sheetId="28" r:id="rId28"/>
+    <sheet name="Kategorije" sheetId="29" r:id="rId29"/>
   </sheets>
 </workbook>
 </file>
@@ -444,19 +446,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
+        <v>M-004 Robno</v>
       </c>
       <c r="B2" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>KIF sada podržava dnevni i mjesečni pazar sa periodom, brojem izvještaja, kasom, poreskim osnovicama, izlaznim PDV-om i raspodjelom naplate na gotovinu, kartice, virman i ostalo. Preklapanje perioda iste kase je blokirano. Ukupan iznos se kaskadno raspoređuje od najveće aktivne stope ka 0%, uz automatski izlazni PDV. Pazar se prikazuje u KIF-u, štampi, Excel izvozu i izlaznom PDV-u. Podešavanja firme imaju posebna dugujuća konta načina naplate, dok prihod i PDV koriste aktivnu KIF šemu.</v>
+        <v>Izlazne fakture imaju pregled, nacrt i brzi editor za robu i usluge, cijene iz šifarnika, Enter navigaciju, brzo dodavanje artikla/usluge i preglednu A4 štampu. Štampa podržava snapshot strana, nacrt, PDV rekapitulaciju i zvanični fiskalni QR/IKOF/JIKR kada postoje. Za firme van Summa fiskalizacije završavanje provjerava lager i PDV period, razdužuje robu, kreira nalog i šalje zapis u KIF kao SOURCE_DOCUMENT bez ponovnog knjiženja.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA kreiranja, izmjene, brisanja, zabrane preklapanja, knjiženja i PDV prikaza pazara; PDV zaključavanje KIF/KUF izmjena.</v>
+        <v>Povezivanje završavanja Summa fakture sa Fiscal API-jem i završni end-to-end QA.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260730170000_kif_pazar je primijenjena, Prisma klijent regenerisan i dev server restartovan. TypeScript, Prisma validacija i lint prolaze bez novih grešaka.</v>
+        <v>Migracije 20260807100000_izlazne_fakture_mvp, 20260807120000_kif_source_document_posting i 20260808100000_invoice_print_snapshots su primijenjene.</v>
       </c>
     </row>
   </sheetData>
@@ -468,6 +470,164 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Partneri</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Zavrsni racun</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Djelimicno implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Arhiva generisanih obrazaca i XML/export.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Partneri</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Zavrsni racun</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Djelimicno implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
@@ -572,7 +732,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E8"/>
   <sheetData>
@@ -678,7 +838,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E9"/>
   <sheetData>
@@ -801,7 +961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E9"/>
   <sheetData>
@@ -924,7 +1084,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E12"/>
   <sheetData>
@@ -1098,7 +1258,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -1393,7 +1553,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z301"/>
   <sheetData>
@@ -1700,7 +1860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z357"/>
   <sheetData>
@@ -5369,7 +5529,52 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>M-010 Računi / KIF-KUF</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C2" t="str">
+        <v>KIF knjiga prikazuje fiskalizovane izlazne račune koji čekaju unos i omogućava grupno preuzimanje kupca, broja, datuma, iznosa i PDV razrade. Izvorni račun i KIF zapis trajno su povezani radi zaštite od duplikata.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Povezati budući ekran izdavanja izlaznih faktura sa lokalnim fiskalnim izvorom i uraditi ručni end-to-end QA na stvarno fiskalizovanom računu.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Migracija 20260804100000_fiskalni_racuni_kif_queue je primijenjena; tenant scope, prava, zaključavanje, PDV stope, duplikati i audit provjeravaju se na backendu.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z365"/>
   <sheetData>
@@ -8787,7 +8992,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z309"/>
   <sheetData>
@@ -9239,7 +9444,7 @@
         <v>Z-017</v>
       </c>
       <c r="B307" t="str">
-        <v>Buduća integracija</v>
+        <v>Integracija u toku</v>
       </c>
       <c r="C307" t="str">
         <v>Fiskalizacija</v>
@@ -9248,16 +9453,19 @@
         <v>Izlazne fakture</v>
       </c>
       <c r="E307" t="str">
-        <v>Fiskalizacija se ne radi u prvoj verziji, ali fakture treba projektovati tako da se kasnije mogu povezati sa fiskalnim API-jem.</v>
+        <v>Produkcijski Summa Fiscal API radi preko HTTPS-a; implementirani su serverski admin klijent, tenant mapiranje, onboarding, kompletna administracija jedinica/ENU-a/operatera/sertifikata i fiskalnog identiteta, readiness, centralna upozorenja, audit filteri, API aplikacije, produkcioni profil, automatski kontrolni test od 1 EUR, activation/production ENU, globalna suspenzija i direktni ili agencijski fiskalni klijenti. Centralni klijent sa platform:admin i konkretnim invoice pravima automatski pokriva sve sadašnje i buduće firme.</v>
       </c>
       <c r="F307" t="str">
-        <v>Ako model fakture nije dobro projektovan, kasnija integracija će biti teža.</v>
+        <v>Direktan poziv iz browsera ili loše mapiran tenant može izložiti ključ, podatke druge firme ili izazvati duplo fiskalizovanje.</v>
       </c>
       <c r="G307" t="str">
-        <v>Zaključeno</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="H307" t="str">
-        <v>MVP 3 / Kasnije</v>
+        <v>MVP 3 / U toku</v>
+      </c>
+      <c r="I307" t="str">
+        <v>Sljedeće je povezivanje izlaznih faktura sa pravima, idempotencyjem i eksplicitnom potvrdom; jednokratne ključeve novih aplikacija treba odmah prenijeti u njihov secret manager.</v>
       </c>
     </row>
     <row r="308">
@@ -9319,69 +9527,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>M-004 Robno</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Robni meni i šifarnici su funkcionalni. Domaća kalkulacija ima obaveznu prodajnu cijenu sa PDV-om, maloprodaju kao default, kompaktne stavke, brzo kreiranje artikla, zavisne troškove i A4 štampu. MAPR link učitava zaglavlje i sve stavke, nudi postojeće/predložene/nove artikle i pamti veze dobavljačevih šifara. Završavanje koristi posebnu šemu iz Robno / Podešavanja, kreira DRAFT nalog i lager, zatim čeka grupno preuzimanje u KUF; preuzeti zapis se ne knjiži ponovo po KUF šemi.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Ručni end-to-end QA MAPR pregleda, završavanja i preuzimanja u KUF sa podešenom robnom šemom; lager lista i kartica artikla; ručna raspodjela zavisnih troškova; uvozna kalkulacija; izlazne fakture i ostali robni dokumenti.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Migracija 20260730130000_kalkulacije_preuzimanje_u_kuf je primijenjena uz backfill četiri postojeća KUF zapisa iz kalkulacija. Prisma klijent je regenerisan, dev server radi, TypeScript je čist i lint nema novih upozorenja; stvarni MAPR primjer sa 28 stavki centovno je usaglašen.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Višestruki QR čitač potvrđen je na 65 stvarnih fajlova, a stvarni import na 145 linkova. Import sada šalje grupe po pet i prikazuje progres; KUF provjerava IIC+PIB+datum u bazi prije MAPR-a i preskače postojeće račune. Neuspjeli fajlovi/linkovi imaju poseban izvještaj, grupni retry i CSV izvoz. Kada novi dobavljač nema zapamćeno KUF konto, svi njegovi računi grupišu se po PIB-u, traže jedan izbor konta i pamte ga za naredne importe. Knjiženje kontroliše svaki KUF račun, koriguje razliku od jednog centa na trošku i za veću razliku jasno označava sporni račun.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Ručni QA novog progres/precheck/retry/CSV toka i grupnog ponovnog importa sa više računa istog novog dobavljača; ručni QA upozorenja za razliku veću od jednog centa; PDV zaključavanje.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Nije potrebna migracija: koristi postojeće fiskalne identifikatore KUF zapisa i firma_komitent.default_kuf_konto_sifra. Read-only simulacija KUF-2026-0004 potvrdila je 133 računa, šest centnih korekcija, bez spornih računa i balans 0 centi. TypeScript je čist, lint nema novih upozorenja.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z336"/>
   <sheetData>
@@ -10780,7 +10926,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z348"/>
   <sheetData>
@@ -12605,7 +12751,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z351"/>
   <sheetData>
@@ -15391,7 +15537,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB350"/>
   <sheetData>
@@ -17329,7 +17475,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -17379,7 +17525,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -17816,7 +17962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z319"/>
   <sheetData>
@@ -18542,7 +18688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -18754,19 +18900,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-004 Robno</v>
+        <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Core implementiran / dorada</v>
       </c>
       <c r="C2" t="str">
-        <v>Robni meni je grupisan na Pregled, Šifarnike, Nabavku, Prodaju, Promet robe i Zalihe. Implementirani su modeli, migracija, prava/audit i ekrani za grupe artikala, artikle/usluge, cijene, jedinice mjere i magacine. Negativan lager se podešava po firmi i opciono po magacinu.</v>
+        <v>KIF sada podržava dnevni i mjesečni pazar sa periodom, brojem izvještaja, kasom, poreskim osnovicama, izlaznim PDV-om i raspodjelom naplate na gotovinu, kartice, virman i ostalo. Preklapanje perioda iste kase je blokirano. Ukupan iznos se kaskadno raspoređuje od najveće aktivne stope ka 0%, uz automatski izlazni PDV. Pazar se prikazuje u KIF-u, štampi, Excel izvozu i izlaznom PDV-u. Podešavanja firme imaju posebna dugujuća konta načina naplate, dok prihod i PDV koriste aktivnu KIF šemu.</v>
       </c>
       <c r="D2" t="str">
-        <v>Stanje/promet zaliha, lager lista, kartica artikla, kalkulacije, izlazne fakture, povrati, prenosi, popis, otpis i nivelacija.</v>
+        <v>Ručni end-to-end QA kreiranja, izmjene, brisanja, zabrane preklapanja, knjiženja i PDV prikaza pazara; PDV zaključavanje KIF/KUF izmjena.</v>
       </c>
       <c r="E2" t="str">
-        <v>Postojeći meni Računi nije mijenjan i ostaje KIF/KUF tok. Sljedeći korak je model lagera prije domaće kalkulacije.</v>
+        <v>Migracija 20260730170000_kif_pazar je primijenjena, Prisma klijent regenerisan i dev server restartovan. TypeScript, Prisma validacija i lint prolaze bez novih grešaka.</v>
       </c>
     </row>
   </sheetData>
@@ -18799,19 +18945,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-003 Nalozi</v>
+        <v>M-004 Robno</v>
       </c>
       <c r="B2" t="str">
-        <v>Početno stanje završeno</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
+        <v>Robni meni i šifarnici su funkcionalni. Domaća kalkulacija ima obaveznu prodajnu cijenu sa PDV-om, maloprodaju kao default, kompaktne stavke, brzo kreiranje artikla, zavisne troškove i A4 štampu. MAPR link učitava zaglavlje i sve stavke, nudi postojeće/predložene/nove artikle i pamti veze dobavljačevih šifara. Završavanje koristi posebnu šemu iz Robno / Podešavanja, kreira DRAFT nalog i lager, zatim čeka grupno preuzimanje u KUF; preuzeti zapis se ne knjiži ponovo po KUF šemi.</v>
       </c>
       <c r="D2" t="str">
-        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
+        <v>Ručni end-to-end QA MAPR pregleda, završavanja i preuzimanja u KUF sa podešenom robnom šemom; lager lista i kartica artikla; ručna raspodjela zavisnih troškova; uvozna kalkulacija; izlazne fakture i ostali robni dokumenti.</v>
       </c>
       <c r="E2" t="str">
-        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
+        <v>Migracija 20260730130000_kalkulacije_preuzimanje_u_kuf je primijenjena uz backfill četiri postojeća KUF zapisa iz kalkulacija. Prisma klijent je regenerisan, dev server radi, TypeScript je čist i lint nema novih upozorenja; stvarni MAPR primjer sa 28 stavki centovno je usaglašen.</v>
       </c>
     </row>
     <row r="3">
@@ -18819,16 +18965,16 @@
         <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B3" t="str">
-        <v>QR čitanje računa završeno</v>
+        <v>Core implementiran / dorada</v>
       </c>
       <c r="C3" t="str">
-        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
+        <v>Višestruki QR čitač potvrđen je na 65 stvarnih fajlova, a stvarni import na 145 linkova. Import sada šalje grupe po pet i prikazuje progres; KUF provjerava IIC+PIB+datum u bazi prije MAPR-a i preskače postojeće račune. Neuspjeli fajlovi/linkovi imaju poseban izvještaj, grupni retry i CSV izvoz. Kada novi dobavljač nema zapamćeno KUF konto, svi njegovi računi grupišu se po PIB-u, traže jedan izbor konta i pamte ga za naredne importe. Knjiženje kontroliše svaki KUF račun, koriguje razliku od jednog centa na trošku i za veću razliku jasno označava sporni račun.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
+        <v>Ručni QA novog progres/precheck/retry/CSV toka i grupnog ponovnog importa sa više računa istog novog dobavljača; ručni QA upozorenja za razliku veću od jednog centa; PDV zaključavanje.</v>
       </c>
       <c r="E3" t="str">
-        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
+        <v>Nije potrebna migracija: koristi postojeće fiskalne identifikatore KUF zapisa i firma_komitent.default_kuf_konto_sifra. Read-only simulacija KUF-2026-0004 potvrdila je 133 računa, šest centnih korekcija, bez spornih računa i balans 0 centi. TypeScript je čist, lint nema novih upozorenja.</v>
       </c>
     </row>
   </sheetData>
@@ -18840,6 +18986,51 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>M-004 Robno</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Robni meni je grupisan na Pregled, Šifarnike, Nabavku, Prodaju, Promet robe i Zalihe. Implementirani su modeli, migracija, prava/audit i ekrani za grupe artikala, artikle/usluge, cijene, jedinice mjere i magacine. Negativan lager se podešava po firmi i opciono po magacinu.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Stanje/promet zaliha, lager lista, kartica artikla, kalkulacije, izlazne fakture, povrati, prenosi, popis, otpis i nivelacija.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Postojeći meni Računi nije mijenjan i ostaje KIF/KUF tok. Sljedeći korak je model lagera prije domaće kalkulacije.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
@@ -18861,36 +19052,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Plate i zaposleni</v>
+        <v>M-003 Nalozi</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Početno stanje završeno</v>
       </c>
       <c r="C2" t="str">
-        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
       </c>
       <c r="D2" t="str">
-        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Firme</v>
+        <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B3" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>QR čitanje računa završeno</v>
       </c>
       <c r="C3" t="str">
-        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
       </c>
       <c r="E3" t="str">
-        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
+        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
       </c>
     </row>
   </sheetData>
@@ -18900,7 +19091,69 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Firme</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -18945,7 +19198,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -18988,162 +19241,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Partneri</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Zavrsni racun</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Djelimicno implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Arhiva generisanih obrazaca i XML/export.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Partneri</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Zavrsni racun</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Djelimicno implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Implement POS fiscalization and accounting flow
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -1555,7 +1555,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z301"/>
+  <dimension ref="A1:Z302"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1853,16 +1853,42 @@
         <v>KIF/KUF knjige po mjesecu i vrsti, PDV razrada, MAPR/SEP import, lokalno QR čitanje PDF/TIFF/JPG/PNG računa, grupni izbor i pamćenje konta za nove KUF dobavljače, šeme kontiranja, automatsko knjiženje, statusi, edit/delete neproknjiženih računa, print i Excel export su implementirani. Ostaju kontrole, XML export, PDV zaključavanje i QA.</v>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>M-011</v>
+      </c>
+      <c r="B302" t="str">
+        <v>POS / Kasa</v>
+      </c>
+      <c r="C302" t="str">
+        <v>Brza mobilna prodaja i fiskalizacija preko postojećeg Fiscal API-ja nad zajedničkim artiklima, cijenama i prodajnim dokumentom.</v>
+      </c>
+      <c r="D302" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Prva funkcionalna faza</v>
+      </c>
+      <c r="F302" t="str">
+        <v>Vlasnik / Kasir / Agencija</v>
+      </c>
+      <c r="G302" t="str">
+        <v>MVP 3</v>
+      </c>
+      <c r="H302" t="str">
+        <v>Postoje mobile-first prodaja, korpa, načini plaćanja, opcioni kupac za gotovinu/karticu i obavezni kupac za virman, POS kasa povezana sa ENU-om, prijava početnog depozita u Test okruženju, kontrolisani retry istog neuspjelog dokumenta, atomarna numeracija, idempotency, istorija pokušaja, fiskalni rezultat, pregled i štampa. POS roba se atomarno razdužuje po prosječnoj nabavnoj cijeni, promet čuva prodaju po artiklu, a minus se može naslijediti sa firme ili podesiti po magacinu kase. Ostaju produkcijska ruta depozita, zbirni KIF/knjiženje, dnevni promet, povrati, smjene i POS Agent.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z301"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z302"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z357"/>
+  <dimension ref="A1:Z358"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5522,9 +5548,47 @@
         <v>Podržani su gotovina, kartice, virman i ostalo; prihodi/PDV koriste KIF šemu, a konta naplate se podešavaju po firmi.</v>
       </c>
     </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>F-096</v>
+      </c>
+      <c r="B358" t="str">
+        <v>POS / Kasa</v>
+      </c>
+      <c r="C358" t="str">
+        <v>Računovodstveni tok po načinu plaćanja</v>
+      </c>
+      <c r="D358" t="str">
+        <v>Fiskalizovani POS virman ulazi pojedinačno u KIF i koristi nalog po šemi izlaznih računa; gotovina i kartica čekaju zbirni dnevni ili mjesečni pazar.</v>
+      </c>
+      <c r="E358" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F358" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="G358" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H358" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I358" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J358" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K358" t="str">
+        <v>M-010,F-062,F-095</v>
+      </c>
+      <c r="L358" t="str">
+        <v>Virman tok i kontrolisani nastavak knjiženja su implementirani. POS dokumenti su isključeni iz kancelarijskog ekrana i akcija izlaznih faktura; gotovina/kartica se ne mogu pojedinačno završavati. KIF razlikuje pojedinačne fiskalne naloge od svog naloga za ručne redove i pazar. Zbirni batch ostaje sljedeća faza.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z357"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z358"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Zavrsi POS storno, izvjestaje i termalnu stampu
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -1867,7 +1867,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="E302" t="str">
-        <v>Prva funkcionalna faza</v>
+        <v>Druga funkcionalna faza</v>
       </c>
       <c r="F302" t="str">
         <v>Vlasnik / Kasir / Agencija</v>
@@ -1876,7 +1876,7 @@
         <v>MVP 3</v>
       </c>
       <c r="H302" t="str">
-        <v>Postoje mobile-first prodaja, korpa, načini plaćanja, opcioni kupac za gotovinu/karticu i obavezni kupac za virman, POS kasa povezana sa ENU-om, prijava početnog depozita u Test okruženju, kontrolisani retry istog neuspjelog dokumenta, atomarna numeracija, idempotency, istorija pokušaja, fiskalni rezultat, pregled i štampa. POS roba se atomarno razdužuje po prosječnoj nabavnoj cijeni, promet čuva prodaju po artiklu, a minus se može naslijediti sa firme ili podesiti po magacinu kase. Ostaju produkcijska ruta depozita, zbirni KIF/knjiženje, dnevni promet, povrati, smjene i POS Agent.</v>
+        <v>Postoje mobile-first prodaja, korpa, načini plaćanja, kupac, POS kasa povezana sa ENU-om, početni depozit u Test okruženju, retry, fiskalizacija, potpuni storno, lager i računovodstveni tok. Virmani ulaze pojedinačno u KIF, a gotovina/kartica kroz zbirni pazar. Dodati su izvještaji po periodu/kasi, plaćanju, PDV-u i artiklima, štampa izvještaja i browser termalna štampa fiskalnog računa za 58/80 mm uz zadržanu A4 opciju. Ostaju produkcijska ruta depozita, reprint audit, djelimični povrat nakon API podrške, smjene i POS Agent.</v>
       </c>
     </row>
   </sheetData>
@@ -1888,7 +1888,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z358"/>
+  <dimension ref="A1:Z360"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5559,13 +5559,13 @@
         <v>Računovodstveni tok po načinu plaćanja</v>
       </c>
       <c r="D358" t="str">
-        <v>Fiskalizovani POS virman ulazi pojedinačno u KIF i koristi nalog po šemi izlaznih računa; gotovina i kartica čekaju zbirni dnevni ili mjesečni pazar.</v>
+        <v>Fiskalizovani POS virman ulazi pojedinačno u KIF i koristi nalog po šemi izlaznih računa; gotovina i kartica ulaze u zbirni dnevni ili mjesečni pazar.</v>
       </c>
       <c r="E358" t="str">
         <v>Vrlo visok</v>
       </c>
       <c r="F358" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Implementirano</v>
       </c>
       <c r="G358" t="str">
         <v>Da</v>
@@ -5583,12 +5583,88 @@
         <v>M-010,F-062,F-095</v>
       </c>
       <c r="L358" t="str">
-        <v>Virman tok i kontrolisani nastavak knjiženja su implementirani. POS dokumenti su isključeni iz kancelarijskog ekrana i akcija izlaznih faktura; gotovina/kartica se ne mogu pojedinačno završavati. KIF razlikuje pojedinačne fiskalne naloge od svog naloga za ručne redove i pazar. Zbirni batch ostaje sljedeća faza.</v>
+        <v>Virman tok ostaje pojedinačan. Zbirna obrada gotovine i kartica kreira idempotentan PAZAR u otvorenom KIF-u, čuva članstvo računa i prati status do zajedničkog KIF naloga i njegovog knjiženja. Automatski POS KIF zapis zaštićen je od ručne izmjene i brisanja.</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>F-097</v>
+      </c>
+      <c r="B359" t="str">
+        <v>POS / Kasa</v>
+      </c>
+      <c r="C359" t="str">
+        <v>Potpuni storno POS računa</v>
+      </c>
+      <c r="D359" t="str">
+        <v>Fiskalizovani POS račun može se potpuno stornirati povezanim negativnim korektivnim dokumentom bez brisanja originala.</v>
+      </c>
+      <c r="E359" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F359" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G359" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H359" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I359" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J359" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K359" t="str">
+        <v>M-011,F-096</v>
+      </c>
+      <c r="L359" t="str">
+        <v>Obavezni razlog i potvrda; Fiscal API storno ruta; povrat robe; obrnuto knjiženje virman računa; inkrementalna korekcija zbirnog pazara; audit i retry. Djelimični povrat čeka API podršku.</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>F-098</v>
+      </c>
+      <c r="B360" t="str">
+        <v>POS / Kasa</v>
+      </c>
+      <c r="C360" t="str">
+        <v>POS izvještaji i termalna štampa</v>
+      </c>
+      <c r="D360" t="str">
+        <v>Promet po periodu i kasi sa neto stornima, plaćanjima, PDV-om i artiklima; fiskalni račun se štampa na 58/80 mm papiru.</v>
+      </c>
+      <c r="E360" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F360" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G360" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H360" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I360" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J360" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K360" t="str">
+        <v>M-011,F-097</v>
+      </c>
+      <c r="L360" t="str">
+        <v>Browser štampa fiskalnog računa čuva A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; stvarni termalni printer i reprint audit ostaju za ručni QA.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z358"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z360"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add POS shifts and warehouse-based pricing
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -1876,7 +1876,7 @@
         <v>MVP 3</v>
       </c>
       <c r="H302" t="str">
-        <v>Postoje mobile-first prodaja, korpa, načini plaćanja, kupac, POS kasa povezana sa ENU-om, početni depozit u Test okruženju, retry, fiskalizacija, potpuni storno, lager i računovodstveni tok. Virmani ulaze pojedinačno u KIF, a gotovina/kartica kroz zbirni pazar. Dodati su izvještaji po periodu/kasi, plaćanju, PDV-u i artiklima, štampa izvještaja i browser termalna štampa fiskalnog računa za 58/80 mm uz zadržanu A4 opciju. Ostaju produkcijska ruta depozita, reprint audit, djelimični povrat nakon API podrške, smjene i POS Agent.</v>
+        <v>Postoje mobile-first prodaja, korpa, načini plaćanja, kupac, POS kasa povezana sa ENU-om, početni depozit u Test okruženju, retry, fiskalizacija, potpuni storno, lager i računovodstveni tok. Virmani ulaze pojedinačno u KIF, a gotovina/kartica kroz zbirni pazar. Dodati su izvještaji po periodu/kasi, browser termalna štampa 58/80 mm i opcione smjene sa presjekom pri predaji kase. Ostaju produkcijska ruta depozita, reprint audit, djelimični povrat nakon API podrške i POS Agent.</v>
       </c>
     </row>
   </sheetData>
@@ -1888,7 +1888,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z360"/>
+  <dimension ref="A1:Z361"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3455,7 +3455,7 @@
         <v>F-039</v>
       </c>
       <c r="L302" t="str">
-        <v>Tabela cijene_artikala modeluje sve tipove; početni UI podržava veleprodajnu i maloprodajnu cijenu, period važenja i unos sa/bez PDV-a. Početne VP/MP cijene mogu se unijeti i prilikom kreiranja artikla.</v>
+        <v>Tabela cijene_artikala modeluje sve tipove; početni UI podržava veleprodajnu i maloprodajnu cijenu, period važenja i unos sa/bez PDV-a. Početne VP/MP cijene mogu se unijeti i prilikom kreiranja artikla. POS bira važeću MP ili VP cijenu prema vrsti magacina povezane kase.</v>
       </c>
     </row>
     <row r="303">
@@ -3493,7 +3493,7 @@
         <v>M-004</v>
       </c>
       <c r="L303" t="str">
-        <v>Implementirani su šifarnik magacina i pravilo negativnog lagera. Veza sa poslovnom jedinicom je odložena dok se uvede njen model.</v>
+        <v>Implementirani su šifarnik magacina, izbor maloprodajnog ili veleprodajnog režima i pravilo negativnog lagera. POS kasa koristi vrstu povezanog magacina. Veza sa poslovnom jedinicom je odložena dok se uvede njen model.</v>
       </c>
     </row>
     <row r="304">
@@ -3551,13 +3551,13 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F305" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Implementirano</v>
       </c>
       <c r="G305" t="str">
         <v>Da</v>
       </c>
       <c r="H305" t="str">
-        <v>Djelimicno</v>
+        <v>Da</v>
       </c>
       <c r="I305" t="str">
         <v>Da</v>
@@ -3569,7 +3569,7 @@
         <v>F-042</v>
       </c>
       <c r="L305" t="str">
-        <v>Podešavanje po firmi i opciono po magacinu je implementirano; sprovođenje pravila slijedi sa dokumentima zaliha.</v>
+        <v>Pravilo firme i opcioni override magacina sprovode se na izlaznim fakturama i POS-u; POS kasa se eksplicitno povezuje sa magacinom prije prodaje robe.</v>
       </c>
     </row>
     <row r="306">
@@ -3835,7 +3835,7 @@
         <v>F-045</v>
       </c>
       <c r="L312" t="str">
-        <v>Podržani su WHOLESALE i RETAIL, uz maloprodaju kao default; maloprodajno stanje prati prodajnu vrijednost, RUC/razliku u cijeni i ukalkulisani PDV.</v>
+        <v>Podržani su WHOLESALE i RETAIL, uz maloprodaju kao default; maloprodajno stanje prati prodajnu vrijednost, RUC/razliku u cijeni i ukalkulisani PDV. POS u maloprodaji čuva konačnu cijenu sa PDV-om i računa osnovicu unazad, a u veleprodaji polazi od cijene bez PDV-a.</v>
       </c>
     </row>
     <row r="313">
@@ -5659,12 +5659,50 @@
         <v>M-011,F-097</v>
       </c>
       <c r="L360" t="str">
-        <v>Browser štampa fiskalnog računa čuva A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; stvarni termalni printer i reprint audit ostaju za ručni QA.</v>
+        <v>Browser štampa fiskalnog računa čuva dvojezičnu srpsko-englesku A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; stvarni termalni printer i reprint audit ostaju za ručni QA.</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>F-099</v>
+      </c>
+      <c r="B361" t="str">
+        <v>POS / Kasa</v>
+      </c>
+      <c r="C361" t="str">
+        <v>Smjenski presjek i predaja kase</v>
+      </c>
+      <c r="D361" t="str">
+        <v>Radnik otvara smjenu sa preuzetom gotovinom, a pri predaji zatvara smjenu i čuva presjek prometa do tog trenutka.</v>
+      </c>
+      <c r="E361" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F361" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G361" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H361" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I361" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J361" t="str">
+        <v>Djelimično</v>
+      </c>
+      <c r="K361" t="str">
+        <v>M-011,F-098</v>
+      </c>
+      <c r="L361" t="str">
+        <v>Jedna otvorena smjena po kasi; presjek čuva račune, plaćanja, ukupan promet i očekivanu gotovinu. Ne mijenja dnevni ili mjesečni KIF zbir.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z360"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z361"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9669,7 +9707,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z336"/>
+  <dimension ref="A1:Z337"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11059,9 +11097,35 @@
         <v>/agencija/racuni/kif/[id]?unos=pazar</v>
       </c>
     </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>E-048</v>
+      </c>
+      <c r="B337" t="str">
+        <v>POS / Kasa</v>
+      </c>
+      <c r="C337" t="str">
+        <v>Smjene i presjeci</v>
+      </c>
+      <c r="D337" t="str">
+        <v>Otvaranje smjene i završni presjek prometa pri predaji kase.</v>
+      </c>
+      <c r="E337" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F337" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G337" t="str">
+        <v>F-099</v>
+      </c>
+      <c r="H337" t="str">
+        <v>/agencija/pos/smjene</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z336"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z337"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -15679,7 +15743,7 @@
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB350"/>
+  <dimension ref="A1:AB351"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -17608,9 +17672,38 @@
         <v>Prisma migracija, validacija šeme, TypeScript i lint prolaze; ruta pazara vraća 200. Ostaje ručni unos i vizuelna potvrda kontrolnih zbirova.</v>
       </c>
     </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>T-081</v>
+      </c>
+      <c r="B351" t="str">
+        <v>POS / Kasa</v>
+      </c>
+      <c r="C351" t="str">
+        <v>Otvaranje i presjek smjene</v>
+      </c>
+      <c r="D351" t="str">
+        <v>Samo jedna smjena može biti otvorena po kasi; zatvaranje čuva zbir računa i plaćanja od otvaranja do presjeka bez promjene KIF batcha.</v>
+      </c>
+      <c r="E351" t="str">
+        <v>F-099</v>
+      </c>
+      <c r="F351" t="str">
+        <v>Djelimično testirano</v>
+      </c>
+      <c r="G351" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="H351">
+        <v>46251.083333333336</v>
+      </c>
+      <c r="I351" t="str">
+        <v>Prisma migracija, TypeScript i lint prolaze; ostaje ručni browser QA otvaranja, prodaje, storna i predaje kase drugom radniku.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB350"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB351"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: update chart of accounts and company purge
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -2733,7 +2733,7 @@
         <v>M-002</v>
       </c>
       <c r="L25" t="str">
-        <v>Globalni osnovni kontni plan implementiran i migration-seedovan iz kontni_plan_GK_KontP.csv: 1514 aktivnih konta. normalni_saldo je podrazumijevani saldo (0/1/2/5 D, 3/4/6 P), nije zabrana knjizenja. Dostupan na /agencija/podesavanja/kontni-plan.</v>
+        <v>Globalni osnovni kontni plan usklađen je sa zadaci/kontni plan.xlsx: 1533 aktivna konta. Puni naziv dolazi iz kolone NAZIV; AK označava obaveznu analitiku, a D korišćenje radne jedinice. Konta uklonjena iz izvora se deaktiviraju radi očuvanja istorije. normalni_saldo je podrazumijevani saldo (0/1/2/5 D, 3/4/6 P), nije zabrana knjiženja. Dostupan na /agencija/podesavanja/kontni-plan.</v>
       </c>
     </row>
     <row r="26">
@@ -5393,7 +5393,7 @@
         <v>M-002</v>
       </c>
       <c r="L353" t="str">
-        <v>Brisanje je jedna backend transakcija sa agencijskim scope-om, audit zapisom i čišćenjem aktivnog konteksta. Zajednički korisnici i globalni/agencijski šifarnici ostaju sačuvani.</v>
+        <v>Brisanje je jedna backend transakcija sa agencijskim scope-om, audit zapisom i čišćenjem aktivnog konteksta. Obuhvata lokalne fiskalne/POS podatke; podaci poslati u zasebni Fiscal API ili Poresku upravu ostaju. Provjera db:check-company-purge pokriva tabele sa firma_id, uz obaveznu ručnu FK provjeru podređenih tabela pri svakoj promjeni šeme.</v>
       </c>
     </row>
     <row r="354">
@@ -17521,10 +17521,10 @@
         <v>Codex</v>
       </c>
       <c r="H345">
-        <v>46227.083333333336</v>
+        <v>46253.083333333336</v>
       </c>
       <c r="I345" t="str">
-        <v>Izolovani integracioni test na dvije privremene firme potvrđuje backend provjeru naziva, brisanje i audit. Dry-run nad stvarnom firmom sa izvodima, nalozima, kontima i agencijskim pravilima prošao je i namjerno je rollbackovan. Ostaje ručni vizuelni QA forme u browseru.</v>
+        <v>Izolovani integracioni test i raniji rollback dry-run potvrđuju osnovni tok. Statička provjera sada potvrđuje svih 53 tabela sa direktnim firma_id, a redosljed je dopunjen lokalnim fiskalnim/POS i podređenim FK tabelama. Ostaju izolovani integracioni test sa fiskalnim/POS zapisima i ručni vizuelni QA; stvarni podaci nijesu brisani.</v>
       </c>
     </row>
     <row r="346">

</xml_diff>

<commit_message>
feat: complete reporting and accounting controls
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,38 +3,42 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-08-20" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-08-19" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-08-08" sheetId="3" r:id="rId3"/>
-    <sheet name="Status 2026-08-07" sheetId="4" r:id="rId4"/>
-    <sheet name="Status 2026-08-04" sheetId="5" r:id="rId5"/>
-    <sheet name="Status 2026-07-30" sheetId="6" r:id="rId6"/>
-    <sheet name="Status 2026-07-29" sheetId="7" r:id="rId7"/>
-    <sheet name="Status 2026-07-26" sheetId="8" r:id="rId8"/>
-    <sheet name="Status 2026-07-25" sheetId="9" r:id="rId9"/>
-    <sheet name="Status 2026-07-24" sheetId="10" r:id="rId10"/>
-    <sheet name="Status 2026-07-09" sheetId="11" r:id="rId11"/>
-    <sheet name="Status 2026-07-07" sheetId="12" r:id="rId12"/>
-    <sheet name="Status 2026-07-06" sheetId="13" r:id="rId13"/>
-    <sheet name="Status 2026-07-05" sheetId="14" r:id="rId14"/>
-    <sheet name="Status 2026-07-02" sheetId="15" r:id="rId15"/>
-    <sheet name="Status 2026-06-30" sheetId="16" r:id="rId16"/>
-    <sheet name="Status 2026-06-29" sheetId="17" r:id="rId17"/>
-    <sheet name="Status 2026-06-28" sheetId="18" r:id="rId18"/>
-    <sheet name="Status 2026-06-25" sheetId="19" r:id="rId19"/>
-    <sheet name="Dashboard" sheetId="20" r:id="rId20"/>
-    <sheet name="Moduli" sheetId="21" r:id="rId21"/>
-    <sheet name="Funkcionalnosti" sheetId="22" r:id="rId22"/>
-    <sheet name="Pravila" sheetId="23" r:id="rId23"/>
-    <sheet name="Zavisnosti" sheetId="24" r:id="rId24"/>
-    <sheet name="Ekrani" sheetId="25" r:id="rId25"/>
-    <sheet name="Baza" sheetId="26" r:id="rId26"/>
-    <sheet name="API" sheetId="27" r:id="rId27"/>
-    <sheet name="Testovi" sheetId="28" r:id="rId28"/>
-    <sheet name="Bugovi" sheetId="29" r:id="rId29"/>
-    <sheet name="Ideje" sheetId="30" r:id="rId30"/>
-    <sheet name="Odluke" sheetId="31" r:id="rId31"/>
-    <sheet name="Kategorije" sheetId="32" r:id="rId32"/>
+    <sheet name="Status 2026-08-31" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-08-30" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-08-25" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-08-23" sheetId="4" r:id="rId4"/>
+    <sheet name="Status 2026-08-20" sheetId="5" r:id="rId5"/>
+    <sheet name="Status 2026-08-19" sheetId="6" r:id="rId6"/>
+    <sheet name="Status 2026-08-08" sheetId="7" r:id="rId7"/>
+    <sheet name="Status 2026-08-07" sheetId="8" r:id="rId8"/>
+    <sheet name="Status 2026-08-04" sheetId="9" r:id="rId9"/>
+    <sheet name="Status 2026-07-30" sheetId="10" r:id="rId10"/>
+    <sheet name="Status 2026-07-29" sheetId="11" r:id="rId11"/>
+    <sheet name="Status 2026-07-26" sheetId="12" r:id="rId12"/>
+    <sheet name="Status 2026-07-25" sheetId="13" r:id="rId13"/>
+    <sheet name="Status 2026-07-24" sheetId="14" r:id="rId14"/>
+    <sheet name="Status 2026-07-09" sheetId="15" r:id="rId15"/>
+    <sheet name="Status 2026-07-07" sheetId="16" r:id="rId16"/>
+    <sheet name="Status 2026-07-06" sheetId="17" r:id="rId17"/>
+    <sheet name="Status 2026-07-05" sheetId="18" r:id="rId18"/>
+    <sheet name="Status 2026-07-02" sheetId="19" r:id="rId19"/>
+    <sheet name="Status 2026-06-30" sheetId="20" r:id="rId20"/>
+    <sheet name="Status 2026-06-29" sheetId="21" r:id="rId21"/>
+    <sheet name="Status 2026-06-28" sheetId="22" r:id="rId22"/>
+    <sheet name="Status 2026-06-25" sheetId="23" r:id="rId23"/>
+    <sheet name="Dashboard" sheetId="24" r:id="rId24"/>
+    <sheet name="Moduli" sheetId="25" r:id="rId25"/>
+    <sheet name="Funkcionalnosti" sheetId="26" r:id="rId26"/>
+    <sheet name="Pravila" sheetId="27" r:id="rId27"/>
+    <sheet name="Zavisnosti" sheetId="28" r:id="rId28"/>
+    <sheet name="Ekrani" sheetId="29" r:id="rId29"/>
+    <sheet name="Baza" sheetId="30" r:id="rId30"/>
+    <sheet name="API" sheetId="31" r:id="rId31"/>
+    <sheet name="Testovi" sheetId="32" r:id="rId32"/>
+    <sheet name="Bugovi" sheetId="33" r:id="rId33"/>
+    <sheet name="Ideje" sheetId="34" r:id="rId34"/>
+    <sheet name="Odluke" sheetId="35" r:id="rId35"/>
+    <sheet name="Kategorije" sheetId="36" r:id="rId36"/>
   </sheets>
 </workbook>
 </file>
@@ -428,6 +432,85 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nalozi / Bruto bilans</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Ispravljeno</v>
+      </c>
+      <c r="C2" t="str">
+        <v>A4 landscape štampa sa osam eksplicitnih kolona, neprelomivim tabularnim iznosima, urednim prelomom naziva konta, ponovljenim zaglavljem i redovima koji se ne cijepaju preko stranice.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Bruto bilans više ne nasljeđuje sedmokolonske širine Bilansa stanja. Nema migracije baze; TypeScript, ESLint i diff provjera prolaze.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Nalozi / Kartica konta</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dugme za štampu prenosi konto, partnera i period na čistu A4 landscape karticu sa početnim saldom, POSTED prometom, tekućim saldom i ukupnim zbirom.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Ruta provjerava agenciju, dodjelu firme, poslovnu godinu, konto i scope partnera. Nema migracije baze; TypeScript i ESLint prolaze.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Završni račun / Kontrole</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Read-only kontrolni centar prikazuje ukupni status i provjere glavne knjige, KIF/KUF-a, dokumenata, izvoda, plata, PDV-a, šablona, rezultatskih konta, klasa 5/6, korekcija, arhive i matičnih podataka. Izvorna PDV konta moraju imati saldo 0,00; klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>XML/export završnog računa ostaje otvoren; po potrebi proširiti dodatnim zakonskim kontrolama.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Svako sporno konto vodi direktno na svoju karticu. Prijavljena ruta vraća HTTP 200; nema migracije baze.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
@@ -449,19 +532,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Fiskalni klijent i agencija</v>
+        <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B2" t="str">
-        <v>Implementirano</v>
+        <v>Core implementiran / dorada</v>
       </c>
       <c r="C2" t="str">
-        <v>Uključivanje fiskalizacije izborom postojeće firme agencije; globalna PIB detekcija; zahtjev i platformsko odobrenje/odbijanje prelaska direktnog klijenta bez duplikata.</v>
+        <v>KIF sada podržava dnevni i mjesečni pazar sa periodom, brojem izvještaja, kasom, poreskim osnovicama, izlaznim PDV-om i raspodjelom naplate na gotovinu, kartice, virman i ostalo. Preklapanje perioda iste kase je blokirano. Ukupan iznos se kaskadno raspoređuje od najveće aktivne stope ka 0%, uz automatski izlazni PDV. Pazar se prikazuje u KIF-u, štampi, Excel izvozu i izlaznom PDV-u. Podešavanja firme imaju posebna dugujuća konta načina naplate, dok prihod i PDV koriste aktivnu KIF šemu.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA transfera na testnoj firmi i naknadna implementacija klijentskog dashboarda sa dugmetom Fiskalizacija.</v>
+        <v>Ručni end-to-end QA kreiranja, izmjene, brisanja, zabrane preklapanja, knjiženja i PDV prikaza pazara; PDV zaključavanje KIF/KUF izmjena.</v>
       </c>
       <c r="E2" t="str">
-        <v>Isti firma_id i Fiscal API veza ostaju kanonski; transfer firm-specific tenant scope-a je auditovan.</v>
+        <v>Migracija 20260730170000_kif_pazar je primijenjena, Prisma klijent regenerisan i dev server restartovan. TypeScript, Prisma validacija i lint prolaze bez novih grešaka.</v>
       </c>
     </row>
   </sheetData>
@@ -471,7 +554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <sheetData>
@@ -494,86 +577,41 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Plate i zaposleni</v>
+        <v>M-004 Robno</v>
       </c>
       <c r="B2" t="str">
         <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+        <v>Robni meni i šifarnici su funkcionalni. Domaća kalkulacija ima obaveznu prodajnu cijenu sa PDV-om, maloprodaju kao default, kompaktne stavke, brzo kreiranje artikla, zavisne troškove i A4 štampu. MAPR link učitava zaglavlje i sve stavke, nudi postojeće/predložene/nove artikle i pamti veze dobavljačevih šifara. Završavanje koristi posebnu šemu iz Robno / Podešavanja, kreira DRAFT nalog i lager, zatim čeka grupno preuzimanje u KUF; preuzeti zapis se ne knjiži ponovo po KUF šemi.</v>
       </c>
       <c r="D2" t="str">
-        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+        <v>Ručni end-to-end QA MAPR pregleda, završavanja i preuzimanja u KUF sa podešenom robnom šemom; lager lista i kartica artikla; ručna raspodjela zavisnih troškova; uvozna kalkulacija; izlazne fakture i ostali robni dokumenti.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+        <v>Migracija 20260730130000_kalkulacije_preuzimanje_u_kuf je primijenjena uz backfill četiri postojeća KUF zapisa iz kalkulacija. Prisma klijent je regenerisan, dev server radi, TypeScript je čist i lint nema novih upozorenja; stvarni MAPR primjer sa 28 stavki centovno je usaglašen.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Firme</v>
+        <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B3" t="str">
         <v>Core implementiran / dorada</v>
       </c>
       <c r="C3" t="str">
-        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+        <v>Višestruki QR čitač potvrđen je na 65 stvarnih fajlova, a stvarni import na 145 linkova. Import sada šalje grupe po pet i prikazuje progres; KUF provjerava IIC+PIB+datum u bazi prije MAPR-a i preskače postojeće račune. Neuspjeli fajlovi/linkovi imaju poseban izvještaj, grupni retry i CSV izvoz. Kada novi dobavljač nema zapamćeno KUF konto, svi njegovi računi grupišu se po PIB-u, traže jedan izbor konta i pamte ga za naredne importe. Knjiženje kontroliše svaki KUF račun, koriguje razliku od jednog centa na trošku i za veću razliku jasno označava sporni račun.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+        <v>Ručni QA novog progres/precheck/retry/CSV toka i grupnog ponovnog importa sa više računa istog novog dobavljača; ručni QA upozorenja za razliku veću od jednog centa; PDV zaključavanje.</v>
       </c>
       <c r="E3" t="str">
-        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
+        <v>Nije potrebna migracija: koristi postojeće fiskalne identifikatore KUF zapisa i firma_komitent.default_kuf_konto_sifra. Read-only simulacija KUF-2026-0004 potvrdila je 133 računa, šest centnih korekcija, bez spornih računa i balans 0 centi. TypeScript je čist, lint nema novih upozorenja.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Plate</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -601,19 +639,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Zavrsni racun</v>
+        <v>M-004 Robno</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimicno implementirano</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
+        <v>Robni meni je grupisan na Pregled, Šifarnike, Nabavku, Prodaju, Promet robe i Zalihe. Implementirani su modeli, migracija, prava/audit i ekrani za grupe artikala, artikle/usluge, cijene, jedinice mjere i magacine. Negativan lager se podešava po firmi i opciono po magacinu.</v>
       </c>
       <c r="D2" t="str">
-        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
+        <v>Stanje/promet zaliha, lager lista, kartica artikla, kalkulacije, izlazne fakture, povrati, prenosi, popis, otpis i nivelacija.</v>
       </c>
       <c r="E2" t="str">
-        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
+        <v>Postojeći meni Računi nije mijenjan i ostaje KIF/KUF tok. Sljedeći korak je model lagera prije domaće kalkulacije.</v>
       </c>
     </row>
   </sheetData>
@@ -625,6 +663,220 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>M-003 Nalozi</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Početno stanje završeno</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>M-010 Računi / KIF-KUF</v>
+      </c>
+      <c r="B3" t="str">
+        <v>QR čitanje računa završeno</v>
+      </c>
+      <c r="C3" t="str">
+        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Firme</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Plate</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Zavrsni racun</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Djelimicno implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
@@ -702,7 +954,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
   <sheetData>
@@ -781,7 +1033,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E8"/>
   <sheetData>
@@ -883,532 +1135,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-30</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Oblast</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Sta je zavrseno</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Sta ostaje</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Preporuceni sljedeci korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C5" t="str">
-        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C7" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C8" t="str">
-        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Redovno održavanje.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Regenerisati Excel nakon svake veće promjene.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-29</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Oblast</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Sta je zavrseno</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Sta ostaje</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Preporuceni sljedeci korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Core zaokruzen</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Core zaokruzen</v>
-      </c>
-      <c r="C6" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>KIF/KUF</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Core implementiran</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C9" t="str">
-        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Regenerisati Excel nakon svake vece promjene.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-28</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Oblast</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Sta je zavrseno</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Sta ostaje</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Preporuceni sljedeci korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Performanse partnera</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Core implementiran</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Pratiti brzinu na produkciji.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Indeksi baze</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>-</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>KIF/KUF uvoz/export</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Core implementiran</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata; XML export.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>QA uvoznih knjizenja i export fajlova.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Dokumentacija</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Uspostavljeno</v>
-      </c>
-      <c r="C8" t="str">
-        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Azurirati uz svaku vecu promjenu.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Prva implementacija</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-25</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Ovaj list je kratki pregled šta je stvarno implementirano u aplikaciji, nezavisno od početne specifikacije.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Oblast</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Šta je završeno</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Šta ostaje</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Preporučeni sljedeći korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Navigacija i kontekst</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Core implementiran</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Fiksni lijevi meni, gornji podmeniji, globalni izbor agencije/firme/godine/korisnika, dodata sekcija Računi.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Sakriti/zaključati menije po pravima i dodati kompletne podmenije budućih modula.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Dorađivati po modulu kad se modul stvarno implementira.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>M-001 Korisnici/agencije/prava</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Login, admin/agencija korisnici, radnici/klijenti, dodjela firmi, matrica prava, audit osnova.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Backend enforcement prava kroz sve rute, pretplate/limiti, statistika radnika, testovi.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Zaključati prava na server actions prije šire produkcije.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>M-002 Firme/kontni plan/partneri</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Firme, IRMS, poslovne godine, banke, ugovor/cijena, globalni kontni plan + override, globalni/agencijski/firmski partneri, import globalnih partnera.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Odgovorna lica, puna izmjena firme, default konta po firmi/dobavljaču, podešavanja firme.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Dovršiti default konta i partner/firma preference koje KIF/KUF već koriste.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>M-003 Nalozi</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Novi/izmjena naloga, nacrt, proknjižavanje, brisanje, partner analitika, datumi stavki, F9/F10, bruto bilans, analitičke kartice, print naloga i bruto bilansa.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Formalni prenos početnog stanja, jači testovi, izvještaji po poslovnoj jedinici, permission checks.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Napisati testove za validaciju stavki i za automatsko knjiženje iz KIF/KUF.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>M-006 Računi KIF/KUF</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Core implementiran / dorada</v>
-      </c>
-      <c r="C9" t="str">
-        <v>PDV stope, KIF/KUF knjige po mjesecu/vrsti, šeme kontiranja, MAPR link/F8, batch import, SEP Excel import za KIF, automatsko knjiženje knjige, edit/delete neproknjiženih, statusi na srpskom, print KIF/KUF.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Kontrole/duplikati, export, PDV zaključavanje, payment status, cache MAPR-a, PDF/QR čitanje, završni QA printa.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Dovršiti kontrole i testove, zatim krenuti PDV prijavu iz KIF/KUF.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>M-004 Robno</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Nije implementirano</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Specifikacija pročitana i unesena u planer.</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Cijeli modul: artikli, magacini, lager, kalkulacije, popis, otpis, nivelacija, automatsko knjiženje.</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Poslije stabilizacije KIF/KUF i PDV osnove krenuti na artikle/magacine.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Izvodi/PDF</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Priprema</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Instaliran pdfjs-dist za buduće čitanje tekstualnih PDF izvoda.</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Parser izvoda, QR iz PDF/TIFF, automatsko knjiženje izvoda.</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Kada se krene na izvode, prvo napraviti parser za jednu banku.</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>PDV/Plate/Završni/Reports</v>
-      </c>
-      <c r="B12" t="str">
-        <v>U planu / djelimično</v>
-      </c>
-      <c r="C12" t="str">
-        <v>PDV stope i bruto bilans postoje; ostalo uglavnom placeholder.</v>
-      </c>
-      <c r="D12" t="str">
-        <v>PDV prijava, plate, završni račun, dashboard i izvještaji.</v>
-      </c>
-      <c r="E12" t="str">
-        <v>PDV prijava treba da dođe poslije finalizacije KIF/KUF kontrola.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1436,36 +1162,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-012 Portal direktnog fiskalnog klijenta</v>
+        <v>Robno / Izvještaji</v>
       </c>
       <c r="B2" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dogovoren je poseban mobile-first /portal sa automatskim kontekstom jedne firme, operativnim dashboardom, POS-om, klasičnim bezgotovinskim fakturama, jedinstvenim pregledom fiskalnih računa, izvještajima, artiklima, kupcima i ograničenim podešavanjima.</v>
+        <v>Lager lista po magacinu i artiklu sa vrijednostima i filterima; kartica artikla sa početnim stanjem perioda, ulazima, izlazima, tekućim stanjem i linkovima na dokumente. Oba prikaza dostupna su u Robnom i centralnim Izvještajima.</v>
       </c>
       <c r="D2" t="str">
-        <v>Implementirati sigurnosni portal guard i zabranu /agencija pristupa, zatim dashboard, oba prodajna toka, izvještaje i šifarnike prema DIRECT_FISCAL_CLIENT_PORTAL_SPEC.md.</v>
+        <v>Live QA sa stvarnim prometima kada lokalna PostgreSQL baza bude dostupna; buduće štampe/exporti po potrebi.</v>
       </c>
       <c r="E2" t="str">
-        <v>Fiskalna konfiguracija, sertifikati, ENU, operateri, aktivacija i suspenzija ostaju isključivo platformskom adminu; direct FISCAL_ONLY dokumenti ne kreiraju KIF ni nalog.</v>
+        <v>Nema migracije baze. TypeScript i ESLint prolaze bez grešaka; ostaju četiri ranija lint upozorenja.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Dokumentacija i planer</v>
+        <v>Centralni izvještaji</v>
       </c>
       <c r="B3" t="str">
-        <v>Usklađeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="C3" t="str">
-        <v>Dodata detaljna implementaciona specifikacija i ažurirani fiskalni README, POS specifikacija, CURRENT_STATE, NEXT_STEPS, SESSION_LOG i arhitektura.</v>
+        <v>Kartica konta ima pretraživ spisak konta lijevo, desni detalj, izbor konta sa prometom/svih aktivnih i mobilni tok lista-detalj. Kartica partnera koristi postojeću analitičku karticu; PDV koristi mjesečni pregled perioda; plate vode na obračune, M-4, OPP-ND i IOPPD.</v>
       </c>
       <c r="D3" t="str">
-        <v>Aplikacijski kod, Prisma šema i migracije nijesu mijenjani.</v>
+        <v>Centralno povezati preostale postojeće izvještaje kupaca, dobavljača i finansijskih obrazaca.</v>
       </c>
       <c r="E3" t="str">
-        <v>Status označava dogovoreni plan, ne završenu funkcionalnost.</v>
+        <v>Nema migracije baze niti dupliranja računice; postojeće backend provjere prava i konteksta ostaju mjerodavne.</v>
       </c>
     </row>
   </sheetData>
@@ -1477,6 +1203,532 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E8"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-30</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C5" t="str">
+        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Nalozi</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Core zaokružen</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core zaokružen</v>
+      </c>
+      <c r="C7" t="str">
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Planer/Dokumentacija</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Ažurirano</v>
+      </c>
+      <c r="C8" t="str">
+        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Redovno održavanje.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Regenerisati Excel nakon svake veće promjene.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Nalozi</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core zaokruzen</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Core zaokruzen</v>
+      </c>
+      <c r="C6" t="str">
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>KIF/KUF</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Planer/Dokumentacija</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Ažurirano</v>
+      </c>
+      <c r="C9" t="str">
+        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Redovno odrzavanje.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Regenerisati Excel nakon svake vece promjene.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Performanse partnera</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pratiti brzinu na produkciji.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Indeksi baze</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KIF/KUF uvoz/export</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kontrole iznosa i duplikata; XML export.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>QA uvoznih knjizenja i export fajlova.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Dokumentacija</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Uspostavljeno</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Redovno odrzavanje.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Azurirati uz svaku vecu promjenu.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Prva implementacija</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E12"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-25</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Ovaj list je kratki pregled šta je stvarno implementirano u aplikaciji, nezavisno od početne specifikacije.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Šta je završeno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Šta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporučeni sljedeći korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Navigacija i kontekst</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Fiksni lijevi meni, gornji podmeniji, globalni izbor agencije/firme/godine/korisnika, dodata sekcija Računi.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Sakriti/zaključati menije po pravima i dodati kompletne podmenije budućih modula.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Dorađivati po modulu kad se modul stvarno implementira.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>M-001 Korisnici/agencije/prava</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Login, admin/agencija korisnici, radnici/klijenti, dodjela firmi, matrica prava, audit osnova.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Backend enforcement prava kroz sve rute, pretplate/limiti, statistika radnika, testovi.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Zaključati prava na server actions prije šire produkcije.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>M-002 Firme/kontni plan/partneri</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Firme, IRMS, poslovne godine, banke, ugovor/cijena, globalni kontni plan + override, globalni/agencijski/firmski partneri, import globalnih partnera.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Odgovorna lica, puna izmjena firme, default konta po firmi/dobavljaču, podešavanja firme.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Dovršiti default konta i partner/firma preference koje KIF/KUF već koriste.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>M-003 Nalozi</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Novi/izmjena naloga, nacrt, proknjižavanje, brisanje, partner analitika, datumi stavki, F9/F10, bruto bilans, analitičke kartice, print naloga i bruto bilansa.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Formalni prenos početnog stanja, jači testovi, izvještaji po poslovnoj jedinici, permission checks.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Napisati testove za validaciju stavki i za automatsko knjiženje iz KIF/KUF.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>M-006 Računi KIF/KUF</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C9" t="str">
+        <v>PDV stope, KIF/KUF knjige po mjesecu/vrsti, šeme kontiranja, MAPR link/F8, batch import, SEP Excel import za KIF, automatsko knjiženje knjige, edit/delete neproknjiženih, statusi na srpskom, print KIF/KUF.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Kontrole/duplikati, export, PDV zaključavanje, payment status, cache MAPR-a, PDF/QR čitanje, završni QA printa.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Dovršiti kontrole i testove, zatim krenuti PDV prijavu iz KIF/KUF.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>M-004 Robno</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Nije implementirano</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Specifikacija pročitana i unesena u planer.</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Cijeli modul: artikli, magacini, lager, kalkulacije, popis, otpis, nivelacija, automatsko knjiženje.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Poslije stabilizacije KIF/KUF i PDV osnove krenuti na artikle/magacine.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Izvodi/PDF</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Priprema</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Instaliran pdfjs-dist za buduće čitanje tekstualnih PDF izvoda.</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Parser izvoda, QR iz PDF/TIFF, automatsko knjiženje izvoda.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Kada se krene na izvode, prvo napraviti parser za jednu banku.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>PDV/Plate/Završni/Reports</v>
+      </c>
+      <c r="B12" t="str">
+        <v>U planu / djelimično</v>
+      </c>
+      <c r="C12" t="str">
+        <v>PDV stope i bruto bilans postoje; ostalo uglavnom placeholder.</v>
+      </c>
+      <c r="D12" t="str">
+        <v>PDV prijava, plate, završni račun, dashboard i izvještaji.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>PDV prijava treba da dođe poslije finalizacije KIF/KUF kontrola.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
     <row r="1">
@@ -1770,7 +2022,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z303"/>
   <sheetData>
@@ -1833,7 +2085,7 @@
         <v>MVP 1</v>
       </c>
       <c r="H5" t="str">
-        <v>Autentifikacija, agencije, korisnici, radnici/klijenti, dodjela firmi, matrica prava i audit osnova postoje. Ostaju kompletan backend enforcement prava, pretplate/limiti i statistika radnika.</v>
+        <v>Autentifikacija, agencije, korisnici, radnici/klijenti, dodjela firmi, matrica prava i audit osnova postoje. Agencijski shell ima sklopivi desktop meni sa pamćenjem izbora i mobilni bočni panel. Ostaju kompletan backend enforcement prava, pretplate/limiti i statistika radnika.</v>
       </c>
     </row>
     <row r="6">
@@ -1885,7 +2137,7 @@
         <v>MVP 1</v>
       </c>
       <c r="H7" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke, prečice F9/F10, bruto bilans, analitičke kartice, print i automatski DRAFT prenos početnog stanja klasa 0-4 su implementirani. Ostaju kontrole po poslovnoj jedinici i dodatni automatizovani testovi.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, vraćanje, brisanje, partner analitika, kupci/dobavljaci zbirno, otvorene stavke, prečice F9/F10, bruto bilans, analitičke kartice, A4 landscape print bruto bilansa i kartice konta te automatski DRAFT prenos početnog stanja klasa 0-4 su implementirani. Ostaju kontrole po poslovnoj jedinici i dodatni automatizovani testovi.</v>
       </c>
     </row>
     <row r="8">
@@ -1911,7 +2163,7 @@
         <v>MVP 1/2</v>
       </c>
       <c r="H8" t="str">
-        <v>Meni i šifarnici su implementirani. Domaća kalkulacija ima nacrt, obaveznu prodajnu cijenu, više PDV stopa, MAPR pregled i povezivanje ili atomarno kreiranje novih artikala, kompaktnu tabelu, zavisne troškove i A4 štampu. Završavanje kreira DRAFT nalog i lager prema posebnoj šemi, a KUF je naknadno preuzima kao knjiženu kroz kalkulaciju bez duplog naloga. Slijede ručni QA, lager lista/kartica, uvozna kalkulacija, izlazne fakture i ostali robni dokumenti.</v>
+        <v>Meni i šifarnici su implementirani. Domaća kalkulacija ima nacrt, obaveznu prodajnu cijenu, više PDV stopa, MAPR pregled i povezivanje ili atomarno kreiranje novih artikala, kompaktnu tabelu, zavisne troškove i A4 štampu. Završavanje kreira DRAFT nalog i lager prema posebnoj šemi, a KUF je naknadno preuzima kao knjiženu kroz kalkulaciju bez duplog naloga. Lager lista i kartica artikla postoje u Robnom i centralnim Izvještajima nad zajedničkim stanjem/prometom. Slijede live QA, uvozna kalkulacija i ostali robni dokumenti.</v>
       </c>
     </row>
     <row r="9">
@@ -1963,7 +2215,7 @@
         <v>MVP 2</v>
       </c>
       <c r="H10" t="str">
-        <v>Prva MVP osnova postoji: tabele i šifarnici za IOPPD, vrste obračuna, poreze, doprinose, prirez, šifre primanja i osnove obračuna; stranice za zaposlene sa dodavanjem, izmjenom, odjavom/reaktivacijom i tabovima aktivni/neaktivni, kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, priprema radnika u nacrtu, kontrole prije obrade, ručne mjesečne korekcije po radniku, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz obračuna; bruto/neto obračun čita važeće stope iz baze i strukturisana pravila osnova za linearne šifre poput ugovora i zakupa, minuli rad se računa progresivno po navršenim godinama staža, a u bazu je importovano svih 108 osnova iz zvaničnog Excel šifarnika, sa originalnim redom sačuvanim u JSON-u pravila i šiframa primanja generisanim za izbor kod radnika. Dodato je 25 obračunskih podšifara iz A_SifR sa hijerarhijom, koeficijentima iznosa/staža, posebnim osnovicama i fondom sati, bez preuzimanja zastarjelih stopa. Podešavanja plata su grupisana: IOPPD šifre otvaraju postojeći šifarnik, a podešavanje knjiženja čuva posebnu šemu D/P konta za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun se akcijom Proknjiži transakcijski pretvara u izbalansiran i odmah POSTED PAYROLL nalog, uz trajnu vezu i blokadu duplog knjiženja. M-4, OPP-ND i IOPPD grupisani su u drugom nivou podmenija Obrasci. IOPPD ima mjesečni pregled, HTML/CSS štampu i XML download. M-4 je završen u dogovorenom obimu: godišnji pregled, matični podaci iz firme, potvrđene uplate, pojedinačni obrazac, Tabela 1 i Tabela 2. OPP-ND razvrstava porez na četiri službene vrste, primjenjuje važeću opštinsku stopu firme i generiše A4 prijavu prema zvaničnom PDF-u. Globalni šifarnik prireza sadrži 21 opštinu sa DJP šiframa, stopama i raspoloživim računima iz stare MDB baze i koristi ga obračun plata, M-4 i OPP-ND. U modulu plata ostaju obustave, opisna pravila koja traže ručne parametre, uplatnice, namjenski storno/vraćanje automatskog naloga te print/export obračuna.</v>
+        <v>Prva MVP osnova postoji: tabele i šifarnici za IOPPD, vrste obračuna, poreze, doprinose, prirez, šifre primanja i osnove obračuna; stranice za zaposlene sa dodavanjem, izmjenom, odjavom/reaktivacijom i tabovima aktivni/neaktivni, kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, priprema radnika u nacrtu, kontrole prije obrade, ručne mjesečne korekcije po radniku, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz obračuna. Stavke podržavaju pojedinačni datum od/do, automatske sate prema periodu i fondu, ručni override sa auditom i radnika koji počne ili završi rad tokom mjeseca. Bruto/neto obračun čita važeće stope iz baze i strukturisana pravila osnova za linearne šifre poput ugovora i zakupa, minuli rad se računa progresivno po navršenim godinama staža, a u bazu je importovano svih 108 osnova iz zvaničnog Excel šifarnika, sa originalnim redom sačuvanim u JSON-u pravila i šiframa primanja generisanim za izbor kod radnika. Dodato je 25 obračunskih podšifara iz A_SifR sa hijerarhijom, koeficijentima iznosa/staža, posebnim osnovicama i fondom sati, bez preuzimanja zastarjelih stopa. Podešavanja plata su grupisana: IOPPD šifre otvaraju postojeći šifarnik, a podešavanje knjiženja čuva posebnu šemu D/P konta za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun se akcijom Proknjiži transakcijski pretvara u izbalansiran i odmah POSTED PAYROLL nalog, uz trajnu vezu i blokadu duplog knjiženja. M-4, OPP-ND i IOPPD grupisani su u drugom nivou podmenija Obrasci. IOPPD ima mjesečni pregled, HTML/CSS štampu i XML download. M-4 je završen u dogovorenom obimu: godišnji pregled, matični podaci iz firme, potvrđene uplate, pojedinačni obrazac, Tabela 1 i Tabela 2. OPP-ND razvrstava porez na četiri službene vrste, primjenjuje važeću opštinsku stopu firme i generiše A4 prijavu prema zvaničnom PDF-u. Globalni šifarnik prireza sadrži 21 opštinu sa DJP šiframa, stopama i raspoloživim računima iz stare MDB baze i koristi ga obračun plata, M-4 i OPP-ND. U modulu plata ostaju kalendar praznika/nestandardnih smjena, obustave, opisna pravila koja traže ručne parametre, uplatnice, namjenski storno/vraćanje automatskog naloga te print/export obračuna.</v>
       </c>
     </row>
     <row r="11">
@@ -2015,7 +2267,7 @@
         <v>MVP 3</v>
       </c>
       <c r="H12" t="str">
-        <v>Prva implementacija Bilansa uspjeha, Bilansa stanja i Statističkog aneksa postoji: šabloni pozicija, obračun iz POSTED naloga, prethodne kolone, podešavanja konta/formula po firmi, trajne ručne korekcije po AOP/koloni, print obrasci, predlog zaključnog naloga za klase 5/6 i arhiva snimljenih obrazaca. Ostaje XML/export.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statistički aneks imaju šablone, obračun iz POSTED naloga, prethodne kolone, podešavanja po firmi, trajne ručne korekcije i print. Objedinjene kontrole provjeravaju glavnu knjigu, pomoćne evidencije, šeme, konta rezultata, zatvaranje klasa 5/6, korekcije, arhivu i matične podatke; postoje i predlog zaključnog naloga i arhiva snimljenih obrazaca. Ostaje XML/export.</v>
       </c>
     </row>
     <row r="13">
@@ -2041,7 +2293,7 @@
         <v>MVP 1/2</v>
       </c>
       <c r="H13" t="str">
-        <v>Bruto bilans i analitičke kartice postoje. Dashboard i ostali izvještaji su uglavnom placeholderi.</v>
+        <v>Bruto bilans i analitičke kartice postoje. Početni agencijski dashboard prikazuje tenant/permission-aware nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF. Centralni Izvještaji imaju funkcionalne kartice konta i partnera, PDV pregled, pregled izvještaja plata, lager listu i karticu artikla preko postojećih zajedničkih prikaza; kupci, dobavljači i finansijski izvještaji ostaju za centralno povezivanje.</v>
       </c>
     </row>
     <row r="301">
@@ -2110,7 +2362,7 @@
         <v>Vrlo visok</v>
       </c>
       <c r="E303" t="str">
-        <v>Specifikacija spremna</v>
+        <v>Implementirano / ručni QA</v>
       </c>
       <c r="F303" t="str">
         <v>Vlasnik / Kasir / Pregled</v>
@@ -2119,7 +2371,7 @@
         <v>MVP 3</v>
       </c>
       <c r="H303" t="str">
-        <v>Implementacija nije započeta. Portal koristi postojeće korisnike, prava, FiskalniIzlazniRacun, artikle, kupce, POS i Fiscal API; sistemski tenant i fiskalna administracija ostaju skriveni.</v>
+        <v>Implementirani su backend guard i automatski kontekst jedne firme/godine, permission-aware navigacija, dashboard, POS, OFFICE fakture, računi, puni storno, A4 i 58/80 mm štampa sa auditom, izvještaji/export, artikli, cijene, kupci i operativna podešavanja. Direktni FISCAL_ONLY tok ne kreira KIF ni nalog; sistemski tenant i fiskalna administracija ostaju skriveni. Otvoreni su live/E2E, cross-tenant/IDOR i stvarni printer QA.</v>
       </c>
     </row>
   </sheetData>
@@ -2129,9 +2381,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z365"/>
+  <dimension ref="A1:Z373"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5902,7 +6154,7 @@
         <v>M-011,F-097</v>
       </c>
       <c r="L360" t="str">
-        <v>Browser štampa fiskalnog računa čuva dvojezičnu srpsko-englesku A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; stvarni termalni printer i reprint audit ostaju za ručni QA.</v>
+        <v>Browser štampa fiskalnog računa čuva dvojezičnu srpsko-englesku A4 opciju i prikazuje QR, IKOF/JIKR, kupca i vezu storna. Izvještaj ima zasebnu štampu; direktni portal auditira otvaranje A4 i 58/80 mm štampe. Stvarni termalni printer i reprint audit agencijskog POS-a ostaju za ručni QA.</v>
       </c>
     </row>
     <row r="361">
@@ -6095,14 +6347,318 @@
         <v>Operativna podešavanja obuhvataju kontakt, glavni račun, kasu, magacin, plaćanje, rok, štampu, smjene, lager i Test depozit. Fiskalna administracija ostaje platformskom adminu; produkcijski depozit čeka API rutu.</v>
       </c>
     </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>F-104</v>
+      </c>
+      <c r="B366" t="str">
+        <v>Plate i zaposleni</v>
+      </c>
+      <c r="C366" t="str">
+        <v>Pojedinačni period i sati radnika</v>
+      </c>
+      <c r="D366" t="str">
+        <v>Obračunska stavka ima datum od/do unutar mjeseca i trajanja zaposlenja; sistem predlaže sate prema radnim danima i fondu, a računovođa može sa auditom ručno promijeniti ili vratiti automatske sate.</v>
+      </c>
+      <c r="E366" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F366" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G366" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H366" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I366" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J366" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K366" t="str">
+        <v>M-006</v>
+      </c>
+      <c r="L366" t="str">
+        <v>Priprema uključuje i radnike koji počnu ili završe radni odnos tokom mjeseca. Testovi pokrivaju početak 17-og, prestanak prije kraja, nekoliko dana rada i period van mjeseca; kalendar praznika i nestandardnih smjena ostaje dorada.</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>F-105</v>
+      </c>
+      <c r="B367" t="str">
+        <v>Korisnici, agencije i prava</v>
+      </c>
+      <c r="C367" t="str">
+        <v>Sklopivi agencijski meni</v>
+      </c>
+      <c r="D367" t="str">
+        <v>Glavni agencijski meni se na desktopu sklapa na ikonice i pamti izbor; na telefonu se otvara kao pristupačan bočni panel preko sadržaja.</v>
+      </c>
+      <c r="E367" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F367" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G367" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H367" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I367" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="J367" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K367" t="str">
+        <v>M-001</v>
+      </c>
+      <c r="L367" t="str">
+        <v>Sadržaj koristi oslobođenu širinu; dostupni su ujednačene SVG ikonice, aktivna stavka, title opisi, aria oznake, Escape i backdrop zatvaranje te reduced-motion stilovi. TypeScript i lint su čisti; browser QA je potvrđen u otvorenom i sklopljenom stanju.</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>F-106</v>
+      </c>
+      <c r="B368" t="str">
+        <v>Izvještaji i dashboard</v>
+      </c>
+      <c r="C368" t="str">
+        <v>Operativne stavke početnog dashboarda</v>
+      </c>
+      <c r="D368" t="str">
+        <v>Početna za aktivnu firmu/godinu prikazuje nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF, umjesto audit logova.</v>
+      </c>
+      <c r="E368" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F368" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G368" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H368" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I368" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J368" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K368" t="str">
+        <v>M-003,M-004,M-009,M-010</v>
+      </c>
+      <c r="L368" t="str">
+        <v>Brojači i najnovije stavke koriste stvarne statuse DRAFT/WAITING_KUF/WAITING_KIF, tenant scope i prava pregleda; redovi vode direktno na izvorni dokument. Browser QA je potvrđen.</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>F-107</v>
+      </c>
+      <c r="B369" t="str">
+        <v>Robno i izvještaji</v>
+      </c>
+      <c r="C369" t="str">
+        <v>Lager lista i kartica artikla</v>
+      </c>
+      <c r="D369" t="str">
+        <v>Lager lista prikazuje stanje i vrijednosti po magacinu/artiklu, a kartica hronološke ulaze, izlaze i saldo za izabrani period.</v>
+      </c>
+      <c r="E369" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F369" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G369" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H369" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I369" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J369" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K369" t="str">
+        <v>M-004,M-009</v>
+      </c>
+      <c r="L369" t="str">
+        <v>Iste serverske komponente koriste se u Robnom i centralnim Izvještajima. Filteri obuhvataju magacin, grupu, artikal, znak stanja i period; kartica računa početno stanje prije perioda i povezuje izvorne dokumente.</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>F-108</v>
+      </c>
+      <c r="B370" t="str">
+        <v>Izvještaji i dashboard</v>
+      </c>
+      <c r="C370" t="str">
+        <v>Centralne kartice konta i partnera, PDV i plate</v>
+      </c>
+      <c r="D370" t="str">
+        <v>Centralni meni izvještaja otvara postojeće funkcionalne kartice glavne knjige, mjesečni PDV pregled i pregled izvještaja plata bez dupliranja poslovne računice.</v>
+      </c>
+      <c r="E370" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F370" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G370" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H370" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I370" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J370" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K370" t="str">
+        <v>M-003,M-006,M-007,M-009</v>
+      </c>
+      <c r="L370" t="str">
+        <v>Kartica konta ima lijevi pretraživ spisak, izbor samo konta sa POSTED prometom ili svih aktivnih konta i desni detalj sa periodom/partnerom; na telefonu radi kao lista pa detalj. Partnerska kartica koristi analitička konta i partnera, PDV postojeće periode/prijave, a plate obračune, M-4, OPP-ND i IOPPD.</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>F-109</v>
+      </c>
+      <c r="B371" t="str">
+        <v>Nalozi / Izvještaji</v>
+      </c>
+      <c r="C371" t="str">
+        <v>Ispravna štampa bruto bilansa</v>
+      </c>
+      <c r="D371" t="str">
+        <v>Bruto bilans se štampa na A4 landscape sa osam stabilnih kolona, neprelomivim iznosima i ponovljenim zaglavljem tabele.</v>
+      </c>
+      <c r="E371" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F371" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G371" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H371" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I371" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="J371" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K371" t="str">
+        <v>M-003,F-038</v>
+      </c>
+      <c r="L371" t="str">
+        <v>Zasebni stil i colgroup odvajaju bruto bilans od sedmokolonskog Bilansa stanja: konto 8%, naziv 26%, šest iznosa po 11%; redovi se ne cijepaju preko stranice.</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>F-110</v>
+      </c>
+      <c r="B372" t="str">
+        <v>Nalozi / Izvještaji</v>
+      </c>
+      <c r="C372" t="str">
+        <v>Štampa kartice konta</v>
+      </c>
+      <c r="D372" t="str">
+        <v>Izabrana kartica konta štampa se sa aktivnim partnerom i periodom, početnim saldom, prometom, tekućim saldom i završnim zbirom.</v>
+      </c>
+      <c r="E372" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F372" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G372" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H372" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I372" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="J372" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K372" t="str">
+        <v>M-003,F-037,F-108</v>
+      </c>
+      <c r="L372" t="str">
+        <v>Čista A4 landscape ruta prikazuje samo POSTED stavke aktivne firme i godine, provjerava tenant/account/partner scope i ponavlja zaglavlje tabele preko stranica.</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>F-111</v>
+      </c>
+      <c r="B373" t="str">
+        <v>Završni račun</v>
+      </c>
+      <c r="C373" t="str">
+        <v>Kontrole spremnosti završnog računa</v>
+      </c>
+      <c r="D373" t="str">
+        <v>Jedinstven ekran provjerava glavnu knjigu, pomoćne evidencije, šeme i zaključna knjiženja prije arhiviranja i zaključivanja godine.</v>
+      </c>
+      <c r="E373" t="str">
+        <v>Vrlo visok</v>
+      </c>
+      <c r="F373" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G373" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H373" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I373" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="J373" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K373" t="str">
+        <v>M-003,M-005,M-006,M-007,M-008,M-010</v>
+      </c>
+      <c r="L373" t="str">
+        <v>Read-only tenant-aware kontrolni centar razdvaja greške/upozorenja/uspjehe i vodi direktno na razrješenje; provjerava POSTED balans, analitiku, nacrte, KIF/KUF, izvode, plate, PDV, šablone, 5990/6990, klase 5/6, korekcije, arhivu i matične podatke. Izvorna PDV konta moraju imati saldo 0,00, klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo; sporna konta vode na karticu.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z365"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z373"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z369"/>
   <sheetData>
@@ -9636,7 +10192,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z310"/>
   <sheetData>
@@ -10200,7 +10756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z342"/>
   <sheetData>
@@ -11755,7 +12311,52 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Dashboard agencije</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Uklonjeni zadnji audit logovi; dodati brojači i liste DRAFT naloga, WAITING_KUF kalkulacija i WAITING_KIF izlaznih računa za aktivnu firmu/godinu; direktni linkovi i permission-aware prazna stanja.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Po potrebi proširiti dashboard rokovima i dodatnim operativnim kontrolama iz postojećih podstranica.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Browser QA potvrđen na aktivnoj firmi/godini; TypeScript, ESLint i diff provjere su čiste.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z348"/>
   <sheetData>
@@ -13580,7 +14181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z351"/>
   <sheetData>
@@ -16366,7 +16967,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB357"/>
   <sheetData>
@@ -18453,7 +19054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -18503,69 +19104,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>M-004 Robno</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Summa izlazna faktura povezana je sa Fiscal API-jem. Jedno dugme automatski koristi Test ili Production, stabilan idempotency ključ i čuva zvanični broj, IKOF, JIKR i QR URL. Poslije fiskalizacije sadržaj je zaključan, a knjiženje se može dovršiti odvojeno.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Ručni end-to-end QA u Test okruženju i kontrolisana produkcijska provjera.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Fiskalni račun se ne šalje iz razvojne provjere; korisnik eksplicitno pokreće slanje dugmetom Fiskalizuj.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>M-011 POS / Kasa</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Prva funkcionalna faza</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Mobile-first POS, povezivanje kase sa Fiscal API objektom/ENU-om/operatorom, zajednički artikli i cijene, korpa, kupac, gotovina/kartica/virman, atomarna numeracija, retry, fiskalni rezultat, pregled, štampa i atomsko razduženje lagera sa podesivim pravilom minusa.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Mobile QA, zbirni KIF/knjiženje, dnevni promet, povrati, smjene i POS Agent.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Koristi FiskalniIzlazniRacun; direktni klijent može dobiti samo POS prava.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -19002,7 +19541,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z321"/>
   <sheetData>
@@ -19774,7 +20313,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -19965,7 +20504,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19986,24 +20525,75 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-004 Robno</v>
+        <v>Direktni fiskalni portal</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Implementirano / ručni QA</v>
       </c>
       <c r="C2" t="str">
-        <v>Izlazne fakture imaju pregled, nacrt i brzi editor za robu i usluge, cijene iz šifarnika, Enter navigaciju, brzo dodavanje artikla/usluge i preglednu A4 štampu. Štampa podržava snapshot strana, nacrt, PDV rekapitulaciju i zvanični fiskalni QR/IKOF/JIKR kada postoje. Za firme van Summa fiskalizacije završavanje provjerava lager i PDV period, razdužuje robu, kreira nalog i šalje zapis u KIF kao SOURCE_DOCUMENT bez ponovnog knjiženja.</v>
+        <v>Backend guard i automatski kontekst; dashboard; POS; OFFICE fakture; računi i puni storno; A4 i 58/80 mm štampa sa auditom; izvještaji/export; artikli, cijene, kupci i operativna podešavanja.</v>
       </c>
       <c r="D2" t="str">
-        <v>Povezivanje završavanja Summa fakture sa Fiscal API-jem i završni end-to-end QA.</v>
+        <v>Kontrolisani live/E2E, cross-tenant/IDOR i stvarni printer QA; e-mail, offline tok, djelimične korekcije, POS Agent i produkcijski depozit.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracije 20260807100000_izlazne_fakture_mvp, 20260807120000_kif_source_document_posting i 20260808100000_invoice_print_snapshots su primijenjene.</v>
+        <v>Status je usklađen isključivo prema provjerenim rutama, servisima, Prisma migracijama i portal unit testovima.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Fiskalni klijent i agencija</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Implementirano / ručni QA</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Uključivanje fiskalizacije postojećoj firmi; PIB zahtjev za transfer; admin odobrenje/odbijanje bez duplikata; uslovno dugme Fiskalizacija na klijentskom dashboardu.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni end-to-end QA uključivanja i transfera na testnoj firmi.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Isti firma_id, Fiscal API veza i fiskalna istorija ostaju kanonski.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Plate — period i sati radnika</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Datum od/do po stavci; presjek sa početkom/prestankom zaposlenja; automatski prijedlog sati; ručni override i vraćanje na auto; serverska validacija i audit.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Kalendar praznika i nestandardnih smjena; ručni end-to-end obračun novog djelimičnog mjeseca.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Automatizovani testovi 5/5; TypeScript i lint čisti; browser QA ručnog override-a bez slanja forme.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Navigacija — sklopivi agencijski meni</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Desktop collapse na ujednačene SVG ikonice sa pamćenjem izbora; automatsko širenje sadržaja; aktivna stavka i tooltip; mobilni drawer sa backdropom i Escape zatvaranjem.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Ručni mobile QA na fizičkom telefonu po potrebi.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>TypeScript, ESLint i diff provjere su čiste; browser QA otvorenog i sklopljenog desktop menija je potvrđen.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -20031,19 +20621,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
+        <v>Fiskalni klijent i agencija</v>
       </c>
       <c r="B2" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>KIF knjiga prikazuje fiskalizovane izlazne račune koji čekaju unos i omogućava grupno preuzimanje kupca, broja, datuma, iznosa i PDV razrade. Izvorni račun i KIF zapis trajno su povezani radi zaštite od duplikata.</v>
+        <v>Uključivanje fiskalizacije izborom postojeće firme agencije; globalna PIB detekcija; zahtjev i platformsko odobrenje/odbijanje prelaska direktnog klijenta bez duplikata.</v>
       </c>
       <c r="D2" t="str">
-        <v>Povezati budući ekran izdavanja izlaznih faktura sa lokalnim fiskalnim izvorom i uraditi ručni end-to-end QA na stvarno fiskalizovanom računu.</v>
+        <v>Ručni end-to-end QA transfera na testnoj firmi i naknadna implementacija klijentskog dashboarda sa dugmetom Fiskalizacija.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260804100000_fiskalni_racuni_kif_queue je primijenjena; tenant scope, prava, zaključavanje, PDV stope, duplikati i audit provjeravaju se na backendu.</v>
+        <v>Isti firma_id i Fiscal API veza ostaju kanonski; transfer firm-specific tenant scope-a je auditovan.</v>
       </c>
     </row>
   </sheetData>
@@ -20055,7 +20645,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20076,24 +20666,41 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
+        <v>M-012 Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="B2" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Specifikacija spremna</v>
       </c>
       <c r="C2" t="str">
-        <v>KIF sada podržava dnevni i mjesečni pazar sa periodom, brojem izvještaja, kasom, poreskim osnovicama, izlaznim PDV-om i raspodjelom naplate na gotovinu, kartice, virman i ostalo. Preklapanje perioda iste kase je blokirano. Ukupan iznos se kaskadno raspoređuje od najveće aktivne stope ka 0%, uz automatski izlazni PDV. Pazar se prikazuje u KIF-u, štampi, Excel izvozu i izlaznom PDV-u. Podešavanja firme imaju posebna dugujuća konta načina naplate, dok prihod i PDV koriste aktivnu KIF šemu.</v>
+        <v>Dogovoren je poseban mobile-first /portal sa automatskim kontekstom jedne firme, operativnim dashboardom, POS-om, klasičnim bezgotovinskim fakturama, jedinstvenim pregledom fiskalnih računa, izvještajima, artiklima, kupcima i ograničenim podešavanjima.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA kreiranja, izmjene, brisanja, zabrane preklapanja, knjiženja i PDV prikaza pazara; PDV zaključavanje KIF/KUF izmjena.</v>
+        <v>Implementirati sigurnosni portal guard i zabranu /agencija pristupa, zatim dashboard, oba prodajna toka, izvještaje i šifarnike prema DIRECT_FISCAL_CLIENT_PORTAL_SPEC.md.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260730170000_kif_pazar je primijenjena, Prisma klijent regenerisan i dev server restartovan. TypeScript, Prisma validacija i lint prolaze bez novih grešaka.</v>
+        <v>Fiskalna konfiguracija, sertifikati, ENU, operateri, aktivacija i suspenzija ostaju isključivo platformskom adminu; direct FISCAL_ONLY dokumenti ne kreiraju KIF ni nalog.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Dokumentacija i planer</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Usklađeno</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dodata detaljna implementaciona specifikacija i ažurirani fiskalni README, POS specifikacija, CURRENT_STATE, NEXT_STEPS, SESSION_LOG i arhitektura.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Aplikacijski kod, Prisma šema i migracije nijesu mijenjani.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Status označava dogovoreni plan, ne završenu funkcionalnost.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -20127,30 +20734,30 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Robni meni i šifarnici su funkcionalni. Domaća kalkulacija ima obaveznu prodajnu cijenu sa PDV-om, maloprodaju kao default, kompaktne stavke, brzo kreiranje artikla, zavisne troškove i A4 štampu. MAPR link učitava zaglavlje i sve stavke, nudi postojeće/predložene/nove artikle i pamti veze dobavljačevih šifara. Završavanje koristi posebnu šemu iz Robno / Podešavanja, kreira DRAFT nalog i lager, zatim čeka grupno preuzimanje u KUF; preuzeti zapis se ne knjiži ponovo po KUF šemi.</v>
+        <v>Summa izlazna faktura povezana je sa Fiscal API-jem. Jedno dugme automatski koristi Test ili Production, stabilan idempotency ključ i čuva zvanični broj, IKOF, JIKR i QR URL. Poslije fiskalizacije sadržaj je zaključan, a knjiženje se može dovršiti odvojeno.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA MAPR pregleda, završavanja i preuzimanja u KUF sa podešenom robnom šemom; lager lista i kartica artikla; ručna raspodjela zavisnih troškova; uvozna kalkulacija; izlazne fakture i ostali robni dokumenti.</v>
+        <v>Ručni end-to-end QA u Test okruženju i kontrolisana produkcijska provjera.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260730130000_kalkulacije_preuzimanje_u_kuf je primijenjena uz backfill četiri postojeća KUF zapisa iz kalkulacija. Prisma klijent je regenerisan, dev server radi, TypeScript je čist i lint nema novih upozorenja; stvarni MAPR primjer sa 28 stavki centovno je usaglašen.</v>
+        <v>Fiskalni račun se ne šalje iz razvojne provjere; korisnik eksplicitno pokreće slanje dugmetom Fiskalizuj.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
+        <v>M-011 POS / Kasa</v>
       </c>
       <c r="B3" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Prva funkcionalna faza</v>
       </c>
       <c r="C3" t="str">
-        <v>Višestruki QR čitač potvrđen je na 65 stvarnih fajlova, a stvarni import na 145 linkova. Import sada šalje grupe po pet i prikazuje progres; KUF provjerava IIC+PIB+datum u bazi prije MAPR-a i preskače postojeće račune. Neuspjeli fajlovi/linkovi imaju poseban izvještaj, grupni retry i CSV izvoz. Kada novi dobavljač nema zapamćeno KUF konto, svi njegovi računi grupišu se po PIB-u, traže jedan izbor konta i pamte ga za naredne importe. Knjiženje kontroliše svaki KUF račun, koriguje razliku od jednog centa na trošku i za veću razliku jasno označava sporni račun.</v>
+        <v>Mobile-first POS, povezivanje kase sa Fiscal API objektom/ENU-om/operatorom, zajednički artikli i cijene, korpa, kupac, gotovina/kartica/virman, atomarna numeracija, retry, fiskalni rezultat, pregled, štampa i atomsko razduženje lagera sa podesivim pravilom minusa.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni QA novog progres/precheck/retry/CSV toka i grupnog ponovnog importa sa više računa istog novog dobavljača; ručni QA upozorenja za razliku veću od jednog centa; PDV zaključavanje.</v>
+        <v>Mobile QA, zbirni KIF/knjiženje, dnevni promet, povrati, smjene i POS Agent.</v>
       </c>
       <c r="E3" t="str">
-        <v>Nije potrebna migracija: koristi postojeće fiskalne identifikatore KUF zapisa i firma_komitent.default_kuf_konto_sifra. Read-only simulacija KUF-2026-0004 potvrdila je 133 računa, šest centnih korekcija, bez spornih računa i balans 0 centi. TypeScript je čist, lint nema novih upozorenja.</v>
+        <v>Koristi FiskalniIzlazniRacun; direktni klijent može dobiti samo POS prava.</v>
       </c>
     </row>
   </sheetData>
@@ -20189,13 +20796,13 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Robni meni je grupisan na Pregled, Šifarnike, Nabavku, Prodaju, Promet robe i Zalihe. Implementirani su modeli, migracija, prava/audit i ekrani za grupe artikala, artikle/usluge, cijene, jedinice mjere i magacine. Negativan lager se podešava po firmi i opciono po magacinu.</v>
+        <v>Izlazne fakture imaju pregled, nacrt i brzi editor za robu i usluge, cijene iz šifarnika, Enter navigaciju, brzo dodavanje artikla/usluge i preglednu A4 štampu. Štampa podržava snapshot strana, nacrt, PDV rekapitulaciju i zvanični fiskalni QR/IKOF/JIKR kada postoje. Za firme van Summa fiskalizacije završavanje provjerava lager i PDV period, razdužuje robu, kreira nalog i šalje zapis u KIF kao SOURCE_DOCUMENT bez ponovnog knjiženja.</v>
       </c>
       <c r="D2" t="str">
-        <v>Stanje/promet zaliha, lager lista, kartica artikla, kalkulacije, izlazne fakture, povrati, prenosi, popis, otpis i nivelacija.</v>
+        <v>Povezivanje završavanja Summa fakture sa Fiscal API-jem i završni end-to-end QA.</v>
       </c>
       <c r="E2" t="str">
-        <v>Postojeći meni Računi nije mijenjan i ostaje KIF/KUF tok. Sljedeći korak je model lagera prije domaće kalkulacije.</v>
+        <v>Migracije 20260807100000_izlazne_fakture_mvp, 20260807120000_kif_source_document_posting i 20260808100000_invoice_print_snapshots su primijenjene.</v>
       </c>
     </row>
   </sheetData>
@@ -20207,7 +20814,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20228,41 +20835,24 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-003 Nalozi</v>
+        <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B2" t="str">
-        <v>Početno stanje završeno</v>
+        <v>Core implementiran / dorada</v>
       </c>
       <c r="C2" t="str">
-        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
+        <v>KIF knjiga prikazuje fiskalizovane izlazne račune koji čekaju unos i omogućava grupno preuzimanje kupca, broja, datuma, iznosa i PDV razrade. Izvorni račun i KIF zapis trajno su povezani radi zaštite od duplikata.</v>
       </c>
       <c r="D2" t="str">
-        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
+        <v>Povezati budući ekran izdavanja izlaznih faktura sa lokalnim fiskalnim izvorom i uraditi ručni end-to-end QA na stvarno fiskalizovanom računu.</v>
       </c>
       <c r="E2" t="str">
-        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
-      </c>
-      <c r="B3" t="str">
-        <v>QR čitanje računa završeno</v>
-      </c>
-      <c r="C3" t="str">
-        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
+        <v>Migracija 20260804100000_fiskalni_racuni_kif_queue je primijenjena; tenant scope, prava, zaključavanje, PDV stope, duplikati i audit provjeravaju se na backendu.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete business units and inventory workflows
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,43 +3,44 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-09-02" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-08-31" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-08-30" sheetId="3" r:id="rId3"/>
-    <sheet name="Status 2026-08-25" sheetId="4" r:id="rId4"/>
-    <sheet name="Status 2026-08-23" sheetId="5" r:id="rId5"/>
-    <sheet name="Status 2026-08-20" sheetId="6" r:id="rId6"/>
-    <sheet name="Status 2026-08-19" sheetId="7" r:id="rId7"/>
-    <sheet name="Status 2026-08-08" sheetId="8" r:id="rId8"/>
-    <sheet name="Status 2026-08-07" sheetId="9" r:id="rId9"/>
-    <sheet name="Status 2026-08-04" sheetId="10" r:id="rId10"/>
-    <sheet name="Status 2026-07-30" sheetId="11" r:id="rId11"/>
-    <sheet name="Status 2026-07-29" sheetId="12" r:id="rId12"/>
-    <sheet name="Status 2026-07-26" sheetId="13" r:id="rId13"/>
-    <sheet name="Status 2026-07-25" sheetId="14" r:id="rId14"/>
-    <sheet name="Status 2026-07-24" sheetId="15" r:id="rId15"/>
-    <sheet name="Status 2026-07-09" sheetId="16" r:id="rId16"/>
-    <sheet name="Status 2026-07-07" sheetId="17" r:id="rId17"/>
-    <sheet name="Status 2026-07-06" sheetId="18" r:id="rId18"/>
-    <sheet name="Status 2026-07-05" sheetId="19" r:id="rId19"/>
-    <sheet name="Status 2026-07-02" sheetId="20" r:id="rId20"/>
-    <sheet name="Status 2026-06-30" sheetId="21" r:id="rId21"/>
-    <sheet name="Status 2026-06-29" sheetId="22" r:id="rId22"/>
-    <sheet name="Status 2026-06-28" sheetId="23" r:id="rId23"/>
-    <sheet name="Status 2026-06-25" sheetId="24" r:id="rId24"/>
-    <sheet name="Dashboard" sheetId="25" r:id="rId25"/>
-    <sheet name="Moduli" sheetId="26" r:id="rId26"/>
-    <sheet name="Funkcionalnosti" sheetId="27" r:id="rId27"/>
-    <sheet name="Pravila" sheetId="28" r:id="rId28"/>
-    <sheet name="Zavisnosti" sheetId="29" r:id="rId29"/>
-    <sheet name="Ekrani" sheetId="30" r:id="rId30"/>
-    <sheet name="Baza" sheetId="31" r:id="rId31"/>
-    <sheet name="API" sheetId="32" r:id="rId32"/>
-    <sheet name="Testovi" sheetId="33" r:id="rId33"/>
-    <sheet name="Bugovi" sheetId="34" r:id="rId34"/>
-    <sheet name="Ideje" sheetId="35" r:id="rId35"/>
-    <sheet name="Odluke" sheetId="36" r:id="rId36"/>
-    <sheet name="Kategorije" sheetId="37" r:id="rId37"/>
+    <sheet name="Status 2026-09-03" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-09-02" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-08-31" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-08-30" sheetId="4" r:id="rId4"/>
+    <sheet name="Status 2026-08-25" sheetId="5" r:id="rId5"/>
+    <sheet name="Status 2026-08-23" sheetId="6" r:id="rId6"/>
+    <sheet name="Status 2026-08-20" sheetId="7" r:id="rId7"/>
+    <sheet name="Status 2026-08-19" sheetId="8" r:id="rId8"/>
+    <sheet name="Status 2026-08-08" sheetId="9" r:id="rId9"/>
+    <sheet name="Status 2026-08-07" sheetId="10" r:id="rId10"/>
+    <sheet name="Status 2026-08-04" sheetId="11" r:id="rId11"/>
+    <sheet name="Status 2026-07-30" sheetId="12" r:id="rId12"/>
+    <sheet name="Status 2026-07-29" sheetId="13" r:id="rId13"/>
+    <sheet name="Status 2026-07-26" sheetId="14" r:id="rId14"/>
+    <sheet name="Status 2026-07-25" sheetId="15" r:id="rId15"/>
+    <sheet name="Status 2026-07-24" sheetId="16" r:id="rId16"/>
+    <sheet name="Status 2026-07-09" sheetId="17" r:id="rId17"/>
+    <sheet name="Status 2026-07-07" sheetId="18" r:id="rId18"/>
+    <sheet name="Status 2026-07-06" sheetId="19" r:id="rId19"/>
+    <sheet name="Status 2026-07-05" sheetId="20" r:id="rId20"/>
+    <sheet name="Status 2026-07-02" sheetId="21" r:id="rId21"/>
+    <sheet name="Status 2026-06-30" sheetId="22" r:id="rId22"/>
+    <sheet name="Status 2026-06-29" sheetId="23" r:id="rId23"/>
+    <sheet name="Status 2026-06-28" sheetId="24" r:id="rId24"/>
+    <sheet name="Status 2026-06-25" sheetId="25" r:id="rId25"/>
+    <sheet name="Dashboard" sheetId="26" r:id="rId26"/>
+    <sheet name="Moduli" sheetId="27" r:id="rId27"/>
+    <sheet name="Funkcionalnosti" sheetId="28" r:id="rId28"/>
+    <sheet name="Pravila" sheetId="29" r:id="rId29"/>
+    <sheet name="Zavisnosti" sheetId="30" r:id="rId30"/>
+    <sheet name="Ekrani" sheetId="31" r:id="rId31"/>
+    <sheet name="Baza" sheetId="32" r:id="rId32"/>
+    <sheet name="API" sheetId="33" r:id="rId33"/>
+    <sheet name="Testovi" sheetId="34" r:id="rId34"/>
+    <sheet name="Bugovi" sheetId="35" r:id="rId35"/>
+    <sheet name="Ideje" sheetId="36" r:id="rId36"/>
+    <sheet name="Odluke" sheetId="37" r:id="rId37"/>
+    <sheet name="Kategorije" sheetId="38" r:id="rId38"/>
   </sheets>
 </workbook>
 </file>
@@ -433,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,41 +455,92 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nalozi / Poslovne jedinice</v>
+        <v>Robno / Prenos robe</v>
       </c>
       <c r="B2" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Firm-specific šifarnik sa pravima i auditom; jedinica prati dokument i svaku stavku naloga, a izvještaji filtriraju POSTED promet po jedinici.</v>
+        <v>Nacrt, zaglavlje, stavke, lista, detalj i A4 štampa; atomarni OUT/IN promet, ažuriranje oba lagera po prosječnoj cijeni, kontrola minusa i DRAFT nalog po firm-specific šemi.</v>
       </c>
       <c r="D2" t="str">
-        <v>Raspodjela jedne stavke dokumenta na više jedinica može se dodati kasnije.</v>
+        <v>Ručni end-to-end QA na stvarnim zalihama i različitim poslovnim jedinicama.</v>
       </c>
       <c r="E2" t="str">
-        <v>Pokriveni su ručni nalozi, KIF/KUF, izlazni/POS računi, izvodi, plate, rezultat po jedinicama i završna kontrola.</v>
+        <v>Migracija 20260903100000_prenosi_robe je primijenjena; automatski test obračuna prolazi 3/3.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Robno / Magacini i kalkulacije</v>
+        <v>Robno / Popis robe</v>
       </c>
       <c r="B3" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C3" t="str">
-        <v>Magacin se opciono vezuje za poslovnu jedinicu. Domaća i MAPR kalkulacija snimaju jedinicu magacina, a njihov nalog je nasljeđuje.</v>
+        <v>Popis po magacinu, knjigovodstveno i stvarno stanje, višak/manjak, vrijednosne korekcije, DRAFT nalog po posebnoj šemi i A4 štampa.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni end-to-end QA na više prodavnica/magacina.</v>
+        <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
       </c>
       <c r="E3" t="str">
-        <v>Istorijska kalkulacija i nalog ne zavise od naknadne promjene veze magacina.</v>
+        <v>Migracija 20260903120000_popisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Robno / Otpis robe</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Nacrt po magacinu, razlozi i stavke, kontrola minusa, razduženje svih vrijednosti lagera, kartični promet, DRAFT nalog po firm-specific šemi i A4 štampa.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Migracija 20260903140000_otpisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Robno / Nivelacija cijena</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Nacrt po maloprodajnom magacinu, stara/nova MPC, promjene MP vrijednosti/RUC-a/PDV-a bez promjene količine, cjenovnik, kartični promet, DRAFT nalog i A4 štampa.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Ručni end-to-end QA sa povećanjem, smanjenjem i mješovitim dokumentom.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Migracija 20260903160000_nivelacije_cijena je primijenjena; automatski test obračuna prolazi 4/4.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Robno / Promet robe</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Pregled sekcije i kompletni tokovi prenosa, popisa sa viškom/manjkom, otpisa i nivelacije.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Ručni end-to-end QA na stvarnim zalihama i podešenim kontima.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Kartica artikla direktno otvara izvorni prenos, popis, otpis i nivelaciju.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -516,19 +568,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
+        <v>M-004 Robno</v>
       </c>
       <c r="B2" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>KIF knjiga prikazuje fiskalizovane izlazne račune koji čekaju unos i omogućava grupno preuzimanje kupca, broja, datuma, iznosa i PDV razrade. Izvorni račun i KIF zapis trajno su povezani radi zaštite od duplikata.</v>
+        <v>Izlazne fakture imaju pregled, nacrt i brzi editor za robu i usluge, cijene iz šifarnika, Enter navigaciju, brzo dodavanje artikla/usluge i preglednu A4 štampu. Štampa podržava snapshot strana, nacrt, PDV rekapitulaciju i zvanični fiskalni QR/IKOF/JIKR kada postoje. Za firme van Summa fiskalizacije završavanje provjerava lager i PDV period, razdužuje robu, kreira nalog i šalje zapis u KIF kao SOURCE_DOCUMENT bez ponovnog knjiženja.</v>
       </c>
       <c r="D2" t="str">
-        <v>Povezati budući ekran izdavanja izlaznih faktura sa lokalnim fiskalnim izvorom i uraditi ručni end-to-end QA na stvarno fiskalizovanom računu.</v>
+        <v>Povezivanje završavanja Summa fakture sa Fiscal API-jem i završni end-to-end QA.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260804100000_fiskalni_racuni_kif_queue je primijenjena; tenant scope, prava, zaključavanje, PDV stope, duplikati i audit provjeravaju se na backendu.</v>
+        <v>Migracije 20260807100000_izlazne_fakture_mvp, 20260807120000_kif_source_document_posting i 20260808100000_invoice_print_snapshots su primijenjene.</v>
       </c>
     </row>
   </sheetData>
@@ -567,13 +619,13 @@
         <v>Core implementiran / dorada</v>
       </c>
       <c r="C2" t="str">
-        <v>KIF sada podržava dnevni i mjesečni pazar sa periodom, brojem izvještaja, kasom, poreskim osnovicama, izlaznim PDV-om i raspodjelom naplate na gotovinu, kartice, virman i ostalo. Preklapanje perioda iste kase je blokirano. Ukupan iznos se kaskadno raspoređuje od najveće aktivne stope ka 0%, uz automatski izlazni PDV. Pazar se prikazuje u KIF-u, štampi, Excel izvozu i izlaznom PDV-u. Podešavanja firme imaju posebna dugujuća konta načina naplate, dok prihod i PDV koriste aktivnu KIF šemu.</v>
+        <v>KIF knjiga prikazuje fiskalizovane izlazne račune koji čekaju unos i omogućava grupno preuzimanje kupca, broja, datuma, iznosa i PDV razrade. Izvorni račun i KIF zapis trajno su povezani radi zaštite od duplikata.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA kreiranja, izmjene, brisanja, zabrane preklapanja, knjiženja i PDV prikaza pazara; PDV zaključavanje KIF/KUF izmjena.</v>
+        <v>Povezati budući ekran izdavanja izlaznih faktura sa lokalnim fiskalnim izvorom i uraditi ručni end-to-end QA na stvarno fiskalizovanom računu.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260730170000_kif_pazar je primijenjena, Prisma klijent regenerisan i dev server restartovan. TypeScript, Prisma validacija i lint prolaze bez novih grešaka.</v>
+        <v>Migracija 20260804100000_fiskalni_racuni_kif_queue je primijenjena; tenant scope, prava, zaključavanje, PDV stope, duplikati i audit provjeravaju se na backendu.</v>
       </c>
     </row>
   </sheetData>
@@ -585,6 +637,51 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>M-010 Računi / KIF-KUF</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C2" t="str">
+        <v>KIF sada podržava dnevni i mjesečni pazar sa periodom, brojem izvještaja, kasom, poreskim osnovicama, izlaznim PDV-om i raspodjelom naplate na gotovinu, kartice, virman i ostalo. Preklapanje perioda iste kase je blokirano. Ukupan iznos se kaskadno raspoređuje od najveće aktivne stope ka 0%, uz automatski izlazni PDV. Pazar se prikazuje u KIF-u, štampi, Excel izvozu i izlaznom PDV-u. Podešavanja firme imaju posebna dugujuća konta načina naplate, dok prihod i PDV koriste aktivnu KIF šemu.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Ručni end-to-end QA kreiranja, izmjene, brisanja, zabrane preklapanja, knjiženja i PDV prikaza pazara; PDV zaključavanje KIF/KUF izmjena.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Migracija 20260730170000_kif_pazar je primijenjena, Prisma klijent regenerisan i dev server restartovan. TypeScript, Prisma validacija i lint prolaze bez novih grešaka.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
@@ -645,7 +742,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -686,68 +783,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>M-003 Nalozi</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Početno stanje završeno</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
-      </c>
-      <c r="B3" t="str">
-        <v>QR čitanje računa završeno</v>
-      </c>
-      <c r="C3" t="str">
-        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -775,36 +810,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Plate i zaposleni</v>
+        <v>M-003 Nalozi</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Početno stanje završeno</v>
       </c>
       <c r="C2" t="str">
-        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
       </c>
       <c r="D2" t="str">
-        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Firme</v>
+        <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B3" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>QR čitanje računa završeno</v>
       </c>
       <c r="C3" t="str">
-        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
       </c>
       <c r="E3" t="str">
-        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
+        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
       </c>
     </row>
   </sheetData>
@@ -816,7 +851,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -837,24 +872,41 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Plate</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="B2" t="str">
         <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
+        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
       </c>
       <c r="D2" t="str">
-        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
+        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
       </c>
       <c r="E2" t="str">
-        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
+        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Firme</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -882,19 +934,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Zavrsni racun</v>
+        <v>Plate</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimicno implementirano</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
+        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
       </c>
       <c r="D2" t="str">
-        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
+        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
       </c>
       <c r="E2" t="str">
-        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
+        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
       </c>
     </row>
   </sheetData>
@@ -906,7 +958,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -927,58 +979,24 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Partneri</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B2" t="str">
-        <v>Implementirano</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
       </c>
       <c r="D2" t="str">
-        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
       </c>
       <c r="E2" t="str">
-        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Zavrsni racun</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Djelimicno implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Arhiva generisanih obrazaca i XML/export.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
+        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1046,13 +1064,13 @@
         <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
       </c>
       <c r="D4" t="str">
-        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
+        <v>Arhiva generisanih obrazaca i XML/export.</v>
       </c>
       <c r="E4" t="str">
-        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
+        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
       </c>
     </row>
   </sheetData>
@@ -1064,7 +1082,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1085,164 +1103,120 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nalozi / Bruto bilans</v>
+        <v>Nalozi / Poslovne jedinice</v>
       </c>
       <c r="B2" t="str">
-        <v>Ispravljeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>A4 landscape štampa sa osam eksplicitnih kolona, neprelomivim tabularnim iznosima, urednim prelomom naziva konta, ponovljenim zaglavljem i redovima koji se ne cijepaju preko stranice.</v>
+        <v>Firm-specific šifarnik sa pravima i auditom; jedinica prati dokument i svaku stavku naloga, a izvještaji filtriraju POSTED promet po jedinici.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
+        <v>Raspodjela jedne stavke dokumenta na više jedinica može se dodati kasnije.</v>
       </c>
       <c r="E2" t="str">
-        <v>Bruto bilans više ne nasljeđuje sedmokolonske širine Bilansa stanja. Nema migracije baze; TypeScript, ESLint i diff provjera prolaze.</v>
+        <v>Pokriveni su ručni nalozi, KIF/KUF, izlazni/POS računi, izvodi, plate, rezultat po jedinicama i završna kontrola; izbor jedinice je skriven firmama bez aktivnih jedinica.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Nalozi / Kartica konta</v>
+        <v>Robno / Magacini i kalkulacije</v>
       </c>
       <c r="B3" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C3" t="str">
-        <v>Dugme za štampu prenosi konto, partnera i period na čistu A4 landscape karticu sa početnim saldom, POSTED prometom, tekućim saldom i ukupnim zbirom.</v>
+        <v>Magacin se opciono vezuje za poslovnu jedinicu. Domaća i MAPR kalkulacija snimaju jedinicu magacina, a njihov nalog je nasljeđuje.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
+        <v>Ručni end-to-end QA na više prodavnica/magacina.</v>
       </c>
       <c r="E3" t="str">
-        <v>Ruta provjerava agenciju, dodjelu firme, poslovnu godinu, konto i scope partnera. Nema migracije baze; TypeScript i ESLint prolaze.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Završni račun / Kontrole</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Read-only kontrolni centar prikazuje ukupni status i provjere glavne knjige, KIF/KUF-a, dokumenata, izvoda, plata, PDV-a, šablona, rezultatskih konta, klasa 5/6, korekcija, arhive i matičnih podataka. Izvorna PDV konta moraju imati saldo 0,00; klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>XML/export završnog računa ostaje otvoren; po potrebi proširiti dodatnim zakonskim kontrolama.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Svako sporno konto vodi direktno na svoju karticu. Prijavljena ruta vraća HTTP 200; nema migracije baze.</v>
+        <v>Istorijska kalkulacija i nalog ne zavise od naknadne promjene veze magacina.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-07-02</v>
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
+        <v>Partneri</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Oblast</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B4" t="str">
-        <v>Status</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Sta je zavrseno</v>
+        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
       </c>
       <c r="D4" t="str">
-        <v>Sta ostaje</v>
+        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
       </c>
       <c r="E4" t="str">
-        <v>Preporuceni sljedeci korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C5" t="str">
-        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C7" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C8" t="str">
-        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Redovno održavanje.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Regenerisati Excel nakon svake veće promjene.</v>
+        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1253,7 +1227,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-30</v>
+        <v>Status projekta na dan 2026-07-02</v>
       </c>
     </row>
     <row r="2">
@@ -1286,13 +1260,13 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
+        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
       </c>
       <c r="D5" t="str">
-        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
+        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
       </c>
       <c r="E5" t="str">
-        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
+        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
       </c>
     </row>
     <row r="6">
@@ -1355,11 +1329,11 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-29</v>
+        <v>Status projekta na dan 2026-06-30</v>
       </c>
     </row>
     <row r="2">
@@ -1386,92 +1360,75 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nalozi</v>
+        <v>Izvodi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core zaokruzen</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
+        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
       </c>
       <c r="D5" t="str">
-        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
       </c>
       <c r="E5" t="str">
-        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
+        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PDV</v>
+        <v>Nalozi</v>
       </c>
       <c r="B6" t="str">
-        <v>Core zaokruzen</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C6" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
       </c>
       <c r="D6" t="str">
-        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
+        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E6" t="str">
-        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
+        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Izvodi</v>
+        <v>PDV</v>
       </c>
       <c r="B7" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C7" t="str">
-        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D7" t="str">
-        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
+        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
       </c>
       <c r="E7" t="str">
-        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
+        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>KIF/KUF</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B8" t="str">
-        <v>Core implementiran</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C8" t="str">
-        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
+        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
       </c>
       <c r="D8" t="str">
-        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
+        <v>Redovno održavanje.</v>
       </c>
       <c r="E8" t="str">
-        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C9" t="str">
-        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Regenerisati Excel nakon svake vece promjene.</v>
+        <v>Regenerisati Excel nakon svake veće promjene.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1482,12 +1439,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-28</v>
+        <v>Status projekta na dan 2026-06-29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
       </c>
     </row>
     <row r="4">
@@ -1509,87 +1466,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Performanse partnera</v>
+        <v>Nalozi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core implementiran</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C5" t="str">
-        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
       </c>
       <c r="D5" t="str">
-        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E5" t="str">
-        <v>Pratiti brzinu na produkciji.</v>
+        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Indeksi baze</v>
+        <v>PDV</v>
       </c>
       <c r="B6" t="str">
-        <v>Implementirano</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C6" t="str">
-        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D6" t="str">
-        <v>-</v>
+        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
       </c>
       <c r="E6" t="str">
-        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIF/KUF uvoz/export</v>
+        <v>Izvodi</v>
       </c>
       <c r="B7" t="str">
-        <v>Core implementiran</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
       </c>
       <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata; XML export.</v>
+        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
       </c>
       <c r="E7" t="str">
-        <v>QA uvoznih knjizenja i export fajlova.</v>
+        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dokumentacija</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="B8" t="str">
-        <v>Uspostavljeno</v>
+        <v>Core implementiran</v>
       </c>
       <c r="C8" t="str">
-        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
       </c>
       <c r="D8" t="str">
-        <v>Redovno odrzavanje.</v>
+        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
       </c>
       <c r="E8" t="str">
-        <v>Azurirati uz svaku vecu promjenu.</v>
+        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PDV</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B9" t="str">
-        <v>Prva implementacija</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C9" t="str">
-        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
       </c>
       <c r="D9" t="str">
-        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+        <v>Redovno odrzavanje.</v>
       </c>
       <c r="E9" t="str">
-        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+        <v>Regenerisati Excel nakon svake vece promjene.</v>
       </c>
     </row>
   </sheetData>
@@ -1601,6 +1558,129 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Performanse partnera</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pratiti brzinu na produkciji.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Indeksi baze</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KIF/KUF uvoz/export</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kontrole iznosa i duplikata; XML export.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>QA uvoznih knjizenja i export fajlova.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Dokumentacija</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Uspostavljeno</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Redovno odrzavanje.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Azurirati uz svaku vecu promjenu.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Prva implementacija</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
@@ -1773,7 +1853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -2068,7 +2148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z303"/>
   <sheetData>
@@ -2209,7 +2289,7 @@
         <v>MVP 1/2</v>
       </c>
       <c r="H8" t="str">
-        <v>Meni i šifarnici su implementirani. Domaća kalkulacija ima nacrt, obaveznu prodajnu cijenu, više PDV stopa, MAPR pregled i povezivanje ili atomarno kreiranje novih artikala, kompaktnu tabelu, zavisne troškove i A4 štampu. Završavanje kreira DRAFT nalog i lager prema posebnoj šemi, a KUF je naknadno preuzima kao knjiženu kroz kalkulaciju bez duplog naloga. Lager lista i kartica artikla postoje u Robnom i centralnim Izvještajima nad zajedničkim stanjem/prometom. Slijede live QA, uvozna kalkulacija i ostali robni dokumenti.</v>
+        <v>Meni i šifarnici su implementirani. Domaća kalkulacija ima MAPR unos, obračun, lager, DRAFT nalog i A4 štampu. Prenos robe, popis, otpis i nivelacija imaju nacrte, robne promete, poslovne jedinice, posebne šeme konta, DRAFT naloge i štampu; popis knjiži višak/manjak, otpis razdužuje zalihe, a nivelacija mijenja MP vrijednost, RUC i PDV bez količinske promjene. Lager lista i kartica artikla postoje u Robnom i centralnim Izvještajima. Slijede live QA, uvozna kalkulacija i povrati.</v>
       </c>
     </row>
     <row r="9">
@@ -2427,7 +2507,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z374"/>
   <sheetData>
@@ -4510,25 +4590,25 @@
         <v>Visok</v>
       </c>
       <c r="F316" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G316" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H316" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I316" t="str">
         <v>Da</v>
       </c>
       <c r="J316" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="K316" t="str">
         <v>F-041,F-042</v>
       </c>
       <c r="L316" t="str">
-        <v>Prenos pravi nalog za knjiženje.</v>
+        <v>Nacrt sa stavkama i štampom; knjiženje atomarno pravi OUT/IN promet po prosječnoj cijeni, ažurira oba lagera, čuva poslovne jedinice i kreira DRAFT WAREHOUSE_TRANSFER nalog po firm-specific šemi.</v>
       </c>
     </row>
     <row r="317">
@@ -4548,25 +4628,25 @@
         <v>Visok</v>
       </c>
       <c r="F317" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G317" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H317" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I317" t="str">
         <v>Da</v>
       </c>
       <c r="J317" t="str">
-        <v>Ne</v>
+        <v>Djelimicno</v>
       </c>
       <c r="K317" t="str">
         <v>F-042</v>
       </c>
       <c r="L317" t="str">
-        <v>Može napraviti višak i manjak.</v>
+        <v>Nacrt snima knjigovodstveno stanje svih aktivnih artikala, podržava grupno prepisivanje praznih količina, ručnu korekciju, osvježavanje snimka, listu, detalj i A4 štampu.</v>
       </c>
     </row>
     <row r="318">
@@ -4586,25 +4666,25 @@
         <v>Visok</v>
       </c>
       <c r="F318" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G318" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H318" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I318" t="str">
         <v>Da</v>
       </c>
       <c r="J318" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="K318" t="str">
         <v>F-055</v>
       </c>
       <c r="L318" t="str">
-        <v>Vrijednost po prosječnoj ili ručnoj cijeni.</v>
+        <v>Višak povećava količinu i sve robne vrijednosti po prosječnoj ili ručnoj cijeni te ulazi u izbalansiran STOCK_COUNT nalog.</v>
       </c>
     </row>
     <row r="319">
@@ -4624,25 +4704,25 @@
         <v>Visok</v>
       </c>
       <c r="F319" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G319" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H319" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I319" t="str">
         <v>Da</v>
       </c>
       <c r="J319" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="K319" t="str">
         <v>F-055</v>
       </c>
       <c r="L319" t="str">
-        <v>U maloprodaji koriguje RUC i ukalkulisani PDV.</v>
+        <v>Manjak proporcionalno smanjuje nabavnu i maloprodajnu vrijednost, RUC i ukalkulisani PDV te ulazi u izbalansiran STOCK_COUNT nalog.</v>
       </c>
     </row>
     <row r="320">
@@ -4662,25 +4742,25 @@
         <v>Visok</v>
       </c>
       <c r="F320" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G320" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H320" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I320" t="str">
         <v>Da</v>
       </c>
       <c r="J320" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="K320" t="str">
         <v>F-042,F-044</v>
       </c>
       <c r="L320" t="str">
-        <v>Ne smije otpisati više od stanja ako je minus blokiran.</v>
+        <v>Nacrt po magacinu sa razlozima i stavkama; knjiženje provjerava negativni lager, koristi prosječnu ili rezervnu nabavnu cijenu, razdužuje količinu i sve vrijednosti zaliha, upisuje kartični promet i kreira DRAFT WRITE_OFF nalog po firm-specific šemi. Dostupna je A4 štampa.</v>
       </c>
     </row>
     <row r="321">
@@ -4700,25 +4780,25 @@
         <v>Visok</v>
       </c>
       <c r="F321" t="str">
-        <v>Zaključeno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G321" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="H321" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="I321" t="str">
         <v>Da</v>
       </c>
       <c r="J321" t="str">
-        <v>Ne</v>
+        <v>Da</v>
       </c>
       <c r="K321" t="str">
         <v>F-042,F-050</v>
       </c>
       <c r="L321" t="str">
-        <v>Pravi nalog za knjiženje.</v>
+        <v>Nacrt po maloprodajnom magacinu pamti staru i novu MPC i početne vrijednosti. Knjiženje ne mijenja količinu ni nabavnu vrijednost, koriguje MP vrijednost, RUC i PDV, ažurira cjenovnik, upisuje kartični promet i kreira izbalansiran DRAFT PRICE_ADJUSTMENT nalog. Dostupna je A4 štampa.</v>
       </c>
     </row>
     <row r="322">
@@ -4788,13 +4868,13 @@
         <v>Da</v>
       </c>
       <c r="J323" t="str">
-        <v>Ne</v>
+        <v>Djelimicno</v>
       </c>
       <c r="K323" t="str">
         <v>F-045,F-052,F-053,F-054,F-055,F-058,F-059</v>
       </c>
       <c r="L323" t="str">
-        <v>Domaća kalkulacija kreira DRAFT nalog CALCULATION prema posebnoj firm-specific šemi iz Robno / Podešavanja. KUF naknadno preuzima kalkulaciju kao već knjižen izvorni dokument, bez ponovnog knjiženja po KUF šemi. Ostali robni dokumenti još nijesu implementirani.</v>
+        <v>Domaća kalkulacija, prenos robe, popis sa razlikama, otpis i nivelacija kreiraju DRAFT naloge prema posebnim firm-specific šemama iz Robno / Podešavanja. KUF naknadno preuzima kalkulaciju bez ponovnog knjiženja. Povrati još nijesu implementirani.</v>
       </c>
     </row>
     <row r="324">
@@ -6580,7 +6660,7 @@
         <v>M-003,M-006,M-007,M-009</v>
       </c>
       <c r="L370" t="str">
-        <v>Kartica konta ima lijevi pretraživ spisak, izbor samo konta sa POSTED prometom ili svih aktivnih konta i desni detalj sa periodom/partnerom; na telefonu radi kao lista pa detalj. Partnerska kartica koristi analitička konta i partnera, PDV postojeće periode/prijave, a plate obračune, M-4, OPP-ND i IOPPD.</v>
+        <v>Kartica konta ima lijevi pretraživ spisak, izbor samo konta sa POSTED prometom ili svih aktivnih konta i desni detalj sa periodom/partnerom; na telefonu radi kao lista pa detalj. Isti master-detail prikaz koristi i ruta pod Nalozima. Partnerska kartica koristi analitička konta i partnera, PDV postojeće periode/prijave, a plate obračune, M-4, OPP-ND i IOPPD.</v>
       </c>
     </row>
     <row r="371">
@@ -6732,7 +6812,7 @@
         <v>F-026,F-029,F-041</v>
       </c>
       <c r="L374" t="str">
-        <v>Kalkulacije i izlazni/POS računi nasljeđuju jedinicu magacina; ručni KIF/KUF, pazar, izvod i plata imaju izbor. KIF/KUF knjiženje čuva jedinicu po stavci, izvještaj računa klasu 6 minus klasu 5, a završna kontrola prijavljuje obaveznu jedinicu koja nedostaje.</v>
+        <v>Kalkulacije i izlazni/POS računi nasljeđuju jedinicu magacina; ručni KIF/KUF, pazar, izvod i plata imaju izbor. KIF/KUF knjiženje čuva jedinicu po stavci, izvještaj računa klasu 6 minus klasu 5, a završna kontrola prijavljuje obaveznu jedinicu koja nedostaje. Izbor se automatski skriva kada firma nema aktivnih jedinica.</v>
       </c>
     </row>
   </sheetData>
@@ -6742,7 +6822,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z369"/>
   <sheetData>
@@ -10276,7 +10356,86 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nalozi / Bruto bilans</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Ispravljeno</v>
+      </c>
+      <c r="C2" t="str">
+        <v>A4 landscape štampa sa osam eksplicitnih kolona, neprelomivim tabularnim iznosima, urednim prelomom naziva konta, ponovljenim zaglavljem i redovima koji se ne cijepaju preko stranice.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Bruto bilans više ne nasljeđuje sedmokolonske širine Bilansa stanja. Nema migracije baze; TypeScript, ESLint i diff provjera prolaze.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Nalozi / Kartica konta</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dugme za štampu prenosi konto, partnera i period na čistu A4 landscape karticu sa početnim saldom, POSTED prometom, tekućim saldom i ukupnim zbirom.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Ruta provjerava agenciju, dodjelu firme, poslovnu godinu, konto i scope partnera. Nema migracije baze; TypeScript i ESLint prolaze.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Završni račun / Kontrole</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Read-only kontrolni centar prikazuje ukupni status i provjere glavne knjige, KIF/KUF-a, dokumenata, izvoda, plata, PDV-a, šablona, rezultatskih konta, klasa 5/6, korekcija, arhive i matičnih podataka. Izvorna PDV konta moraju imati saldo 0,00; klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>XML/export završnog računa ostaje otvoren; po potrebi proširiti dodatnim zakonskim kontrolama.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Svako sporno konto vodi direktno na svoju karticu. Prijavljena ruta vraća HTTP 200; nema migracije baze.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z310"/>
   <sheetData>
@@ -10840,69 +10999,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Robno / Izvještaji</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Lager lista po magacinu i artiklu sa vrijednostima i filterima; kartica artikla sa početnim stanjem perioda, ulazima, izlazima, tekućim stanjem i linkovima na dokumente. Oba prikaza dostupna su u Robnom i centralnim Izvještajima.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Live QA sa stvarnim prometima kada lokalna PostgreSQL baza bude dostupna; buduće štampe/exporti po potrebi.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Nema migracije baze. TypeScript i ESLint prolaze bez grešaka; ostaju četiri ranija lint upozorenja.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Centralni izvještaji</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Kartica konta ima pretraživ spisak konta lijevo, desni detalj, izbor konta sa prometom/svih aktivnih i mobilni tok lista-detalj. Kartica partnera koristi postojeću analitičku karticu; PDV koristi mjesečni pregled perioda; plate vode na obračune, M-4, OPP-ND i IOPPD.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Centralno povezati preostale postojeće izvještaje kupaca, dobavljača i finansijskih obrazaca.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Nema migracije baze niti dupliranja računice; postojeće backend provjere prava i konteksta ostaju mjerodavne.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z342"/>
   <sheetData>
@@ -12457,7 +12554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z349"/>
   <sheetData>
@@ -14308,7 +14405,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z351"/>
   <sheetData>
@@ -17094,7 +17191,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB357"/>
   <sheetData>
@@ -19181,7 +19278,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -19231,7 +19328,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -19668,7 +19765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z321"/>
   <sheetData>
@@ -20440,7 +20537,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -20631,6 +20728,68 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Robno / Izvještaji</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Lager lista po magacinu i artiklu sa vrijednostima i filterima; kartica artikla sa početnim stanjem perioda, ulazima, izlazima, tekućim stanjem i linkovima na dokumente. Oba prikaza dostupna su u Robnom i centralnim Izvještajima.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Live QA sa stvarnim prometima kada lokalna PostgreSQL baza bude dostupna; buduće štampe/exporti po potrebi.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Nema migracije baze. TypeScript i ESLint prolaze bez grešaka; ostaju četiri ranija lint upozorenja.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Centralni izvještaji</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Kartica konta ima pretraživ spisak konta lijevo, desni detalj, izbor konta sa prometom/svih aktivnih i mobilni tok lista-detalj. Kartica partnera koristi postojeću analitičku karticu; PDV koristi mjesečni pregled perioda; plate vode na obračune, M-4, OPP-ND i IOPPD.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Centralno povezati preostale postojeće izvještaje kupaca, dobavljača i finansijskih obrazaca.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Nema migracije baze niti dupliranja računice; postojeće backend provjere prava i konteksta ostaju mjerodavne.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
@@ -20674,7 +20833,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
   <sheetData>
@@ -20770,7 +20929,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -20811,68 +20970,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>M-012 Portal direktnog fiskalnog klijenta</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Specifikacija spremna</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Dogovoren je poseban mobile-first /portal sa automatskim kontekstom jedne firme, operativnim dashboardom, POS-om, klasičnim bezgotovinskim fakturama, jedinstvenim pregledom fiskalnih računa, izvještajima, artiklima, kupcima i ograničenim podešavanjima.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Implementirati sigurnosni portal guard i zabranu /agencija pristupa, zatim dashboard, oba prodajna toka, izvještaje i šifarnike prema DIRECT_FISCAL_CLIENT_PORTAL_SPEC.md.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Fiskalna konfiguracija, sertifikati, ENU, operateri, aktivacija i suspenzija ostaju isključivo platformskom adminu; direct FISCAL_ONLY dokumenti ne kreiraju KIF ni nalog.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Dokumentacija i planer</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Usklađeno</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Dodata detaljna implementaciona specifikacija i ažurirani fiskalni README, POS specifikacija, CURRENT_STATE, NEXT_STEPS, SESSION_LOG i arhitektura.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Aplikacijski kod, Prisma šema i migracije nijesu mijenjani.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Status označava dogovoreni plan, ne završenu funkcionalnost.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -20900,36 +20997,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-004 Robno</v>
+        <v>M-012 Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Specifikacija spremna</v>
       </c>
       <c r="C2" t="str">
-        <v>Summa izlazna faktura povezana je sa Fiscal API-jem. Jedno dugme automatski koristi Test ili Production, stabilan idempotency ključ i čuva zvanični broj, IKOF, JIKR i QR URL. Poslije fiskalizacije sadržaj je zaključan, a knjiženje se može dovršiti odvojeno.</v>
+        <v>Dogovoren je poseban mobile-first /portal sa automatskim kontekstom jedne firme, operativnim dashboardom, POS-om, klasičnim bezgotovinskim fakturama, jedinstvenim pregledom fiskalnih računa, izvještajima, artiklima, kupcima i ograničenim podešavanjima.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA u Test okruženju i kontrolisana produkcijska provjera.</v>
+        <v>Implementirati sigurnosni portal guard i zabranu /agencija pristupa, zatim dashboard, oba prodajna toka, izvještaje i šifarnike prema DIRECT_FISCAL_CLIENT_PORTAL_SPEC.md.</v>
       </c>
       <c r="E2" t="str">
-        <v>Fiskalni račun se ne šalje iz razvojne provjere; korisnik eksplicitno pokreće slanje dugmetom Fiskalizuj.</v>
+        <v>Fiskalna konfiguracija, sertifikati, ENU, operateri, aktivacija i suspenzija ostaju isključivo platformskom adminu; direct FISCAL_ONLY dokumenti ne kreiraju KIF ni nalog.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>M-011 POS / Kasa</v>
+        <v>Dokumentacija i planer</v>
       </c>
       <c r="B3" t="str">
-        <v>Prva funkcionalna faza</v>
+        <v>Usklađeno</v>
       </c>
       <c r="C3" t="str">
-        <v>Mobile-first POS, povezivanje kase sa Fiscal API objektom/ENU-om/operatorom, zajednički artikli i cijene, korpa, kupac, gotovina/kartica/virman, atomarna numeracija, retry, fiskalni rezultat, pregled, štampa i atomsko razduženje lagera sa podesivim pravilom minusa.</v>
+        <v>Dodata detaljna implementaciona specifikacija i ažurirani fiskalni README, POS specifikacija, CURRENT_STATE, NEXT_STEPS, SESSION_LOG i arhitektura.</v>
       </c>
       <c r="D3" t="str">
-        <v>Mobile QA, zbirni KIF/knjiženje, dnevni promet, povrati, smjene i POS Agent.</v>
+        <v>Aplikacijski kod, Prisma šema i migracije nijesu mijenjani.</v>
       </c>
       <c r="E3" t="str">
-        <v>Koristi FiskalniIzlazniRacun; direktni klijent može dobiti samo POS prava.</v>
+        <v>Status označava dogovoreni plan, ne završenu funkcionalnost.</v>
       </c>
     </row>
   </sheetData>
@@ -20941,7 +21038,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20968,18 +21065,35 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Izlazne fakture imaju pregled, nacrt i brzi editor za robu i usluge, cijene iz šifarnika, Enter navigaciju, brzo dodavanje artikla/usluge i preglednu A4 štampu. Štampa podržava snapshot strana, nacrt, PDV rekapitulaciju i zvanični fiskalni QR/IKOF/JIKR kada postoje. Za firme van Summa fiskalizacije završavanje provjerava lager i PDV period, razdužuje robu, kreira nalog i šalje zapis u KIF kao SOURCE_DOCUMENT bez ponovnog knjiženja.</v>
+        <v>Summa izlazna faktura povezana je sa Fiscal API-jem. Jedno dugme automatski koristi Test ili Production, stabilan idempotency ključ i čuva zvanični broj, IKOF, JIKR i QR URL. Poslije fiskalizacije sadržaj je zaključan, a knjiženje se može dovršiti odvojeno.</v>
       </c>
       <c r="D2" t="str">
-        <v>Povezivanje završavanja Summa fakture sa Fiscal API-jem i završni end-to-end QA.</v>
+        <v>Ručni end-to-end QA u Test okruženju i kontrolisana produkcijska provjera.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracije 20260807100000_izlazne_fakture_mvp, 20260807120000_kif_source_document_posting i 20260808100000_invoice_print_snapshots su primijenjene.</v>
+        <v>Fiskalni račun se ne šalje iz razvojne provjere; korisnik eksplicitno pokreće slanje dugmetom Fiskalizuj.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>M-011 POS / Kasa</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Prva funkcionalna faza</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Mobile-first POS, povezivanje kase sa Fiscal API objektom/ENU-om/operatorom, zajednički artikli i cijene, korpa, kupac, gotovina/kartica/virman, atomarna numeracija, retry, fiskalni rezultat, pregled, štampa i atomsko razduženje lagera sa podesivim pravilom minusa.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Mobile QA, zbirni KIF/knjiženje, dnevni promet, povrati, smjene i POS Agent.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Koristi FiskalniIzlazniRacun; direktni klijent može dobiti samo POS prava.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add financial statements XML export and polish agency UI
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -434,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -455,92 +455,109 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Robno / Prenos robe</v>
+        <v>Završni račun / XML</v>
       </c>
       <c r="B2" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Nacrt, zaglavlje, stavke, lista, detalj i A4 štampa; atomarni OUT/IN promet, ažuriranje oba lagera po prosječnoj cijeni, kontrola minusa i DRAFT nalog po firm-specific šemi.</v>
+        <v>XML BS/BU/SA sa korekcijama i uporednim kolonama; nulte ostale sekcije; zaglavlje i audit.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA na stvarnim zalihama i različitim poslovnim jedinicama.</v>
+        <v>Probni portal uvoz i provjera identifikatora/datuma.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260903100000_prenosi_robe je primijenjena; automatski test obračuna prolazi 3/3.</v>
+        <v>6 testova uključujući stvarnu XSD validaciju; bez migracije.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Robno / Popis robe</v>
+        <v>Robno / Prenos robe</v>
       </c>
       <c r="B3" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C3" t="str">
-        <v>Popis po magacinu, knjigovodstveno i stvarno stanje, višak/manjak, vrijednosne korekcije, DRAFT nalog po posebnoj šemi i A4 štampa.</v>
+        <v>Nacrt, zaglavlje, stavke, lista, detalj i A4 štampa; atomarni OUT/IN promet, ažuriranje oba lagera po prosječnoj cijeni, kontrola minusa i DRAFT nalog po firm-specific šemi.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
+        <v>Ručni end-to-end QA na stvarnim zalihama i različitim poslovnim jedinicama.</v>
       </c>
       <c r="E3" t="str">
-        <v>Migracija 20260903120000_popisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
+        <v>Migracija 20260903100000_prenosi_robe je primijenjena; automatski test obračuna prolazi 3/3.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Robno / Otpis robe</v>
+        <v>Robno / Popis robe</v>
       </c>
       <c r="B4" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Nacrt po magacinu, razlozi i stavke, kontrola minusa, razduženje svih vrijednosti lagera, kartični promet, DRAFT nalog po firm-specific šemi i A4 štampa.</v>
+        <v>Popis po magacinu, knjigovodstveno i stvarno stanje, višak/manjak, vrijednosne korekcije, DRAFT nalog po posebnoj šemi i A4 štampa.</v>
       </c>
       <c r="D4" t="str">
         <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
       </c>
       <c r="E4" t="str">
-        <v>Migracija 20260903140000_otpisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
+        <v>Migracija 20260903120000_popisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Robno / Nivelacija cijena</v>
+        <v>Robno / Otpis robe</v>
       </c>
       <c r="B5" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>Nacrt po maloprodajnom magacinu, stara/nova MPC, promjene MP vrijednosti/RUC-a/PDV-a bez promjene količine, cjenovnik, kartični promet, DRAFT nalog i A4 štampa.</v>
+        <v>Nacrt po magacinu, razlozi i stavke, kontrola minusa, razduženje svih vrijednosti lagera, kartični promet, DRAFT nalog po firm-specific šemi i A4 štampa.</v>
       </c>
       <c r="D5" t="str">
-        <v>Ručni end-to-end QA sa povećanjem, smanjenjem i mješovitim dokumentom.</v>
+        <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
       </c>
       <c r="E5" t="str">
-        <v>Migracija 20260903160000_nivelacije_cijena je primijenjena; automatski test obračuna prolazi 4/4.</v>
+        <v>Migracija 20260903140000_otpisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Robno / Nivelacija cijena</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Nacrt po maloprodajnom magacinu, stara/nova MPC, promjene MP vrijednosti/RUC-a/PDV-a bez promjene količine, cjenovnik, kartični promet, DRAFT nalog i A4 štampa.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Ručni end-to-end QA sa povećanjem, smanjenjem i mješovitim dokumentom.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Migracija 20260903160000_nivelacije_cijena je primijenjena; automatski test obračuna prolazi 4/4.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>Robno / Promet robe</v>
       </c>
-      <c r="B6" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C6" t="str">
+      <c r="B7" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C7" t="str">
         <v>Pregled sekcije i kompletni tokovi prenosa, popisa sa viškom/manjkom, otpisa i nivelacije.</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D7" t="str">
         <v>Ručni end-to-end QA na stvarnim zalihama i podešenim kontima.</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E7" t="str">
         <v>Kartica artikla direktno otvara izvorni prenos, popis, otpis i nivelaciju.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2393,7 +2410,7 @@
         <v>MVP 3</v>
       </c>
       <c r="H12" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statistički aneks imaju šablone, obračun iz POSTED naloga, prethodne kolone, podešavanja po firmi, trajne ručne korekcije i print. Objedinjene kontrole provjeravaju glavnu knjigu, pomoćne evidencije, šeme, konta rezultata, zatvaranje klasa 5/6, korekcije, arhivu i matične podatke; postoje i predlog zaključnog naloga i arhiva snimljenih obrazaca. Ostaje XML/export.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statistički aneks imaju šablone, obračun iz POSTED naloga, prethodne kolone, podešavanja po firmi, trajne ručne korekcije i print. Objedinjene kontrole provjeravaju glavnu knjigu, pomoćne evidencije, šeme, konta rezultata, zatvaranje klasa 5/6, korekcije, arhivu i matične podatke; postoje i predlog zaključnog naloga i arhiva snimljenih obrazaca. XML izvoz BS/BU/SA sa nultim nekorišćenim sekcijama i XSD testom je implementiran; ostaje portal QA.</v>
       </c>
     </row>
     <row r="13">
@@ -2509,7 +2526,7 @@
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z374"/>
+  <dimension ref="A1:Z375"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6815,9 +6832,47 @@
         <v>Kalkulacije i izlazni/POS računi nasljeđuju jedinicu magacina; ručni KIF/KUF, pazar, izvod i plata imaju izbor. KIF/KUF knjiženje čuva jedinicu po stavci, izvještaj računa klasu 6 minus klasu 5, a završna kontrola prijavljuje obaveznu jedinicu koja nedostaje. Izbor se automatski skriva kada firma nema aktivnih jedinica.</v>
       </c>
     </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>F-113</v>
+      </c>
+      <c r="B375" t="str">
+        <v>Završni račun</v>
+      </c>
+      <c r="C375" t="str">
+        <v>XML izvoz finansijskih iskaza</v>
+      </c>
+      <c r="D375" t="str">
+        <v>BS/BU/SA sa korekcijama i uporednim kolonama; ostale sekcije nulte prema potvrđenom obimu.</v>
+      </c>
+      <c r="E375" t="str">
+        <v>Visok</v>
+      </c>
+      <c r="F375" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="G375" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H375" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I375" t="str">
+        <v>Ne</v>
+      </c>
+      <c r="J375" t="str">
+        <v>Da</v>
+      </c>
+      <c r="K375" t="str">
+        <v>M-008</v>
+      </c>
+      <c r="L375" t="str">
+        <v>Zaglavlje za pregled; view/export scope i audit; XSD test. Portal QA ostaje otvoren.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z374"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z375"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: unify agency permissions and reporting
</commit_message>
<xml_diff>
--- a/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
+++ b/zadaci/Planer_Racunovodstveni_Program_AZURIRAN_M1-M3.xlsx
@@ -3,44 +3,45 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Status 2026-09-03" sheetId="1" r:id="rId1"/>
-    <sheet name="Status 2026-09-02" sheetId="2" r:id="rId2"/>
-    <sheet name="Status 2026-08-31" sheetId="3" r:id="rId3"/>
-    <sheet name="Status 2026-08-30" sheetId="4" r:id="rId4"/>
-    <sheet name="Status 2026-08-25" sheetId="5" r:id="rId5"/>
-    <sheet name="Status 2026-08-23" sheetId="6" r:id="rId6"/>
-    <sheet name="Status 2026-08-20" sheetId="7" r:id="rId7"/>
-    <sheet name="Status 2026-08-19" sheetId="8" r:id="rId8"/>
-    <sheet name="Status 2026-08-08" sheetId="9" r:id="rId9"/>
-    <sheet name="Status 2026-08-07" sheetId="10" r:id="rId10"/>
-    <sheet name="Status 2026-08-04" sheetId="11" r:id="rId11"/>
-    <sheet name="Status 2026-07-30" sheetId="12" r:id="rId12"/>
-    <sheet name="Status 2026-07-29" sheetId="13" r:id="rId13"/>
-    <sheet name="Status 2026-07-26" sheetId="14" r:id="rId14"/>
-    <sheet name="Status 2026-07-25" sheetId="15" r:id="rId15"/>
-    <sheet name="Status 2026-07-24" sheetId="16" r:id="rId16"/>
-    <sheet name="Status 2026-07-09" sheetId="17" r:id="rId17"/>
-    <sheet name="Status 2026-07-07" sheetId="18" r:id="rId18"/>
-    <sheet name="Status 2026-07-06" sheetId="19" r:id="rId19"/>
-    <sheet name="Status 2026-07-05" sheetId="20" r:id="rId20"/>
-    <sheet name="Status 2026-07-02" sheetId="21" r:id="rId21"/>
-    <sheet name="Status 2026-06-30" sheetId="22" r:id="rId22"/>
-    <sheet name="Status 2026-06-29" sheetId="23" r:id="rId23"/>
-    <sheet name="Status 2026-06-28" sheetId="24" r:id="rId24"/>
-    <sheet name="Status 2026-06-25" sheetId="25" r:id="rId25"/>
-    <sheet name="Dashboard" sheetId="26" r:id="rId26"/>
-    <sheet name="Moduli" sheetId="27" r:id="rId27"/>
-    <sheet name="Funkcionalnosti" sheetId="28" r:id="rId28"/>
-    <sheet name="Pravila" sheetId="29" r:id="rId29"/>
-    <sheet name="Zavisnosti" sheetId="30" r:id="rId30"/>
-    <sheet name="Ekrani" sheetId="31" r:id="rId31"/>
-    <sheet name="Baza" sheetId="32" r:id="rId32"/>
-    <sheet name="API" sheetId="33" r:id="rId33"/>
-    <sheet name="Testovi" sheetId="34" r:id="rId34"/>
-    <sheet name="Bugovi" sheetId="35" r:id="rId35"/>
-    <sheet name="Ideje" sheetId="36" r:id="rId36"/>
-    <sheet name="Odluke" sheetId="37" r:id="rId37"/>
-    <sheet name="Kategorije" sheetId="38" r:id="rId38"/>
+    <sheet name="Status 2026-09-04" sheetId="1" r:id="rId1"/>
+    <sheet name="Status 2026-09-03" sheetId="2" r:id="rId2"/>
+    <sheet name="Status 2026-09-02" sheetId="3" r:id="rId3"/>
+    <sheet name="Status 2026-08-31" sheetId="4" r:id="rId4"/>
+    <sheet name="Status 2026-08-30" sheetId="5" r:id="rId5"/>
+    <sheet name="Status 2026-08-25" sheetId="6" r:id="rId6"/>
+    <sheet name="Status 2026-08-23" sheetId="7" r:id="rId7"/>
+    <sheet name="Status 2026-08-20" sheetId="8" r:id="rId8"/>
+    <sheet name="Status 2026-08-19" sheetId="9" r:id="rId9"/>
+    <sheet name="Status 2026-08-08" sheetId="10" r:id="rId10"/>
+    <sheet name="Status 2026-08-07" sheetId="11" r:id="rId11"/>
+    <sheet name="Status 2026-08-04" sheetId="12" r:id="rId12"/>
+    <sheet name="Status 2026-07-30" sheetId="13" r:id="rId13"/>
+    <sheet name="Status 2026-07-29" sheetId="14" r:id="rId14"/>
+    <sheet name="Status 2026-07-26" sheetId="15" r:id="rId15"/>
+    <sheet name="Status 2026-07-25" sheetId="16" r:id="rId16"/>
+    <sheet name="Status 2026-07-24" sheetId="17" r:id="rId17"/>
+    <sheet name="Status 2026-07-09" sheetId="18" r:id="rId18"/>
+    <sheet name="Status 2026-07-07" sheetId="19" r:id="rId19"/>
+    <sheet name="Status 2026-07-06" sheetId="20" r:id="rId20"/>
+    <sheet name="Status 2026-07-05" sheetId="21" r:id="rId21"/>
+    <sheet name="Status 2026-07-02" sheetId="22" r:id="rId22"/>
+    <sheet name="Status 2026-06-30" sheetId="23" r:id="rId23"/>
+    <sheet name="Status 2026-06-29" sheetId="24" r:id="rId24"/>
+    <sheet name="Status 2026-06-28" sheetId="25" r:id="rId25"/>
+    <sheet name="Status 2026-06-25" sheetId="26" r:id="rId26"/>
+    <sheet name="Dashboard" sheetId="27" r:id="rId27"/>
+    <sheet name="Moduli" sheetId="28" r:id="rId28"/>
+    <sheet name="Funkcionalnosti" sheetId="29" r:id="rId29"/>
+    <sheet name="Pravila" sheetId="30" r:id="rId30"/>
+    <sheet name="Zavisnosti" sheetId="31" r:id="rId31"/>
+    <sheet name="Ekrani" sheetId="32" r:id="rId32"/>
+    <sheet name="Baza" sheetId="33" r:id="rId33"/>
+    <sheet name="API" sheetId="34" r:id="rId34"/>
+    <sheet name="Testovi" sheetId="35" r:id="rId35"/>
+    <sheet name="Bugovi" sheetId="36" r:id="rId36"/>
+    <sheet name="Ideje" sheetId="37" r:id="rId37"/>
+    <sheet name="Odluke" sheetId="38" r:id="rId38"/>
+    <sheet name="Kategorije" sheetId="39" r:id="rId39"/>
   </sheets>
 </workbook>
 </file>
@@ -434,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -455,116 +456,48 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Završni račun / XML</v>
+        <v>Izvještaji / Bruto bilans</v>
       </c>
       <c r="B2" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>XML BS/BU/SA sa korekcijama i uporednim kolonama; nulte ostale sekcije; zaglavlje i audit.</v>
+        <v>Centralna ruta koristi postojeći Bruto bilans iz Naloga sa svim filterima, nivoima zbira, poslovnim jedinicama i A4 štampom; konto otvara centralnu karticu uz prenesene filtere.</v>
       </c>
       <c r="D2" t="str">
-        <v>Probni portal uvoz i provjera identifikatora/datuma.</v>
+        <v>Formalni QA na većem setu podataka ostaje u postojećem planu testova.</v>
       </c>
       <c r="E2" t="str">
-        <v>6 testova uključujući stvarnu XSD validaciju; bez migracije.</v>
+        <v>Nema dupliranja poslovne logike ni migracije baze; TypeScript, ESLint i diff provjera prolaze.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Robno / Prenos robe</v>
+        <v>Korisnici i prava</v>
       </c>
       <c r="B3" t="str">
-        <v>Implementirano</v>
+        <v>Core implementiran / dorada</v>
       </c>
       <c r="C3" t="str">
-        <v>Nacrt, zaglavlje, stavke, lista, detalj i A4 štampa; atomarni OUT/IN promet, ažuriranje oba lagera po prosječnoj cijeni, kontrola minusa i DRAFT nalog po firm-specific šemi.</v>
+        <v>Uklonjena su legacy moze_da_* prava; KorisnikPravo je jedini izvor dozvola. View filtrira glavni meni po aktivnoj firmi, matrica ima cancel, ručni nalozi provjeravaju prava na backendu, a admin-only statistika radnika koristi aktivnost_dogadjaji sa periodom i poslovnim filterima.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni end-to-end QA na stvarnim zalihama i različitim poslovnim jedinicama.</v>
+        <v>Auditirati preostale poslovne rute i dodati integracione permission testove.</v>
       </c>
       <c r="E3" t="str">
-        <v>Migracija 20260903100000_prenosi_robe je primijenjena; automatski test obračuna prolazi 3/3.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Robno / Popis robe</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Popis po magacinu, knjigovodstveno i stvarno stanje, višak/manjak, vrijednosne korekcije, DRAFT nalog po posebnoj šemi i A4 štampa.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Migracija 20260903120000_popisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Robno / Otpis robe</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Nacrt po magacinu, razlozi i stavke, kontrola minusa, razduženje svih vrijednosti lagera, kartični promet, DRAFT nalog po firm-specific šemi i A4 štampa.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Migracija 20260903140000_otpisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Robno / Nivelacija cijena</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Nacrt po maloprodajnom magacinu, stara/nova MPC, promjene MP vrijednosti/RUC-a/PDV-a bez promjene količine, cjenovnik, kartični promet, DRAFT nalog i A4 štampa.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Ručni end-to-end QA sa povećanjem, smanjenjem i mješovitim dokumentom.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Migracija 20260903160000_nivelacije_cijena je primijenjena; automatski test obračuna prolazi 4/4.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Robno / Promet robe</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Pregled sekcije i kompletni tokovi prenosa, popisa sa viškom/manjkom, otpisa i nivelacije.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Ručni end-to-end QA na stvarnim zalihama i podešenim kontima.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Kartica artikla direktno otvara izvorni prenos, popis, otpis i nivelaciju.</v>
+        <v>Backfill ne dira već podešene matrice; radnik firmu bira u gornjoj traci, dok su Firme, Korisnici i prava, glavna Podešavanja, podešavanja poslovnih modula i Aktivnosti radnika samo za admina agencije.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -591,18 +524,35 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Izlazne fakture imaju pregled, nacrt i brzi editor za robu i usluge, cijene iz šifarnika, Enter navigaciju, brzo dodavanje artikla/usluge i preglednu A4 štampu. Štampa podržava snapshot strana, nacrt, PDV rekapitulaciju i zvanični fiskalni QR/IKOF/JIKR kada postoje. Za firme van Summa fiskalizacije završavanje provjerava lager i PDV period, razdužuje robu, kreira nalog i šalje zapis u KIF kao SOURCE_DOCUMENT bez ponovnog knjiženja.</v>
+        <v>Summa izlazna faktura povezana je sa Fiscal API-jem. Jedno dugme automatski koristi Test ili Production, stabilan idempotency ključ i čuva zvanični broj, IKOF, JIKR i QR URL. Poslije fiskalizacije sadržaj je zaključan, a knjiženje se može dovršiti odvojeno.</v>
       </c>
       <c r="D2" t="str">
-        <v>Povezivanje završavanja Summa fakture sa Fiscal API-jem i završni end-to-end QA.</v>
+        <v>Ručni end-to-end QA u Test okruženju i kontrolisana produkcijska provjera.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracije 20260807100000_izlazne_fakture_mvp, 20260807120000_kif_source_document_posting i 20260808100000_invoice_print_snapshots su primijenjene.</v>
+        <v>Fiskalni račun se ne šalje iz razvojne provjere; korisnik eksplicitno pokreće slanje dugmetom Fiskalizuj.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>M-011 POS / Kasa</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Prva funkcionalna faza</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Mobile-first POS, povezivanje kase sa Fiscal API objektom/ENU-om/operatorom, zajednički artikli i cijene, korpa, kupac, gotovina/kartica/virman, atomarna numeracija, retry, fiskalni rezultat, pregled, štampa i atomsko razduženje lagera sa podesivim pravilom minusa.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Mobile QA, zbirni KIF/knjiženje, dnevni promet, povrati, smjene i POS Agent.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Koristi FiskalniIzlazniRacun; direktni klijent može dobiti samo POS prava.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -630,19 +580,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
+        <v>M-004 Robno</v>
       </c>
       <c r="B2" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>KIF knjiga prikazuje fiskalizovane izlazne račune koji čekaju unos i omogućava grupno preuzimanje kupca, broja, datuma, iznosa i PDV razrade. Izvorni račun i KIF zapis trajno su povezani radi zaštite od duplikata.</v>
+        <v>Izlazne fakture imaju pregled, nacrt i brzi editor za robu i usluge, cijene iz šifarnika, Enter navigaciju, brzo dodavanje artikla/usluge i preglednu A4 štampu. Štampa podržava snapshot strana, nacrt, PDV rekapitulaciju i zvanični fiskalni QR/IKOF/JIKR kada postoje. Za firme van Summa fiskalizacije završavanje provjerava lager i PDV period, razdužuje robu, kreira nalog i šalje zapis u KIF kao SOURCE_DOCUMENT bez ponovnog knjiženja.</v>
       </c>
       <c r="D2" t="str">
-        <v>Povezati budući ekran izdavanja izlaznih faktura sa lokalnim fiskalnim izvorom i uraditi ručni end-to-end QA na stvarno fiskalizovanom računu.</v>
+        <v>Povezivanje završavanja Summa fakture sa Fiscal API-jem i završni end-to-end QA.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260804100000_fiskalni_racuni_kif_queue je primijenjena; tenant scope, prava, zaključavanje, PDV stope, duplikati i audit provjeravaju se na backendu.</v>
+        <v>Migracije 20260807100000_izlazne_fakture_mvp, 20260807120000_kif_source_document_posting i 20260808100000_invoice_print_snapshots su primijenjene.</v>
       </c>
     </row>
   </sheetData>
@@ -681,13 +631,13 @@
         <v>Core implementiran / dorada</v>
       </c>
       <c r="C2" t="str">
-        <v>KIF sada podržava dnevni i mjesečni pazar sa periodom, brojem izvještaja, kasom, poreskim osnovicama, izlaznim PDV-om i raspodjelom naplate na gotovinu, kartice, virman i ostalo. Preklapanje perioda iste kase je blokirano. Ukupan iznos se kaskadno raspoređuje od najveće aktivne stope ka 0%, uz automatski izlazni PDV. Pazar se prikazuje u KIF-u, štampi, Excel izvozu i izlaznom PDV-u. Podešavanja firme imaju posebna dugujuća konta načina naplate, dok prihod i PDV koriste aktivnu KIF šemu.</v>
+        <v>KIF knjiga prikazuje fiskalizovane izlazne račune koji čekaju unos i omogućava grupno preuzimanje kupca, broja, datuma, iznosa i PDV razrade. Izvorni račun i KIF zapis trajno su povezani radi zaštite od duplikata.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA kreiranja, izmjene, brisanja, zabrane preklapanja, knjiženja i PDV prikaza pazara; PDV zaključavanje KIF/KUF izmjena.</v>
+        <v>Povezati budući ekran izdavanja izlaznih faktura sa lokalnim fiskalnim izvorom i uraditi ručni end-to-end QA na stvarno fiskalizovanom računu.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracija 20260730170000_kif_pazar je primijenjena, Prisma klijent regenerisan i dev server restartovan. TypeScript, Prisma validacija i lint prolaze bez novih grešaka.</v>
+        <v>Migracija 20260804100000_fiskalni_racuni_kif_queue je primijenjena; tenant scope, prava, zaključavanje, PDV stope, duplikati i audit provjeravaju se na backendu.</v>
       </c>
     </row>
   </sheetData>
@@ -699,6 +649,51 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>M-010 Računi / KIF-KUF</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C2" t="str">
+        <v>KIF sada podržava dnevni i mjesečni pazar sa periodom, brojem izvještaja, kasom, poreskim osnovicama, izlaznim PDV-om i raspodjelom naplate na gotovinu, kartice, virman i ostalo. Preklapanje perioda iste kase je blokirano. Ukupan iznos se kaskadno raspoređuje od najveće aktivne stope ka 0%, uz automatski izlazni PDV. Pazar se prikazuje u KIF-u, štampi, Excel izvozu i izlaznom PDV-u. Podešavanja firme imaju posebna dugujuća konta načina naplate, dok prihod i PDV koriste aktivnu KIF šemu.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Ručni end-to-end QA kreiranja, izmjene, brisanja, zabrane preklapanja, knjiženja i PDV prikaza pazara; PDV zaključavanje KIF/KUF izmjena.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Migracija 20260730170000_kif_pazar je primijenjena, Prisma klijent regenerisan i dev server restartovan. TypeScript, Prisma validacija i lint prolaze bez novih grešaka.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
@@ -759,7 +754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -800,68 +795,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>M-003 Nalozi</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Početno stanje završeno</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>M-010 Računi / KIF-KUF</v>
-      </c>
-      <c r="B3" t="str">
-        <v>QR čitanje računa završeno</v>
-      </c>
-      <c r="C3" t="str">
-        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -889,36 +822,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Plate i zaposleni</v>
+        <v>M-003 Nalozi</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Početno stanje završeno</v>
       </c>
       <c r="C2" t="str">
-        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
+        <v>Automatski prenos POSTED salda prethodne godine za klase 0-4, grupisanje po kontu i partneru, numerisan DRAFT nalog, pregled stavki, upozorenje za klase 5/6, provjere prava/scope-a/zaključavanja/balansa i zaštita od duplikata.</v>
       </c>
       <c r="D2" t="str">
-        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
+        <v>Kontrole po poslovnoj jedinici, trajni automatizovani test i test konkurentnih zahtjeva.</v>
       </c>
       <c r="E2" t="str">
-        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+        <v>Rollback integracioni test 2026-07-25 potvrdio je prenos, partner analitiku, isključenje klasa 5/6 i balans bez zadržavanja testnih podataka.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Firme</v>
+        <v>M-010 Računi / KIF-KUF</v>
       </c>
       <c r="B3" t="str">
-        <v>Core implementiran / dorada</v>
+        <v>QR čitanje računa završeno</v>
       </c>
       <c r="C3" t="str">
-        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+        <v>KUF forma lokalno čita MAPR QR kod iz PDF, TIFF, JPG i PNG računa bez čuvanja originala. Za male QR kodove koristi visoku rezoluciju, Chrome/ZXing dekodere, zone, uvećavanje i kontrast. Import stranica prihvata više fajlova, dopisuje jedinstvene linkove i prikazuje status po fajlu prije stvarnog importa.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+        <v>Ručni QA na većem uzorku stvarnih skenova i višestraničnih dokumenata.</v>
       </c>
       <c r="E3" t="str">
-        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
+        <v>Podržano do 20 MB po fajlu i do osam PDF/TIFF stranica; Racun_izlaza(18).pdf potvrđen je kroz ZXing pri renderu od 3000 px.</v>
       </c>
     </row>
   </sheetData>
@@ -930,7 +863,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -951,24 +884,41 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Plate</v>
+        <v>Plate i zaposleni</v>
       </c>
       <c r="B2" t="str">
         <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
+        <v>Podešavanje knjiženja više nije placeholder: firma i poslovna godina imaju odvojenu šemu za redovan rad, ugovor o djelu, zakup i ostale ugovore. Obrađeni obračun akcijom Proknjiži kreira izbalansiran i odmah POSTED PAYROLL nalog. M-4, OPP-ND i IOPPD grupisani su u podmeniju Obrasci; OPP-ND razvrstava mjesečni porez po četiri službene vrste i generiše zvaničnu A4 prijavu prireza po opštinskoj stopi.</v>
       </c>
       <c r="D2" t="str">
-        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
+        <v>Obustave, uplatnice, namjenski storno/vraćanje automatskog naloga i print/export obračuna.</v>
       </c>
       <c r="E2" t="str">
-        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
+        <v>Migracije kontiranja i veze naloga su primijenjene. OPP-ND koristi postojeće obračune i opštinski šifarnik pa ne traži novu tabelu; završni render je vizuelno upoređen sa dostavljenim PDF-om.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Firme</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Core implementiran / dorada</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Na detalju firme dodat je odvojeni opasni odjeljak za trajno brisanje testne firme. Admin agencije mora unijeti potpuno isti puni naziv; backend ponavlja provjeru unutar jedne transakcije i zaključava firmu kroz agencijski scope. Brišu se samo firmine poslovne godine, nalozi, KIF/KUF, PDV, izvodi, plate/M-4, konta, bankovni računi, partneri koji pripadaju firmi, korisničke veze, ugovor, odgovorna lica, finansijski izvještaji i ostala firm-specific podešavanja. Zajednički korisnici i globalni/agencijski šifarnici ostaju.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni vizuelni QA forme u browseru i puni ekran za više odgovornih/kontakt lica.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Izolovani integracioni test potvrdio je da pogrešan naziv ne briše firmu, tačan naziv je briše, a agencijski audit zapis ostaje. Aktivni kontekst firme/godine se čisti kada se obriše trenutno izabrana firma.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -996,19 +946,19 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Zavrsni racun</v>
+        <v>Plate</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimicno implementirano</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
+        <v>Dodata prva MVP osnova: migracija 20260709100000_plate_mvp uvodi šifarnike IOPPD šifara, vrsta obračuna, poreskih razreda, doprinosa, prireza i šifri primanja; tabele zaposlenih, obračuna i obračunskih stavki; /agencija/plate za dodavanje, izmjenu, odjavu i reaktivaciju zaposlenih uz tabove aktivni/neaktivni; /agencija/plate/obracun za kategorije obračuna redovan rad/ugovor o djelu/zakup/ostali ugovori, redovan obračun 001, pripremu radnika, kontrole prije obrade, ručne mjesečne korekcije, dodatne stavke, brisanje obračuna i ručno dodavanje/izbacivanje radnika iz postojećeg obračuna; /agencija/plate/podesavanja za pregled šifarnika i ažuriranje IOPPD osnova obračuna; /agencija/plate/ioppd za mjesečni pregled IOPPD-a, /stampa/plate/ioppd za HTML/CSS štampu opšteg i posebnog dijela i /api/plate/ioppd/xml za XML download. Migracije 20260719130000_plate_osnove_obracuna i 20260719133000_plate_osnove_full_import uvode osnove, pravila i stope, te importuju svih 108 šifara iz zvaničnog Excel dokumenta.</v>
       </c>
       <c r="D2" t="str">
-        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
+        <v>Povezati IOPPD osnove direktno u algoritme za zakup/ugovore, zatim obustave, ručni QA IOPPD XML upload-a na portalu, uplatnice, automatski PAYROLL nalog, print/export i arhiva obračuna.</v>
       </c>
       <c r="E2" t="str">
-        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
+        <v>Bruto/neto servis čita važeće stope iz baze i podržava proporcionalni obračun po satima/fondu; minuli rad se računa progresivno po navršenim godinama staža, po potrebi izvodi godine iz datuma zaposlenja, i dodaje na osnovnu zaradu prije bruto/neto preračuna; originalni red svake osnove iz Excel šifarnika čuva se u JSON-u pravila; obračun više ne briše ručne korekcije nego računa iz pripremljenih mjesečnih stavki; obrada se blokira ako postoje kontrolne greške; IOPPD mjesečni pregled sabira sve obrađene obračune istog mjeseca.</v>
       </c>
     </row>
   </sheetData>
@@ -1020,7 +970,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1041,65 +991,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Partneri</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B2" t="str">
-        <v>Implementirano</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+        <v>Dodato snimanje zavrsnog racuna u arhivu: tabela finansijski_izvjestaj_arhive cuva JSON snapshot Bilansa stanja, Bilansa uspjeha i Statistickog aneksa za aktivnu firmu/godinu; /agencija/zavrsni-racun/arhiva prikazuje snimljene zavrsne racune, a /arhiva/[id] prikazuje zamrznuti snapshot.</v>
       </c>
       <c r="D2" t="str">
-        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+        <v>XML/export zavrsnog racuna i eventualna stampana verzija direktno iz arhivskog snimka.</v>
       </c>
       <c r="E2" t="str">
-        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Zavrsni racun</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Djelimicno implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Arhiva generisanih obrazaca i XML/export.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
+        <v>Live obrasci se i dalje preracunavaju iz bruto bilansa i sacuvanih rucnih korekcija; arhiva se ne preracunava.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1120,41 +1036,109 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Nalozi / Poslovne jedinice</v>
+        <v>Završni račun / XML</v>
       </c>
       <c r="B2" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C2" t="str">
-        <v>Firm-specific šifarnik sa pravima i auditom; jedinica prati dokument i svaku stavku naloga, a izvještaji filtriraju POSTED promet po jedinici.</v>
+        <v>XML BS/BU/SA sa korekcijama i uporednim kolonama; nulte ostale sekcije; zaglavlje i audit.</v>
       </c>
       <c r="D2" t="str">
-        <v>Raspodjela jedne stavke dokumenta na više jedinica može se dodati kasnije.</v>
+        <v>Probni portal uvoz i provjera identifikatora/datuma.</v>
       </c>
       <c r="E2" t="str">
-        <v>Pokriveni su ručni nalozi, KIF/KUF, izlazni/POS računi, izvodi, plate, rezultat po jedinicama i završna kontrola; izbor jedinice je skriven firmama bez aktivnih jedinica.</v>
+        <v>6 testova uključujući stvarnu XSD validaciju; bez migracije.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Robno / Magacini i kalkulacije</v>
+        <v>Robno / Prenos robe</v>
       </c>
       <c r="B3" t="str">
         <v>Implementirano</v>
       </c>
       <c r="C3" t="str">
-        <v>Magacin se opciono vezuje za poslovnu jedinicu. Domaća i MAPR kalkulacija snimaju jedinicu magacina, a njihov nalog je nasljeđuje.</v>
+        <v>Nacrt, zaglavlje, stavke, lista, detalj i A4 štampa; atomarni OUT/IN promet, ažuriranje oba lagera po prosječnoj cijeni, kontrola minusa i DRAFT nalog po firm-specific šemi.</v>
       </c>
       <c r="D3" t="str">
-        <v>Ručni end-to-end QA na više prodavnica/magacina.</v>
+        <v>Ručni end-to-end QA na stvarnim zalihama i različitim poslovnim jedinicama.</v>
       </c>
       <c r="E3" t="str">
-        <v>Istorijska kalkulacija i nalog ne zavise od naknadne promjene veze magacina.</v>
+        <v>Migracija 20260903100000_prenosi_robe je primijenjena; automatski test obračuna prolazi 3/3.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Robno / Popis robe</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Popis po magacinu, knjigovodstveno i stvarno stanje, višak/manjak, vrijednosne korekcije, DRAFT nalog po posebnoj šemi i A4 štampa.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Migracija 20260903120000_popisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Robno / Otpis robe</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Nacrt po magacinu, razlozi i stavke, kontrola minusa, razduženje svih vrijednosti lagera, kartični promet, DRAFT nalog po firm-specific šemi i A4 štampa.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Ručni end-to-end QA na stvarnom lageru i podešenim kontima.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Migracija 20260903140000_otpisi_robe je primijenjena; automatski test obračuna prolazi 4/4.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Robno / Nivelacija cijena</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Nacrt po maloprodajnom magacinu, stara/nova MPC, promjene MP vrijednosti/RUC-a/PDV-a bez promjene količine, cjenovnik, kartični promet, DRAFT nalog i A4 štampa.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Ručni end-to-end QA sa povećanjem, smanjenjem i mješovitim dokumentom.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Migracija 20260903160000_nivelacije_cijena je primijenjena; automatski test obračuna prolazi 4/4.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Robno / Promet robe</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Pregled sekcije i kompletni tokovi prenosa, popisa sa viškom/manjkom, otpisa i nivelacije.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Ručni end-to-end QA na stvarnim zalihama i podešenim kontima.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Kartica artikla direktno otvara izvorni prenos, popis, otpis i nivelaciju.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1222,13 +1206,13 @@
         <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
+        <v>Bilans uspjeha, Bilans stanja i Statisticki aneks imaju sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, podesavanja konta/formula po firmi, tab UI u obrascima, HTML/CSS print obrasce, trajne rucne korekcije po AOP/koloni i predlog zakljucnog naloga za klase 5/6.</v>
       </c>
       <c r="D4" t="str">
-        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
+        <v>Arhiva generisanih obrazaca i XML/export.</v>
       </c>
       <c r="E4" t="str">
-        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
+        <v>Rucne korekcije se cuvaju u finansijski_izvjestaj_korekcije; zakljucno knjizenje izuzima postojece FINAL_ACCOUNT naloge i cuva predlog kao nacrt naloga.</v>
       </c>
     </row>
   </sheetData>
@@ -1240,106 +1224,79 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-07-02</v>
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
+        <v>Partneri</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Polja za izbor partnera u KIF/KUF, izvodima i stavkama naloga imaju + Novi partner i modal za brzi unos; endpoint /api/partners/quick-create kreira/povezuje partnera u aktivnoj firmi.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Dodatni UX: IRMS dopuna direktno iz quick modal-a i naprednija provjera duplikata po nazivu.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Novi partner se odmah selektuje u polju iz kog je dodat.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Izvodi</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Djelimično implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>NLB XML/PDF, Erste HTM, CKB PDF, Hipotekarna PDF, Lovćen PDF i Prva banka PDF parseri rade; predlog naloga podržava osnovno zatvaranje otvorenih KIF/KUF računa preko bank_statement_line_allocations; status plaćanja računa se osvježava na UNPAID/PARTIALLY_PAID/PAID/OVERPAID.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Parseri za ostale banke, split alokacije jedne uplate na više računa, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Osnovna alokacija je po jednoj stavci izvoda na jedan račun istog partnera.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Oblast</v>
+        <v>Zavrsni racun</v>
       </c>
       <c r="B4" t="str">
-        <v>Status</v>
+        <v>Djelimicno implementirano</v>
       </c>
       <c r="C4" t="str">
-        <v>Sta je zavrseno</v>
+        <v>Dodate tabele za sablone finansijskih izvjestaja i prva implementacija Bilansa uspjeha, Bilansa stanja i Statistickog aneksa: sistemske seme pozicija, obracun iz POSTED naloga, poredjenje sa prethodnim kolonama, stranica Obrasci, podesavanja konta/formula po firmi i HTML/CSS print obrasci.</v>
       </c>
       <c r="D4" t="str">
-        <v>Sta ostaje</v>
+        <v>Rucni iznosi, arhiva generisanih obrazaca, XML/export i zakljucna knjizenja.</v>
       </c>
       <c r="E4" t="str">
-        <v>Preporuceni sljedeci korak</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Izvodi</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Djelimično implementirano</v>
-      </c>
-      <c r="C5" t="str">
-        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Nalozi</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PDV</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Core zaokružen</v>
-      </c>
-      <c r="C7" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C8" t="str">
-        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Redovno održavanje.</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Regenerisati Excel nakon svake veće promjene.</v>
+        <v>Bilans uspjeha izuzima pocetno stanje i nalog zavrsnog racuna; Bilans stanja prikazuje tekucu, prethodnu krajnju i prethodnu pocetnu kolonu; Statisticki aneks ima tekucu i prethodnu godinu.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1350,7 +1307,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-30</v>
+        <v>Status projekta na dan 2026-07-02</v>
       </c>
     </row>
     <row r="2">
@@ -1383,13 +1340,13 @@
         <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
+        <v>NLB XML, Erste HTM i CKB PDF parseri rade; batch upload postoji; CKB ukupni priliv i odliv čita iz zaglavlja PDF izvoda; pravila knjiženja mogu biti zajednička za agenciju ili specifična za firmu; pravila čuvaju account_code i automatski se povezuju na firma_konta aktivne firme; ručno naučeni žiro računi partnera čuvaju se zajednički kad je moguće; interni prenosi između sopstvenih računa firme prepoznaju se prije običnih pravila.</v>
       </c>
       <c r="D5" t="str">
-        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
+        <v>Parseri za ostale banke, alokacije na KIF/KUF fakture, vraćanje proknjiženog izvoda u nacrt i dodatni QA pravila.</v>
       </c>
       <c r="E5" t="str">
-        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
+        <v>Testirati uvoz više NLB/Erste/CKB izvoda na više firmi i provjeriti da zajednička pravila ne dupliraju račune komitenata.</v>
       </c>
     </row>
     <row r="6">
@@ -1452,11 +1409,11 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-29</v>
+        <v>Status projekta na dan 2026-06-30</v>
       </c>
     </row>
     <row r="2">
@@ -1483,92 +1440,75 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Nalozi</v>
+        <v>Izvodi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core zaokruzen</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C5" t="str">
-        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
+        <v>NLB XML parser radi; konto banke i konta stavki u predlogu čuvaju se preko šifre i automatski se povezuju na firma_konta; nalog knjiži banku zbirno po ukupnom prilivu/odlivu; dodate stranice Obrada stavki, Parseri banaka, Pravila knjiženja kao kandidati, Žiro računi komitenata, Kartica banke i Kontrole.</v>
       </c>
       <c r="D5" t="str">
-        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
+        <v>Parseri za druge banke, učenje žiro računa iz UI-a, trajna pravila knjiženja, alokacije na KIF/KUF fakture i vraćanje proknjiženog izvoda u nacrt.</v>
       </c>
       <c r="E5" t="str">
-        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
+        <v>Ručni QA: uvoz više NLB XML izvoda, čuvanje predloga, knjiženje READY izvoda i provjera naloga.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>PDV</v>
+        <v>Nalozi</v>
       </c>
       <c r="B6" t="str">
-        <v>Core zaokruzen</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C6" t="str">
-        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
+        <v>Ručni nalozi, nacrti, proknjižavanje, otvorene stavke na broju dokumenta, analitičke kartice, kupci/dobavljači zbirno i bruto bilans rade.</v>
       </c>
       <c r="D6" t="str">
-        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
+        <v>Formalni unos/prenos početnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E6" t="str">
-        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
+        <v>Nastaviti da izvodi koriste postojeći nalog IZV, bez posebnog ručnog toka.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Izvodi</v>
+        <v>PDV</v>
       </c>
       <c r="B7" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Core zaokružen</v>
       </c>
       <c r="C7" t="str">
-        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podešavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D7" t="str">
-        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
+        <v>Zaključavanje perioda i ručni QA XML upload-a na portalu.</v>
       </c>
       <c r="E7" t="str">
-        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
+        <v>Zaključati periodni tok poslije stabilizacije izvoda.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>KIF/KUF</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B8" t="str">
-        <v>Core implementiran</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C8" t="str">
-        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
+        <v>CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md, docs/accounting/izvodi.md i planer CSV usklađeni sa najnovijim radom na izvodima.</v>
       </c>
       <c r="D8" t="str">
-        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
+        <v>Redovno održavanje.</v>
       </c>
       <c r="E8" t="str">
-        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Planer/Dokumentacija</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Ažurirano</v>
-      </c>
-      <c r="C9" t="str">
-        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Redovno odrzavanje.</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Regenerisati Excel nakon svake vece promjene.</v>
+        <v>Regenerisati Excel nakon svake veće promjene.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1579,12 +1519,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status projekta na dan 2026-06-28</v>
+        <v>Status projekta na dan 2026-06-29</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+        <v>Kratki pregled stvarno implementiranog stanja i dogovorenog sljedećeg fokusa.</v>
       </c>
     </row>
     <row r="4">
@@ -1606,87 +1546,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Performanse partnera</v>
+        <v>Nalozi</v>
       </c>
       <c r="B5" t="str">
-        <v>Core implementiran</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C5" t="str">
-        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+        <v>Rucni nalozi, nacrti, proknjizavanje, otvorene stavke na broju dokumenta, analiticke kartice, kupci/dobavljaci zbirno po kontima sa partner analitikom i bruto bilans rade.</v>
       </c>
       <c r="D5" t="str">
-        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+        <v>Formalni unos/prenos pocetnog stanja, testovi i dodatne kontrole po poslovnoj jedinici.</v>
       </c>
       <c r="E5" t="str">
-        <v>Pratiti brzinu na produkciji.</v>
+        <v>Nalog IZV koristiti kao osnovu za ručno knjiženje izvoda; modul izvoda ne treba duplirati taj tok.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Indeksi baze</v>
+        <v>PDV</v>
       </c>
       <c r="B6" t="str">
-        <v>Implementirano</v>
+        <v>Core zaokruzen</v>
       </c>
       <c r="C6" t="str">
-        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+        <v>PDV periodi, ulazni/izlazni PDV, prijava po portalu, XML PR_PDV_2025, podesavanja knjiženja po stopama, osnovno knjiženje i kontrole postoje.</v>
       </c>
       <c r="D6" t="str">
-        <v>-</v>
+        <v>Zakljucavanje perioda i rucni QA XML upload-a na portalu.</v>
       </c>
       <c r="E6" t="str">
-        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+        <v>Zakljucati periodni tok poslije izvoda ili u stabilizaciji.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>KIF/KUF uvoz/export</v>
+        <v>Izvodi</v>
       </c>
       <c r="B7" t="str">
-        <v>Core implementiran</v>
+        <v>Djelimično implementirano</v>
       </c>
       <c r="C7" t="str">
-        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+        <v>Dodate tabele bank_statements, bank_statement_lines i partner_bank_accounts; /agencija/izvodi ima uvoz/paste teksta, NLB XML parser, pregled izvoda, tab Stavke izvoda, tab Predlog naloga, izbor partnera/konta i knjiženje READY izvoda u poseban IZV nalog.</v>
       </c>
       <c r="D7" t="str">
-        <v>Kontrole iznosa i duplikata; XML export.</v>
+        <v>Parseri za ostale banke, učenje žiro računa iz UI-a, alokacije na KIF/KUF fakture, pravila knjiženja, kartica banke i ručni QA.</v>
       </c>
       <c r="E7" t="str">
-        <v>QA uvoznih knjizenja i export fajlova.</v>
+        <v>Sljedeće ručno testirati NLB XML uvoz i dodati mapping/učenje žiro računa.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Dokumentacija</v>
+        <v>KIF/KUF</v>
       </c>
       <c r="B8" t="str">
-        <v>Uspostavljeno</v>
+        <v>Core implementiran</v>
       </c>
       <c r="C8" t="str">
-        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+        <v>Mjesečne knjige, vrste, seme, uvoz/izvoz, knjizenje i statusi postoje.</v>
       </c>
       <c r="D8" t="str">
-        <v>Redovno odrzavanje.</v>
+        <v>Kontrole duplikata/iznosa, payment status koji ce izvodi azurirati.</v>
       </c>
       <c r="E8" t="str">
-        <v>Azurirati uz svaku vecu promjenu.</v>
+        <v>Pripremiti status placanja i otvorene iznose kada krenu alokacije izvoda.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>PDV</v>
+        <v>Planer/Dokumentacija</v>
       </c>
       <c r="B9" t="str">
-        <v>Prva implementacija</v>
+        <v>Ažurirano</v>
       </c>
       <c r="C9" t="str">
-        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+        <v>docs/accounting/izvodi.md, NEXT_STEPS.md, CURRENT_STATE.md, SESSION_LOG.md i planer CSV usklađeni sa finalnom specifikacijom izvoda.</v>
       </c>
       <c r="D9" t="str">
-        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+        <v>Redovno odrzavanje.</v>
       </c>
       <c r="E9" t="str">
-        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+        <v>Regenerisati Excel nakon svake vece promjene.</v>
       </c>
     </row>
   </sheetData>
@@ -1698,6 +1638,129 @@
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Status projekta na dan 2026-06-28</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Kratki pregled stvarno implementiranog stanja (nezavisno od pocetne specifikacije).</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Oblast</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sta je zavrseno</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Sta ostaje</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Preporuceni sljedeci korak</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Performanse partnera</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Pretraga partnera u nalozima (novi/[id]) i filteru analitickih kartica prebacena na async (/api/partners/search); vise se ne ucitava ~64k partnera. Nove komponente JournalPartnerCell i PartnerFilterSelect.</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Eventualno cache rezultata i prikaz scope-a u dropdownu.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pratiti brzinu na produkciji.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Indeksi baze</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Migracija 20260628120000_komitent_pretraga_indeksi: pg_trgm GIN na komitenti.naziv + btree na pib i scope.</v>
+      </c>
+      <c r="D6" t="str">
+        <v>-</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Po potrebi indeksi na agencija_id/firma_id.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>KIF/KUF uvoz/export</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Core implementiran</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Konfigurabilna sema za uvoz (KUF): 5 konta, smjer D/P i partner po stavci; carina kao zasebna stavka troska, carinska obaveza na partnera CARINA. Dodat Excel export KIF/KUF pregleda po datumskom filteru.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Kontrole iznosa i duplikata; XML export.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>QA uvoznih knjizenja i export fajlova.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Dokumentacija</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Uspostavljeno</v>
+      </c>
+      <c r="C8" t="str">
+        <v>AGENTS.md, CURRENT_STATE.md, NEXT_STEPS.md, SESSION_LOG.md i docs/ (architecture + accounting). Pointeri za Copilot i Claude. Planer se vodi kao CSV izvor (zadaci/planer) + skripta za regeneraciju Excela.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Redovno odrzavanje.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Azurirati uz svaku vecu promjenu.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PDV</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Prva implementacija</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dodati mjesečni PDV periodi, ulazni/izlazni PDV pregledi iz KIF/KUF po datumu knjige, PDV prijava po portal layout-u, automatski preračuni, XML snapshot, podešavanja knjiženja D/P+konto po aktivnim stopama i osnovno knjiženje prijave.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Finalno IRMS XML mapiranje, zaključavanje perioda, ručni QA na stvarnim podacima.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Provjeriti konta 2700/4700 i nalog knjiženja.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
@@ -1870,7 +1933,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -2165,7 +2228,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z303"/>
   <sheetData>
@@ -2228,7 +2291,7 @@
         <v>MVP 1</v>
       </c>
       <c r="H5" t="str">
-        <v>Autentifikacija, agencije, korisnici, radnici/klijenti, dodjela firmi, matrica prava i audit osnova postoje. Agencijski shell ima sklopivi desktop meni sa pamćenjem izbora i mobilni bočni panel. Ostaju kompletan backend enforcement prava, pretplate/limiti i statistika radnika.</v>
+        <v>Autentifikacija, agencije, korisnici, radnici/klijenti, dodjela firmi i audit osnova postoje. KorisnikPravo je jedini izvor dozvola, view filtrira glavni meni po aktivnoj firmi, a ručni nalozi provjeravaju akcije na backendu. Agencijski shell ima sklopivi desktop meni i mobilni panel. Ostaju audit preostalih ruta, pretplate/limiti i statistika radnika.</v>
       </c>
     </row>
     <row r="6">
@@ -2436,7 +2499,7 @@
         <v>MVP 1/2</v>
       </c>
       <c r="H13" t="str">
-        <v>Bruto bilans i analitičke kartice postoje. Početni agencijski dashboard prikazuje tenant/permission-aware nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF. Centralni Izvještaji imaju funkcionalne kartice konta i partnera, PDV pregled, pregled izvještaja plata, lager listu i karticu artikla preko postojećih zajedničkih prikaza; kupci, dobavljači i finansijski izvještaji ostaju za centralno povezivanje.</v>
+        <v>Početna centralnih Izvještaja prikazuje postojeći Bruto bilans sa filterima, nivoima zbira, štampom i drill-downom na centralnu karticu konta. Početni agencijski dashboard prikazuje tenant/permission-aware nacrte naloga, kalkulacije koje čekaju KUF i izlazne račune koji čekaju KIF. Centralni Izvještaji imaju i funkcionalne kartice konta i partnera, PDV pregled, pregled izvještaja plata, lager listu i karticu artikla preko postojećih zajedničkih prikaza; kupci, dobavljači i finansijski izvještaji ostaju za centralno povezivanje.</v>
       </c>
     </row>
     <row r="301">
@@ -2524,7 +2587,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z375"/>
   <sheetData>
@@ -2877,7 +2940,7 @@
         <v>F-005</v>
       </c>
       <c r="L12" t="str">
-        <v>Matrica prava postoji; backend enforcement po modulima treba dodatno zakljucati.</v>
+        <v>KorisnikPravo je jedini izvor dozvola; view upravlja glavnim menijem, matrica uključuje cancel, a ručni nalozi su zaključani po akcijama. Administrativna podešavanja poslovnih modula vidljiva su i izvršiva samo adminu agencije. Audit preostalih operativnih ruta i jači testovi ostaju.</v>
       </c>
     </row>
     <row r="13">
@@ -2897,25 +2960,25 @@
         <v>Visok</v>
       </c>
       <c r="F13" t="str">
-        <v>U izradi</v>
+        <v>Implementirano</v>
       </c>
       <c r="G13" t="str">
+        <v>Da</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Da</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Da</v>
+      </c>
+      <c r="J13" t="str">
         <v>Djelimicno</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Djelimicno</v>
-      </c>
-      <c r="I13" t="str">
-        <v>Da</v>
-      </c>
-      <c r="J13" t="str">
-        <v>Ne</v>
       </c>
       <c r="K13" t="str">
         <v>F-005,F-034</v>
       </c>
       <c r="L13" t="str">
-        <v>Postoji osnova aktivnosti/audit; statistika ucinka nije poseban kompletan ekran.</v>
+        <v>Admin-only /agencija/aktivnosti ima brze periode, od-do i filtere radnika, firme, modula i akcije; prikazuje zbir, učinak po radniku, dnevni trend, module i hronologiju iz activity events. Tačnost zavisi od audit pokrića poslovnih akcija, koje se nastavlja širiti.</v>
       </c>
     </row>
     <row r="14">
@@ -4017,7 +4080,7 @@
         <v>F-029,F-034</v>
       </c>
       <c r="L42" t="str">
-        <v>Bruto bilans ima filtere, nivoe zbira, samo zbir, globalni zbir, klik na konto ka analitici i print varijantu.</v>
+        <v>Bruto bilans ima filtere, nivoe zbira, samo zbir, globalni zbir, klik na konto ka analitici i print varijantu; isti prikaz je povezan i kao početna stranica centralnih Izvještaja.</v>
       </c>
     </row>
     <row r="301">
@@ -6877,7 +6940,69 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nalozi / Poslovne jedinice</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Firm-specific šifarnik sa pravima i auditom; jedinica prati dokument i svaku stavku naloga, a izvještaji filtriraju POSTED promet po jedinici.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Raspodjela jedne stavke dokumenta na više jedinica može se dodati kasnije.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Pokriveni su ručni nalozi, KIF/KUF, izlazni/POS računi, izvodi, plate, rezultat po jedinicama i završna kontrola; izbor jedinice je skriven firmama bez aktivnih jedinica.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Robno / Magacini i kalkulacije</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Magacin se opciono vezuje za poslovnu jedinicu. Domaća i MAPR kalkulacija snimaju jedinicu magacina, a njihov nalog je nasljeđuje.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni end-to-end QA na više prodavnica/magacina.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Istorijska kalkulacija i nalog ne zavise od naknadne promjene veze magacina.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z369"/>
   <sheetData>
@@ -10411,86 +10536,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Nalozi / Bruto bilans</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Ispravljeno</v>
-      </c>
-      <c r="C2" t="str">
-        <v>A4 landscape štampa sa osam eksplicitnih kolona, neprelomivim tabularnim iznosima, urednim prelomom naziva konta, ponovljenim zaglavljem i redovima koji se ne cijepaju preko stranice.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Bruto bilans više ne nasljeđuje sedmokolonske širine Bilansa stanja. Nema migracije baze; TypeScript, ESLint i diff provjera prolaze.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Nalozi / Kartica konta</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Dugme za štampu prenosi konto, partnera i period na čistu A4 landscape karticu sa početnim saldom, POSTED prometom, tekućim saldom i ukupnim zbirom.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Ruta provjerava agenciju, dodjelu firme, poslovnu godinu, konto i scope partnera. Nema migracije baze; TypeScript i ESLint prolaze.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Završni račun / Kontrole</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Read-only kontrolni centar prikazuje ukupni status i provjere glavne knjige, KIF/KUF-a, dokumenata, izvoda, plata, PDV-a, šablona, rezultatskih konta, klasa 5/6, korekcija, arhive i matičnih podataka. Izvorna PDV konta moraju imati saldo 0,00; klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>XML/export završnog računa ostaje otvoren; po potrebi proširiti dodatnim zakonskim kontrolama.</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Svako sporno konto vodi direktno na svoju karticu. Prijavljena ruta vraća HTTP 200; nema migracije baze.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z310"/>
   <sheetData>
@@ -11054,7 +11100,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z342"/>
   <sheetData>
@@ -11163,13 +11209,13 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F7" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G7" t="str">
         <v>F-007,F-008</v>
       </c>
       <c r="H7" t="str">
-        <v>Matrica prava postoji; enforcement prava treba dodatno zakljucati.</v>
+        <v>Matrica ima pregled, unos, izmjenu, brisanje, knjiženje, storniranje, izvoz i administraciju; pravo pregleda određuje prikaz glavnog menija po aktivnoj firmi.</v>
       </c>
     </row>
     <row r="8">
@@ -11475,13 +11521,13 @@
         <v>Vrlo visok</v>
       </c>
       <c r="F19" t="str">
-        <v>Nije poceto</v>
+        <v>Implementirano</v>
       </c>
       <c r="G19" t="str">
         <v>F-038</v>
       </c>
       <c r="H19" t="str">
-        <v>Bruto bilans jos nije implementiran.</v>
+        <v>Dostupan u Nalozima i centralnim Izvještajima preko iste serverske komponente; ima filtere, nivoe zbira, drill-down na karticu konta i A4 štampu.</v>
       </c>
     </row>
     <row r="20">
@@ -12609,7 +12655,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z349"/>
   <sheetData>
@@ -12732,10 +12778,10 @@
         <v>Korisnici i prava</v>
       </c>
       <c r="F8" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G8" t="str">
-        <v>Prava su implementirana kao korisnik_prava po modulu/akciji.</v>
+        <v>Prava su implementirana kao korisnik_prava po modulu i akcijama view/create/update/delete/post/cancel/export/manage.</v>
       </c>
     </row>
     <row r="9">
@@ -12758,7 +12804,7 @@
         <v>Implementirano</v>
       </c>
       <c r="G9" t="str">
-        <v>Dodijeljena prava postoje kroz korisnik_prava.</v>
+        <v>Dodijeljena prava postoje isključivo kroz korisnik_prava; korisnik_firma čuva samo dodjelu, vrstu pristupa, glavnog radnika i period važenja.</v>
       </c>
     </row>
     <row r="10">
@@ -14460,7 +14506,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z351"/>
   <sheetData>
@@ -14734,7 +14780,7 @@
         <v>Korisnici i prava</v>
       </c>
       <c r="F13" t="str">
-        <v>Implementirano djelimicno</v>
+        <v>Implementirano</v>
       </c>
       <c r="G13" t="str">
         <v>F-008</v>
@@ -14743,7 +14789,7 @@
         <v>Djelimicno</v>
       </c>
       <c r="I13" t="str">
-        <v>Matrica prava se cuva; enforcement treba dodatno zakljucati.</v>
+        <v>Matrica je jedini izvor prava i upravlja glavnim menijem; audit backend provjera preostalih poslovnih ruta ostaje zaseban stabilizacioni zadatak.</v>
       </c>
     </row>
     <row r="14">
@@ -17246,7 +17292,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB357"/>
   <sheetData>
@@ -17819,10 +17865,16 @@
         <v>F-030,R-038</v>
       </c>
       <c r="F26" t="str">
-        <v>Nije poceto</v>
+        <v>Djelimicno testirano</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Codex</v>
+      </c>
+      <c r="H26">
+        <v>46270.083333333336</v>
       </c>
       <c r="I26" t="str">
-        <v>Detaljna prava za reopen jos nisu implementirana.</v>
+        <v>Server action provjerava pravo nalozi:update; potreban je jos integracioni test sa radnikom bez tog prava.</v>
       </c>
     </row>
     <row r="27">
@@ -19333,7 +19385,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -19383,7 +19435,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z308"/>
   <sheetData>
@@ -19820,7 +19872,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z321"/>
   <sheetData>
@@ -20592,7 +20644,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Z300"/>
   <sheetData>
@@ -20783,6 +20835,85 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Modul</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Otvoreno</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Napomena</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Nalozi / Bruto bilans</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Ispravljeno</v>
+      </c>
+      <c r="C2" t="str">
+        <v>A4 landscape štampa sa osam eksplicitnih kolona, neprelomivim tabularnim iznosima, urednim prelomom naziva konta, ponovljenim zaglavljem i redovima koji se ne cijepaju preko stranice.</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Bruto bilans više ne nasljeđuje sedmokolonske širine Bilansa stanja. Nema migracije baze; TypeScript, ESLint i diff provjera prolaze.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Nalozi / Kartica konta</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dugme za štampu prenosi konto, partnera i period na čistu A4 landscape karticu sa početnim saldom, POSTED prometom, tekućim saldom i ukupnim zbirom.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ručni pregled sistemskog print dijaloga po potrebi.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Ruta provjerava agenciju, dodjelu firme, poslovnu godinu, konto i scope partnera. Nema migracije baze; TypeScript i ESLint prolaze.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Završni račun / Kontrole</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Implementirano</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Read-only kontrolni centar prikazuje ukupni status i provjere glavne knjige, KIF/KUF-a, dokumenata, izvoda, plata, PDV-a, šablona, rezultatskih konta, klasa 5/6, korekcija, arhive i matičnih podataka. Izvorna PDV konta moraju imati saldo 0,00; klasa 5 dugovni/nulti, a klasa 6 potražni/nulti saldo.</v>
+      </c>
+      <c r="D4" t="str">
+        <v>XML/export završnog računa ostaje otvoren; po potrebi proširiti dodatnim zakonskim kontrolama.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Svako sporno konto vodi direktno na svoju karticu. Prijavljena ruta vraća HTTP 200; nema migracije baze.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
@@ -20843,7 +20974,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -20888,7 +21019,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
   <sheetData>
@@ -20984,7 +21115,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetData>
@@ -21025,68 +21156,6 @@
   </sheetData>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Modul</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Implementirano</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Otvoreno</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Napomena</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>M-012 Portal direktnog fiskalnog klijenta</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Specifikacija spremna</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Dogovoren je poseban mobile-first /portal sa automatskim kontekstom jedne firme, operativnim dashboardom, POS-om, klasičnim bezgotovinskim fakturama, jedinstvenim pregledom fiskalnih računa, izvještajima, artiklima, kupcima i ograničenim podešavanjima.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Implementirati sigurnosni portal guard i zabranu /agencija pristupa, zatim dashboard, oba prodajna toka, izvještaje i šifarnike prema DIRECT_FISCAL_CLIENT_PORTAL_SPEC.md.</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Fiskalna konfiguracija, sertifikati, ENU, operateri, aktivacija i suspenzija ostaju isključivo platformskom adminu; direct FISCAL_ONLY dokumenti ne kreiraju KIF ni nalog.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Dokumentacija i planer</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Usklađeno</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Dodata detaljna implementaciona specifikacija i ažurirani fiskalni README, POS specifikacija, CURRENT_STATE, NEXT_STEPS, SESSION_LOG i arhitektura.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Aplikacijski kod, Prisma šema i migracije nijesu mijenjani.</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Status označava dogovoreni plan, ne završenu funkcionalnost.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -21114,36 +21183,36 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>M-004 Robno</v>
+        <v>M-012 Portal direktnog fiskalnog klijenta</v>
       </c>
       <c r="B2" t="str">
-        <v>Djelimično implementirano</v>
+        <v>Specifikacija spremna</v>
       </c>
       <c r="C2" t="str">
-        <v>Summa izlazna faktura povezana je sa Fiscal API-jem. Jedno dugme automatski koristi Test ili Production, stabilan idempotency ključ i čuva zvanični broj, IKOF, JIKR i QR URL. Poslije fiskalizacije sadržaj je zaključan, a knjiženje se može dovršiti odvojeno.</v>
+        <v>Dogovoren je poseban mobile-first /portal sa automatskim kontekstom jedne firme, operativnim dashboardom, POS-om, klasičnim bezgotovinskim fakturama, jedinstvenim pregledom fiskalnih računa, izvještajima, artiklima, kupcima i ograničenim podešavanjima.</v>
       </c>
       <c r="D2" t="str">
-        <v>Ručni end-to-end QA u Test okruženju i kontrolisana produkcijska provjera.</v>
+        <v>Implementirati sigurnosni portal guard i zabranu /agencija pristupa, zatim dashboard, oba prodajna toka, izvještaje i šifarnike prema DIRECT_FISCAL_CLIENT_PORTAL_SPEC.md.</v>
       </c>
       <c r="E2" t="str">
-        <v>Fiskalni račun se ne šalje iz razvojne provjere; korisnik eksplicitno pokreće slanje dugmetom Fiskalizuj.</v>
+        <v>Fiskalna konfiguracija, sertifikati, ENU, operateri, aktivacija i suspenzija ostaju isključivo platformskom adminu; direct FISCAL_ONLY dokumenti ne kreiraju KIF ni nalog.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>M-011 POS / Kasa</v>
+        <v>Dokumentacija i planer</v>
       </c>
       <c r="B3" t="str">
-        <v>Prva funkcionalna faza</v>
+        <v>Usklađeno</v>
       </c>
       <c r="C3" t="str">
-        <v>Mobile-first POS, povezivanje kase sa Fiscal API objektom/ENU-om/operatorom, zajednički artikli i cijene, korpa, kupac, gotovina/kartica/virman, atomarna numeracija, retry, fiskalni rezultat, pregled, štampa i atomsko razduženje lagera sa podesivim pravilom minusa.</v>
+        <v>Dodata detaljna implementaciona specifikacija i ažurirani fiskalni README, POS specifikacija, CURRENT_STATE, NEXT_STEPS, SESSION_LOG i arhitektura.</v>
       </c>
       <c r="D3" t="str">
-        <v>Mobile QA, zbirni KIF/knjiženje, dnevni promet, povrati, smjene i POS Agent.</v>
+        <v>Aplikacijski kod, Prisma šema i migracije nijesu mijenjani.</v>
       </c>
       <c r="E3" t="str">
-        <v>Koristi FiskalniIzlazniRacun; direktni klijent može dobiti samo POS prava.</v>
+        <v>Status označava dogovoreni plan, ne završenu funkcionalnost.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>